<commit_message>
modified:   Ferrite Transformer Calculation.xlsx 	modified:   README.md 	deleted:    hardware/XF-1.0/XF-1.0-backups/XF-1.0-2025-07-15_095716.zip 	new file:   hardware/XF-1.0/XF-1.0-backups/XF-1.0-2025-07-15_145509.zip 	new file:   hardware/XF-1.0/XF-1.0-backups/XF-1.0-2025-07-15_150114.zip 	new file:   hardware/XF-1.0/XF-1.0-backups/XF-1.0-2025-07-15_150614.zip 	new file:   hardware/XF-1.0/XF-1.0-backups/XF-1.0-2025-07-15_151503.zip 	new file:   hardware/XF-1.0/XF-1.0-backups/XF-1.0-2025-07-15_152320.zip 	new file:   hardware/XF-1.0/XF-1.0-backups/XF-1.0-2025-07-15_154638.zip 	modified:   hardware/XF-1.0/XF-1.0.kicad_pcb 	modified:   hardware/XF-1.0/XF-1.0.kicad_prl 	modified:   hardware/XF-1.0/XF-1.0.kicad_pro 	modified:   hardware/XF-1.0/XF-1.0.kicad_sch 	modified:   hardware/XF-1.0/_autosave-XF-1.0.kicad_sch 	modified:   hardware/XF-1.0/fp-info-cache
</commit_message>
<xml_diff>
--- a/Ferrite Transformer Calculation.xlsx
+++ b/Ferrite Transformer Calculation.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="27660" windowHeight="12960" activeTab="2"/>
+    <workbookView windowWidth="28800" windowHeight="12960" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="ETD" sheetId="1" r:id="rId1"/>
@@ -1043,6 +1043,13 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
       <t>R</t>
     </r>
     <r>
@@ -1062,6 +1069,13 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
       <t>R</t>
     </r>
     <r>
@@ -1154,7 +1168,7 @@
         <charset val="134"/>
         <scheme val="minor"/>
       </rPr>
-      <t xml:space="preserve"> √2</t>
+      <t xml:space="preserve"> √2 / 2πf</t>
     </r>
   </si>
   <si>
@@ -1165,6 +1179,13 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
       <t>C</t>
     </r>
     <r>
@@ -1218,6 +1239,13 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
       <t>C</t>
     </r>
     <r>
@@ -1271,6 +1299,13 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
       <t>L</t>
     </r>
     <r>
@@ -1287,6 +1322,13 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
       <t>C</t>
     </r>
     <r>
@@ -1303,6 +1345,13 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
       <t>C</t>
     </r>
     <r>
@@ -1340,6 +1389,13 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
       <t>Q = R</t>
     </r>
     <r>
@@ -1387,6 +1443,13 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
       <t>f₀ = 1/(2π√LC</t>
     </r>
     <r>
@@ -1413,6 +1476,13 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
       <t>⍵</t>
     </r>
     <r>
@@ -1505,7 +1575,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
-  <numFmts count="14">
+  <numFmts count="16">
     <numFmt numFmtId="41" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;_);_(@_)"/>
     <numFmt numFmtId="42" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
     <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
@@ -1514,12 +1584,14 @@
     <numFmt numFmtId="178" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="179" formatCode="_ * #,##0.0000_ ;_ * \-#,##0.0000_ ;_ * &quot;-&quot;??.0000_ ;_ @_ "/>
     <numFmt numFmtId="180" formatCode="0.0000_ "/>
-    <numFmt numFmtId="181" formatCode="_ * #,##0.0_ ;_ * \-#,##0.0_ ;_ * &quot;-&quot;??.0_ ;_ @_ "/>
-    <numFmt numFmtId="182" formatCode="_ * #,##0.000_ ;_ * \-#,##0.000_ ;_ * &quot;-&quot;??.000_ ;_ @_ "/>
-    <numFmt numFmtId="183" formatCode="_ * #,##0.00000000_ ;_ * \-#,##0.00000000_ ;_ * &quot;-&quot;??.00000000_ ;_ @_ "/>
-    <numFmt numFmtId="184" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??.00_ ;_ @_ "/>
-    <numFmt numFmtId="185" formatCode="_(* #,##0.0000_);_(* \(#,##0.0000\);_(* &quot;-&quot;_);_(@_)"/>
-    <numFmt numFmtId="186" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;_);_(@_)"/>
+    <numFmt numFmtId="181" formatCode="_ * #,##0.0000000_ ;_ * \-#,##0.0000000_ ;_ * &quot;-&quot;??.0000000_ ;_ @_ "/>
+    <numFmt numFmtId="182" formatCode="_ * #,##0.0_ ;_ * \-#,##0.0_ ;_ * &quot;-&quot;??.0_ ;_ @_ "/>
+    <numFmt numFmtId="183" formatCode="_ * #,##0.000000000000_ ;_ * \-#,##0.000000000000_ ;_ * &quot;-&quot;??.000000000000_ ;_ @_ "/>
+    <numFmt numFmtId="184" formatCode="_ * #,##0.000_ ;_ * \-#,##0.000_ ;_ * &quot;-&quot;??.000_ ;_ @_ "/>
+    <numFmt numFmtId="185" formatCode="_ * #,##0.00000000_ ;_ * \-#,##0.00000000_ ;_ * &quot;-&quot;??.00000000_ ;_ @_ "/>
+    <numFmt numFmtId="186" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??.00_ ;_ @_ "/>
+    <numFmt numFmtId="187" formatCode="_(* #,##0.0000_);_(* \(#,##0.0000\);_(* &quot;-&quot;_);_(@_)"/>
+    <numFmt numFmtId="188" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;_);_(@_)"/>
   </numFmts>
   <fonts count="31">
     <font>
@@ -1701,6 +1773,13 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <b/>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial Bold"/>
+      <charset val="134"/>
+    </font>
+    <font>
       <vertAlign val="subscript"/>
       <sz val="10"/>
       <color theme="1"/>
@@ -1716,19 +1795,10 @@
       <charset val="134"/>
     </font>
     <font>
-      <b/>
       <vertAlign val="superscript"/>
       <sz val="10"/>
       <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="10"/>
-      <color theme="1"/>
-      <name val="Arial Bold"/>
+      <name val="Arial"/>
       <charset val="134"/>
     </font>
     <font>
@@ -1740,11 +1810,13 @@
       <charset val="134"/>
     </font>
     <font>
+      <b/>
       <vertAlign val="superscript"/>
       <sz val="10"/>
       <color theme="1"/>
-      <name val="Arial"/>
+      <name val="Calibri"/>
       <charset val="134"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <vertAlign val="superscript"/>
@@ -2205,7 +2277,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -2218,9 +2290,6 @@
     <xf numFmtId="10" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
@@ -2236,13 +2305,13 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="179" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="180" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="181" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="178" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -2251,31 +2320,31 @@
     <xf numFmtId="178" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="181" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1">
+    <xf numFmtId="182" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="183" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="179" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="182" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="183" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="184" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="185" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="186" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -2296,16 +2365,16 @@
     <xf numFmtId="41" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="185" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1">
+    <xf numFmtId="187" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="41" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="185" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="187" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="186" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1">
+    <xf numFmtId="188" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="180" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1">
@@ -2950,6 +3019,11 @@
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
     <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext uri="{0b15fc19-7d7d-44ad-8c2d-2c3a37ce22c3}">
+        <chartProps xmlns="https://web.wps.cn/et/2018/main" chartId="{7a78da87-5feb-4af1-b1e6-2ebcd56edc5b}"/>
+      </c:ext>
+    </c:extLst>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -3824,471 +3898,471 @@
   <dimension ref="A1:U33"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="5.5625" style="27" customWidth="1"/>
-    <col min="2" max="4" width="10.5625" style="27" customWidth="1"/>
-    <col min="5" max="5" width="20.5625" style="27" customWidth="1"/>
-    <col min="6" max="6" width="15.5625" style="27" customWidth="1"/>
-    <col min="7" max="7" width="30.5625" style="29" customWidth="1"/>
-    <col min="8" max="8" width="10.5625" style="27" customWidth="1"/>
-    <col min="9" max="9" width="15.5625" style="5" customWidth="1"/>
-    <col min="10" max="13" width="10.5625" style="5" customWidth="1"/>
-    <col min="14" max="14" width="9" style="5"/>
-    <col min="15" max="15" width="20.5625" style="5" customWidth="1"/>
-    <col min="16" max="17" width="10.5625" style="5" customWidth="1"/>
-    <col min="18" max="16384" width="9" style="5"/>
+    <col min="1" max="1" width="5.5625" style="26" customWidth="1"/>
+    <col min="2" max="4" width="10.5625" style="26" customWidth="1"/>
+    <col min="5" max="5" width="20.5625" style="26" customWidth="1"/>
+    <col min="6" max="6" width="15.5625" style="26" customWidth="1"/>
+    <col min="7" max="7" width="30.5625" style="28" customWidth="1"/>
+    <col min="8" max="8" width="10.5625" style="26" customWidth="1"/>
+    <col min="9" max="9" width="15.5625" style="4" customWidth="1"/>
+    <col min="10" max="13" width="10.5625" style="4" customWidth="1"/>
+    <col min="14" max="14" width="9" style="4"/>
+    <col min="15" max="15" width="20.5625" style="4" customWidth="1"/>
+    <col min="16" max="17" width="10.5625" style="4" customWidth="1"/>
+    <col min="18" max="16384" width="9" style="4"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8">
-      <c r="A1" s="5"/>
-      <c r="B1" s="5"/>
-      <c r="C1" s="5"/>
-      <c r="D1" s="5"/>
-      <c r="E1" s="5"/>
-      <c r="F1" s="5"/>
-      <c r="G1" s="24"/>
-      <c r="H1" s="5"/>
-    </row>
-    <row r="2" s="28" customFormat="1" ht="18" spans="1:21">
-      <c r="A2" s="24" t="s">
+      <c r="A1" s="4"/>
+      <c r="B1" s="4"/>
+      <c r="C1" s="4"/>
+      <c r="D1" s="4"/>
+      <c r="E1" s="4"/>
+      <c r="F1" s="4"/>
+      <c r="G1" s="23"/>
+      <c r="H1" s="4"/>
+    </row>
+    <row r="2" s="27" customFormat="1" ht="18" spans="1:21">
+      <c r="A2" s="23" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="25" t="s">
+      <c r="B2" s="24" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="25" t="s">
+      <c r="C2" s="24" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="25" t="s">
+      <c r="D2" s="24" t="s">
         <v>3</v>
       </c>
-      <c r="E2" s="25" t="s">
+      <c r="E2" s="24" t="s">
         <v>4</v>
       </c>
-      <c r="F2" s="25" t="s">
+      <c r="F2" s="24" t="s">
         <v>5</v>
       </c>
-      <c r="G2" s="24" t="s">
+      <c r="G2" s="23" t="s">
         <v>6</v>
       </c>
-      <c r="H2" s="25" t="s">
+      <c r="H2" s="24" t="s">
         <v>7</v>
       </c>
-      <c r="I2" s="24" t="s">
+      <c r="I2" s="23" t="s">
         <v>8</v>
       </c>
-      <c r="J2" s="24" t="s">
+      <c r="J2" s="23" t="s">
         <v>9</v>
       </c>
-      <c r="K2" s="24" t="s">
+      <c r="K2" s="23" t="s">
         <v>10</v>
       </c>
-      <c r="L2" s="24" t="s">
+      <c r="L2" s="23" t="s">
         <v>11</v>
       </c>
-      <c r="M2" s="24" t="s">
+      <c r="M2" s="23" t="s">
         <v>12</v>
       </c>
-      <c r="N2" s="24" t="s">
+      <c r="N2" s="23" t="s">
         <v>13</v>
       </c>
-      <c r="O2" s="24" t="s">
+      <c r="O2" s="23" t="s">
         <v>14</v>
       </c>
-      <c r="P2" s="24" t="s">
+      <c r="P2" s="23" t="s">
         <v>15</v>
       </c>
-      <c r="Q2" s="24" t="s">
+      <c r="Q2" s="23" t="s">
         <v>16</v>
       </c>
-      <c r="R2" s="24" t="s">
+      <c r="R2" s="23" t="s">
         <v>17</v>
       </c>
-      <c r="S2" s="24" t="s">
+      <c r="S2" s="23" t="s">
         <v>18</v>
       </c>
-      <c r="T2" s="24" t="s">
+      <c r="T2" s="23" t="s">
         <v>17</v>
       </c>
-      <c r="U2" s="24" t="s">
+      <c r="U2" s="23" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="3" spans="1:21">
-      <c r="A3" s="26">
+      <c r="A3" s="25">
         <v>1</v>
       </c>
-      <c r="B3" s="26">
+      <c r="B3" s="25">
         <v>72</v>
       </c>
-      <c r="C3" s="26">
+      <c r="C3" s="25">
         <v>400000</v>
       </c>
-      <c r="D3" s="26">
+      <c r="D3" s="25">
         <v>10</v>
       </c>
-      <c r="E3" s="30">
+      <c r="E3" s="29">
         <f>3.14*POWER(D3,2)/4</f>
         <v>78.5</v>
       </c>
-      <c r="F3" s="30">
+      <c r="F3" s="29">
         <v>1898.58</v>
       </c>
-      <c r="G3" s="31">
+      <c r="G3" s="30">
         <f>(B3*POWER(10,10))/(4*C3*F3*E3)</f>
         <v>3.01935345175506</v>
       </c>
-      <c r="H3" s="32" t="str">
+      <c r="H3" s="31" t="str">
         <f>IF((B3*POWER(10,10))/(4*C3*G3*E3)&gt;1200,IF((B3*POWER(10,10))/(4*C3*G3*E3)&lt;2000,"OK","NG"),"NG")</f>
         <v>OK</v>
       </c>
-      <c r="I3" s="27">
+      <c r="I3" s="26">
         <f>B3/G3</f>
         <v>23.8461648</v>
       </c>
-      <c r="J3" s="27">
+      <c r="J3" s="26">
         <f>B3*3</f>
         <v>216</v>
       </c>
-      <c r="K3" s="33">
+      <c r="K3" s="32">
         <v>0.5</v>
       </c>
-      <c r="L3" s="27">
+      <c r="L3" s="26">
         <f>J3*K3</f>
         <v>108</v>
       </c>
-      <c r="M3" s="33">
+      <c r="M3" s="32">
         <f>L3/B3</f>
         <v>1.5</v>
       </c>
-      <c r="N3" s="27">
+      <c r="N3" s="26">
         <f>J3/I3</f>
         <v>9.05806035526518</v>
       </c>
-      <c r="O3" s="27">
+      <c r="O3" s="26">
         <v>1.5</v>
       </c>
-      <c r="P3" s="34">
+      <c r="P3" s="33">
         <f>SQRT((M3*0.9/(O3+5))/0.9)</f>
         <v>0.480384461415261</v>
       </c>
-      <c r="Q3" s="34">
+      <c r="Q3" s="33">
         <f>SQRT((K3*0.9/(O3+5))/0.9)</f>
         <v>0.277350098112615</v>
       </c>
-      <c r="R3" s="5">
+      <c r="R3" s="4">
         <v>1</v>
       </c>
-      <c r="S3" s="5">
+      <c r="S3" s="4">
         <v>1</v>
       </c>
-      <c r="T3" s="5">
+      <c r="T3" s="4">
         <f>IF(((M3*0.9/(O3+5)))/(R3*R3*1)&lt;1,1,((M3*0.9/(O3+5))/(R3*R3*1)))</f>
         <v>1</v>
       </c>
-      <c r="U3" s="5">
+      <c r="U3" s="4">
         <f>IF(((K3*0.9/(O3+5)))/(S3*S3*1)&lt;1,1,((K3*0.9/(O3+5))/(S3*S3*1)))</f>
         <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:8">
-      <c r="A4" s="26"/>
-      <c r="B4" s="26"/>
-      <c r="C4" s="26"/>
-      <c r="D4" s="26"/>
-      <c r="E4" s="26"/>
-      <c r="F4" s="26"/>
-      <c r="G4" s="31"/>
-      <c r="H4" s="26"/>
+      <c r="A4" s="25"/>
+      <c r="B4" s="25"/>
+      <c r="C4" s="25"/>
+      <c r="D4" s="25"/>
+      <c r="E4" s="25"/>
+      <c r="F4" s="25"/>
+      <c r="G4" s="30"/>
+      <c r="H4" s="25"/>
     </row>
     <row r="5" spans="1:8">
-      <c r="A5" s="26"/>
-      <c r="B5" s="26"/>
-      <c r="C5" s="26"/>
-      <c r="D5" s="26"/>
-      <c r="E5" s="26"/>
-      <c r="F5" s="26"/>
-      <c r="G5" s="31"/>
-      <c r="H5" s="26"/>
+      <c r="A5" s="25"/>
+      <c r="B5" s="25"/>
+      <c r="C5" s="25"/>
+      <c r="D5" s="25"/>
+      <c r="E5" s="25"/>
+      <c r="F5" s="25"/>
+      <c r="G5" s="30"/>
+      <c r="H5" s="25"/>
     </row>
     <row r="6" spans="1:8">
-      <c r="A6" s="26"/>
-      <c r="B6" s="26"/>
-      <c r="C6" s="26"/>
-      <c r="D6" s="26"/>
-      <c r="E6" s="26"/>
-      <c r="F6" s="26"/>
-      <c r="G6" s="31"/>
-      <c r="H6" s="26"/>
+      <c r="A6" s="25"/>
+      <c r="B6" s="25"/>
+      <c r="C6" s="25"/>
+      <c r="D6" s="25"/>
+      <c r="E6" s="25"/>
+      <c r="F6" s="25"/>
+      <c r="G6" s="30"/>
+      <c r="H6" s="25"/>
     </row>
     <row r="7" spans="1:8">
-      <c r="A7" s="26"/>
-      <c r="B7" s="26"/>
-      <c r="C7" s="26"/>
-      <c r="D7" s="26"/>
-      <c r="E7" s="26"/>
-      <c r="F7" s="26"/>
-      <c r="G7" s="31"/>
-      <c r="H7" s="26"/>
+      <c r="A7" s="25"/>
+      <c r="B7" s="25"/>
+      <c r="C7" s="25"/>
+      <c r="D7" s="25"/>
+      <c r="E7" s="25"/>
+      <c r="F7" s="25"/>
+      <c r="G7" s="30"/>
+      <c r="H7" s="25"/>
     </row>
     <row r="8" spans="1:8">
-      <c r="A8" s="26"/>
-      <c r="B8" s="26"/>
-      <c r="C8" s="26"/>
-      <c r="D8" s="26"/>
-      <c r="E8" s="26"/>
-      <c r="F8" s="26"/>
-      <c r="G8" s="31"/>
-      <c r="H8" s="26"/>
+      <c r="A8" s="25"/>
+      <c r="B8" s="25"/>
+      <c r="C8" s="25"/>
+      <c r="D8" s="25"/>
+      <c r="E8" s="25"/>
+      <c r="F8" s="25"/>
+      <c r="G8" s="30"/>
+      <c r="H8" s="25"/>
     </row>
     <row r="9" spans="1:8">
-      <c r="A9" s="26"/>
-      <c r="B9" s="26"/>
-      <c r="C9" s="26"/>
-      <c r="D9" s="26"/>
-      <c r="E9" s="26"/>
-      <c r="F9" s="26"/>
-      <c r="G9" s="31"/>
-      <c r="H9" s="26"/>
+      <c r="A9" s="25"/>
+      <c r="B9" s="25"/>
+      <c r="C9" s="25"/>
+      <c r="D9" s="25"/>
+      <c r="E9" s="25"/>
+      <c r="F9" s="25"/>
+      <c r="G9" s="30"/>
+      <c r="H9" s="25"/>
     </row>
     <row r="10" spans="1:8">
-      <c r="A10" s="26"/>
-      <c r="B10" s="26"/>
-      <c r="C10" s="26"/>
-      <c r="D10" s="26"/>
-      <c r="E10" s="26"/>
-      <c r="F10" s="26"/>
-      <c r="G10" s="31"/>
-      <c r="H10" s="26"/>
+      <c r="A10" s="25"/>
+      <c r="B10" s="25"/>
+      <c r="C10" s="25"/>
+      <c r="D10" s="25"/>
+      <c r="E10" s="25"/>
+      <c r="F10" s="25"/>
+      <c r="G10" s="30"/>
+      <c r="H10" s="25"/>
     </row>
     <row r="11" spans="1:8">
-      <c r="A11" s="26"/>
-      <c r="B11" s="26"/>
-      <c r="C11" s="26"/>
-      <c r="D11" s="26"/>
-      <c r="E11" s="26"/>
-      <c r="F11" s="26"/>
-      <c r="G11" s="31"/>
-      <c r="H11" s="26"/>
+      <c r="A11" s="25"/>
+      <c r="B11" s="25"/>
+      <c r="C11" s="25"/>
+      <c r="D11" s="25"/>
+      <c r="E11" s="25"/>
+      <c r="F11" s="25"/>
+      <c r="G11" s="30"/>
+      <c r="H11" s="25"/>
     </row>
     <row r="12" spans="1:8">
-      <c r="A12" s="26"/>
-      <c r="B12" s="26"/>
-      <c r="C12" s="26"/>
-      <c r="D12" s="26"/>
-      <c r="E12" s="26"/>
-      <c r="F12" s="26"/>
-      <c r="G12" s="31"/>
-      <c r="H12" s="26"/>
+      <c r="A12" s="25"/>
+      <c r="B12" s="25"/>
+      <c r="C12" s="25"/>
+      <c r="D12" s="25"/>
+      <c r="E12" s="25"/>
+      <c r="F12" s="25"/>
+      <c r="G12" s="30"/>
+      <c r="H12" s="25"/>
     </row>
     <row r="13" spans="1:8">
-      <c r="A13" s="26"/>
-      <c r="B13" s="26"/>
-      <c r="C13" s="26"/>
-      <c r="D13" s="26"/>
-      <c r="E13" s="26"/>
-      <c r="F13" s="26"/>
-      <c r="G13" s="31"/>
-      <c r="H13" s="26"/>
+      <c r="A13" s="25"/>
+      <c r="B13" s="25"/>
+      <c r="C13" s="25"/>
+      <c r="D13" s="25"/>
+      <c r="E13" s="25"/>
+      <c r="F13" s="25"/>
+      <c r="G13" s="30"/>
+      <c r="H13" s="25"/>
     </row>
     <row r="14" spans="1:8">
-      <c r="A14" s="26"/>
-      <c r="B14" s="26"/>
-      <c r="C14" s="26"/>
-      <c r="D14" s="26"/>
-      <c r="E14" s="26"/>
-      <c r="F14" s="26"/>
-      <c r="G14" s="31"/>
-      <c r="H14" s="26"/>
+      <c r="A14" s="25"/>
+      <c r="B14" s="25"/>
+      <c r="C14" s="25"/>
+      <c r="D14" s="25"/>
+      <c r="E14" s="25"/>
+      <c r="F14" s="25"/>
+      <c r="G14" s="30"/>
+      <c r="H14" s="25"/>
     </row>
     <row r="15" spans="1:8">
-      <c r="A15" s="26"/>
-      <c r="B15" s="26"/>
-      <c r="C15" s="26"/>
-      <c r="D15" s="26"/>
-      <c r="E15" s="26"/>
-      <c r="F15" s="26"/>
-      <c r="G15" s="31"/>
-      <c r="H15" s="26"/>
+      <c r="A15" s="25"/>
+      <c r="B15" s="25"/>
+      <c r="C15" s="25"/>
+      <c r="D15" s="25"/>
+      <c r="E15" s="25"/>
+      <c r="F15" s="25"/>
+      <c r="G15" s="30"/>
+      <c r="H15" s="25"/>
     </row>
     <row r="16" spans="1:8">
-      <c r="A16" s="26"/>
-      <c r="B16" s="26"/>
-      <c r="C16" s="26"/>
-      <c r="D16" s="26"/>
-      <c r="E16" s="26"/>
-      <c r="F16" s="26"/>
-      <c r="G16" s="31"/>
-      <c r="H16" s="26"/>
+      <c r="A16" s="25"/>
+      <c r="B16" s="25"/>
+      <c r="C16" s="25"/>
+      <c r="D16" s="25"/>
+      <c r="E16" s="25"/>
+      <c r="F16" s="25"/>
+      <c r="G16" s="30"/>
+      <c r="H16" s="25"/>
     </row>
     <row r="17" spans="1:8">
-      <c r="A17" s="26"/>
-      <c r="B17" s="26"/>
-      <c r="C17" s="26"/>
-      <c r="D17" s="26"/>
-      <c r="E17" s="26"/>
-      <c r="F17" s="26"/>
-      <c r="G17" s="31"/>
-      <c r="H17" s="26"/>
+      <c r="A17" s="25"/>
+      <c r="B17" s="25"/>
+      <c r="C17" s="25"/>
+      <c r="D17" s="25"/>
+      <c r="E17" s="25"/>
+      <c r="F17" s="25"/>
+      <c r="G17" s="30"/>
+      <c r="H17" s="25"/>
     </row>
     <row r="18" spans="1:8">
-      <c r="A18" s="26"/>
-      <c r="B18" s="26"/>
-      <c r="C18" s="26"/>
-      <c r="D18" s="26"/>
-      <c r="E18" s="26"/>
-      <c r="F18" s="26"/>
-      <c r="G18" s="31"/>
-      <c r="H18" s="26"/>
+      <c r="A18" s="25"/>
+      <c r="B18" s="25"/>
+      <c r="C18" s="25"/>
+      <c r="D18" s="25"/>
+      <c r="E18" s="25"/>
+      <c r="F18" s="25"/>
+      <c r="G18" s="30"/>
+      <c r="H18" s="25"/>
     </row>
     <row r="19" spans="1:8">
-      <c r="A19" s="26"/>
-      <c r="B19" s="26"/>
-      <c r="C19" s="26"/>
-      <c r="D19" s="26"/>
-      <c r="E19" s="26"/>
-      <c r="F19" s="26"/>
-      <c r="G19" s="31"/>
-      <c r="H19" s="26"/>
+      <c r="A19" s="25"/>
+      <c r="B19" s="25"/>
+      <c r="C19" s="25"/>
+      <c r="D19" s="25"/>
+      <c r="E19" s="25"/>
+      <c r="F19" s="25"/>
+      <c r="G19" s="30"/>
+      <c r="H19" s="25"/>
     </row>
     <row r="20" spans="1:8">
-      <c r="A20" s="26"/>
-      <c r="B20" s="26"/>
-      <c r="C20" s="26"/>
-      <c r="D20" s="26"/>
-      <c r="E20" s="26"/>
-      <c r="F20" s="26"/>
-      <c r="G20" s="31"/>
-      <c r="H20" s="26"/>
+      <c r="A20" s="25"/>
+      <c r="B20" s="25"/>
+      <c r="C20" s="25"/>
+      <c r="D20" s="25"/>
+      <c r="E20" s="25"/>
+      <c r="F20" s="25"/>
+      <c r="G20" s="30"/>
+      <c r="H20" s="25"/>
     </row>
     <row r="21" spans="1:8">
-      <c r="A21" s="26"/>
-      <c r="B21" s="26"/>
-      <c r="C21" s="26"/>
-      <c r="D21" s="26"/>
-      <c r="E21" s="26"/>
-      <c r="F21" s="26"/>
-      <c r="G21" s="31"/>
-      <c r="H21" s="26"/>
+      <c r="A21" s="25"/>
+      <c r="B21" s="25"/>
+      <c r="C21" s="25"/>
+      <c r="D21" s="25"/>
+      <c r="E21" s="25"/>
+      <c r="F21" s="25"/>
+      <c r="G21" s="30"/>
+      <c r="H21" s="25"/>
     </row>
     <row r="22" spans="1:8">
-      <c r="A22" s="26"/>
-      <c r="B22" s="26"/>
-      <c r="C22" s="26"/>
-      <c r="D22" s="26"/>
-      <c r="E22" s="26"/>
-      <c r="F22" s="26"/>
-      <c r="G22" s="31"/>
-      <c r="H22" s="26"/>
+      <c r="A22" s="25"/>
+      <c r="B22" s="25"/>
+      <c r="C22" s="25"/>
+      <c r="D22" s="25"/>
+      <c r="E22" s="25"/>
+      <c r="F22" s="25"/>
+      <c r="G22" s="30"/>
+      <c r="H22" s="25"/>
     </row>
     <row r="23" spans="1:8">
-      <c r="A23" s="26"/>
-      <c r="B23" s="26"/>
-      <c r="C23" s="26"/>
-      <c r="D23" s="26"/>
-      <c r="E23" s="26"/>
-      <c r="F23" s="26"/>
-      <c r="G23" s="31"/>
-      <c r="H23" s="26"/>
+      <c r="A23" s="25"/>
+      <c r="B23" s="25"/>
+      <c r="C23" s="25"/>
+      <c r="D23" s="25"/>
+      <c r="E23" s="25"/>
+      <c r="F23" s="25"/>
+      <c r="G23" s="30"/>
+      <c r="H23" s="25"/>
     </row>
     <row r="24" spans="1:8">
-      <c r="A24" s="26"/>
-      <c r="B24" s="26"/>
-      <c r="C24" s="26"/>
-      <c r="D24" s="26"/>
-      <c r="E24" s="26"/>
-      <c r="F24" s="26"/>
-      <c r="G24" s="31"/>
-      <c r="H24" s="26"/>
+      <c r="A24" s="25"/>
+      <c r="B24" s="25"/>
+      <c r="C24" s="25"/>
+      <c r="D24" s="25"/>
+      <c r="E24" s="25"/>
+      <c r="F24" s="25"/>
+      <c r="G24" s="30"/>
+      <c r="H24" s="25"/>
     </row>
     <row r="25" spans="1:8">
-      <c r="A25" s="26"/>
-      <c r="B25" s="26"/>
-      <c r="C25" s="26"/>
-      <c r="D25" s="26"/>
-      <c r="E25" s="26"/>
-      <c r="F25" s="26"/>
-      <c r="G25" s="31"/>
-      <c r="H25" s="26"/>
+      <c r="A25" s="25"/>
+      <c r="B25" s="25"/>
+      <c r="C25" s="25"/>
+      <c r="D25" s="25"/>
+      <c r="E25" s="25"/>
+      <c r="F25" s="25"/>
+      <c r="G25" s="30"/>
+      <c r="H25" s="25"/>
     </row>
     <row r="26" spans="1:8">
-      <c r="A26" s="26"/>
-      <c r="B26" s="26"/>
-      <c r="C26" s="26"/>
-      <c r="D26" s="26"/>
-      <c r="E26" s="26"/>
-      <c r="F26" s="26"/>
-      <c r="G26" s="31"/>
-      <c r="H26" s="26"/>
+      <c r="A26" s="25"/>
+      <c r="B26" s="25"/>
+      <c r="C26" s="25"/>
+      <c r="D26" s="25"/>
+      <c r="E26" s="25"/>
+      <c r="F26" s="25"/>
+      <c r="G26" s="30"/>
+      <c r="H26" s="25"/>
     </row>
     <row r="27" spans="1:8">
-      <c r="A27" s="26"/>
-      <c r="B27" s="26"/>
-      <c r="C27" s="26"/>
-      <c r="D27" s="26"/>
-      <c r="E27" s="26"/>
-      <c r="F27" s="26"/>
-      <c r="G27" s="31"/>
-      <c r="H27" s="26"/>
+      <c r="A27" s="25"/>
+      <c r="B27" s="25"/>
+      <c r="C27" s="25"/>
+      <c r="D27" s="25"/>
+      <c r="E27" s="25"/>
+      <c r="F27" s="25"/>
+      <c r="G27" s="30"/>
+      <c r="H27" s="25"/>
     </row>
     <row r="28" spans="1:8">
-      <c r="A28" s="26"/>
-      <c r="B28" s="26"/>
-      <c r="C28" s="26"/>
-      <c r="D28" s="26"/>
-      <c r="E28" s="26"/>
-      <c r="F28" s="26"/>
-      <c r="G28" s="31"/>
-      <c r="H28" s="26"/>
+      <c r="A28" s="25"/>
+      <c r="B28" s="25"/>
+      <c r="C28" s="25"/>
+      <c r="D28" s="25"/>
+      <c r="E28" s="25"/>
+      <c r="F28" s="25"/>
+      <c r="G28" s="30"/>
+      <c r="H28" s="25"/>
     </row>
     <row r="29" spans="1:8">
-      <c r="A29" s="26"/>
-      <c r="B29" s="26"/>
-      <c r="C29" s="26"/>
-      <c r="D29" s="26"/>
-      <c r="E29" s="26"/>
-      <c r="F29" s="26"/>
-      <c r="G29" s="31"/>
-      <c r="H29" s="26"/>
+      <c r="A29" s="25"/>
+      <c r="B29" s="25"/>
+      <c r="C29" s="25"/>
+      <c r="D29" s="25"/>
+      <c r="E29" s="25"/>
+      <c r="F29" s="25"/>
+      <c r="G29" s="30"/>
+      <c r="H29" s="25"/>
     </row>
     <row r="30" spans="1:8">
-      <c r="A30" s="26"/>
-      <c r="B30" s="26"/>
-      <c r="C30" s="26"/>
-      <c r="D30" s="26"/>
-      <c r="E30" s="26"/>
-      <c r="F30" s="26"/>
-      <c r="G30" s="31"/>
-      <c r="H30" s="26"/>
+      <c r="A30" s="25"/>
+      <c r="B30" s="25"/>
+      <c r="C30" s="25"/>
+      <c r="D30" s="25"/>
+      <c r="E30" s="25"/>
+      <c r="F30" s="25"/>
+      <c r="G30" s="30"/>
+      <c r="H30" s="25"/>
     </row>
     <row r="31" spans="1:8">
-      <c r="A31" s="26"/>
-      <c r="B31" s="26"/>
-      <c r="C31" s="26"/>
-      <c r="D31" s="26"/>
-      <c r="E31" s="26"/>
-      <c r="F31" s="26"/>
-      <c r="G31" s="31"/>
-      <c r="H31" s="26"/>
+      <c r="A31" s="25"/>
+      <c r="B31" s="25"/>
+      <c r="C31" s="25"/>
+      <c r="D31" s="25"/>
+      <c r="E31" s="25"/>
+      <c r="F31" s="25"/>
+      <c r="G31" s="30"/>
+      <c r="H31" s="25"/>
     </row>
     <row r="32" spans="1:8">
-      <c r="A32" s="26"/>
-      <c r="B32" s="26"/>
-      <c r="C32" s="26"/>
-      <c r="D32" s="26"/>
-      <c r="E32" s="26"/>
-      <c r="F32" s="26"/>
-      <c r="G32" s="31"/>
-      <c r="H32" s="26"/>
+      <c r="A32" s="25"/>
+      <c r="B32" s="25"/>
+      <c r="C32" s="25"/>
+      <c r="D32" s="25"/>
+      <c r="E32" s="25"/>
+      <c r="F32" s="25"/>
+      <c r="G32" s="30"/>
+      <c r="H32" s="25"/>
     </row>
     <row r="33" spans="1:8">
-      <c r="A33" s="26"/>
-      <c r="B33" s="26"/>
-      <c r="C33" s="26"/>
-      <c r="D33" s="26"/>
-      <c r="E33" s="26"/>
-      <c r="F33" s="26"/>
-      <c r="G33" s="31"/>
-      <c r="H33" s="26"/>
+      <c r="A33" s="25"/>
+      <c r="B33" s="25"/>
+      <c r="C33" s="25"/>
+      <c r="D33" s="25"/>
+      <c r="E33" s="25"/>
+      <c r="F33" s="25"/>
+      <c r="G33" s="30"/>
+      <c r="H33" s="25"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4302,237 +4376,237 @@
   <dimension ref="A2:T6"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4" outlineLevelRow="5"/>
   <cols>
-    <col min="1" max="1" width="5.5625" style="5" customWidth="1"/>
-    <col min="2" max="7" width="10.5625" style="5" customWidth="1"/>
-    <col min="8" max="8" width="20.5625" style="5" customWidth="1"/>
-    <col min="9" max="9" width="15.5625" style="5" customWidth="1"/>
-    <col min="10" max="10" width="30.5625" style="5" customWidth="1"/>
-    <col min="11" max="11" width="9" style="5"/>
-    <col min="12" max="12" width="15.5625" style="5" customWidth="1"/>
-    <col min="13" max="16" width="10.5625" style="5" customWidth="1"/>
-    <col min="17" max="17" width="9" style="5"/>
-    <col min="18" max="18" width="20.5625" style="5" customWidth="1"/>
-    <col min="19" max="20" width="10.5625" style="5" customWidth="1"/>
-    <col min="21" max="16384" width="9" style="5"/>
+    <col min="1" max="1" width="5.5625" style="4" customWidth="1"/>
+    <col min="2" max="7" width="10.5625" style="4" customWidth="1"/>
+    <col min="8" max="8" width="20.5625" style="4" customWidth="1"/>
+    <col min="9" max="9" width="15.5625" style="4" customWidth="1"/>
+    <col min="10" max="10" width="30.5625" style="4" customWidth="1"/>
+    <col min="11" max="11" width="9" style="4"/>
+    <col min="12" max="12" width="15.5625" style="4" customWidth="1"/>
+    <col min="13" max="16" width="10.5625" style="4" customWidth="1"/>
+    <col min="17" max="17" width="9" style="4"/>
+    <col min="18" max="18" width="20.5625" style="4" customWidth="1"/>
+    <col min="19" max="20" width="10.5625" style="4" customWidth="1"/>
+    <col min="21" max="16384" width="9" style="4"/>
   </cols>
   <sheetData>
     <row r="2" ht="18" spans="1:20">
-      <c r="A2" s="24" t="s">
+      <c r="A2" s="23" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="25" t="s">
+      <c r="B2" s="24" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="25" t="s">
+      <c r="C2" s="24" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="25"/>
-      <c r="E2" s="25" t="s">
+      <c r="D2" s="24"/>
+      <c r="E2" s="24" t="s">
         <v>19</v>
       </c>
-      <c r="F2" s="25" t="s">
+      <c r="F2" s="24" t="s">
         <v>20</v>
       </c>
-      <c r="G2" s="25" t="s">
+      <c r="G2" s="24" t="s">
         <v>21</v>
       </c>
-      <c r="H2" s="25" t="s">
+      <c r="H2" s="24" t="s">
         <v>22</v>
       </c>
-      <c r="I2" s="25" t="s">
+      <c r="I2" s="24" t="s">
         <v>5</v>
       </c>
-      <c r="J2" s="24" t="s">
+      <c r="J2" s="23" t="s">
         <v>23</v>
       </c>
-      <c r="L2" s="24" t="s">
+      <c r="L2" s="23" t="s">
         <v>8</v>
       </c>
-      <c r="M2" s="24" t="s">
+      <c r="M2" s="23" t="s">
         <v>9</v>
       </c>
-      <c r="N2" s="24" t="s">
+      <c r="N2" s="23" t="s">
         <v>10</v>
       </c>
-      <c r="O2" s="24" t="s">
+      <c r="O2" s="23" t="s">
         <v>11</v>
       </c>
-      <c r="P2" s="24" t="s">
+      <c r="P2" s="23" t="s">
         <v>12</v>
       </c>
-      <c r="Q2" s="24" t="s">
+      <c r="Q2" s="23" t="s">
         <v>13</v>
       </c>
-      <c r="R2" s="24" t="s">
+      <c r="R2" s="23" t="s">
         <v>14</v>
       </c>
-      <c r="S2" s="24" t="s">
+      <c r="S2" s="23" t="s">
         <v>15</v>
       </c>
-      <c r="T2" s="24" t="s">
+      <c r="T2" s="23" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="3" spans="1:17">
-      <c r="A3" s="26">
+      <c r="A3" s="25">
         <v>1</v>
       </c>
-      <c r="B3" s="26">
+      <c r="B3" s="25">
         <v>72</v>
       </c>
-      <c r="C3" s="26">
+      <c r="C3" s="25">
         <v>400000</v>
       </c>
-      <c r="D3" s="26" t="s">
+      <c r="D3" s="25" t="s">
         <v>24</v>
       </c>
-      <c r="E3" s="5">
+      <c r="E3" s="4">
         <v>25</v>
       </c>
-      <c r="F3" s="5">
+      <c r="F3" s="4">
         <v>40</v>
       </c>
-      <c r="G3" s="5">
+      <c r="G3" s="4">
         <v>15</v>
       </c>
-      <c r="H3" s="5">
+      <c r="H3" s="4">
         <f t="shared" ref="H3:H6" si="0">(F3-E3)*G3/2</f>
         <v>112.5</v>
       </c>
-      <c r="I3" s="5">
+      <c r="I3" s="4">
         <v>1800</v>
       </c>
-      <c r="J3" s="5">
+      <c r="J3" s="4">
         <f t="shared" ref="J3:J6" si="1">(B3*0.5*POWER(10,10))/(2*C3*I3*H3)</f>
         <v>2.22222222222222</v>
       </c>
-      <c r="L3" s="27">
+      <c r="L3" s="26">
         <f t="shared" ref="L3:L6" si="2">B3/J3</f>
         <v>32.4</v>
       </c>
-      <c r="M3" s="5">
+      <c r="M3" s="4">
         <v>216</v>
       </c>
-      <c r="Q3" s="27">
+      <c r="Q3" s="26">
         <f t="shared" ref="Q3:Q6" si="3">M3/L3</f>
         <v>6.66666666666667</v>
       </c>
     </row>
     <row r="4" spans="2:17">
-      <c r="B4" s="26">
+      <c r="B4" s="25">
         <v>72</v>
       </c>
-      <c r="C4" s="26">
+      <c r="C4" s="25">
         <v>400000</v>
       </c>
-      <c r="D4" s="26"/>
-      <c r="E4" s="5">
+      <c r="D4" s="25"/>
+      <c r="E4" s="4">
         <v>23.13</v>
       </c>
-      <c r="F4" s="5">
+      <c r="F4" s="4">
         <v>39.88</v>
       </c>
-      <c r="G4" s="5">
+      <c r="G4" s="4">
         <v>14.48</v>
       </c>
-      <c r="H4" s="5">
+      <c r="H4" s="4">
         <f t="shared" si="0"/>
         <v>121.27</v>
       </c>
-      <c r="I4" s="5">
+      <c r="I4" s="4">
         <v>600</v>
       </c>
-      <c r="J4" s="5">
+      <c r="J4" s="4">
         <f t="shared" si="1"/>
         <v>6.18454687886534</v>
       </c>
-      <c r="L4" s="27">
+      <c r="L4" s="26">
         <f t="shared" si="2"/>
         <v>11.64192</v>
       </c>
-      <c r="M4" s="5">
+      <c r="M4" s="4">
         <v>216</v>
       </c>
-      <c r="Q4" s="27">
+      <c r="Q4" s="26">
         <f t="shared" si="3"/>
         <v>18.553640636596</v>
       </c>
     </row>
     <row r="5" spans="2:17">
-      <c r="B5" s="26">
+      <c r="B5" s="25">
         <v>72</v>
       </c>
-      <c r="C5" s="26">
+      <c r="C5" s="25">
         <v>400000</v>
       </c>
-      <c r="D5" s="26"/>
-      <c r="E5" s="5">
+      <c r="D5" s="25"/>
+      <c r="E5" s="4">
         <v>23.13</v>
       </c>
-      <c r="F5" s="5">
+      <c r="F5" s="4">
         <v>39.88</v>
       </c>
-      <c r="G5" s="5">
+      <c r="G5" s="4">
         <v>14.48</v>
       </c>
-      <c r="H5" s="5">
+      <c r="H5" s="4">
         <f t="shared" si="0"/>
         <v>121.27</v>
       </c>
-      <c r="I5" s="5">
+      <c r="I5" s="4">
         <v>350</v>
       </c>
-      <c r="J5" s="5">
+      <c r="J5" s="4">
         <f t="shared" si="1"/>
         <v>10.6020803637692</v>
       </c>
-      <c r="L5" s="27">
+      <c r="L5" s="26">
         <f t="shared" si="2"/>
         <v>6.79112</v>
       </c>
-      <c r="M5" s="5">
+      <c r="M5" s="4">
         <v>216</v>
       </c>
-      <c r="Q5" s="27">
+      <c r="Q5" s="26">
         <f t="shared" si="3"/>
         <v>31.8062410913075</v>
       </c>
     </row>
     <row r="6" spans="2:17">
-      <c r="B6" s="26">
+      <c r="B6" s="25">
         <v>72</v>
       </c>
-      <c r="C6" s="26">
+      <c r="C6" s="25">
         <v>400000</v>
       </c>
-      <c r="E6" s="5">
+      <c r="E6" s="4">
         <v>23.3</v>
       </c>
-      <c r="F6" s="5">
+      <c r="F6" s="4">
         <v>40.4</v>
       </c>
-      <c r="G6" s="5">
+      <c r="G6" s="4">
         <v>15.1</v>
       </c>
-      <c r="H6" s="5">
+      <c r="H6" s="4">
         <f t="shared" si="0"/>
         <v>129.105</v>
       </c>
-      <c r="I6" s="5">
+      <c r="I6" s="4">
         <v>350</v>
       </c>
-      <c r="J6" s="5">
+      <c r="J6" s="4">
         <f t="shared" si="1"/>
         <v>9.95867151322014</v>
       </c>
-      <c r="L6" s="27">
+      <c r="L6" s="26">
         <f t="shared" si="2"/>
         <v>7.22988</v>
       </c>
-      <c r="M6" s="5">
+      <c r="M6" s="4">
         <v>216</v>
       </c>
-      <c r="Q6" s="27">
+      <c r="Q6" s="26">
         <f t="shared" si="3"/>
         <v>29.8760145396604</v>
       </c>
@@ -4549,906 +4623,925 @@
   <dimension ref="B3:Y38"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="5.5625" style="5" customWidth="1"/>
-    <col min="2" max="2" width="15.5625" style="6" customWidth="1"/>
-    <col min="3" max="3" width="15.5625" style="5" customWidth="1"/>
-    <col min="4" max="4" width="5.5625" style="5" customWidth="1"/>
-    <col min="5" max="12" width="18.5625" style="5" customWidth="1"/>
-    <col min="13" max="13" width="5.2265625" style="5" customWidth="1"/>
-    <col min="14" max="14" width="25.4375" style="5" customWidth="1"/>
-    <col min="15" max="17" width="5.5625" style="5" customWidth="1"/>
-    <col min="18" max="18" width="15.5625" style="5" customWidth="1"/>
-    <col min="19" max="20" width="9" style="5"/>
-    <col min="21" max="22" width="20.5625" style="5" customWidth="1"/>
-    <col min="23" max="23" width="9" style="5"/>
-    <col min="24" max="24" width="11.125" style="5"/>
-    <col min="25" max="16384" width="9" style="5"/>
+    <col min="1" max="1" width="5.5625" style="4" customWidth="1"/>
+    <col min="2" max="2" width="15.5625" style="5" customWidth="1"/>
+    <col min="3" max="3" width="15.5625" style="4" customWidth="1"/>
+    <col min="4" max="4" width="5.5625" style="4" customWidth="1"/>
+    <col min="5" max="12" width="18.5625" style="4" customWidth="1"/>
+    <col min="13" max="13" width="5.2265625" style="4" customWidth="1"/>
+    <col min="14" max="14" width="25.4375" style="4" customWidth="1"/>
+    <col min="15" max="17" width="5.5625" style="4" customWidth="1"/>
+    <col min="18" max="18" width="15.5625" style="4" customWidth="1"/>
+    <col min="19" max="20" width="9" style="4"/>
+    <col min="21" max="22" width="20.5625" style="4" customWidth="1"/>
+    <col min="23" max="23" width="9" style="4"/>
+    <col min="24" max="24" width="11.125" style="4"/>
+    <col min="25" max="16384" width="9" style="4"/>
   </cols>
   <sheetData>
     <row r="3" spans="2:4">
-      <c r="B3" s="7" t="s">
+      <c r="B3" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="C3" s="8">
+      <c r="C3" s="7">
         <v>400000</v>
       </c>
-      <c r="D3" s="8" t="s">
+      <c r="D3" s="7" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="4" customHeight="1" spans="2:4">
-      <c r="B4" s="7" t="s">
+      <c r="B4" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="C4" s="8">
+      <c r="C4" s="7">
         <v>100</v>
       </c>
-      <c r="D4" s="8" t="s">
+      <c r="D4" s="7" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="5" customHeight="1" spans="2:4">
-      <c r="B5" s="7" t="s">
+      <c r="B5" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="C5" s="8">
+      <c r="C5" s="7">
         <f>C4/2</f>
         <v>50</v>
       </c>
-      <c r="D5" s="8" t="s">
+      <c r="D5" s="7" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="6" customHeight="1" spans="2:4">
-      <c r="B6" s="7"/>
-      <c r="C6" s="8"/>
-      <c r="D6" s="8"/>
+      <c r="B6" s="6"/>
+      <c r="C6" s="7"/>
+      <c r="D6" s="7"/>
     </row>
     <row r="7" spans="2:4">
-      <c r="B7" s="9" t="s">
+      <c r="B7" s="8" t="s">
         <v>30</v>
       </c>
-      <c r="D7" s="8"/>
+      <c r="D7" s="7"/>
     </row>
     <row r="8" ht="18" spans="2:24">
-      <c r="B8" s="10" t="s">
+      <c r="B8" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="C8" s="11">
+      <c r="C8" s="9">
         <f>((C5*SQRT(2))/(2*3.14*C3))*1000000</f>
         <v>28.1491553020122</v>
       </c>
-      <c r="D8" s="8" t="s">
+      <c r="D8" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="M8" s="18"/>
-      <c r="N8" s="8" t="s">
+      <c r="F8" s="4">
+        <f>50*SQRT(2)</f>
+        <v>70.7106781186548</v>
+      </c>
+      <c r="G8" s="4">
+        <f>1/G9</f>
+        <v>5.62983106040245e-9</v>
+      </c>
+      <c r="M8" s="17"/>
+      <c r="N8" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="O8" s="21">
+      <c r="O8" s="20">
         <v>1.4</v>
       </c>
-      <c r="P8" s="8"/>
-      <c r="S8" s="8"/>
-      <c r="T8" s="18"/>
-      <c r="U8" s="18"/>
-      <c r="V8" s="8"/>
-      <c r="W8" s="8"/>
-      <c r="X8" s="8"/>
+      <c r="P8" s="7"/>
+      <c r="S8" s="7"/>
+      <c r="T8" s="17"/>
+      <c r="U8" s="17"/>
+      <c r="V8" s="7"/>
+      <c r="W8" s="7"/>
+      <c r="X8" s="7"/>
     </row>
     <row r="9" ht="18" spans="2:24">
-      <c r="B9" s="10" t="s">
+      <c r="B9" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="C9" s="12">
+      <c r="C9" s="10">
         <f>(1/(2*3.14*C3*C5*SQRT(2)))*1000000000</f>
         <v>5.62983106040245</v>
       </c>
-      <c r="D9" s="8" t="s">
+      <c r="D9" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="M9" s="16"/>
-      <c r="N9" s="8" t="s">
+      <c r="F9" s="4">
+        <f>2*3.14*400000</f>
+        <v>2512000</v>
+      </c>
+      <c r="G9" s="4">
+        <f>F8*F9</f>
+        <v>177625223.434061</v>
+      </c>
+      <c r="M9" s="15"/>
+      <c r="N9" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="O9" s="21">
+      <c r="O9" s="20">
         <v>0.707</v>
       </c>
-      <c r="P9" s="22"/>
-      <c r="S9" s="8"/>
-      <c r="T9" s="11"/>
-      <c r="U9" s="11"/>
-      <c r="V9" s="23"/>
-      <c r="W9" s="23"/>
-      <c r="X9" s="8"/>
+      <c r="P9" s="21"/>
+      <c r="S9" s="7"/>
+      <c r="T9" s="9"/>
+      <c r="U9" s="9"/>
+      <c r="V9" s="22"/>
+      <c r="W9" s="22"/>
+      <c r="X9" s="7"/>
     </row>
     <row r="10" ht="18" spans="2:24">
-      <c r="B10" s="7" t="s">
+      <c r="B10" s="6" t="s">
         <v>37</v>
       </c>
       <c r="C10" s="11">
         <f>C9/2</f>
         <v>2.81491553020122</v>
       </c>
-      <c r="D10" s="8" t="s">
+      <c r="D10" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="E10" s="16"/>
-      <c r="F10" s="8"/>
-      <c r="G10" s="8"/>
-      <c r="H10" s="8"/>
-      <c r="I10" s="8"/>
-      <c r="J10" s="11"/>
-      <c r="K10" s="11"/>
-      <c r="L10" s="16"/>
-      <c r="M10" s="16"/>
-      <c r="N10" s="8" t="s">
+      <c r="E10" s="15"/>
+      <c r="F10" s="16">
+        <f>F8/F9</f>
+        <v>2.81491553020122e-5</v>
+      </c>
+      <c r="G10" s="7"/>
+      <c r="H10" s="7"/>
+      <c r="I10" s="7"/>
+      <c r="J10" s="9"/>
+      <c r="K10" s="9"/>
+      <c r="L10" s="15"/>
+      <c r="M10" s="15"/>
+      <c r="N10" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="O10" s="21">
+      <c r="O10" s="20">
         <v>0.3</v>
       </c>
-      <c r="P10" s="8"/>
-      <c r="S10" s="8"/>
-      <c r="T10" s="8"/>
-      <c r="U10" s="8"/>
-      <c r="V10" s="8"/>
-      <c r="W10" s="8"/>
-      <c r="X10" s="8"/>
+      <c r="P10" s="7"/>
+      <c r="S10" s="7"/>
+      <c r="T10" s="7"/>
+      <c r="U10" s="7"/>
+      <c r="V10" s="7"/>
+      <c r="W10" s="7"/>
+      <c r="X10" s="7"/>
     </row>
     <row r="11" spans="2:24">
-      <c r="B11" s="13"/>
-      <c r="C11" s="8"/>
-      <c r="D11" s="8"/>
-      <c r="J11" s="11"/>
-      <c r="K11" s="11"/>
-      <c r="L11" s="16"/>
-      <c r="M11" s="16"/>
-      <c r="N11" s="8"/>
-      <c r="O11" s="8"/>
-      <c r="P11" s="8"/>
-      <c r="Q11" s="8"/>
-      <c r="R11" s="8"/>
-      <c r="S11" s="8"/>
-      <c r="T11" s="8"/>
-      <c r="U11" s="8"/>
-      <c r="V11" s="8"/>
-      <c r="W11" s="8"/>
-      <c r="X11" s="8"/>
+      <c r="B11" s="12"/>
+      <c r="C11" s="7"/>
+      <c r="D11" s="7"/>
+      <c r="J11" s="9"/>
+      <c r="K11" s="9"/>
+      <c r="L11" s="15"/>
+      <c r="M11" s="15"/>
+      <c r="N11" s="7"/>
+      <c r="O11" s="7"/>
+      <c r="P11" s="7"/>
+      <c r="Q11" s="7"/>
+      <c r="R11" s="7"/>
+      <c r="S11" s="7"/>
+      <c r="T11" s="7"/>
+      <c r="U11" s="7"/>
+      <c r="V11" s="7"/>
+      <c r="W11" s="7"/>
+      <c r="X11" s="7"/>
     </row>
     <row r="12" spans="2:24">
-      <c r="B12" s="9" t="s">
+      <c r="B12" s="8" t="s">
         <v>39</v>
       </c>
-      <c r="C12" s="14"/>
-      <c r="D12" s="8"/>
+      <c r="C12" s="13"/>
+      <c r="D12" s="7"/>
       <c r="E12" s="17"/>
       <c r="F12" s="17"/>
       <c r="G12" s="17"/>
       <c r="H12" s="17"/>
-      <c r="I12" s="18"/>
-      <c r="J12" s="19"/>
-      <c r="K12" s="19"/>
-      <c r="L12" s="20"/>
-      <c r="M12" s="20"/>
-      <c r="N12" s="8"/>
-      <c r="O12" s="8"/>
-      <c r="P12" s="8"/>
-      <c r="Q12" s="8"/>
-      <c r="R12" s="8"/>
-      <c r="S12" s="8"/>
-      <c r="T12" s="8"/>
-      <c r="U12" s="8"/>
-      <c r="V12" s="8"/>
-      <c r="W12" s="8"/>
-      <c r="X12" s="8"/>
+      <c r="I12" s="17"/>
+      <c r="J12" s="18"/>
+      <c r="K12" s="18"/>
+      <c r="L12" s="19"/>
+      <c r="M12" s="19"/>
+      <c r="N12" s="7"/>
+      <c r="O12" s="7"/>
+      <c r="P12" s="7"/>
+      <c r="Q12" s="7"/>
+      <c r="R12" s="7"/>
+      <c r="S12" s="7"/>
+      <c r="T12" s="7"/>
+      <c r="U12" s="7"/>
+      <c r="V12" s="7"/>
+      <c r="W12" s="7"/>
+      <c r="X12" s="7"/>
     </row>
     <row r="13" ht="18" spans="2:24">
-      <c r="B13" s="10" t="s">
+      <c r="B13" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="C13" s="8">
+      <c r="C13" s="7">
         <v>29</v>
       </c>
-      <c r="D13" s="8" t="s">
+      <c r="D13" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="J13" s="11"/>
-      <c r="K13" s="11"/>
-      <c r="L13" s="16"/>
-      <c r="M13" s="16"/>
-      <c r="N13" s="8"/>
-      <c r="O13" s="8"/>
-      <c r="P13" s="8"/>
-      <c r="Q13" s="8"/>
-      <c r="R13" s="8"/>
-      <c r="S13" s="8"/>
-      <c r="T13" s="8"/>
-      <c r="U13" s="8"/>
-      <c r="V13" s="8"/>
-      <c r="W13" s="8"/>
-      <c r="X13" s="8"/>
+      <c r="J13" s="9"/>
+      <c r="K13" s="9"/>
+      <c r="L13" s="15"/>
+      <c r="M13" s="15"/>
+      <c r="N13" s="7"/>
+      <c r="O13" s="7"/>
+      <c r="P13" s="7"/>
+      <c r="Q13" s="7"/>
+      <c r="R13" s="7"/>
+      <c r="S13" s="7"/>
+      <c r="T13" s="7"/>
+      <c r="U13" s="7"/>
+      <c r="V13" s="7"/>
+      <c r="W13" s="7"/>
+      <c r="X13" s="7"/>
     </row>
     <row r="14" ht="18" spans="2:24">
-      <c r="B14" s="7" t="s">
+      <c r="B14" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="C14" s="15">
+      <c r="C14" s="14">
         <v>2.7</v>
       </c>
-      <c r="D14" s="8" t="s">
+      <c r="D14" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="E14" s="16"/>
-      <c r="F14" s="8"/>
-      <c r="G14" s="8"/>
-      <c r="H14" s="8"/>
-      <c r="I14" s="8"/>
-      <c r="J14" s="11"/>
-      <c r="K14" s="11"/>
-      <c r="L14" s="16"/>
-      <c r="M14" s="16"/>
-      <c r="N14" s="8"/>
-      <c r="O14" s="8"/>
-      <c r="P14" s="8"/>
-      <c r="Q14" s="8"/>
-      <c r="R14" s="8"/>
-      <c r="S14" s="8"/>
-      <c r="T14" s="8"/>
-      <c r="U14" s="8"/>
-      <c r="V14" s="8"/>
-      <c r="W14" s="8"/>
-      <c r="X14" s="8"/>
+      <c r="E14" s="15"/>
+      <c r="F14" s="7"/>
+      <c r="G14" s="7"/>
+      <c r="H14" s="7"/>
+      <c r="I14" s="7"/>
+      <c r="J14" s="9"/>
+      <c r="K14" s="9"/>
+      <c r="L14" s="15"/>
+      <c r="M14" s="15"/>
+      <c r="N14" s="7"/>
+      <c r="O14" s="7"/>
+      <c r="P14" s="7"/>
+      <c r="Q14" s="7"/>
+      <c r="R14" s="7"/>
+      <c r="S14" s="7"/>
+      <c r="T14" s="7"/>
+      <c r="U14" s="7"/>
+      <c r="V14" s="7"/>
+      <c r="W14" s="7"/>
+      <c r="X14" s="7"/>
     </row>
     <row r="15" ht="18" spans="2:25">
-      <c r="B15" s="7" t="s">
+      <c r="B15" s="6" t="s">
         <v>42</v>
       </c>
-      <c r="C15" s="15">
+      <c r="C15" s="14">
         <f>2*C14</f>
         <v>5.4</v>
       </c>
-      <c r="D15" s="8" t="s">
+      <c r="D15" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="E15" s="8"/>
-      <c r="F15" s="16"/>
-      <c r="G15" s="16"/>
-      <c r="H15" s="16"/>
-      <c r="I15" s="16"/>
-      <c r="J15" s="8"/>
-      <c r="K15" s="11"/>
-      <c r="L15" s="11"/>
-      <c r="M15" s="11"/>
-      <c r="N15" s="11"/>
-      <c r="O15" s="8"/>
-      <c r="P15" s="8"/>
-      <c r="Q15" s="8"/>
-      <c r="R15" s="8"/>
-      <c r="S15" s="8"/>
-      <c r="T15" s="8"/>
-      <c r="U15" s="8"/>
-      <c r="V15" s="8"/>
-      <c r="W15" s="8"/>
-      <c r="X15" s="8"/>
-      <c r="Y15" s="8"/>
+      <c r="E15" s="7"/>
+      <c r="F15" s="15"/>
+      <c r="G15" s="15"/>
+      <c r="H15" s="15"/>
+      <c r="I15" s="15"/>
+      <c r="J15" s="7"/>
+      <c r="K15" s="9"/>
+      <c r="L15" s="9"/>
+      <c r="M15" s="9"/>
+      <c r="N15" s="9"/>
+      <c r="O15" s="7"/>
+      <c r="P15" s="7"/>
+      <c r="Q15" s="7"/>
+      <c r="R15" s="7"/>
+      <c r="S15" s="7"/>
+      <c r="T15" s="7"/>
+      <c r="U15" s="7"/>
+      <c r="V15" s="7"/>
+      <c r="W15" s="7"/>
+      <c r="X15" s="7"/>
+      <c r="Y15" s="7"/>
     </row>
     <row r="16" ht="18" spans="2:25">
-      <c r="B16" s="7" t="s">
+      <c r="B16" s="6" t="s">
         <v>43</v>
       </c>
-      <c r="C16" s="11">
+      <c r="C16" s="9">
         <f>C5*SQRT((C15/(POWER(10,9))/(C13/POWER(10,6))))</f>
         <v>0.682288239221013</v>
       </c>
-      <c r="D16" s="8"/>
-      <c r="E16" s="8"/>
-      <c r="F16" s="8"/>
-      <c r="G16" s="8"/>
-      <c r="H16" s="8"/>
-      <c r="I16" s="8"/>
-      <c r="J16" s="8"/>
-      <c r="K16" s="8"/>
-      <c r="L16" s="8"/>
-      <c r="M16" s="8"/>
-      <c r="N16" s="8"/>
-      <c r="O16" s="8"/>
-      <c r="P16" s="8"/>
-      <c r="Q16" s="8"/>
-      <c r="R16" s="8"/>
-      <c r="S16" s="8"/>
-      <c r="T16" s="8"/>
-      <c r="U16" s="8"/>
-      <c r="V16" s="8"/>
-      <c r="W16" s="8"/>
-      <c r="X16" s="8"/>
-      <c r="Y16" s="8"/>
+      <c r="D16" s="7"/>
+      <c r="E16" s="7"/>
+      <c r="F16" s="7"/>
+      <c r="G16" s="7"/>
+      <c r="H16" s="7"/>
+      <c r="I16" s="7"/>
+      <c r="J16" s="7"/>
+      <c r="K16" s="7"/>
+      <c r="L16" s="7"/>
+      <c r="M16" s="7"/>
+      <c r="N16" s="7"/>
+      <c r="O16" s="7"/>
+      <c r="P16" s="7"/>
+      <c r="Q16" s="7"/>
+      <c r="R16" s="7"/>
+      <c r="S16" s="7"/>
+      <c r="T16" s="7"/>
+      <c r="U16" s="7"/>
+      <c r="V16" s="7"/>
+      <c r="W16" s="7"/>
+      <c r="X16" s="7"/>
+      <c r="Y16" s="7"/>
     </row>
     <row r="17" ht="18" spans="2:25">
-      <c r="B17" s="7" t="s">
+      <c r="B17" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="C17" s="11">
+      <c r="C17" s="9">
         <f>1/(2*3.14*SQRT((C13/POWER(10,6))*(C15/POWER(10,9))))</f>
         <v>402387.496591775</v>
       </c>
-      <c r="D17" s="8" t="s">
+      <c r="D17" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="E17" s="8"/>
-      <c r="F17" s="8"/>
-      <c r="G17" s="8"/>
-      <c r="H17" s="8"/>
-      <c r="I17" s="8"/>
-      <c r="J17" s="8"/>
-      <c r="K17" s="8"/>
-      <c r="L17" s="8"/>
-      <c r="M17" s="8"/>
-      <c r="N17" s="8"/>
-      <c r="O17" s="8"/>
-      <c r="P17" s="8"/>
-      <c r="Q17" s="8"/>
-      <c r="R17" s="8"/>
-      <c r="S17" s="8"/>
-      <c r="T17" s="8"/>
-      <c r="U17" s="8"/>
-      <c r="V17" s="8"/>
-      <c r="W17" s="8"/>
-      <c r="X17" s="8"/>
-      <c r="Y17" s="8"/>
+      <c r="E17" s="7"/>
+      <c r="F17" s="7"/>
+      <c r="G17" s="7"/>
+      <c r="H17" s="7"/>
+      <c r="I17" s="7"/>
+      <c r="J17" s="7"/>
+      <c r="K17" s="7"/>
+      <c r="L17" s="7"/>
+      <c r="M17" s="7"/>
+      <c r="N17" s="7"/>
+      <c r="O17" s="7"/>
+      <c r="P17" s="7"/>
+      <c r="Q17" s="7"/>
+      <c r="R17" s="7"/>
+      <c r="S17" s="7"/>
+      <c r="T17" s="7"/>
+      <c r="U17" s="7"/>
+      <c r="V17" s="7"/>
+      <c r="W17" s="7"/>
+      <c r="X17" s="7"/>
+      <c r="Y17" s="7"/>
     </row>
     <row r="18" ht="18" spans="2:25">
-      <c r="B18" s="10" t="s">
+      <c r="B18" s="6" t="s">
         <v>45</v>
       </c>
-      <c r="C18" s="11">
+      <c r="C18" s="9">
         <f>20*LOG10(C16)</f>
         <v>-3.3206422940395</v>
       </c>
-      <c r="D18" s="8" t="s">
+      <c r="D18" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="E18" s="8"/>
-      <c r="F18" s="8"/>
-      <c r="G18" s="8"/>
-      <c r="H18" s="8"/>
-      <c r="I18" s="8"/>
-      <c r="J18" s="8"/>
-      <c r="K18" s="8"/>
-      <c r="L18" s="8"/>
-      <c r="M18" s="8"/>
-      <c r="N18" s="8"/>
-      <c r="O18" s="8"/>
-      <c r="P18" s="8"/>
-      <c r="Q18" s="8"/>
-      <c r="R18" s="8"/>
-      <c r="S18" s="8"/>
-      <c r="T18" s="8"/>
-      <c r="U18" s="8"/>
-      <c r="V18" s="8"/>
-      <c r="W18" s="8"/>
-      <c r="X18" s="8"/>
-      <c r="Y18" s="8"/>
+      <c r="E18" s="7"/>
+      <c r="F18" s="7"/>
+      <c r="G18" s="7"/>
+      <c r="H18" s="7"/>
+      <c r="I18" s="7"/>
+      <c r="J18" s="7"/>
+      <c r="K18" s="7"/>
+      <c r="L18" s="7"/>
+      <c r="M18" s="7"/>
+      <c r="N18" s="7"/>
+      <c r="O18" s="7"/>
+      <c r="P18" s="7"/>
+      <c r="Q18" s="7"/>
+      <c r="R18" s="7"/>
+      <c r="S18" s="7"/>
+      <c r="T18" s="7"/>
+      <c r="U18" s="7"/>
+      <c r="V18" s="7"/>
+      <c r="W18" s="7"/>
+      <c r="X18" s="7"/>
+      <c r="Y18" s="7"/>
     </row>
     <row r="19" spans="2:25">
-      <c r="B19" s="13"/>
-      <c r="C19" s="8"/>
-      <c r="D19" s="8"/>
-      <c r="E19" s="8"/>
-      <c r="F19" s="8"/>
-      <c r="G19" s="8"/>
-      <c r="H19" s="8"/>
-      <c r="I19" s="8"/>
-      <c r="J19" s="8"/>
-      <c r="K19" s="8"/>
-      <c r="L19" s="8"/>
-      <c r="M19" s="8"/>
-      <c r="N19" s="8"/>
-      <c r="O19" s="8"/>
-      <c r="P19" s="8"/>
-      <c r="Q19" s="8"/>
-      <c r="R19" s="8"/>
-      <c r="S19" s="8"/>
-      <c r="T19" s="8"/>
-      <c r="U19" s="8"/>
-      <c r="V19" s="8"/>
-      <c r="W19" s="8"/>
-      <c r="X19" s="8"/>
-      <c r="Y19" s="8"/>
+      <c r="B19" s="12"/>
+      <c r="C19" s="7"/>
+      <c r="D19" s="7"/>
+      <c r="E19" s="7"/>
+      <c r="F19" s="7"/>
+      <c r="G19" s="7"/>
+      <c r="H19" s="7"/>
+      <c r="I19" s="7"/>
+      <c r="J19" s="7"/>
+      <c r="K19" s="7"/>
+      <c r="L19" s="7"/>
+      <c r="M19" s="7"/>
+      <c r="N19" s="7"/>
+      <c r="O19" s="7"/>
+      <c r="P19" s="7"/>
+      <c r="Q19" s="7"/>
+      <c r="R19" s="7"/>
+      <c r="S19" s="7"/>
+      <c r="T19" s="7"/>
+      <c r="U19" s="7"/>
+      <c r="V19" s="7"/>
+      <c r="W19" s="7"/>
+      <c r="X19" s="7"/>
+      <c r="Y19" s="7"/>
     </row>
     <row r="20" spans="2:25">
-      <c r="B20" s="13"/>
-      <c r="C20" s="8"/>
-      <c r="D20" s="8"/>
-      <c r="E20" s="8"/>
-      <c r="F20" s="8"/>
-      <c r="G20" s="8"/>
-      <c r="H20" s="8"/>
-      <c r="I20" s="8"/>
-      <c r="J20" s="8"/>
-      <c r="K20" s="8"/>
-      <c r="L20" s="8"/>
-      <c r="M20" s="8"/>
-      <c r="N20" s="8"/>
-      <c r="O20" s="8"/>
-      <c r="P20" s="8"/>
-      <c r="Q20" s="8"/>
-      <c r="R20" s="8"/>
-      <c r="S20" s="8"/>
-      <c r="T20" s="8"/>
-      <c r="U20" s="8"/>
-      <c r="V20" s="8"/>
-      <c r="W20" s="8"/>
-      <c r="X20" s="8"/>
-      <c r="Y20" s="8"/>
+      <c r="B20" s="12"/>
+      <c r="C20" s="7"/>
+      <c r="D20" s="7"/>
+      <c r="E20" s="7"/>
+      <c r="F20" s="7"/>
+      <c r="G20" s="7"/>
+      <c r="H20" s="7"/>
+      <c r="I20" s="7"/>
+      <c r="J20" s="7"/>
+      <c r="K20" s="7"/>
+      <c r="L20" s="7"/>
+      <c r="M20" s="7"/>
+      <c r="N20" s="7"/>
+      <c r="O20" s="7"/>
+      <c r="P20" s="7"/>
+      <c r="Q20" s="7"/>
+      <c r="R20" s="7"/>
+      <c r="S20" s="7"/>
+      <c r="T20" s="7"/>
+      <c r="U20" s="7"/>
+      <c r="V20" s="7"/>
+      <c r="W20" s="7"/>
+      <c r="X20" s="7"/>
+      <c r="Y20" s="7"/>
     </row>
     <row r="21" spans="2:25">
-      <c r="B21" s="13"/>
-      <c r="C21" s="8"/>
-      <c r="D21" s="8"/>
-      <c r="E21" s="8"/>
-      <c r="F21" s="8"/>
-      <c r="G21" s="8"/>
-      <c r="H21" s="8"/>
-      <c r="I21" s="8"/>
-      <c r="J21" s="8"/>
-      <c r="K21" s="8"/>
-      <c r="L21" s="8"/>
-      <c r="M21" s="8"/>
-      <c r="N21" s="8"/>
-      <c r="O21" s="8"/>
-      <c r="P21" s="8"/>
-      <c r="Q21" s="8"/>
-      <c r="R21" s="8"/>
-      <c r="S21" s="8"/>
-      <c r="T21" s="8"/>
-      <c r="U21" s="8"/>
-      <c r="V21" s="8"/>
-      <c r="W21" s="8"/>
-      <c r="X21" s="8"/>
-      <c r="Y21" s="8"/>
+      <c r="B21" s="12"/>
+      <c r="C21" s="7"/>
+      <c r="D21" s="7"/>
+      <c r="E21" s="7"/>
+      <c r="F21" s="7"/>
+      <c r="G21" s="7"/>
+      <c r="H21" s="7"/>
+      <c r="I21" s="7"/>
+      <c r="J21" s="7"/>
+      <c r="K21" s="7"/>
+      <c r="L21" s="7"/>
+      <c r="M21" s="7"/>
+      <c r="N21" s="7"/>
+      <c r="O21" s="7"/>
+      <c r="P21" s="7"/>
+      <c r="Q21" s="7"/>
+      <c r="R21" s="7"/>
+      <c r="S21" s="7"/>
+      <c r="T21" s="7"/>
+      <c r="U21" s="7"/>
+      <c r="V21" s="7"/>
+      <c r="W21" s="7"/>
+      <c r="X21" s="7"/>
+      <c r="Y21" s="7"/>
     </row>
     <row r="22" spans="2:25">
-      <c r="B22" s="13"/>
-      <c r="C22" s="8"/>
-      <c r="D22" s="8"/>
-      <c r="E22" s="8"/>
-      <c r="F22" s="8"/>
-      <c r="G22" s="8"/>
-      <c r="H22" s="8"/>
-      <c r="I22" s="8"/>
-      <c r="J22" s="8"/>
-      <c r="K22" s="8"/>
-      <c r="L22" s="8"/>
-      <c r="M22" s="8"/>
-      <c r="N22" s="8"/>
-      <c r="O22" s="8"/>
-      <c r="P22" s="8"/>
-      <c r="Q22" s="8"/>
-      <c r="R22" s="8"/>
-      <c r="S22" s="8"/>
-      <c r="T22" s="8"/>
-      <c r="U22" s="8"/>
-      <c r="V22" s="8"/>
-      <c r="W22" s="8"/>
-      <c r="X22" s="8"/>
-      <c r="Y22" s="8"/>
+      <c r="B22" s="12"/>
+      <c r="C22" s="7"/>
+      <c r="D22" s="7"/>
+      <c r="E22" s="7"/>
+      <c r="F22" s="7"/>
+      <c r="G22" s="7"/>
+      <c r="H22" s="7"/>
+      <c r="I22" s="7"/>
+      <c r="J22" s="7"/>
+      <c r="K22" s="7"/>
+      <c r="L22" s="7"/>
+      <c r="M22" s="7"/>
+      <c r="N22" s="7"/>
+      <c r="O22" s="7"/>
+      <c r="P22" s="7"/>
+      <c r="Q22" s="7"/>
+      <c r="R22" s="7"/>
+      <c r="S22" s="7"/>
+      <c r="T22" s="7"/>
+      <c r="U22" s="7"/>
+      <c r="V22" s="7"/>
+      <c r="W22" s="7"/>
+      <c r="X22" s="7"/>
+      <c r="Y22" s="7"/>
     </row>
     <row r="23" spans="2:25">
-      <c r="B23" s="13"/>
-      <c r="C23" s="8"/>
-      <c r="D23" s="8"/>
-      <c r="E23" s="8"/>
-      <c r="F23" s="8"/>
-      <c r="G23" s="8"/>
-      <c r="H23" s="8"/>
-      <c r="I23" s="8"/>
-      <c r="J23" s="8"/>
-      <c r="K23" s="8"/>
-      <c r="L23" s="8"/>
-      <c r="M23" s="8"/>
-      <c r="N23" s="8"/>
-      <c r="O23" s="8"/>
-      <c r="P23" s="8"/>
-      <c r="Q23" s="8"/>
-      <c r="R23" s="8"/>
-      <c r="S23" s="8"/>
-      <c r="T23" s="8"/>
-      <c r="U23" s="8"/>
-      <c r="V23" s="8"/>
-      <c r="W23" s="8"/>
-      <c r="X23" s="8"/>
-      <c r="Y23" s="8"/>
+      <c r="B23" s="12"/>
+      <c r="C23" s="7"/>
+      <c r="D23" s="7"/>
+      <c r="E23" s="7"/>
+      <c r="F23" s="7"/>
+      <c r="G23" s="7"/>
+      <c r="H23" s="7"/>
+      <c r="I23" s="7"/>
+      <c r="J23" s="7"/>
+      <c r="K23" s="7"/>
+      <c r="L23" s="7"/>
+      <c r="M23" s="7"/>
+      <c r="N23" s="7"/>
+      <c r="O23" s="7"/>
+      <c r="P23" s="7"/>
+      <c r="Q23" s="7"/>
+      <c r="R23" s="7"/>
+      <c r="S23" s="7"/>
+      <c r="T23" s="7"/>
+      <c r="U23" s="7"/>
+      <c r="V23" s="7"/>
+      <c r="W23" s="7"/>
+      <c r="X23" s="7"/>
+      <c r="Y23" s="7"/>
     </row>
     <row r="24" spans="2:25">
-      <c r="B24" s="13"/>
-      <c r="C24" s="8"/>
-      <c r="D24" s="8"/>
-      <c r="E24" s="8"/>
-      <c r="F24" s="8"/>
-      <c r="G24" s="8"/>
-      <c r="H24" s="8"/>
-      <c r="I24" s="8"/>
-      <c r="J24" s="8"/>
-      <c r="K24" s="8"/>
-      <c r="L24" s="8"/>
-      <c r="M24" s="8"/>
-      <c r="N24" s="8"/>
-      <c r="O24" s="8"/>
-      <c r="P24" s="8"/>
-      <c r="Q24" s="8"/>
-      <c r="R24" s="8"/>
-      <c r="S24" s="8"/>
-      <c r="T24" s="8"/>
-      <c r="U24" s="8"/>
-      <c r="V24" s="8"/>
-      <c r="W24" s="8"/>
-      <c r="X24" s="8"/>
-      <c r="Y24" s="8"/>
+      <c r="B24" s="12"/>
+      <c r="C24" s="7"/>
+      <c r="D24" s="7"/>
+      <c r="E24" s="7"/>
+      <c r="F24" s="7"/>
+      <c r="G24" s="7"/>
+      <c r="H24" s="7"/>
+      <c r="I24" s="7"/>
+      <c r="J24" s="7"/>
+      <c r="K24" s="7"/>
+      <c r="L24" s="7"/>
+      <c r="M24" s="7"/>
+      <c r="N24" s="7"/>
+      <c r="O24" s="7"/>
+      <c r="P24" s="7"/>
+      <c r="Q24" s="7"/>
+      <c r="R24" s="7"/>
+      <c r="S24" s="7"/>
+      <c r="T24" s="7"/>
+      <c r="U24" s="7"/>
+      <c r="V24" s="7"/>
+      <c r="W24" s="7"/>
+      <c r="X24" s="7"/>
+      <c r="Y24" s="7"/>
     </row>
     <row r="25" spans="2:25">
-      <c r="B25" s="13"/>
-      <c r="C25" s="8"/>
-      <c r="D25" s="8"/>
-      <c r="E25" s="8"/>
-      <c r="F25" s="8"/>
-      <c r="G25" s="8"/>
-      <c r="H25" s="8"/>
-      <c r="I25" s="8"/>
-      <c r="J25" s="8"/>
-      <c r="K25" s="8"/>
-      <c r="L25" s="8"/>
-      <c r="M25" s="8"/>
-      <c r="N25" s="8"/>
-      <c r="O25" s="8"/>
-      <c r="P25" s="8"/>
-      <c r="Q25" s="8"/>
-      <c r="R25" s="8"/>
-      <c r="S25" s="8"/>
-      <c r="T25" s="8"/>
-      <c r="U25" s="8"/>
-      <c r="V25" s="8"/>
-      <c r="W25" s="8"/>
-      <c r="X25" s="8"/>
-      <c r="Y25" s="8"/>
+      <c r="B25" s="12"/>
+      <c r="C25" s="7"/>
+      <c r="D25" s="7"/>
+      <c r="E25" s="7"/>
+      <c r="F25" s="7"/>
+      <c r="G25" s="7"/>
+      <c r="H25" s="7"/>
+      <c r="I25" s="7"/>
+      <c r="J25" s="7"/>
+      <c r="K25" s="7"/>
+      <c r="L25" s="7"/>
+      <c r="M25" s="7"/>
+      <c r="N25" s="7"/>
+      <c r="O25" s="7"/>
+      <c r="P25" s="7"/>
+      <c r="Q25" s="7"/>
+      <c r="R25" s="7"/>
+      <c r="S25" s="7"/>
+      <c r="T25" s="7"/>
+      <c r="U25" s="7"/>
+      <c r="V25" s="7"/>
+      <c r="W25" s="7"/>
+      <c r="X25" s="7"/>
+      <c r="Y25" s="7"/>
     </row>
     <row r="26" spans="2:25">
-      <c r="B26" s="13"/>
-      <c r="C26" s="8"/>
-      <c r="D26" s="8"/>
-      <c r="E26" s="8"/>
-      <c r="F26" s="8"/>
-      <c r="G26" s="8"/>
-      <c r="H26" s="8"/>
-      <c r="I26" s="8"/>
-      <c r="J26" s="8"/>
-      <c r="K26" s="8"/>
-      <c r="L26" s="8"/>
-      <c r="M26" s="8"/>
-      <c r="N26" s="8"/>
-      <c r="O26" s="8"/>
-      <c r="P26" s="8"/>
-      <c r="Q26" s="8"/>
-      <c r="R26" s="8"/>
-      <c r="S26" s="8"/>
-      <c r="T26" s="8"/>
-      <c r="U26" s="8"/>
-      <c r="V26" s="8"/>
-      <c r="W26" s="8"/>
-      <c r="X26" s="8"/>
-      <c r="Y26" s="8"/>
+      <c r="B26" s="12"/>
+      <c r="C26" s="7"/>
+      <c r="D26" s="7"/>
+      <c r="E26" s="7"/>
+      <c r="F26" s="7"/>
+      <c r="G26" s="7"/>
+      <c r="H26" s="7"/>
+      <c r="I26" s="7"/>
+      <c r="J26" s="7"/>
+      <c r="K26" s="7"/>
+      <c r="L26" s="7"/>
+      <c r="M26" s="7"/>
+      <c r="N26" s="7"/>
+      <c r="O26" s="7"/>
+      <c r="P26" s="7"/>
+      <c r="Q26" s="7"/>
+      <c r="R26" s="7"/>
+      <c r="S26" s="7"/>
+      <c r="T26" s="7"/>
+      <c r="U26" s="7"/>
+      <c r="V26" s="7"/>
+      <c r="W26" s="7"/>
+      <c r="X26" s="7"/>
+      <c r="Y26" s="7"/>
     </row>
     <row r="27" spans="2:25">
-      <c r="B27" s="13"/>
-      <c r="C27" s="8"/>
-      <c r="D27" s="8"/>
-      <c r="E27" s="8"/>
-      <c r="F27" s="8"/>
-      <c r="G27" s="8"/>
-      <c r="H27" s="8"/>
-      <c r="I27" s="8"/>
-      <c r="J27" s="8"/>
-      <c r="K27" s="8"/>
-      <c r="L27" s="8"/>
-      <c r="M27" s="8"/>
-      <c r="N27" s="8"/>
-      <c r="O27" s="8"/>
-      <c r="P27" s="8"/>
-      <c r="Q27" s="8"/>
-      <c r="R27" s="8"/>
-      <c r="S27" s="8"/>
-      <c r="T27" s="8"/>
-      <c r="U27" s="8"/>
-      <c r="V27" s="8"/>
-      <c r="W27" s="8"/>
-      <c r="X27" s="8"/>
-      <c r="Y27" s="8"/>
+      <c r="B27" s="12"/>
+      <c r="C27" s="7"/>
+      <c r="D27" s="7"/>
+      <c r="E27" s="7"/>
+      <c r="F27" s="7"/>
+      <c r="G27" s="7"/>
+      <c r="H27" s="7"/>
+      <c r="I27" s="7"/>
+      <c r="J27" s="7"/>
+      <c r="K27" s="7"/>
+      <c r="L27" s="7"/>
+      <c r="M27" s="7"/>
+      <c r="N27" s="7"/>
+      <c r="O27" s="7"/>
+      <c r="P27" s="7"/>
+      <c r="Q27" s="7"/>
+      <c r="R27" s="7"/>
+      <c r="S27" s="7"/>
+      <c r="T27" s="7"/>
+      <c r="U27" s="7"/>
+      <c r="V27" s="7"/>
+      <c r="W27" s="7"/>
+      <c r="X27" s="7"/>
+      <c r="Y27" s="7"/>
     </row>
     <row r="28" spans="2:25">
-      <c r="B28" s="13"/>
-      <c r="C28" s="8"/>
-      <c r="D28" s="8"/>
-      <c r="E28" s="8"/>
-      <c r="F28" s="8"/>
-      <c r="G28" s="8"/>
-      <c r="H28" s="8"/>
-      <c r="I28" s="8"/>
-      <c r="J28" s="8"/>
-      <c r="K28" s="8"/>
-      <c r="L28" s="8"/>
-      <c r="M28" s="8"/>
-      <c r="N28" s="8"/>
-      <c r="O28" s="8"/>
-      <c r="P28" s="8"/>
-      <c r="Q28" s="8"/>
-      <c r="R28" s="8"/>
-      <c r="S28" s="8"/>
-      <c r="T28" s="8"/>
-      <c r="U28" s="8"/>
-      <c r="V28" s="8"/>
-      <c r="W28" s="8"/>
-      <c r="X28" s="8"/>
-      <c r="Y28" s="8"/>
+      <c r="B28" s="12"/>
+      <c r="C28" s="7"/>
+      <c r="D28" s="7"/>
+      <c r="E28" s="7"/>
+      <c r="F28" s="7"/>
+      <c r="G28" s="7"/>
+      <c r="H28" s="7"/>
+      <c r="I28" s="7"/>
+      <c r="J28" s="7"/>
+      <c r="K28" s="7"/>
+      <c r="L28" s="7"/>
+      <c r="M28" s="7"/>
+      <c r="N28" s="7"/>
+      <c r="O28" s="7"/>
+      <c r="P28" s="7"/>
+      <c r="Q28" s="7"/>
+      <c r="R28" s="7"/>
+      <c r="S28" s="7"/>
+      <c r="T28" s="7"/>
+      <c r="U28" s="7"/>
+      <c r="V28" s="7"/>
+      <c r="W28" s="7"/>
+      <c r="X28" s="7"/>
+      <c r="Y28" s="7"/>
     </row>
     <row r="29" spans="2:25">
-      <c r="B29" s="13"/>
-      <c r="C29" s="8"/>
-      <c r="D29" s="8"/>
-      <c r="E29" s="8"/>
-      <c r="F29" s="8"/>
-      <c r="G29" s="8"/>
-      <c r="H29" s="8"/>
-      <c r="I29" s="8"/>
-      <c r="J29" s="8"/>
-      <c r="K29" s="8"/>
-      <c r="L29" s="8"/>
-      <c r="M29" s="8"/>
-      <c r="N29" s="8"/>
-      <c r="O29" s="8"/>
-      <c r="P29" s="8"/>
-      <c r="Q29" s="8"/>
-      <c r="R29" s="8"/>
-      <c r="S29" s="8"/>
-      <c r="T29" s="8"/>
-      <c r="U29" s="8"/>
-      <c r="V29" s="8"/>
-      <c r="W29" s="8"/>
-      <c r="X29" s="8"/>
-      <c r="Y29" s="8"/>
+      <c r="B29" s="12"/>
+      <c r="C29" s="7"/>
+      <c r="D29" s="7"/>
+      <c r="E29" s="7"/>
+      <c r="F29" s="7"/>
+      <c r="G29" s="7"/>
+      <c r="H29" s="7"/>
+      <c r="I29" s="7"/>
+      <c r="J29" s="7"/>
+      <c r="K29" s="7"/>
+      <c r="L29" s="7"/>
+      <c r="M29" s="7"/>
+      <c r="N29" s="7"/>
+      <c r="O29" s="7"/>
+      <c r="P29" s="7"/>
+      <c r="Q29" s="7"/>
+      <c r="R29" s="7"/>
+      <c r="S29" s="7"/>
+      <c r="T29" s="7"/>
+      <c r="U29" s="7"/>
+      <c r="V29" s="7"/>
+      <c r="W29" s="7"/>
+      <c r="X29" s="7"/>
+      <c r="Y29" s="7"/>
     </row>
     <row r="30" spans="2:25">
-      <c r="B30" s="13"/>
-      <c r="C30" s="8"/>
-      <c r="D30" s="8"/>
-      <c r="E30" s="8"/>
-      <c r="F30" s="8"/>
-      <c r="G30" s="8"/>
-      <c r="H30" s="8"/>
-      <c r="I30" s="8"/>
-      <c r="J30" s="8"/>
-      <c r="K30" s="8"/>
-      <c r="L30" s="8"/>
-      <c r="M30" s="8"/>
-      <c r="N30" s="8"/>
-      <c r="O30" s="8"/>
-      <c r="P30" s="8"/>
-      <c r="Q30" s="8"/>
-      <c r="R30" s="8"/>
-      <c r="S30" s="8"/>
-      <c r="T30" s="8"/>
-      <c r="U30" s="8"/>
-      <c r="V30" s="8"/>
-      <c r="W30" s="8"/>
-      <c r="X30" s="8"/>
-      <c r="Y30" s="8"/>
+      <c r="B30" s="12"/>
+      <c r="C30" s="7"/>
+      <c r="D30" s="7"/>
+      <c r="E30" s="7"/>
+      <c r="F30" s="7"/>
+      <c r="G30" s="7"/>
+      <c r="H30" s="7"/>
+      <c r="I30" s="7"/>
+      <c r="J30" s="7"/>
+      <c r="K30" s="7"/>
+      <c r="L30" s="7"/>
+      <c r="M30" s="7"/>
+      <c r="N30" s="7"/>
+      <c r="O30" s="7"/>
+      <c r="P30" s="7"/>
+      <c r="Q30" s="7"/>
+      <c r="R30" s="7"/>
+      <c r="S30" s="7"/>
+      <c r="T30" s="7"/>
+      <c r="U30" s="7"/>
+      <c r="V30" s="7"/>
+      <c r="W30" s="7"/>
+      <c r="X30" s="7"/>
+      <c r="Y30" s="7"/>
     </row>
     <row r="31" spans="2:25">
-      <c r="B31" s="13"/>
-      <c r="C31" s="8"/>
-      <c r="D31" s="8"/>
-      <c r="E31" s="8"/>
-      <c r="F31" s="8"/>
-      <c r="G31" s="8"/>
-      <c r="H31" s="8"/>
-      <c r="I31" s="8"/>
-      <c r="J31" s="8"/>
-      <c r="K31" s="8"/>
-      <c r="L31" s="8"/>
-      <c r="M31" s="8"/>
-      <c r="N31" s="8"/>
-      <c r="O31" s="8"/>
-      <c r="P31" s="8"/>
-      <c r="Q31" s="8"/>
-      <c r="R31" s="8"/>
-      <c r="S31" s="8"/>
-      <c r="T31" s="8"/>
-      <c r="U31" s="8"/>
-      <c r="V31" s="8"/>
-      <c r="W31" s="8"/>
-      <c r="X31" s="8"/>
-      <c r="Y31" s="8"/>
+      <c r="B31" s="12"/>
+      <c r="C31" s="7"/>
+      <c r="D31" s="7"/>
+      <c r="E31" s="7"/>
+      <c r="F31" s="7"/>
+      <c r="G31" s="7"/>
+      <c r="H31" s="7"/>
+      <c r="I31" s="7"/>
+      <c r="J31" s="7"/>
+      <c r="K31" s="7"/>
+      <c r="L31" s="7"/>
+      <c r="M31" s="7"/>
+      <c r="N31" s="7"/>
+      <c r="O31" s="7"/>
+      <c r="P31" s="7"/>
+      <c r="Q31" s="7"/>
+      <c r="R31" s="7"/>
+      <c r="S31" s="7"/>
+      <c r="T31" s="7"/>
+      <c r="U31" s="7"/>
+      <c r="V31" s="7"/>
+      <c r="W31" s="7"/>
+      <c r="X31" s="7"/>
+      <c r="Y31" s="7"/>
     </row>
     <row r="32" spans="2:25">
-      <c r="B32" s="13"/>
-      <c r="C32" s="8"/>
-      <c r="D32" s="8"/>
-      <c r="E32" s="8"/>
-      <c r="F32" s="8"/>
-      <c r="G32" s="8"/>
-      <c r="H32" s="8"/>
-      <c r="I32" s="8"/>
-      <c r="J32" s="8"/>
-      <c r="K32" s="8"/>
-      <c r="L32" s="8"/>
-      <c r="M32" s="8"/>
-      <c r="N32" s="8"/>
-      <c r="O32" s="8"/>
-      <c r="P32" s="8"/>
-      <c r="Q32" s="8"/>
-      <c r="R32" s="8"/>
-      <c r="S32" s="8"/>
-      <c r="T32" s="8"/>
-      <c r="U32" s="8"/>
-      <c r="V32" s="8"/>
-      <c r="W32" s="8"/>
-      <c r="X32" s="8"/>
-      <c r="Y32" s="8"/>
+      <c r="B32" s="12"/>
+      <c r="C32" s="7"/>
+      <c r="D32" s="7"/>
+      <c r="E32" s="7"/>
+      <c r="F32" s="7"/>
+      <c r="G32" s="7"/>
+      <c r="H32" s="7"/>
+      <c r="I32" s="7"/>
+      <c r="J32" s="7"/>
+      <c r="K32" s="7"/>
+      <c r="L32" s="7"/>
+      <c r="M32" s="7"/>
+      <c r="N32" s="7"/>
+      <c r="O32" s="7"/>
+      <c r="P32" s="7"/>
+      <c r="Q32" s="7"/>
+      <c r="R32" s="7"/>
+      <c r="S32" s="7"/>
+      <c r="T32" s="7"/>
+      <c r="U32" s="7"/>
+      <c r="V32" s="7"/>
+      <c r="W32" s="7"/>
+      <c r="X32" s="7"/>
+      <c r="Y32" s="7"/>
     </row>
     <row r="33" spans="2:25">
-      <c r="B33" s="13"/>
-      <c r="C33" s="8"/>
-      <c r="D33" s="8"/>
-      <c r="E33" s="8"/>
-      <c r="F33" s="8"/>
-      <c r="G33" s="8"/>
-      <c r="H33" s="8"/>
-      <c r="I33" s="8"/>
-      <c r="J33" s="8"/>
-      <c r="K33" s="8"/>
-      <c r="L33" s="8"/>
-      <c r="M33" s="8"/>
-      <c r="N33" s="8"/>
-      <c r="O33" s="8"/>
-      <c r="P33" s="8"/>
-      <c r="Q33" s="8"/>
-      <c r="R33" s="8"/>
-      <c r="S33" s="8"/>
-      <c r="T33" s="8"/>
-      <c r="U33" s="8"/>
-      <c r="V33" s="8"/>
-      <c r="W33" s="8"/>
-      <c r="X33" s="8"/>
-      <c r="Y33" s="8"/>
+      <c r="B33" s="12"/>
+      <c r="C33" s="7"/>
+      <c r="D33" s="7"/>
+      <c r="E33" s="7"/>
+      <c r="F33" s="7"/>
+      <c r="G33" s="7"/>
+      <c r="H33" s="7"/>
+      <c r="I33" s="7"/>
+      <c r="J33" s="7"/>
+      <c r="K33" s="7"/>
+      <c r="L33" s="7"/>
+      <c r="M33" s="7"/>
+      <c r="N33" s="7"/>
+      <c r="O33" s="7"/>
+      <c r="P33" s="7"/>
+      <c r="Q33" s="7"/>
+      <c r="R33" s="7"/>
+      <c r="S33" s="7"/>
+      <c r="T33" s="7"/>
+      <c r="U33" s="7"/>
+      <c r="V33" s="7"/>
+      <c r="W33" s="7"/>
+      <c r="X33" s="7"/>
+      <c r="Y33" s="7"/>
     </row>
     <row r="34" spans="2:25">
-      <c r="B34" s="13"/>
-      <c r="C34" s="8"/>
-      <c r="D34" s="8"/>
-      <c r="E34" s="8"/>
-      <c r="F34" s="8"/>
-      <c r="G34" s="8"/>
-      <c r="H34" s="8"/>
-      <c r="I34" s="8"/>
-      <c r="J34" s="8"/>
-      <c r="K34" s="8"/>
-      <c r="L34" s="8"/>
-      <c r="M34" s="8"/>
-      <c r="N34" s="8"/>
-      <c r="O34" s="8"/>
-      <c r="P34" s="8"/>
-      <c r="Q34" s="8"/>
-      <c r="R34" s="8"/>
-      <c r="S34" s="8"/>
-      <c r="T34" s="8"/>
-      <c r="U34" s="8"/>
-      <c r="V34" s="8"/>
-      <c r="W34" s="8"/>
-      <c r="X34" s="8"/>
-      <c r="Y34" s="8"/>
+      <c r="B34" s="12"/>
+      <c r="C34" s="7"/>
+      <c r="D34" s="7"/>
+      <c r="E34" s="7"/>
+      <c r="F34" s="7"/>
+      <c r="G34" s="7"/>
+      <c r="H34" s="7"/>
+      <c r="I34" s="7"/>
+      <c r="J34" s="7"/>
+      <c r="K34" s="7"/>
+      <c r="L34" s="7"/>
+      <c r="M34" s="7"/>
+      <c r="N34" s="7"/>
+      <c r="O34" s="7"/>
+      <c r="P34" s="7"/>
+      <c r="Q34" s="7"/>
+      <c r="R34" s="7"/>
+      <c r="S34" s="7"/>
+      <c r="T34" s="7"/>
+      <c r="U34" s="7"/>
+      <c r="V34" s="7"/>
+      <c r="W34" s="7"/>
+      <c r="X34" s="7"/>
+      <c r="Y34" s="7"/>
     </row>
     <row r="35" spans="2:25">
-      <c r="B35" s="13"/>
-      <c r="C35" s="8"/>
-      <c r="D35" s="8"/>
-      <c r="E35" s="8"/>
-      <c r="F35" s="8"/>
-      <c r="G35" s="8"/>
-      <c r="H35" s="8"/>
-      <c r="I35" s="8"/>
-      <c r="J35" s="8"/>
-      <c r="K35" s="8"/>
-      <c r="L35" s="8"/>
-      <c r="M35" s="8"/>
-      <c r="N35" s="8"/>
-      <c r="O35" s="8"/>
-      <c r="P35" s="8"/>
-      <c r="Q35" s="8"/>
-      <c r="R35" s="8"/>
-      <c r="S35" s="8"/>
-      <c r="T35" s="8"/>
-      <c r="U35" s="8"/>
-      <c r="V35" s="8"/>
-      <c r="W35" s="8"/>
-      <c r="X35" s="8"/>
-      <c r="Y35" s="8"/>
+      <c r="B35" s="12"/>
+      <c r="C35" s="7"/>
+      <c r="D35" s="7"/>
+      <c r="E35" s="7"/>
+      <c r="F35" s="7"/>
+      <c r="G35" s="7"/>
+      <c r="H35" s="7"/>
+      <c r="I35" s="7"/>
+      <c r="J35" s="7"/>
+      <c r="K35" s="7"/>
+      <c r="L35" s="7"/>
+      <c r="M35" s="7"/>
+      <c r="N35" s="7"/>
+      <c r="O35" s="7"/>
+      <c r="P35" s="7"/>
+      <c r="Q35" s="7"/>
+      <c r="R35" s="7"/>
+      <c r="S35" s="7"/>
+      <c r="T35" s="7"/>
+      <c r="U35" s="7"/>
+      <c r="V35" s="7"/>
+      <c r="W35" s="7"/>
+      <c r="X35" s="7"/>
+      <c r="Y35" s="7"/>
     </row>
     <row r="36" spans="2:25">
-      <c r="B36" s="13"/>
-      <c r="C36" s="8"/>
-      <c r="D36" s="8"/>
-      <c r="E36" s="8"/>
-      <c r="F36" s="8"/>
-      <c r="G36" s="8"/>
-      <c r="H36" s="8"/>
-      <c r="I36" s="8"/>
-      <c r="J36" s="8"/>
-      <c r="K36" s="8"/>
-      <c r="L36" s="8"/>
-      <c r="M36" s="8"/>
-      <c r="N36" s="8"/>
-      <c r="O36" s="8"/>
-      <c r="P36" s="8"/>
-      <c r="Q36" s="8"/>
-      <c r="R36" s="8"/>
-      <c r="S36" s="8"/>
-      <c r="T36" s="8"/>
-      <c r="U36" s="8"/>
-      <c r="V36" s="8"/>
-      <c r="W36" s="8"/>
-      <c r="X36" s="8"/>
-      <c r="Y36" s="8"/>
+      <c r="B36" s="12"/>
+      <c r="C36" s="7"/>
+      <c r="D36" s="7"/>
+      <c r="E36" s="7"/>
+      <c r="F36" s="7"/>
+      <c r="G36" s="7"/>
+      <c r="H36" s="7"/>
+      <c r="I36" s="7"/>
+      <c r="J36" s="7"/>
+      <c r="K36" s="7"/>
+      <c r="L36" s="7"/>
+      <c r="M36" s="7"/>
+      <c r="N36" s="7"/>
+      <c r="O36" s="7"/>
+      <c r="P36" s="7"/>
+      <c r="Q36" s="7"/>
+      <c r="R36" s="7"/>
+      <c r="S36" s="7"/>
+      <c r="T36" s="7"/>
+      <c r="U36" s="7"/>
+      <c r="V36" s="7"/>
+      <c r="W36" s="7"/>
+      <c r="X36" s="7"/>
+      <c r="Y36" s="7"/>
     </row>
     <row r="37" spans="2:25">
-      <c r="B37" s="13"/>
-      <c r="C37" s="8"/>
-      <c r="D37" s="8"/>
-      <c r="E37" s="8"/>
-      <c r="F37" s="8"/>
-      <c r="G37" s="8"/>
-      <c r="H37" s="8"/>
-      <c r="I37" s="8"/>
-      <c r="J37" s="8"/>
-      <c r="K37" s="8"/>
-      <c r="L37" s="8"/>
-      <c r="M37" s="8"/>
-      <c r="N37" s="8"/>
-      <c r="O37" s="8"/>
-      <c r="P37" s="8"/>
-      <c r="Q37" s="8"/>
-      <c r="R37" s="8"/>
-      <c r="S37" s="8"/>
-      <c r="T37" s="8"/>
-      <c r="U37" s="8"/>
-      <c r="V37" s="8"/>
-      <c r="W37" s="8"/>
-      <c r="X37" s="8"/>
-      <c r="Y37" s="8"/>
+      <c r="B37" s="12"/>
+      <c r="C37" s="7"/>
+      <c r="D37" s="7"/>
+      <c r="E37" s="7"/>
+      <c r="F37" s="7"/>
+      <c r="G37" s="7"/>
+      <c r="H37" s="7"/>
+      <c r="I37" s="7"/>
+      <c r="J37" s="7"/>
+      <c r="K37" s="7"/>
+      <c r="L37" s="7"/>
+      <c r="M37" s="7"/>
+      <c r="N37" s="7"/>
+      <c r="O37" s="7"/>
+      <c r="P37" s="7"/>
+      <c r="Q37" s="7"/>
+      <c r="R37" s="7"/>
+      <c r="S37" s="7"/>
+      <c r="T37" s="7"/>
+      <c r="U37" s="7"/>
+      <c r="V37" s="7"/>
+      <c r="W37" s="7"/>
+      <c r="X37" s="7"/>
+      <c r="Y37" s="7"/>
     </row>
     <row r="38" spans="2:25">
-      <c r="B38" s="13"/>
-      <c r="C38" s="8"/>
-      <c r="D38" s="8"/>
-      <c r="E38" s="8"/>
-      <c r="F38" s="8"/>
-      <c r="G38" s="8"/>
-      <c r="H38" s="8"/>
-      <c r="I38" s="8"/>
-      <c r="J38" s="8"/>
-      <c r="K38" s="8"/>
-      <c r="L38" s="8"/>
-      <c r="M38" s="8"/>
-      <c r="N38" s="8"/>
-      <c r="O38" s="8"/>
-      <c r="P38" s="8"/>
-      <c r="Q38" s="8"/>
-      <c r="R38" s="8"/>
-      <c r="S38" s="8"/>
-      <c r="T38" s="8"/>
-      <c r="U38" s="8"/>
-      <c r="V38" s="8"/>
-      <c r="W38" s="8"/>
-      <c r="X38" s="8"/>
-      <c r="Y38" s="8"/>
+      <c r="B38" s="12"/>
+      <c r="C38" s="7"/>
+      <c r="D38" s="7"/>
+      <c r="E38" s="7"/>
+      <c r="F38" s="7"/>
+      <c r="G38" s="7"/>
+      <c r="H38" s="7"/>
+      <c r="I38" s="7"/>
+      <c r="J38" s="7"/>
+      <c r="K38" s="7"/>
+      <c r="L38" s="7"/>
+      <c r="M38" s="7"/>
+      <c r="N38" s="7"/>
+      <c r="O38" s="7"/>
+      <c r="P38" s="7"/>
+      <c r="Q38" s="7"/>
+      <c r="R38" s="7"/>
+      <c r="S38" s="7"/>
+      <c r="T38" s="7"/>
+      <c r="U38" s="7"/>
+      <c r="V38" s="7"/>
+      <c r="W38" s="7"/>
+      <c r="X38" s="7"/>
+      <c r="Y38" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -5489,7 +5582,7 @@
       <c r="E2" s="3">
         <v>0.989</v>
       </c>
-      <c r="F2" s="4" t="s">
+      <c r="F2" s="2" t="s">
         <v>49</v>
       </c>
     </row>
@@ -5506,7 +5599,7 @@
       <c r="E3" s="3">
         <v>0.977</v>
       </c>
-      <c r="F3" s="4" t="s">
+      <c r="F3" s="2" t="s">
         <v>49</v>
       </c>
     </row>
@@ -5523,7 +5616,7 @@
       <c r="E4" s="3">
         <v>0.912</v>
       </c>
-      <c r="F4" s="4" t="s">
+      <c r="F4" s="2" t="s">
         <v>50</v>
       </c>
     </row>
@@ -5540,7 +5633,7 @@
       <c r="E5" s="3">
         <v>0.813</v>
       </c>
-      <c r="F5" s="4" t="s">
+      <c r="F5" s="2" t="s">
         <v>51</v>
       </c>
     </row>
@@ -5557,7 +5650,7 @@
       <c r="E6" s="3">
         <v>0.692</v>
       </c>
-      <c r="F6" s="4" t="s">
+      <c r="F6" s="2" t="s">
         <v>51</v>
       </c>
     </row>
@@ -5574,7 +5667,7 @@
       <c r="E7" s="3">
         <v>0.724</v>
       </c>
-      <c r="F7" s="4" t="s">
+      <c r="F7" s="2" t="s">
         <v>52</v>
       </c>
     </row>
@@ -5591,7 +5684,7 @@
       <c r="E8" s="3">
         <v>0.708</v>
       </c>
-      <c r="F8" s="4" t="s">
+      <c r="F8" s="2" t="s">
         <v>53</v>
       </c>
     </row>
@@ -5608,7 +5701,7 @@
       <c r="E9" s="3">
         <v>0.668</v>
       </c>
-      <c r="F9" s="4" t="s">
+      <c r="F9" s="2" t="s">
         <v>54</v>
       </c>
     </row>
@@ -5625,7 +5718,7 @@
       <c r="E10" s="3">
         <v>0.617</v>
       </c>
-      <c r="F10" s="4" t="s">
+      <c r="F10" s="2" t="s">
         <v>55</v>
       </c>
     </row>
@@ -5642,7 +5735,7 @@
       <c r="E11" s="3">
         <v>0.585</v>
       </c>
-      <c r="F11" s="4" t="s">
+      <c r="F11" s="2" t="s">
         <v>56</v>
       </c>
     </row>
@@ -5659,7 +5752,7 @@
       <c r="E12" s="3">
         <v>0.544</v>
       </c>
-      <c r="F12" s="4" t="s">
+      <c r="F12" s="2" t="s">
         <v>55</v>
       </c>
     </row>
@@ -5676,7 +5769,7 @@
       <c r="E13" s="3">
         <v>0.501</v>
       </c>
-      <c r="F13" s="4" t="s">
+      <c r="F13" s="2" t="s">
         <v>57</v>
       </c>
     </row>
@@ -5693,7 +5786,7 @@
       <c r="E14" s="3">
         <v>0.407</v>
       </c>
-      <c r="F14" s="4" t="s">
+      <c r="F14" s="2" t="s">
         <v>57</v>
       </c>
     </row>
@@ -5710,7 +5803,7 @@
       <c r="E15" s="3">
         <v>0.307</v>
       </c>
-      <c r="F15" s="4" t="s">
+      <c r="F15" s="2" t="s">
         <v>58</v>
       </c>
     </row>
@@ -5727,7 +5820,7 @@
       <c r="E16" s="3">
         <v>0.221</v>
       </c>
-      <c r="F16" s="4" t="s">
+      <c r="F16" s="2" t="s">
         <v>58</v>
       </c>
     </row>
@@ -5744,7 +5837,7 @@
       <c r="E17" s="3">
         <v>0.151</v>
       </c>
-      <c r="F17" s="4" t="s">
+      <c r="F17" s="2" t="s">
         <v>59</v>
       </c>
     </row>
@@ -5761,7 +5854,7 @@
       <c r="E18" s="3">
         <v>0.1</v>
       </c>
-      <c r="F18" s="4" t="s">
+      <c r="F18" s="2" t="s">
         <v>59</v>
       </c>
     </row>

</xml_diff>

<commit_message>
modified:   Ferrite Transformer Calculation.xlsx
</commit_message>
<xml_diff>
--- a/Ferrite Transformer Calculation.xlsx
+++ b/Ferrite Transformer Calculation.xlsx
@@ -4396,7 +4396,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A2:T12"/>
+  <dimension ref="A2:U12"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="5.5625" style="4" customWidth="1"/>
@@ -4470,7 +4470,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="3" spans="1:20">
+    <row r="3" spans="1:21">
       <c r="A3" s="25">
         <v>1</v>
       </c>
@@ -4526,16 +4526,19 @@
         <v>6.66666666666667</v>
       </c>
       <c r="R3" s="30">
-        <f>P3</f>
-        <v>1.5</v>
+        <v>2.5</v>
       </c>
       <c r="S3" s="29">
         <f>SQRT((P3*0.9/(R3+5))/0.9)</f>
-        <v>0.480384461415261</v>
+        <v>0.447213595499958</v>
       </c>
       <c r="T3" s="29">
         <f>SQRT((N3*0.9/(R3+5))/0.9)</f>
-        <v>0.277350098112615</v>
+        <v>0.258198889747161</v>
+      </c>
+      <c r="U3" s="30">
+        <f>P3/R3</f>
+        <v>0.6</v>
       </c>
     </row>
     <row r="4" spans="1:20">
@@ -4592,16 +4595,15 @@
         <v>30.2521008403361</v>
       </c>
       <c r="R4" s="30">
-        <f t="shared" ref="R4:R9" si="6">P4</f>
-        <v>1.5</v>
+        <v>2.5</v>
       </c>
       <c r="S4" s="29">
-        <f t="shared" ref="S4:S9" si="7">SQRT((P4*0.9/(R4+5))/0.9)</f>
-        <v>0.480384461415261</v>
+        <f t="shared" ref="S4:S9" si="6">SQRT((P4*0.9/(R4+5))/0.9)</f>
+        <v>0.447213595499958</v>
       </c>
       <c r="T4" s="29">
-        <f t="shared" ref="T4:T9" si="8">SQRT((N4*0.9/(R4+5))/0.9)</f>
-        <v>0.277350098112615</v>
+        <f t="shared" ref="T4:T9" si="7">SQRT((N4*0.9/(R4+5))/0.9)</f>
+        <v>0.258198889747161</v>
       </c>
     </row>
     <row r="5" spans="2:20">
@@ -4655,16 +4657,15 @@
         <v>18.553640636596</v>
       </c>
       <c r="R5" s="30">
+        <v>2.5</v>
+      </c>
+      <c r="S5" s="29">
         <f t="shared" si="6"/>
-        <v>1.5</v>
-      </c>
-      <c r="S5" s="29">
+        <v>0.447213595499958</v>
+      </c>
+      <c r="T5" s="29">
         <f t="shared" si="7"/>
-        <v>0.480384461415261</v>
-      </c>
-      <c r="T5" s="29">
-        <f t="shared" si="8"/>
-        <v>0.277350098112615</v>
+        <v>0.258198889747161</v>
       </c>
     </row>
     <row r="6" spans="2:20">
@@ -4718,16 +4719,15 @@
         <v>31.8062410913075</v>
       </c>
       <c r="R6" s="30">
+        <v>2.5</v>
+      </c>
+      <c r="S6" s="29">
         <f t="shared" si="6"/>
-        <v>1.5</v>
-      </c>
-      <c r="S6" s="29">
+        <v>0.447213595499958</v>
+      </c>
+      <c r="T6" s="29">
         <f t="shared" si="7"/>
-        <v>0.480384461415261</v>
-      </c>
-      <c r="T6" s="29">
-        <f t="shared" si="8"/>
-        <v>0.277350098112615</v>
+        <v>0.258198889747161</v>
       </c>
     </row>
     <row r="7" spans="2:20">
@@ -4783,16 +4783,15 @@
         <v>29.8760145396604</v>
       </c>
       <c r="R7" s="30">
+        <v>2.5</v>
+      </c>
+      <c r="S7" s="29">
         <f t="shared" si="6"/>
-        <v>1.5</v>
-      </c>
-      <c r="S7" s="29">
+        <v>0.447213595499958</v>
+      </c>
+      <c r="T7" s="29">
         <f t="shared" si="7"/>
-        <v>0.480384461415261</v>
-      </c>
-      <c r="T7" s="29">
-        <f t="shared" si="8"/>
-        <v>0.277350098112615</v>
+        <v>0.258198889747161</v>
       </c>
     </row>
     <row r="8" spans="2:20">
@@ -4848,16 +4847,15 @@
         <v>98.396501457726</v>
       </c>
       <c r="R8" s="30">
+        <v>2.5</v>
+      </c>
+      <c r="S8" s="29">
         <f t="shared" si="6"/>
-        <v>1.5</v>
-      </c>
-      <c r="S8" s="29">
+        <v>0.447213595499958</v>
+      </c>
+      <c r="T8" s="29">
         <f t="shared" si="7"/>
-        <v>0.480384461415261</v>
-      </c>
-      <c r="T8" s="29">
-        <f t="shared" si="8"/>
-        <v>0.277350098112615</v>
+        <v>0.258198889747161</v>
       </c>
     </row>
     <row r="9" spans="2:20">
@@ -4910,16 +4908,15 @@
         <v>29.9270113445541</v>
       </c>
       <c r="R9" s="30">
+        <v>2.5</v>
+      </c>
+      <c r="S9" s="29">
         <f t="shared" si="6"/>
-        <v>1.5</v>
-      </c>
-      <c r="S9" s="29">
+        <v>0.447213595499958</v>
+      </c>
+      <c r="T9" s="29">
         <f t="shared" si="7"/>
-        <v>0.480384461415261</v>
-      </c>
-      <c r="T9" s="29">
-        <f t="shared" si="8"/>
-        <v>0.277350098112615</v>
+        <v>0.258198889747161</v>
       </c>
     </row>
     <row r="10" spans="10:10">

</xml_diff>

<commit_message>
modified:   Ferrite Transformer Calculation.xlsx 	modified:   README.md
</commit_message>
<xml_diff>
--- a/Ferrite Transformer Calculation.xlsx
+++ b/Ferrite Transformer Calculation.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="28800" windowHeight="12960" activeTab="1"/>
+    <workbookView windowWidth="28800" windowHeight="13060" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="ETD" sheetId="1" r:id="rId1"/>
@@ -1358,13 +1358,6 @@
   </si>
   <si>
     <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <charset val="134"/>
-        <scheme val="minor"/>
-      </rPr>
       <t>C</t>
     </r>
     <r>
@@ -1386,7 +1379,7 @@
         <charset val="134"/>
         <scheme val="minor"/>
       </rPr>
-      <t xml:space="preserve"> = C</t>
+      <t xml:space="preserve"> = 2 C</t>
     </r>
     <r>
       <rPr>
@@ -1588,7 +1581,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
-  <numFmts count="17">
+  <numFmts count="19">
     <numFmt numFmtId="41" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;_);_(@_)"/>
     <numFmt numFmtId="42" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
     <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
@@ -1600,12 +1593,14 @@
     <numFmt numFmtId="181" formatCode="_ * #,##0.0000000_ ;_ * \-#,##0.0000000_ ;_ * &quot;-&quot;??.0000000_ ;_ @_ "/>
     <numFmt numFmtId="182" formatCode="_ * #,##0.0_ ;_ * \-#,##0.0_ ;_ * &quot;-&quot;??.0_ ;_ @_ "/>
     <numFmt numFmtId="183" formatCode="_ * #,##0.000000000000_ ;_ * \-#,##0.000000000000_ ;_ * &quot;-&quot;??.000000000000_ ;_ @_ "/>
-    <numFmt numFmtId="184" formatCode="_ * #,##0.000_ ;_ * \-#,##0.000_ ;_ * &quot;-&quot;??.000_ ;_ @_ "/>
-    <numFmt numFmtId="185" formatCode="_ * #,##0.00000000_ ;_ * \-#,##0.00000000_ ;_ * &quot;-&quot;??.00000000_ ;_ @_ "/>
-    <numFmt numFmtId="186" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??.00_ ;_ @_ "/>
-    <numFmt numFmtId="187" formatCode="0.00_ "/>
-    <numFmt numFmtId="188" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;_);_(@_)"/>
-    <numFmt numFmtId="189" formatCode="_(* #,##0.0000_);_(* \(#,##0.0000\);_(* &quot;-&quot;_);_(@_)"/>
+    <numFmt numFmtId="184" formatCode="0.0000000000E+00"/>
+    <numFmt numFmtId="185" formatCode="_ * #,##0.00000000000000_ ;_ * \-#,##0.00000000000000_ ;_ * &quot;-&quot;??.00000000000000_ ;_ @_ "/>
+    <numFmt numFmtId="186" formatCode="_ * #,##0.000_ ;_ * \-#,##0.000_ ;_ * &quot;-&quot;??.000_ ;_ @_ "/>
+    <numFmt numFmtId="187" formatCode="_ * #,##0.00000000_ ;_ * \-#,##0.00000000_ ;_ * &quot;-&quot;??.00000000_ ;_ @_ "/>
+    <numFmt numFmtId="188" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??.00_ ;_ @_ "/>
+    <numFmt numFmtId="189" formatCode="0.00_ "/>
+    <numFmt numFmtId="190" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;_);_(@_)"/>
+    <numFmt numFmtId="191" formatCode="_(* #,##0.0000_);_(* \(#,##0.0000\);_(* &quot;-&quot;_);_(@_)"/>
   </numFmts>
   <fonts count="31">
     <font>
@@ -1790,6 +1785,20 @@
       <vertAlign val="subscript"/>
       <sz val="10"/>
       <color theme="1"/>
+      <name val="Arial"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial Bold"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <vertAlign val="subscript"/>
+      <sz val="10"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -1803,26 +1812,13 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <vertAlign val="subscript"/>
-      <sz val="10"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-      <charset val="134"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="10"/>
-      <color theme="1"/>
-      <name val="Arial Bold"/>
-      <charset val="134"/>
-    </font>
-    <font>
       <b/>
       <vertAlign val="superscript"/>
       <sz val="10"/>
       <color theme="1"/>
-      <name val="Arial Bold"/>
+      <name val="Calibri"/>
       <charset val="134"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <vertAlign val="superscript"/>
@@ -1836,9 +1832,8 @@
       <vertAlign val="superscript"/>
       <sz val="10"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="Arial Bold"/>
       <charset val="134"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="33">
@@ -2291,7 +2286,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -2346,19 +2341,28 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="184" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="182" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="185" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="179" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="184" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="185" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="186" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="187" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="188" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -2379,10 +2383,10 @@
     <xf numFmtId="176" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="187" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="188" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1">
+    <xf numFmtId="189" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="190" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -2391,13 +2395,13 @@
     <xf numFmtId="41" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="189" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1">
+    <xf numFmtId="191" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="41" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="189" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="191" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="180" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1">
@@ -3921,12 +3925,12 @@
   <dimension ref="A1:U33"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="5.5625" style="26" customWidth="1"/>
-    <col min="2" max="4" width="10.5625" style="26" customWidth="1"/>
-    <col min="5" max="5" width="20.5625" style="26" customWidth="1"/>
-    <col min="6" max="6" width="15.5625" style="26" customWidth="1"/>
-    <col min="7" max="7" width="30.5625" style="32" customWidth="1"/>
-    <col min="8" max="8" width="10.5625" style="26" customWidth="1"/>
+    <col min="1" max="1" width="5.5625" style="29" customWidth="1"/>
+    <col min="2" max="4" width="10.5625" style="29" customWidth="1"/>
+    <col min="5" max="5" width="20.5625" style="29" customWidth="1"/>
+    <col min="6" max="6" width="15.5625" style="29" customWidth="1"/>
+    <col min="7" max="7" width="30.5625" style="35" customWidth="1"/>
+    <col min="8" max="8" width="10.5625" style="29" customWidth="1"/>
     <col min="9" max="9" width="15.5625" style="4" customWidth="1"/>
     <col min="10" max="13" width="10.5625" style="4" customWidth="1"/>
     <col min="14" max="14" width="9" style="4"/>
@@ -3942,133 +3946,133 @@
       <c r="D1" s="4"/>
       <c r="E1" s="4"/>
       <c r="F1" s="4"/>
-      <c r="G1" s="23"/>
+      <c r="G1" s="26"/>
       <c r="H1" s="4"/>
     </row>
-    <row r="2" s="31" customFormat="1" ht="18" spans="1:21">
-      <c r="A2" s="23" t="s">
+    <row r="2" s="34" customFormat="1" ht="18" spans="1:21">
+      <c r="A2" s="26" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="24" t="s">
+      <c r="B2" s="27" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="24" t="s">
+      <c r="C2" s="27" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="24" t="s">
+      <c r="D2" s="27" t="s">
         <v>3</v>
       </c>
-      <c r="E2" s="24" t="s">
+      <c r="E2" s="27" t="s">
         <v>4</v>
       </c>
-      <c r="F2" s="24" t="s">
+      <c r="F2" s="27" t="s">
         <v>5</v>
       </c>
-      <c r="G2" s="23" t="s">
+      <c r="G2" s="26" t="s">
         <v>6</v>
       </c>
-      <c r="H2" s="24" t="s">
+      <c r="H2" s="27" t="s">
         <v>7</v>
       </c>
-      <c r="I2" s="23" t="s">
+      <c r="I2" s="26" t="s">
         <v>8</v>
       </c>
-      <c r="J2" s="23" t="s">
+      <c r="J2" s="26" t="s">
         <v>9</v>
       </c>
-      <c r="K2" s="23" t="s">
+      <c r="K2" s="26" t="s">
         <v>10</v>
       </c>
-      <c r="L2" s="23" t="s">
+      <c r="L2" s="26" t="s">
         <v>11</v>
       </c>
-      <c r="M2" s="23" t="s">
+      <c r="M2" s="26" t="s">
         <v>12</v>
       </c>
-      <c r="N2" s="23" t="s">
+      <c r="N2" s="26" t="s">
         <v>13</v>
       </c>
-      <c r="O2" s="23" t="s">
+      <c r="O2" s="26" t="s">
         <v>14</v>
       </c>
-      <c r="P2" s="23" t="s">
+      <c r="P2" s="26" t="s">
         <v>15</v>
       </c>
-      <c r="Q2" s="23" t="s">
+      <c r="Q2" s="26" t="s">
         <v>16</v>
       </c>
-      <c r="R2" s="23" t="s">
+      <c r="R2" s="26" t="s">
         <v>17</v>
       </c>
-      <c r="S2" s="23" t="s">
+      <c r="S2" s="26" t="s">
         <v>18</v>
       </c>
-      <c r="T2" s="23" t="s">
+      <c r="T2" s="26" t="s">
         <v>17</v>
       </c>
-      <c r="U2" s="23" t="s">
+      <c r="U2" s="26" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="3" spans="1:21">
-      <c r="A3" s="25">
+      <c r="A3" s="28">
         <v>1</v>
       </c>
-      <c r="B3" s="25">
+      <c r="B3" s="28">
         <v>72</v>
       </c>
-      <c r="C3" s="25">
+      <c r="C3" s="28">
         <v>400000</v>
       </c>
-      <c r="D3" s="25">
+      <c r="D3" s="28">
         <v>10</v>
       </c>
-      <c r="E3" s="33">
+      <c r="E3" s="36">
         <f>3.14*POWER(D3,2)/4</f>
         <v>78.5</v>
       </c>
-      <c r="F3" s="33">
+      <c r="F3" s="36">
         <v>1898.58</v>
       </c>
-      <c r="G3" s="34">
+      <c r="G3" s="37">
         <f>(B3*POWER(10,10))/(4*C3*F3*E3)</f>
         <v>3.01935345175506</v>
       </c>
-      <c r="H3" s="35" t="str">
+      <c r="H3" s="38" t="str">
         <f>IF((B3*POWER(10,10))/(4*C3*G3*E3)&gt;1200,IF((B3*POWER(10,10))/(4*C3*G3*E3)&lt;2000,"OK","NG"),"NG")</f>
         <v>OK</v>
       </c>
-      <c r="I3" s="26">
+      <c r="I3" s="29">
         <f>B3/G3</f>
         <v>23.8461648</v>
       </c>
-      <c r="J3" s="26">
+      <c r="J3" s="29">
         <f>B3*3</f>
         <v>216</v>
       </c>
-      <c r="K3" s="30">
+      <c r="K3" s="33">
         <v>0.5</v>
       </c>
-      <c r="L3" s="26">
+      <c r="L3" s="29">
         <f>J3*K3</f>
         <v>108</v>
       </c>
-      <c r="M3" s="30">
+      <c r="M3" s="33">
         <f>L3/B3</f>
         <v>1.5</v>
       </c>
-      <c r="N3" s="26">
+      <c r="N3" s="29">
         <f>J3/I3</f>
         <v>9.05806035526518</v>
       </c>
-      <c r="O3" s="26">
+      <c r="O3" s="29">
         <v>1.5</v>
       </c>
-      <c r="P3" s="36">
+      <c r="P3" s="39">
         <f>SQRT((M3*0.9/(O3+5))/0.9)</f>
         <v>0.480384461415261</v>
       </c>
-      <c r="Q3" s="36">
+      <c r="Q3" s="39">
         <f>SQRT((K3*0.9/(O3+5))/0.9)</f>
         <v>0.277350098112615</v>
       </c>
@@ -4088,304 +4092,304 @@
       </c>
     </row>
     <row r="4" spans="1:8">
-      <c r="A4" s="25"/>
-      <c r="B4" s="25"/>
-      <c r="C4" s="25"/>
-      <c r="D4" s="25"/>
-      <c r="E4" s="25"/>
-      <c r="F4" s="25"/>
-      <c r="G4" s="34"/>
-      <c r="H4" s="25"/>
+      <c r="A4" s="28"/>
+      <c r="B4" s="28"/>
+      <c r="C4" s="28"/>
+      <c r="D4" s="28"/>
+      <c r="E4" s="28"/>
+      <c r="F4" s="28"/>
+      <c r="G4" s="37"/>
+      <c r="H4" s="28"/>
     </row>
     <row r="5" spans="1:8">
-      <c r="A5" s="25"/>
-      <c r="B5" s="25"/>
-      <c r="C5" s="25"/>
-      <c r="D5" s="25"/>
-      <c r="E5" s="25"/>
-      <c r="F5" s="25"/>
-      <c r="G5" s="34"/>
-      <c r="H5" s="25"/>
+      <c r="A5" s="28"/>
+      <c r="B5" s="28"/>
+      <c r="C5" s="28"/>
+      <c r="D5" s="28"/>
+      <c r="E5" s="28"/>
+      <c r="F5" s="28"/>
+      <c r="G5" s="37"/>
+      <c r="H5" s="28"/>
     </row>
     <row r="6" spans="1:8">
-      <c r="A6" s="25"/>
-      <c r="B6" s="25"/>
-      <c r="C6" s="25"/>
-      <c r="D6" s="25"/>
-      <c r="E6" s="25"/>
-      <c r="F6" s="25"/>
-      <c r="G6" s="34"/>
-      <c r="H6" s="25"/>
+      <c r="A6" s="28"/>
+      <c r="B6" s="28"/>
+      <c r="C6" s="28"/>
+      <c r="D6" s="28"/>
+      <c r="E6" s="28"/>
+      <c r="F6" s="28"/>
+      <c r="G6" s="37"/>
+      <c r="H6" s="28"/>
     </row>
     <row r="7" spans="1:8">
-      <c r="A7" s="25"/>
-      <c r="B7" s="25"/>
-      <c r="C7" s="25"/>
-      <c r="D7" s="25"/>
-      <c r="E7" s="25"/>
-      <c r="F7" s="25"/>
-      <c r="G7" s="34"/>
-      <c r="H7" s="25"/>
+      <c r="A7" s="28"/>
+      <c r="B7" s="28"/>
+      <c r="C7" s="28"/>
+      <c r="D7" s="28"/>
+      <c r="E7" s="28"/>
+      <c r="F7" s="28"/>
+      <c r="G7" s="37"/>
+      <c r="H7" s="28"/>
     </row>
     <row r="8" spans="1:8">
-      <c r="A8" s="25"/>
-      <c r="B8" s="25"/>
-      <c r="C8" s="25"/>
-      <c r="D8" s="25"/>
-      <c r="E8" s="25"/>
-      <c r="F8" s="25"/>
-      <c r="G8" s="34"/>
-      <c r="H8" s="25"/>
+      <c r="A8" s="28"/>
+      <c r="B8" s="28"/>
+      <c r="C8" s="28"/>
+      <c r="D8" s="28"/>
+      <c r="E8" s="28"/>
+      <c r="F8" s="28"/>
+      <c r="G8" s="37"/>
+      <c r="H8" s="28"/>
     </row>
     <row r="9" spans="1:8">
-      <c r="A9" s="25"/>
-      <c r="B9" s="25"/>
-      <c r="C9" s="25"/>
-      <c r="D9" s="25"/>
-      <c r="E9" s="25"/>
-      <c r="F9" s="25"/>
-      <c r="G9" s="34"/>
-      <c r="H9" s="25"/>
+      <c r="A9" s="28"/>
+      <c r="B9" s="28"/>
+      <c r="C9" s="28"/>
+      <c r="D9" s="28"/>
+      <c r="E9" s="28"/>
+      <c r="F9" s="28"/>
+      <c r="G9" s="37"/>
+      <c r="H9" s="28"/>
     </row>
     <row r="10" spans="1:8">
-      <c r="A10" s="25"/>
-      <c r="B10" s="25"/>
-      <c r="C10" s="25"/>
-      <c r="D10" s="25"/>
-      <c r="E10" s="25"/>
-      <c r="F10" s="25"/>
-      <c r="G10" s="34"/>
-      <c r="H10" s="25"/>
+      <c r="A10" s="28"/>
+      <c r="B10" s="28"/>
+      <c r="C10" s="28"/>
+      <c r="D10" s="28"/>
+      <c r="E10" s="28"/>
+      <c r="F10" s="28"/>
+      <c r="G10" s="37"/>
+      <c r="H10" s="28"/>
     </row>
     <row r="11" spans="1:8">
-      <c r="A11" s="25"/>
-      <c r="B11" s="25"/>
-      <c r="C11" s="25"/>
-      <c r="D11" s="25"/>
-      <c r="E11" s="25"/>
-      <c r="F11" s="25"/>
-      <c r="G11" s="34"/>
-      <c r="H11" s="25"/>
+      <c r="A11" s="28"/>
+      <c r="B11" s="28"/>
+      <c r="C11" s="28"/>
+      <c r="D11" s="28"/>
+      <c r="E11" s="28"/>
+      <c r="F11" s="28"/>
+      <c r="G11" s="37"/>
+      <c r="H11" s="28"/>
     </row>
     <row r="12" spans="1:8">
-      <c r="A12" s="25"/>
-      <c r="B12" s="25"/>
-      <c r="C12" s="25"/>
-      <c r="D12" s="25"/>
-      <c r="E12" s="25"/>
-      <c r="F12" s="25"/>
-      <c r="G12" s="34"/>
-      <c r="H12" s="25"/>
+      <c r="A12" s="28"/>
+      <c r="B12" s="28"/>
+      <c r="C12" s="28"/>
+      <c r="D12" s="28"/>
+      <c r="E12" s="28"/>
+      <c r="F12" s="28"/>
+      <c r="G12" s="37"/>
+      <c r="H12" s="28"/>
     </row>
     <row r="13" spans="1:8">
-      <c r="A13" s="25"/>
-      <c r="B13" s="25"/>
-      <c r="C13" s="25"/>
-      <c r="D13" s="25"/>
-      <c r="E13" s="25"/>
-      <c r="F13" s="25"/>
-      <c r="G13" s="34"/>
-      <c r="H13" s="25"/>
+      <c r="A13" s="28"/>
+      <c r="B13" s="28"/>
+      <c r="C13" s="28"/>
+      <c r="D13" s="28"/>
+      <c r="E13" s="28"/>
+      <c r="F13" s="28"/>
+      <c r="G13" s="37"/>
+      <c r="H13" s="28"/>
     </row>
     <row r="14" spans="1:8">
-      <c r="A14" s="25"/>
-      <c r="B14" s="25"/>
-      <c r="C14" s="25"/>
-      <c r="D14" s="25"/>
-      <c r="E14" s="25"/>
-      <c r="F14" s="25"/>
-      <c r="G14" s="34"/>
-      <c r="H14" s="25"/>
+      <c r="A14" s="28"/>
+      <c r="B14" s="28"/>
+      <c r="C14" s="28"/>
+      <c r="D14" s="28"/>
+      <c r="E14" s="28"/>
+      <c r="F14" s="28"/>
+      <c r="G14" s="37"/>
+      <c r="H14" s="28"/>
     </row>
     <row r="15" spans="1:8">
-      <c r="A15" s="25"/>
-      <c r="B15" s="25"/>
-      <c r="C15" s="25"/>
-      <c r="D15" s="25"/>
-      <c r="E15" s="25"/>
-      <c r="F15" s="25"/>
-      <c r="G15" s="34"/>
-      <c r="H15" s="25"/>
+      <c r="A15" s="28"/>
+      <c r="B15" s="28"/>
+      <c r="C15" s="28"/>
+      <c r="D15" s="28"/>
+      <c r="E15" s="28"/>
+      <c r="F15" s="28"/>
+      <c r="G15" s="37"/>
+      <c r="H15" s="28"/>
     </row>
     <row r="16" spans="1:8">
-      <c r="A16" s="25"/>
-      <c r="B16" s="25"/>
-      <c r="C16" s="25"/>
-      <c r="D16" s="25"/>
-      <c r="E16" s="25"/>
-      <c r="F16" s="25"/>
-      <c r="G16" s="34"/>
-      <c r="H16" s="25"/>
+      <c r="A16" s="28"/>
+      <c r="B16" s="28"/>
+      <c r="C16" s="28"/>
+      <c r="D16" s="28"/>
+      <c r="E16" s="28"/>
+      <c r="F16" s="28"/>
+      <c r="G16" s="37"/>
+      <c r="H16" s="28"/>
     </row>
     <row r="17" spans="1:8">
-      <c r="A17" s="25"/>
-      <c r="B17" s="25"/>
-      <c r="C17" s="25"/>
-      <c r="D17" s="25"/>
-      <c r="E17" s="25"/>
-      <c r="F17" s="25"/>
-      <c r="G17" s="34"/>
-      <c r="H17" s="25"/>
+      <c r="A17" s="28"/>
+      <c r="B17" s="28"/>
+      <c r="C17" s="28"/>
+      <c r="D17" s="28"/>
+      <c r="E17" s="28"/>
+      <c r="F17" s="28"/>
+      <c r="G17" s="37"/>
+      <c r="H17" s="28"/>
     </row>
     <row r="18" spans="1:8">
-      <c r="A18" s="25"/>
-      <c r="B18" s="25"/>
-      <c r="C18" s="25"/>
-      <c r="D18" s="25"/>
-      <c r="E18" s="25"/>
-      <c r="F18" s="25"/>
-      <c r="G18" s="34"/>
-      <c r="H18" s="25"/>
+      <c r="A18" s="28"/>
+      <c r="B18" s="28"/>
+      <c r="C18" s="28"/>
+      <c r="D18" s="28"/>
+      <c r="E18" s="28"/>
+      <c r="F18" s="28"/>
+      <c r="G18" s="37"/>
+      <c r="H18" s="28"/>
     </row>
     <row r="19" spans="1:8">
-      <c r="A19" s="25"/>
-      <c r="B19" s="25"/>
-      <c r="C19" s="25"/>
-      <c r="D19" s="25"/>
-      <c r="E19" s="25"/>
-      <c r="F19" s="25"/>
-      <c r="G19" s="34"/>
-      <c r="H19" s="25"/>
+      <c r="A19" s="28"/>
+      <c r="B19" s="28"/>
+      <c r="C19" s="28"/>
+      <c r="D19" s="28"/>
+      <c r="E19" s="28"/>
+      <c r="F19" s="28"/>
+      <c r="G19" s="37"/>
+      <c r="H19" s="28"/>
     </row>
     <row r="20" spans="1:8">
-      <c r="A20" s="25"/>
-      <c r="B20" s="25"/>
-      <c r="C20" s="25"/>
-      <c r="D20" s="25"/>
-      <c r="E20" s="25"/>
-      <c r="F20" s="25"/>
-      <c r="G20" s="34"/>
-      <c r="H20" s="25"/>
+      <c r="A20" s="28"/>
+      <c r="B20" s="28"/>
+      <c r="C20" s="28"/>
+      <c r="D20" s="28"/>
+      <c r="E20" s="28"/>
+      <c r="F20" s="28"/>
+      <c r="G20" s="37"/>
+      <c r="H20" s="28"/>
     </row>
     <row r="21" spans="1:8">
-      <c r="A21" s="25"/>
-      <c r="B21" s="25"/>
-      <c r="C21" s="25"/>
-      <c r="D21" s="25"/>
-      <c r="E21" s="25"/>
-      <c r="F21" s="25"/>
-      <c r="G21" s="34"/>
-      <c r="H21" s="25"/>
+      <c r="A21" s="28"/>
+      <c r="B21" s="28"/>
+      <c r="C21" s="28"/>
+      <c r="D21" s="28"/>
+      <c r="E21" s="28"/>
+      <c r="F21" s="28"/>
+      <c r="G21" s="37"/>
+      <c r="H21" s="28"/>
     </row>
     <row r="22" spans="1:8">
-      <c r="A22" s="25"/>
-      <c r="B22" s="25"/>
-      <c r="C22" s="25"/>
-      <c r="D22" s="25"/>
-      <c r="E22" s="25"/>
-      <c r="F22" s="25"/>
-      <c r="G22" s="34"/>
-      <c r="H22" s="25"/>
+      <c r="A22" s="28"/>
+      <c r="B22" s="28"/>
+      <c r="C22" s="28"/>
+      <c r="D22" s="28"/>
+      <c r="E22" s="28"/>
+      <c r="F22" s="28"/>
+      <c r="G22" s="37"/>
+      <c r="H22" s="28"/>
     </row>
     <row r="23" spans="1:8">
-      <c r="A23" s="25"/>
-      <c r="B23" s="25"/>
-      <c r="C23" s="25"/>
-      <c r="D23" s="25"/>
-      <c r="E23" s="25"/>
-      <c r="F23" s="25"/>
-      <c r="G23" s="34"/>
-      <c r="H23" s="25"/>
+      <c r="A23" s="28"/>
+      <c r="B23" s="28"/>
+      <c r="C23" s="28"/>
+      <c r="D23" s="28"/>
+      <c r="E23" s="28"/>
+      <c r="F23" s="28"/>
+      <c r="G23" s="37"/>
+      <c r="H23" s="28"/>
     </row>
     <row r="24" spans="1:8">
-      <c r="A24" s="25"/>
-      <c r="B24" s="25"/>
-      <c r="C24" s="25"/>
-      <c r="D24" s="25"/>
-      <c r="E24" s="25"/>
-      <c r="F24" s="25"/>
-      <c r="G24" s="34"/>
-      <c r="H24" s="25"/>
+      <c r="A24" s="28"/>
+      <c r="B24" s="28"/>
+      <c r="C24" s="28"/>
+      <c r="D24" s="28"/>
+      <c r="E24" s="28"/>
+      <c r="F24" s="28"/>
+      <c r="G24" s="37"/>
+      <c r="H24" s="28"/>
     </row>
     <row r="25" spans="1:8">
-      <c r="A25" s="25"/>
-      <c r="B25" s="25"/>
-      <c r="C25" s="25"/>
-      <c r="D25" s="25"/>
-      <c r="E25" s="25"/>
-      <c r="F25" s="25"/>
-      <c r="G25" s="34"/>
-      <c r="H25" s="25"/>
+      <c r="A25" s="28"/>
+      <c r="B25" s="28"/>
+      <c r="C25" s="28"/>
+      <c r="D25" s="28"/>
+      <c r="E25" s="28"/>
+      <c r="F25" s="28"/>
+      <c r="G25" s="37"/>
+      <c r="H25" s="28"/>
     </row>
     <row r="26" spans="1:8">
-      <c r="A26" s="25"/>
-      <c r="B26" s="25"/>
-      <c r="C26" s="25"/>
-      <c r="D26" s="25"/>
-      <c r="E26" s="25"/>
-      <c r="F26" s="25"/>
-      <c r="G26" s="34"/>
-      <c r="H26" s="25"/>
+      <c r="A26" s="28"/>
+      <c r="B26" s="28"/>
+      <c r="C26" s="28"/>
+      <c r="D26" s="28"/>
+      <c r="E26" s="28"/>
+      <c r="F26" s="28"/>
+      <c r="G26" s="37"/>
+      <c r="H26" s="28"/>
     </row>
     <row r="27" spans="1:8">
-      <c r="A27" s="25"/>
-      <c r="B27" s="25"/>
-      <c r="C27" s="25"/>
-      <c r="D27" s="25"/>
-      <c r="E27" s="25"/>
-      <c r="F27" s="25"/>
-      <c r="G27" s="34"/>
-      <c r="H27" s="25"/>
+      <c r="A27" s="28"/>
+      <c r="B27" s="28"/>
+      <c r="C27" s="28"/>
+      <c r="D27" s="28"/>
+      <c r="E27" s="28"/>
+      <c r="F27" s="28"/>
+      <c r="G27" s="37"/>
+      <c r="H27" s="28"/>
     </row>
     <row r="28" spans="1:8">
-      <c r="A28" s="25"/>
-      <c r="B28" s="25"/>
-      <c r="C28" s="25"/>
-      <c r="D28" s="25"/>
-      <c r="E28" s="25"/>
-      <c r="F28" s="25"/>
-      <c r="G28" s="34"/>
-      <c r="H28" s="25"/>
+      <c r="A28" s="28"/>
+      <c r="B28" s="28"/>
+      <c r="C28" s="28"/>
+      <c r="D28" s="28"/>
+      <c r="E28" s="28"/>
+      <c r="F28" s="28"/>
+      <c r="G28" s="37"/>
+      <c r="H28" s="28"/>
     </row>
     <row r="29" spans="1:8">
-      <c r="A29" s="25"/>
-      <c r="B29" s="25"/>
-      <c r="C29" s="25"/>
-      <c r="D29" s="25"/>
-      <c r="E29" s="25"/>
-      <c r="F29" s="25"/>
-      <c r="G29" s="34"/>
-      <c r="H29" s="25"/>
+      <c r="A29" s="28"/>
+      <c r="B29" s="28"/>
+      <c r="C29" s="28"/>
+      <c r="D29" s="28"/>
+      <c r="E29" s="28"/>
+      <c r="F29" s="28"/>
+      <c r="G29" s="37"/>
+      <c r="H29" s="28"/>
     </row>
     <row r="30" spans="1:8">
-      <c r="A30" s="25"/>
-      <c r="B30" s="25"/>
-      <c r="C30" s="25"/>
-      <c r="D30" s="25"/>
-      <c r="E30" s="25"/>
-      <c r="F30" s="25"/>
-      <c r="G30" s="34"/>
-      <c r="H30" s="25"/>
+      <c r="A30" s="28"/>
+      <c r="B30" s="28"/>
+      <c r="C30" s="28"/>
+      <c r="D30" s="28"/>
+      <c r="E30" s="28"/>
+      <c r="F30" s="28"/>
+      <c r="G30" s="37"/>
+      <c r="H30" s="28"/>
     </row>
     <row r="31" spans="1:8">
-      <c r="A31" s="25"/>
-      <c r="B31" s="25"/>
-      <c r="C31" s="25"/>
-      <c r="D31" s="25"/>
-      <c r="E31" s="25"/>
-      <c r="F31" s="25"/>
-      <c r="G31" s="34"/>
-      <c r="H31" s="25"/>
+      <c r="A31" s="28"/>
+      <c r="B31" s="28"/>
+      <c r="C31" s="28"/>
+      <c r="D31" s="28"/>
+      <c r="E31" s="28"/>
+      <c r="F31" s="28"/>
+      <c r="G31" s="37"/>
+      <c r="H31" s="28"/>
     </row>
     <row r="32" spans="1:8">
-      <c r="A32" s="25"/>
-      <c r="B32" s="25"/>
-      <c r="C32" s="25"/>
-      <c r="D32" s="25"/>
-      <c r="E32" s="25"/>
-      <c r="F32" s="25"/>
-      <c r="G32" s="34"/>
-      <c r="H32" s="25"/>
+      <c r="A32" s="28"/>
+      <c r="B32" s="28"/>
+      <c r="C32" s="28"/>
+      <c r="D32" s="28"/>
+      <c r="E32" s="28"/>
+      <c r="F32" s="28"/>
+      <c r="G32" s="37"/>
+      <c r="H32" s="28"/>
     </row>
     <row r="33" spans="1:8">
-      <c r="A33" s="25"/>
-      <c r="B33" s="25"/>
-      <c r="C33" s="25"/>
-      <c r="D33" s="25"/>
-      <c r="E33" s="25"/>
-      <c r="F33" s="25"/>
-      <c r="G33" s="34"/>
-      <c r="H33" s="25"/>
+      <c r="A33" s="28"/>
+      <c r="B33" s="28"/>
+      <c r="C33" s="28"/>
+      <c r="D33" s="28"/>
+      <c r="E33" s="28"/>
+      <c r="F33" s="28"/>
+      <c r="G33" s="37"/>
+      <c r="H33" s="28"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4414,73 +4418,73 @@
   </cols>
   <sheetData>
     <row r="2" ht="18" spans="1:20">
-      <c r="A2" s="23" t="s">
+      <c r="A2" s="26" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="24" t="s">
+      <c r="B2" s="27" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="24" t="s">
+      <c r="C2" s="27" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="24"/>
-      <c r="E2" s="24" t="s">
+      <c r="D2" s="27"/>
+      <c r="E2" s="27" t="s">
         <v>19</v>
       </c>
-      <c r="F2" s="24" t="s">
+      <c r="F2" s="27" t="s">
         <v>20</v>
       </c>
-      <c r="G2" s="24" t="s">
+      <c r="G2" s="27" t="s">
         <v>21</v>
       </c>
-      <c r="H2" s="24" t="s">
+      <c r="H2" s="27" t="s">
         <v>22</v>
       </c>
-      <c r="I2" s="24" t="s">
+      <c r="I2" s="27" t="s">
         <v>5</v>
       </c>
-      <c r="J2" s="23" t="s">
+      <c r="J2" s="26" t="s">
         <v>23</v>
       </c>
-      <c r="L2" s="23" t="s">
+      <c r="L2" s="26" t="s">
         <v>8</v>
       </c>
-      <c r="M2" s="23" t="s">
+      <c r="M2" s="26" t="s">
         <v>9</v>
       </c>
-      <c r="N2" s="23" t="s">
+      <c r="N2" s="26" t="s">
         <v>10</v>
       </c>
-      <c r="O2" s="23" t="s">
+      <c r="O2" s="26" t="s">
         <v>11</v>
       </c>
-      <c r="P2" s="23" t="s">
+      <c r="P2" s="26" t="s">
         <v>12</v>
       </c>
-      <c r="Q2" s="23" t="s">
+      <c r="Q2" s="26" t="s">
         <v>13</v>
       </c>
-      <c r="R2" s="23" t="s">
+      <c r="R2" s="26" t="s">
         <v>14</v>
       </c>
-      <c r="S2" s="23" t="s">
+      <c r="S2" s="26" t="s">
         <v>15</v>
       </c>
-      <c r="T2" s="23" t="s">
+      <c r="T2" s="26" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="3" spans="1:21">
-      <c r="A3" s="25">
+      <c r="A3" s="28">
         <v>1</v>
       </c>
-      <c r="B3" s="25">
+      <c r="B3" s="28">
         <v>72</v>
       </c>
-      <c r="C3" s="25">
+      <c r="C3" s="28">
         <v>400000</v>
       </c>
-      <c r="D3" s="25" t="s">
+      <c r="D3" s="28" t="s">
         <v>24</v>
       </c>
       <c r="E3" s="4">
@@ -4503,53 +4507,53 @@
         <f>(B3*0.5*POWER(10,10))/(2*C3*I3*H3)</f>
         <v>2.22222222222222</v>
       </c>
-      <c r="L3" s="26">
+      <c r="L3" s="29">
         <f>B3/J3</f>
         <v>32.4</v>
       </c>
       <c r="M3" s="4">
         <v>216</v>
       </c>
-      <c r="N3" s="29">
+      <c r="N3" s="32">
         <v>0.5</v>
       </c>
       <c r="O3" s="4">
         <f>M3*N3</f>
         <v>108</v>
       </c>
-      <c r="P3" s="30">
+      <c r="P3" s="33">
         <f>O3/B3</f>
         <v>1.5</v>
       </c>
-      <c r="Q3" s="26">
+      <c r="Q3" s="29">
         <f>M3/L3</f>
         <v>6.66666666666667</v>
       </c>
-      <c r="R3" s="30">
+      <c r="R3" s="33">
         <v>2.5</v>
       </c>
-      <c r="S3" s="29">
+      <c r="S3" s="32">
         <f>SQRT((P3*0.9/(R3+5))/0.9)</f>
         <v>0.447213595499958</v>
       </c>
-      <c r="T3" s="29">
+      <c r="T3" s="32">
         <f>SQRT((N3*0.9/(R3+5))/0.9)</f>
         <v>0.258198889747161</v>
       </c>
-      <c r="U3" s="30">
+      <c r="U3" s="33">
         <f>P3/R3</f>
         <v>0.6</v>
       </c>
     </row>
     <row r="4" spans="1:20">
-      <c r="A4" s="25"/>
-      <c r="B4" s="25">
+      <c r="A4" s="28"/>
+      <c r="B4" s="28">
         <v>72</v>
       </c>
-      <c r="C4" s="25">
+      <c r="C4" s="28">
         <v>400000</v>
       </c>
-      <c r="D4" s="25" t="s">
+      <c r="D4" s="28" t="s">
         <v>24</v>
       </c>
       <c r="E4" s="4">
@@ -4572,48 +4576,48 @@
         <f t="shared" ref="J4:J9" si="1">(B4*0.5*POWER(10,10))/(2*C4*I4*H4)</f>
         <v>10.0840336134454</v>
       </c>
-      <c r="L4" s="26">
+      <c r="L4" s="29">
         <f t="shared" ref="L4:L9" si="2">B4/J4</f>
         <v>7.14</v>
       </c>
       <c r="M4" s="4">
         <v>216</v>
       </c>
-      <c r="N4" s="29">
+      <c r="N4" s="32">
         <v>0.5</v>
       </c>
       <c r="O4" s="4">
         <f t="shared" ref="O4:O9" si="3">M4*N4</f>
         <v>108</v>
       </c>
-      <c r="P4" s="30">
+      <c r="P4" s="33">
         <f t="shared" ref="P4:P9" si="4">O4/B4</f>
         <v>1.5</v>
       </c>
-      <c r="Q4" s="26">
+      <c r="Q4" s="29">
         <f t="shared" ref="Q4:Q9" si="5">M4/L4</f>
         <v>30.2521008403361</v>
       </c>
-      <c r="R4" s="30">
+      <c r="R4" s="33">
         <v>2.5</v>
       </c>
-      <c r="S4" s="29">
+      <c r="S4" s="32">
         <f t="shared" ref="S4:S9" si="6">SQRT((P4*0.9/(R4+5))/0.9)</f>
         <v>0.447213595499958</v>
       </c>
-      <c r="T4" s="29">
+      <c r="T4" s="32">
         <f t="shared" ref="T4:T9" si="7">SQRT((N4*0.9/(R4+5))/0.9)</f>
         <v>0.258198889747161</v>
       </c>
     </row>
     <row r="5" spans="2:20">
-      <c r="B5" s="25">
+      <c r="B5" s="28">
         <v>72</v>
       </c>
-      <c r="C5" s="25">
+      <c r="C5" s="28">
         <v>400000</v>
       </c>
-      <c r="D5" s="25"/>
+      <c r="D5" s="28"/>
       <c r="E5" s="4">
         <v>23.13</v>
       </c>
@@ -4634,48 +4638,48 @@
         <f t="shared" si="1"/>
         <v>6.18454687886534</v>
       </c>
-      <c r="L5" s="26">
+      <c r="L5" s="29">
         <f t="shared" si="2"/>
         <v>11.64192</v>
       </c>
       <c r="M5" s="4">
         <v>216</v>
       </c>
-      <c r="N5" s="29">
+      <c r="N5" s="32">
         <v>0.5</v>
       </c>
       <c r="O5" s="4">
         <f t="shared" si="3"/>
         <v>108</v>
       </c>
-      <c r="P5" s="30">
+      <c r="P5" s="33">
         <f t="shared" si="4"/>
         <v>1.5</v>
       </c>
-      <c r="Q5" s="26">
+      <c r="Q5" s="29">
         <f t="shared" si="5"/>
         <v>18.553640636596</v>
       </c>
-      <c r="R5" s="30">
+      <c r="R5" s="33">
         <v>2.5</v>
       </c>
-      <c r="S5" s="29">
+      <c r="S5" s="32">
         <f t="shared" si="6"/>
         <v>0.447213595499958</v>
       </c>
-      <c r="T5" s="29">
+      <c r="T5" s="32">
         <f t="shared" si="7"/>
         <v>0.258198889747161</v>
       </c>
     </row>
     <row r="6" spans="2:20">
-      <c r="B6" s="25">
+      <c r="B6" s="28">
         <v>72</v>
       </c>
-      <c r="C6" s="25">
+      <c r="C6" s="28">
         <v>400000</v>
       </c>
-      <c r="D6" s="25"/>
+      <c r="D6" s="28"/>
       <c r="E6" s="4">
         <v>23.13</v>
       </c>
@@ -4696,45 +4700,45 @@
         <f t="shared" si="1"/>
         <v>10.6020803637692</v>
       </c>
-      <c r="L6" s="26">
+      <c r="L6" s="29">
         <f t="shared" si="2"/>
         <v>6.79112</v>
       </c>
       <c r="M6" s="4">
         <v>216</v>
       </c>
-      <c r="N6" s="29">
+      <c r="N6" s="32">
         <v>0.5</v>
       </c>
       <c r="O6" s="4">
         <f t="shared" si="3"/>
         <v>108</v>
       </c>
-      <c r="P6" s="30">
+      <c r="P6" s="33">
         <f t="shared" si="4"/>
         <v>1.5</v>
       </c>
-      <c r="Q6" s="26">
+      <c r="Q6" s="29">
         <f t="shared" si="5"/>
         <v>31.8062410913075</v>
       </c>
-      <c r="R6" s="30">
+      <c r="R6" s="33">
         <v>2.5</v>
       </c>
-      <c r="S6" s="29">
+      <c r="S6" s="32">
         <f t="shared" si="6"/>
         <v>0.447213595499958</v>
       </c>
-      <c r="T6" s="29">
+      <c r="T6" s="32">
         <f t="shared" si="7"/>
         <v>0.258198889747161</v>
       </c>
     </row>
     <row r="7" spans="2:20">
-      <c r="B7" s="25">
+      <c r="B7" s="28">
         <v>72</v>
       </c>
-      <c r="C7" s="25">
+      <c r="C7" s="28">
         <v>400000</v>
       </c>
       <c r="D7" s="4" t="s">
@@ -4760,45 +4764,45 @@
         <f t="shared" si="1"/>
         <v>9.95867151322014</v>
       </c>
-      <c r="L7" s="26">
+      <c r="L7" s="29">
         <f t="shared" si="2"/>
         <v>7.22988</v>
       </c>
       <c r="M7" s="4">
         <v>216</v>
       </c>
-      <c r="N7" s="29">
+      <c r="N7" s="32">
         <v>0.5</v>
       </c>
       <c r="O7" s="4">
         <f t="shared" si="3"/>
         <v>108</v>
       </c>
-      <c r="P7" s="30">
+      <c r="P7" s="33">
         <f t="shared" si="4"/>
         <v>1.5</v>
       </c>
-      <c r="Q7" s="26">
+      <c r="Q7" s="29">
         <f t="shared" si="5"/>
         <v>29.8760145396604</v>
       </c>
-      <c r="R7" s="30">
+      <c r="R7" s="33">
         <v>2.5</v>
       </c>
-      <c r="S7" s="29">
+      <c r="S7" s="32">
         <f t="shared" si="6"/>
         <v>0.447213595499958</v>
       </c>
-      <c r="T7" s="29">
+      <c r="T7" s="32">
         <f t="shared" si="7"/>
         <v>0.258198889747161</v>
       </c>
     </row>
     <row r="8" spans="2:20">
-      <c r="B8" s="25">
+      <c r="B8" s="28">
         <v>72</v>
       </c>
-      <c r="C8" s="25">
+      <c r="C8" s="28">
         <v>400000</v>
       </c>
       <c r="D8" s="4" t="s">
@@ -4824,45 +4828,45 @@
         <f t="shared" si="1"/>
         <v>32.798833819242</v>
       </c>
-      <c r="L8" s="26">
+      <c r="L8" s="29">
         <f t="shared" si="2"/>
         <v>2.1952</v>
       </c>
       <c r="M8" s="4">
         <v>216</v>
       </c>
-      <c r="N8" s="29">
+      <c r="N8" s="32">
         <v>0.5</v>
       </c>
       <c r="O8" s="4">
         <f t="shared" si="3"/>
         <v>108</v>
       </c>
-      <c r="P8" s="30">
+      <c r="P8" s="33">
         <f t="shared" si="4"/>
         <v>1.5</v>
       </c>
-      <c r="Q8" s="26">
+      <c r="Q8" s="29">
         <f t="shared" si="5"/>
         <v>98.396501457726</v>
       </c>
-      <c r="R8" s="30">
+      <c r="R8" s="33">
         <v>2.5</v>
       </c>
-      <c r="S8" s="29">
+      <c r="S8" s="32">
         <f t="shared" si="6"/>
         <v>0.447213595499958</v>
       </c>
-      <c r="T8" s="29">
+      <c r="T8" s="32">
         <f t="shared" si="7"/>
         <v>0.258198889747161</v>
       </c>
     </row>
     <row r="9" spans="2:20">
-      <c r="B9" s="25">
+      <c r="B9" s="28">
         <v>72</v>
       </c>
-      <c r="C9" s="25">
+      <c r="C9" s="28">
         <v>400000</v>
       </c>
       <c r="E9" s="4">
@@ -4885,48 +4889,48 @@
         <f t="shared" si="1"/>
         <v>9.9756704481847</v>
       </c>
-      <c r="L9" s="26">
+      <c r="L9" s="29">
         <f t="shared" si="2"/>
         <v>7.21756</v>
       </c>
       <c r="M9" s="4">
         <v>216</v>
       </c>
-      <c r="N9" s="29">
+      <c r="N9" s="32">
         <v>0.5</v>
       </c>
       <c r="O9" s="4">
         <f t="shared" si="3"/>
         <v>108</v>
       </c>
-      <c r="P9" s="30">
+      <c r="P9" s="33">
         <f t="shared" si="4"/>
         <v>1.5</v>
       </c>
-      <c r="Q9" s="26">
+      <c r="Q9" s="29">
         <f t="shared" si="5"/>
         <v>29.9270113445541</v>
       </c>
-      <c r="R9" s="30">
+      <c r="R9" s="33">
         <v>2.5</v>
       </c>
-      <c r="S9" s="29">
+      <c r="S9" s="32">
         <f t="shared" si="6"/>
         <v>0.447213595499958</v>
       </c>
-      <c r="T9" s="29">
+      <c r="T9" s="32">
         <f t="shared" si="7"/>
         <v>0.258198889747161</v>
       </c>
     </row>
     <row r="10" spans="10:10">
-      <c r="J10" s="27"/>
+      <c r="J10" s="30"/>
     </row>
     <row r="11" spans="10:10">
-      <c r="J11" s="26"/>
+      <c r="J11" s="29"/>
     </row>
     <row r="12" spans="10:10">
-      <c r="J12" s="28"/>
+      <c r="J12" s="31"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4944,7 +4948,9 @@
     <col min="2" max="2" width="15.5625" style="5" customWidth="1"/>
     <col min="3" max="3" width="15.5625" style="4" customWidth="1"/>
     <col min="4" max="4" width="5.5625" style="4" customWidth="1"/>
-    <col min="5" max="12" width="18.5625" style="4" customWidth="1"/>
+    <col min="5" max="5" width="18.5625" style="4" customWidth="1"/>
+    <col min="6" max="6" width="34.6015625" style="4" customWidth="1"/>
+    <col min="7" max="12" width="18.5625" style="4" customWidth="1"/>
     <col min="13" max="13" width="5.2265625" style="4" customWidth="1"/>
     <col min="14" max="14" width="25.4375" style="4" customWidth="1"/>
     <col min="15" max="17" width="5.5625" style="4" customWidth="1"/>
@@ -5024,7 +5030,7 @@
       <c r="N8" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="O8" s="20">
+      <c r="O8" s="23">
         <v>1.4</v>
       </c>
       <c r="P8" s="7"/>
@@ -5058,15 +5064,15 @@
       <c r="N9" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="O9" s="20">
+      <c r="O9" s="23">
         <v>0.707</v>
       </c>
-      <c r="P9" s="21"/>
+      <c r="P9" s="24"/>
       <c r="S9" s="7"/>
       <c r="T9" s="9"/>
       <c r="U9" s="9"/>
-      <c r="V9" s="22"/>
-      <c r="W9" s="22"/>
+      <c r="V9" s="25"/>
+      <c r="W9" s="25"/>
       <c r="X9" s="7"/>
     </row>
     <row r="10" ht="18" spans="2:24">
@@ -5095,7 +5101,7 @@
       <c r="N10" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="O10" s="20">
+      <c r="O10" s="23">
         <v>0.3</v>
       </c>
       <c r="P10" s="7"/>
@@ -5137,10 +5143,10 @@
       <c r="G12" s="17"/>
       <c r="H12" s="17"/>
       <c r="I12" s="17"/>
-      <c r="J12" s="18"/>
-      <c r="K12" s="18"/>
-      <c r="L12" s="19"/>
-      <c r="M12" s="19"/>
+      <c r="J12" s="21"/>
+      <c r="K12" s="21"/>
+      <c r="L12" s="22"/>
+      <c r="M12" s="22"/>
       <c r="N12" s="7"/>
       <c r="O12" s="7"/>
       <c r="P12" s="7"/>
@@ -5162,6 +5168,14 @@
       </c>
       <c r="D13" s="7" t="s">
         <v>34</v>
+      </c>
+      <c r="F13" s="18">
+        <f>SQRT(C13*C15*10^-(15))</f>
+        <v>3.95727178748188e-7</v>
+      </c>
+      <c r="G13" s="19">
+        <f>C13*C15</f>
+        <v>156.6</v>
       </c>
       <c r="J13" s="9"/>
       <c r="K13" s="9"/>
@@ -5190,7 +5204,10 @@
         <v>37</v>
       </c>
       <c r="E14" s="15"/>
-      <c r="F14" s="7"/>
+      <c r="F14" s="20">
+        <f>2*3.14*F13</f>
+        <v>2.48516668253862e-6</v>
+      </c>
       <c r="G14" s="7"/>
       <c r="H14" s="7"/>
       <c r="I14" s="7"/>
@@ -5222,7 +5239,10 @@
         <v>37</v>
       </c>
       <c r="E15" s="7"/>
-      <c r="F15" s="15"/>
+      <c r="F15" s="20">
+        <f>1/F14</f>
+        <v>402387.496591775</v>
+      </c>
       <c r="G15" s="15"/>
       <c r="H15" s="15"/>
       <c r="I15" s="15"/>
@@ -5248,13 +5268,19 @@
         <v>45</v>
       </c>
       <c r="C16" s="9">
-        <f>C5*SQRT((C15/(POWER(10,9))/(C13/POWER(10,6))))</f>
+        <f>C5*SQRT((C15*(POWER(10,-9))/(C13*POWER(10,-6))))</f>
         <v>0.682288239221013</v>
       </c>
       <c r="D16" s="7"/>
       <c r="E16" s="7"/>
-      <c r="F16" s="7"/>
-      <c r="G16" s="7"/>
+      <c r="F16" s="11">
+        <f>(C15*POWER(10,-9))/(C13*POWER(10,-6))</f>
+        <v>0.000186206896551724</v>
+      </c>
+      <c r="G16" s="11">
+        <f>SQRT(F16)</f>
+        <v>0.0136457647844203</v>
+      </c>
       <c r="H16" s="7"/>
       <c r="I16" s="7"/>
       <c r="J16" s="7"/>
@@ -5287,7 +5313,10 @@
       </c>
       <c r="E17" s="7"/>
       <c r="F17" s="7"/>
-      <c r="G17" s="7"/>
+      <c r="G17" s="7">
+        <f>50/G16</f>
+        <v>3664.1405439647</v>
+      </c>
       <c r="H17" s="7"/>
       <c r="I17" s="7"/>
       <c r="J17" s="7"/>

</xml_diff>

<commit_message>
modified:   Ferrite Transformer Calculation.xlsx 	modified:   log.md
</commit_message>
<xml_diff>
--- a/Ferrite Transformer Calculation.xlsx
+++ b/Ferrite Transformer Calculation.xlsx
@@ -4,13 +4,14 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="28800" windowHeight="13060" activeTab="2"/>
+    <workbookView windowWidth="28800" windowHeight="13060" activeTab="4"/>
   </bookViews>
   <sheets>
     <sheet name="ETD" sheetId="1" r:id="rId1"/>
     <sheet name="Toroid" sheetId="2" r:id="rId2"/>
     <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
     <sheet name="Sheet1" sheetId="4" r:id="rId4"/>
+    <sheet name="Sheet2" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -30,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="66">
   <si>
     <t>#</t>
   </si>
@@ -1575,32 +1576,45 @@
   </si>
   <si>
     <t>Very high attenuation</t>
+  </si>
+  <si>
+    <t>S</t>
+  </si>
+  <si>
+    <t>RBTL</t>
+  </si>
+  <si>
+    <t>LBTL</t>
+  </si>
+  <si>
+    <t>CBTL</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
-  <numFmts count="19">
+  <numFmts count="20">
     <numFmt numFmtId="41" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;_);_(@_)"/>
     <numFmt numFmtId="42" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
     <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="178" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="179" formatCode="_ * #,##0.0000_ ;_ * \-#,##0.0000_ ;_ * &quot;-&quot;??.0000_ ;_ @_ "/>
-    <numFmt numFmtId="180" formatCode="0.0000_ "/>
-    <numFmt numFmtId="181" formatCode="_ * #,##0.0000000_ ;_ * \-#,##0.0000000_ ;_ * &quot;-&quot;??.0000000_ ;_ @_ "/>
-    <numFmt numFmtId="182" formatCode="_ * #,##0.0_ ;_ * \-#,##0.0_ ;_ * &quot;-&quot;??.0_ ;_ @_ "/>
-    <numFmt numFmtId="183" formatCode="_ * #,##0.000000000000_ ;_ * \-#,##0.000000000000_ ;_ * &quot;-&quot;??.000000000000_ ;_ @_ "/>
-    <numFmt numFmtId="184" formatCode="0.0000000000E+00"/>
-    <numFmt numFmtId="185" formatCode="_ * #,##0.00000000000000_ ;_ * \-#,##0.00000000000000_ ;_ * &quot;-&quot;??.00000000000000_ ;_ @_ "/>
-    <numFmt numFmtId="186" formatCode="_ * #,##0.000_ ;_ * \-#,##0.000_ ;_ * &quot;-&quot;??.000_ ;_ @_ "/>
-    <numFmt numFmtId="187" formatCode="_ * #,##0.00000000_ ;_ * \-#,##0.00000000_ ;_ * &quot;-&quot;??.00000000_ ;_ @_ "/>
-    <numFmt numFmtId="188" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??.00_ ;_ @_ "/>
-    <numFmt numFmtId="189" formatCode="0.00_ "/>
-    <numFmt numFmtId="190" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;_);_(@_)"/>
-    <numFmt numFmtId="191" formatCode="_(* #,##0.0000_);_(* \(#,##0.0000\);_(* &quot;-&quot;_);_(@_)"/>
+    <numFmt numFmtId="178" formatCode="0.000000_ "/>
+    <numFmt numFmtId="179" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="180" formatCode="_ * #,##0.0000_ ;_ * \-#,##0.0000_ ;_ * &quot;-&quot;??.0000_ ;_ @_ "/>
+    <numFmt numFmtId="181" formatCode="0.0000_ "/>
+    <numFmt numFmtId="182" formatCode="_ * #,##0.0000000_ ;_ * \-#,##0.0000000_ ;_ * &quot;-&quot;??.0000000_ ;_ @_ "/>
+    <numFmt numFmtId="183" formatCode="_ * #,##0.0_ ;_ * \-#,##0.0_ ;_ * &quot;-&quot;??.0_ ;_ @_ "/>
+    <numFmt numFmtId="184" formatCode="_ * #,##0.000000000000_ ;_ * \-#,##0.000000000000_ ;_ * &quot;-&quot;??.000000000000_ ;_ @_ "/>
+    <numFmt numFmtId="185" formatCode="0.0000000000E+00"/>
+    <numFmt numFmtId="186" formatCode="_ * #,##0.00000000000000_ ;_ * \-#,##0.00000000000000_ ;_ * &quot;-&quot;??.00000000000000_ ;_ @_ "/>
+    <numFmt numFmtId="187" formatCode="_ * #,##0.000_ ;_ * \-#,##0.000_ ;_ * &quot;-&quot;??.000_ ;_ @_ "/>
+    <numFmt numFmtId="188" formatCode="_ * #,##0.00000000_ ;_ * \-#,##0.00000000_ ;_ * &quot;-&quot;??.00000000_ ;_ @_ "/>
+    <numFmt numFmtId="189" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??.00_ ;_ @_ "/>
+    <numFmt numFmtId="190" formatCode="0.00_ "/>
+    <numFmt numFmtId="191" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;_);_(@_)"/>
+    <numFmt numFmtId="192" formatCode="_(* #,##0.0000_);_(* \(#,##0.0000\);_(* &quot;-&quot;_);_(@_)"/>
   </numFmts>
   <fonts count="31">
     <font>
@@ -2286,8 +2300,11 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="178" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1">
@@ -2308,61 +2325,61 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="178" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1">
+    <xf numFmtId="179" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="179" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="180" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="181" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="178" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="182" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="178" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1">
+    <xf numFmtId="179" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="183" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="183" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1">
+    <xf numFmtId="184" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="184" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="185" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="179" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1">
+    <xf numFmtId="185" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="183" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="186" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="180" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="186" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="187" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="188" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="189" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -2383,10 +2400,10 @@
     <xf numFmtId="176" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="189" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="190" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="191" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -2395,16 +2412,16 @@
     <xf numFmtId="41" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="191" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1">
+    <xf numFmtId="192" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="41" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="191" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="192" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="180" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1">
+    <xf numFmtId="181" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -3925,471 +3942,471 @@
   <dimension ref="A1:U33"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="5.5625" style="29" customWidth="1"/>
-    <col min="2" max="4" width="10.5625" style="29" customWidth="1"/>
-    <col min="5" max="5" width="20.5625" style="29" customWidth="1"/>
-    <col min="6" max="6" width="15.5625" style="29" customWidth="1"/>
-    <col min="7" max="7" width="30.5625" style="35" customWidth="1"/>
-    <col min="8" max="8" width="10.5625" style="29" customWidth="1"/>
-    <col min="9" max="9" width="15.5625" style="4" customWidth="1"/>
-    <col min="10" max="13" width="10.5625" style="4" customWidth="1"/>
-    <col min="14" max="14" width="9" style="4"/>
-    <col min="15" max="15" width="20.5625" style="4" customWidth="1"/>
-    <col min="16" max="17" width="10.5625" style="4" customWidth="1"/>
-    <col min="18" max="16384" width="9" style="4"/>
+    <col min="1" max="1" width="5.5625" style="30" customWidth="1"/>
+    <col min="2" max="4" width="10.5625" style="30" customWidth="1"/>
+    <col min="5" max="5" width="20.5625" style="30" customWidth="1"/>
+    <col min="6" max="6" width="15.5625" style="30" customWidth="1"/>
+    <col min="7" max="7" width="30.5625" style="36" customWidth="1"/>
+    <col min="8" max="8" width="10.5625" style="30" customWidth="1"/>
+    <col min="9" max="9" width="15.5625" style="5" customWidth="1"/>
+    <col min="10" max="13" width="10.5625" style="5" customWidth="1"/>
+    <col min="14" max="14" width="9" style="5"/>
+    <col min="15" max="15" width="20.5625" style="5" customWidth="1"/>
+    <col min="16" max="17" width="10.5625" style="5" customWidth="1"/>
+    <col min="18" max="16384" width="9" style="5"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8">
-      <c r="A1" s="4"/>
-      <c r="B1" s="4"/>
-      <c r="C1" s="4"/>
-      <c r="D1" s="4"/>
-      <c r="E1" s="4"/>
-      <c r="F1" s="4"/>
-      <c r="G1" s="26"/>
-      <c r="H1" s="4"/>
-    </row>
-    <row r="2" s="34" customFormat="1" ht="18" spans="1:21">
-      <c r="A2" s="26" t="s">
+      <c r="A1" s="5"/>
+      <c r="B1" s="5"/>
+      <c r="C1" s="5"/>
+      <c r="D1" s="5"/>
+      <c r="E1" s="5"/>
+      <c r="F1" s="5"/>
+      <c r="G1" s="27"/>
+      <c r="H1" s="5"/>
+    </row>
+    <row r="2" s="35" customFormat="1" ht="18" spans="1:21">
+      <c r="A2" s="27" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="27" t="s">
+      <c r="B2" s="28" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="27" t="s">
+      <c r="C2" s="28" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="27" t="s">
+      <c r="D2" s="28" t="s">
         <v>3</v>
       </c>
-      <c r="E2" s="27" t="s">
+      <c r="E2" s="28" t="s">
         <v>4</v>
       </c>
-      <c r="F2" s="27" t="s">
+      <c r="F2" s="28" t="s">
         <v>5</v>
       </c>
-      <c r="G2" s="26" t="s">
+      <c r="G2" s="27" t="s">
         <v>6</v>
       </c>
-      <c r="H2" s="27" t="s">
+      <c r="H2" s="28" t="s">
         <v>7</v>
       </c>
-      <c r="I2" s="26" t="s">
+      <c r="I2" s="27" t="s">
         <v>8</v>
       </c>
-      <c r="J2" s="26" t="s">
+      <c r="J2" s="27" t="s">
         <v>9</v>
       </c>
-      <c r="K2" s="26" t="s">
+      <c r="K2" s="27" t="s">
         <v>10</v>
       </c>
-      <c r="L2" s="26" t="s">
+      <c r="L2" s="27" t="s">
         <v>11</v>
       </c>
-      <c r="M2" s="26" t="s">
+      <c r="M2" s="27" t="s">
         <v>12</v>
       </c>
-      <c r="N2" s="26" t="s">
+      <c r="N2" s="27" t="s">
         <v>13</v>
       </c>
-      <c r="O2" s="26" t="s">
+      <c r="O2" s="27" t="s">
         <v>14</v>
       </c>
-      <c r="P2" s="26" t="s">
+      <c r="P2" s="27" t="s">
         <v>15</v>
       </c>
-      <c r="Q2" s="26" t="s">
+      <c r="Q2" s="27" t="s">
         <v>16</v>
       </c>
-      <c r="R2" s="26" t="s">
+      <c r="R2" s="27" t="s">
         <v>17</v>
       </c>
-      <c r="S2" s="26" t="s">
+      <c r="S2" s="27" t="s">
         <v>18</v>
       </c>
-      <c r="T2" s="26" t="s">
+      <c r="T2" s="27" t="s">
         <v>17</v>
       </c>
-      <c r="U2" s="26" t="s">
+      <c r="U2" s="27" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="3" spans="1:21">
-      <c r="A3" s="28">
+      <c r="A3" s="29">
         <v>1</v>
       </c>
-      <c r="B3" s="28">
+      <c r="B3" s="29">
         <v>72</v>
       </c>
-      <c r="C3" s="28">
+      <c r="C3" s="29">
         <v>400000</v>
       </c>
-      <c r="D3" s="28">
+      <c r="D3" s="29">
         <v>10</v>
       </c>
-      <c r="E3" s="36">
+      <c r="E3" s="37">
         <f>3.14*POWER(D3,2)/4</f>
         <v>78.5</v>
       </c>
-      <c r="F3" s="36">
+      <c r="F3" s="37">
         <v>1898.58</v>
       </c>
-      <c r="G3" s="37">
+      <c r="G3" s="38">
         <f>(B3*POWER(10,10))/(4*C3*F3*E3)</f>
         <v>3.01935345175506</v>
       </c>
-      <c r="H3" s="38" t="str">
+      <c r="H3" s="39" t="str">
         <f>IF((B3*POWER(10,10))/(4*C3*G3*E3)&gt;1200,IF((B3*POWER(10,10))/(4*C3*G3*E3)&lt;2000,"OK","NG"),"NG")</f>
         <v>OK</v>
       </c>
-      <c r="I3" s="29">
+      <c r="I3" s="30">
         <f>B3/G3</f>
         <v>23.8461648</v>
       </c>
-      <c r="J3" s="29">
+      <c r="J3" s="30">
         <f>B3*3</f>
         <v>216</v>
       </c>
-      <c r="K3" s="33">
+      <c r="K3" s="34">
         <v>0.5</v>
       </c>
-      <c r="L3" s="29">
+      <c r="L3" s="30">
         <f>J3*K3</f>
         <v>108</v>
       </c>
-      <c r="M3" s="33">
+      <c r="M3" s="34">
         <f>L3/B3</f>
         <v>1.5</v>
       </c>
-      <c r="N3" s="29">
+      <c r="N3" s="30">
         <f>J3/I3</f>
         <v>9.05806035526518</v>
       </c>
-      <c r="O3" s="29">
+      <c r="O3" s="30">
         <v>1.5</v>
       </c>
-      <c r="P3" s="39">
+      <c r="P3" s="40">
         <f>SQRT((M3*0.9/(O3+5))/0.9)</f>
         <v>0.480384461415261</v>
       </c>
-      <c r="Q3" s="39">
+      <c r="Q3" s="40">
         <f>SQRT((K3*0.9/(O3+5))/0.9)</f>
         <v>0.277350098112615</v>
       </c>
-      <c r="R3" s="4">
+      <c r="R3" s="5">
         <v>1</v>
       </c>
-      <c r="S3" s="4">
+      <c r="S3" s="5">
         <v>1</v>
       </c>
-      <c r="T3" s="4">
+      <c r="T3" s="5">
         <f>IF(((M3*0.9/(O3+5)))/(R3*R3*1)&lt;1,1,((M3*0.9/(O3+5))/(R3*R3*1)))</f>
         <v>1</v>
       </c>
-      <c r="U3" s="4">
+      <c r="U3" s="5">
         <f>IF(((K3*0.9/(O3+5)))/(S3*S3*1)&lt;1,1,((K3*0.9/(O3+5))/(S3*S3*1)))</f>
         <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:8">
-      <c r="A4" s="28"/>
-      <c r="B4" s="28"/>
-      <c r="C4" s="28"/>
-      <c r="D4" s="28"/>
-      <c r="E4" s="28"/>
-      <c r="F4" s="28"/>
-      <c r="G4" s="37"/>
-      <c r="H4" s="28"/>
+      <c r="A4" s="29"/>
+      <c r="B4" s="29"/>
+      <c r="C4" s="29"/>
+      <c r="D4" s="29"/>
+      <c r="E4" s="29"/>
+      <c r="F4" s="29"/>
+      <c r="G4" s="38"/>
+      <c r="H4" s="29"/>
     </row>
     <row r="5" spans="1:8">
-      <c r="A5" s="28"/>
-      <c r="B5" s="28"/>
-      <c r="C5" s="28"/>
-      <c r="D5" s="28"/>
-      <c r="E5" s="28"/>
-      <c r="F5" s="28"/>
-      <c r="G5" s="37"/>
-      <c r="H5" s="28"/>
+      <c r="A5" s="29"/>
+      <c r="B5" s="29"/>
+      <c r="C5" s="29"/>
+      <c r="D5" s="29"/>
+      <c r="E5" s="29"/>
+      <c r="F5" s="29"/>
+      <c r="G5" s="38"/>
+      <c r="H5" s="29"/>
     </row>
     <row r="6" spans="1:8">
-      <c r="A6" s="28"/>
-      <c r="B6" s="28"/>
-      <c r="C6" s="28"/>
-      <c r="D6" s="28"/>
-      <c r="E6" s="28"/>
-      <c r="F6" s="28"/>
-      <c r="G6" s="37"/>
-      <c r="H6" s="28"/>
+      <c r="A6" s="29"/>
+      <c r="B6" s="29"/>
+      <c r="C6" s="29"/>
+      <c r="D6" s="29"/>
+      <c r="E6" s="29"/>
+      <c r="F6" s="29"/>
+      <c r="G6" s="38"/>
+      <c r="H6" s="29"/>
     </row>
     <row r="7" spans="1:8">
-      <c r="A7" s="28"/>
-      <c r="B7" s="28"/>
-      <c r="C7" s="28"/>
-      <c r="D7" s="28"/>
-      <c r="E7" s="28"/>
-      <c r="F7" s="28"/>
-      <c r="G7" s="37"/>
-      <c r="H7" s="28"/>
+      <c r="A7" s="29"/>
+      <c r="B7" s="29"/>
+      <c r="C7" s="29"/>
+      <c r="D7" s="29"/>
+      <c r="E7" s="29"/>
+      <c r="F7" s="29"/>
+      <c r="G7" s="38"/>
+      <c r="H7" s="29"/>
     </row>
     <row r="8" spans="1:8">
-      <c r="A8" s="28"/>
-      <c r="B8" s="28"/>
-      <c r="C8" s="28"/>
-      <c r="D8" s="28"/>
-      <c r="E8" s="28"/>
-      <c r="F8" s="28"/>
-      <c r="G8" s="37"/>
-      <c r="H8" s="28"/>
+      <c r="A8" s="29"/>
+      <c r="B8" s="29"/>
+      <c r="C8" s="29"/>
+      <c r="D8" s="29"/>
+      <c r="E8" s="29"/>
+      <c r="F8" s="29"/>
+      <c r="G8" s="38"/>
+      <c r="H8" s="29"/>
     </row>
     <row r="9" spans="1:8">
-      <c r="A9" s="28"/>
-      <c r="B9" s="28"/>
-      <c r="C9" s="28"/>
-      <c r="D9" s="28"/>
-      <c r="E9" s="28"/>
-      <c r="F9" s="28"/>
-      <c r="G9" s="37"/>
-      <c r="H9" s="28"/>
+      <c r="A9" s="29"/>
+      <c r="B9" s="29"/>
+      <c r="C9" s="29"/>
+      <c r="D9" s="29"/>
+      <c r="E9" s="29"/>
+      <c r="F9" s="29"/>
+      <c r="G9" s="38"/>
+      <c r="H9" s="29"/>
     </row>
     <row r="10" spans="1:8">
-      <c r="A10" s="28"/>
-      <c r="B10" s="28"/>
-      <c r="C10" s="28"/>
-      <c r="D10" s="28"/>
-      <c r="E10" s="28"/>
-      <c r="F10" s="28"/>
-      <c r="G10" s="37"/>
-      <c r="H10" s="28"/>
+      <c r="A10" s="29"/>
+      <c r="B10" s="29"/>
+      <c r="C10" s="29"/>
+      <c r="D10" s="29"/>
+      <c r="E10" s="29"/>
+      <c r="F10" s="29"/>
+      <c r="G10" s="38"/>
+      <c r="H10" s="29"/>
     </row>
     <row r="11" spans="1:8">
-      <c r="A11" s="28"/>
-      <c r="B11" s="28"/>
-      <c r="C11" s="28"/>
-      <c r="D11" s="28"/>
-      <c r="E11" s="28"/>
-      <c r="F11" s="28"/>
-      <c r="G11" s="37"/>
-      <c r="H11" s="28"/>
+      <c r="A11" s="29"/>
+      <c r="B11" s="29"/>
+      <c r="C11" s="29"/>
+      <c r="D11" s="29"/>
+      <c r="E11" s="29"/>
+      <c r="F11" s="29"/>
+      <c r="G11" s="38"/>
+      <c r="H11" s="29"/>
     </row>
     <row r="12" spans="1:8">
-      <c r="A12" s="28"/>
-      <c r="B12" s="28"/>
-      <c r="C12" s="28"/>
-      <c r="D12" s="28"/>
-      <c r="E12" s="28"/>
-      <c r="F12" s="28"/>
-      <c r="G12" s="37"/>
-      <c r="H12" s="28"/>
+      <c r="A12" s="29"/>
+      <c r="B12" s="29"/>
+      <c r="C12" s="29"/>
+      <c r="D12" s="29"/>
+      <c r="E12" s="29"/>
+      <c r="F12" s="29"/>
+      <c r="G12" s="38"/>
+      <c r="H12" s="29"/>
     </row>
     <row r="13" spans="1:8">
-      <c r="A13" s="28"/>
-      <c r="B13" s="28"/>
-      <c r="C13" s="28"/>
-      <c r="D13" s="28"/>
-      <c r="E13" s="28"/>
-      <c r="F13" s="28"/>
-      <c r="G13" s="37"/>
-      <c r="H13" s="28"/>
+      <c r="A13" s="29"/>
+      <c r="B13" s="29"/>
+      <c r="C13" s="29"/>
+      <c r="D13" s="29"/>
+      <c r="E13" s="29"/>
+      <c r="F13" s="29"/>
+      <c r="G13" s="38"/>
+      <c r="H13" s="29"/>
     </row>
     <row r="14" spans="1:8">
-      <c r="A14" s="28"/>
-      <c r="B14" s="28"/>
-      <c r="C14" s="28"/>
-      <c r="D14" s="28"/>
-      <c r="E14" s="28"/>
-      <c r="F14" s="28"/>
-      <c r="G14" s="37"/>
-      <c r="H14" s="28"/>
+      <c r="A14" s="29"/>
+      <c r="B14" s="29"/>
+      <c r="C14" s="29"/>
+      <c r="D14" s="29"/>
+      <c r="E14" s="29"/>
+      <c r="F14" s="29"/>
+      <c r="G14" s="38"/>
+      <c r="H14" s="29"/>
     </row>
     <row r="15" spans="1:8">
-      <c r="A15" s="28"/>
-      <c r="B15" s="28"/>
-      <c r="C15" s="28"/>
-      <c r="D15" s="28"/>
-      <c r="E15" s="28"/>
-      <c r="F15" s="28"/>
-      <c r="G15" s="37"/>
-      <c r="H15" s="28"/>
+      <c r="A15" s="29"/>
+      <c r="B15" s="29"/>
+      <c r="C15" s="29"/>
+      <c r="D15" s="29"/>
+      <c r="E15" s="29"/>
+      <c r="F15" s="29"/>
+      <c r="G15" s="38"/>
+      <c r="H15" s="29"/>
     </row>
     <row r="16" spans="1:8">
-      <c r="A16" s="28"/>
-      <c r="B16" s="28"/>
-      <c r="C16" s="28"/>
-      <c r="D16" s="28"/>
-      <c r="E16" s="28"/>
-      <c r="F16" s="28"/>
-      <c r="G16" s="37"/>
-      <c r="H16" s="28"/>
+      <c r="A16" s="29"/>
+      <c r="B16" s="29"/>
+      <c r="C16" s="29"/>
+      <c r="D16" s="29"/>
+      <c r="E16" s="29"/>
+      <c r="F16" s="29"/>
+      <c r="G16" s="38"/>
+      <c r="H16" s="29"/>
     </row>
     <row r="17" spans="1:8">
-      <c r="A17" s="28"/>
-      <c r="B17" s="28"/>
-      <c r="C17" s="28"/>
-      <c r="D17" s="28"/>
-      <c r="E17" s="28"/>
-      <c r="F17" s="28"/>
-      <c r="G17" s="37"/>
-      <c r="H17" s="28"/>
+      <c r="A17" s="29"/>
+      <c r="B17" s="29"/>
+      <c r="C17" s="29"/>
+      <c r="D17" s="29"/>
+      <c r="E17" s="29"/>
+      <c r="F17" s="29"/>
+      <c r="G17" s="38"/>
+      <c r="H17" s="29"/>
     </row>
     <row r="18" spans="1:8">
-      <c r="A18" s="28"/>
-      <c r="B18" s="28"/>
-      <c r="C18" s="28"/>
-      <c r="D18" s="28"/>
-      <c r="E18" s="28"/>
-      <c r="F18" s="28"/>
-      <c r="G18" s="37"/>
-      <c r="H18" s="28"/>
+      <c r="A18" s="29"/>
+      <c r="B18" s="29"/>
+      <c r="C18" s="29"/>
+      <c r="D18" s="29"/>
+      <c r="E18" s="29"/>
+      <c r="F18" s="29"/>
+      <c r="G18" s="38"/>
+      <c r="H18" s="29"/>
     </row>
     <row r="19" spans="1:8">
-      <c r="A19" s="28"/>
-      <c r="B19" s="28"/>
-      <c r="C19" s="28"/>
-      <c r="D19" s="28"/>
-      <c r="E19" s="28"/>
-      <c r="F19" s="28"/>
-      <c r="G19" s="37"/>
-      <c r="H19" s="28"/>
+      <c r="A19" s="29"/>
+      <c r="B19" s="29"/>
+      <c r="C19" s="29"/>
+      <c r="D19" s="29"/>
+      <c r="E19" s="29"/>
+      <c r="F19" s="29"/>
+      <c r="G19" s="38"/>
+      <c r="H19" s="29"/>
     </row>
     <row r="20" spans="1:8">
-      <c r="A20" s="28"/>
-      <c r="B20" s="28"/>
-      <c r="C20" s="28"/>
-      <c r="D20" s="28"/>
-      <c r="E20" s="28"/>
-      <c r="F20" s="28"/>
-      <c r="G20" s="37"/>
-      <c r="H20" s="28"/>
+      <c r="A20" s="29"/>
+      <c r="B20" s="29"/>
+      <c r="C20" s="29"/>
+      <c r="D20" s="29"/>
+      <c r="E20" s="29"/>
+      <c r="F20" s="29"/>
+      <c r="G20" s="38"/>
+      <c r="H20" s="29"/>
     </row>
     <row r="21" spans="1:8">
-      <c r="A21" s="28"/>
-      <c r="B21" s="28"/>
-      <c r="C21" s="28"/>
-      <c r="D21" s="28"/>
-      <c r="E21" s="28"/>
-      <c r="F21" s="28"/>
-      <c r="G21" s="37"/>
-      <c r="H21" s="28"/>
+      <c r="A21" s="29"/>
+      <c r="B21" s="29"/>
+      <c r="C21" s="29"/>
+      <c r="D21" s="29"/>
+      <c r="E21" s="29"/>
+      <c r="F21" s="29"/>
+      <c r="G21" s="38"/>
+      <c r="H21" s="29"/>
     </row>
     <row r="22" spans="1:8">
-      <c r="A22" s="28"/>
-      <c r="B22" s="28"/>
-      <c r="C22" s="28"/>
-      <c r="D22" s="28"/>
-      <c r="E22" s="28"/>
-      <c r="F22" s="28"/>
-      <c r="G22" s="37"/>
-      <c r="H22" s="28"/>
+      <c r="A22" s="29"/>
+      <c r="B22" s="29"/>
+      <c r="C22" s="29"/>
+      <c r="D22" s="29"/>
+      <c r="E22" s="29"/>
+      <c r="F22" s="29"/>
+      <c r="G22" s="38"/>
+      <c r="H22" s="29"/>
     </row>
     <row r="23" spans="1:8">
-      <c r="A23" s="28"/>
-      <c r="B23" s="28"/>
-      <c r="C23" s="28"/>
-      <c r="D23" s="28"/>
-      <c r="E23" s="28"/>
-      <c r="F23" s="28"/>
-      <c r="G23" s="37"/>
-      <c r="H23" s="28"/>
+      <c r="A23" s="29"/>
+      <c r="B23" s="29"/>
+      <c r="C23" s="29"/>
+      <c r="D23" s="29"/>
+      <c r="E23" s="29"/>
+      <c r="F23" s="29"/>
+      <c r="G23" s="38"/>
+      <c r="H23" s="29"/>
     </row>
     <row r="24" spans="1:8">
-      <c r="A24" s="28"/>
-      <c r="B24" s="28"/>
-      <c r="C24" s="28"/>
-      <c r="D24" s="28"/>
-      <c r="E24" s="28"/>
-      <c r="F24" s="28"/>
-      <c r="G24" s="37"/>
-      <c r="H24" s="28"/>
+      <c r="A24" s="29"/>
+      <c r="B24" s="29"/>
+      <c r="C24" s="29"/>
+      <c r="D24" s="29"/>
+      <c r="E24" s="29"/>
+      <c r="F24" s="29"/>
+      <c r="G24" s="38"/>
+      <c r="H24" s="29"/>
     </row>
     <row r="25" spans="1:8">
-      <c r="A25" s="28"/>
-      <c r="B25" s="28"/>
-      <c r="C25" s="28"/>
-      <c r="D25" s="28"/>
-      <c r="E25" s="28"/>
-      <c r="F25" s="28"/>
-      <c r="G25" s="37"/>
-      <c r="H25" s="28"/>
+      <c r="A25" s="29"/>
+      <c r="B25" s="29"/>
+      <c r="C25" s="29"/>
+      <c r="D25" s="29"/>
+      <c r="E25" s="29"/>
+      <c r="F25" s="29"/>
+      <c r="G25" s="38"/>
+      <c r="H25" s="29"/>
     </row>
     <row r="26" spans="1:8">
-      <c r="A26" s="28"/>
-      <c r="B26" s="28"/>
-      <c r="C26" s="28"/>
-      <c r="D26" s="28"/>
-      <c r="E26" s="28"/>
-      <c r="F26" s="28"/>
-      <c r="G26" s="37"/>
-      <c r="H26" s="28"/>
+      <c r="A26" s="29"/>
+      <c r="B26" s="29"/>
+      <c r="C26" s="29"/>
+      <c r="D26" s="29"/>
+      <c r="E26" s="29"/>
+      <c r="F26" s="29"/>
+      <c r="G26" s="38"/>
+      <c r="H26" s="29"/>
     </row>
     <row r="27" spans="1:8">
-      <c r="A27" s="28"/>
-      <c r="B27" s="28"/>
-      <c r="C27" s="28"/>
-      <c r="D27" s="28"/>
-      <c r="E27" s="28"/>
-      <c r="F27" s="28"/>
-      <c r="G27" s="37"/>
-      <c r="H27" s="28"/>
+      <c r="A27" s="29"/>
+      <c r="B27" s="29"/>
+      <c r="C27" s="29"/>
+      <c r="D27" s="29"/>
+      <c r="E27" s="29"/>
+      <c r="F27" s="29"/>
+      <c r="G27" s="38"/>
+      <c r="H27" s="29"/>
     </row>
     <row r="28" spans="1:8">
-      <c r="A28" s="28"/>
-      <c r="B28" s="28"/>
-      <c r="C28" s="28"/>
-      <c r="D28" s="28"/>
-      <c r="E28" s="28"/>
-      <c r="F28" s="28"/>
-      <c r="G28" s="37"/>
-      <c r="H28" s="28"/>
+      <c r="A28" s="29"/>
+      <c r="B28" s="29"/>
+      <c r="C28" s="29"/>
+      <c r="D28" s="29"/>
+      <c r="E28" s="29"/>
+      <c r="F28" s="29"/>
+      <c r="G28" s="38"/>
+      <c r="H28" s="29"/>
     </row>
     <row r="29" spans="1:8">
-      <c r="A29" s="28"/>
-      <c r="B29" s="28"/>
-      <c r="C29" s="28"/>
-      <c r="D29" s="28"/>
-      <c r="E29" s="28"/>
-      <c r="F29" s="28"/>
-      <c r="G29" s="37"/>
-      <c r="H29" s="28"/>
+      <c r="A29" s="29"/>
+      <c r="B29" s="29"/>
+      <c r="C29" s="29"/>
+      <c r="D29" s="29"/>
+      <c r="E29" s="29"/>
+      <c r="F29" s="29"/>
+      <c r="G29" s="38"/>
+      <c r="H29" s="29"/>
     </row>
     <row r="30" spans="1:8">
-      <c r="A30" s="28"/>
-      <c r="B30" s="28"/>
-      <c r="C30" s="28"/>
-      <c r="D30" s="28"/>
-      <c r="E30" s="28"/>
-      <c r="F30" s="28"/>
-      <c r="G30" s="37"/>
-      <c r="H30" s="28"/>
+      <c r="A30" s="29"/>
+      <c r="B30" s="29"/>
+      <c r="C30" s="29"/>
+      <c r="D30" s="29"/>
+      <c r="E30" s="29"/>
+      <c r="F30" s="29"/>
+      <c r="G30" s="38"/>
+      <c r="H30" s="29"/>
     </row>
     <row r="31" spans="1:8">
-      <c r="A31" s="28"/>
-      <c r="B31" s="28"/>
-      <c r="C31" s="28"/>
-      <c r="D31" s="28"/>
-      <c r="E31" s="28"/>
-      <c r="F31" s="28"/>
-      <c r="G31" s="37"/>
-      <c r="H31" s="28"/>
+      <c r="A31" s="29"/>
+      <c r="B31" s="29"/>
+      <c r="C31" s="29"/>
+      <c r="D31" s="29"/>
+      <c r="E31" s="29"/>
+      <c r="F31" s="29"/>
+      <c r="G31" s="38"/>
+      <c r="H31" s="29"/>
     </row>
     <row r="32" spans="1:8">
-      <c r="A32" s="28"/>
-      <c r="B32" s="28"/>
-      <c r="C32" s="28"/>
-      <c r="D32" s="28"/>
-      <c r="E32" s="28"/>
-      <c r="F32" s="28"/>
-      <c r="G32" s="37"/>
-      <c r="H32" s="28"/>
+      <c r="A32" s="29"/>
+      <c r="B32" s="29"/>
+      <c r="C32" s="29"/>
+      <c r="D32" s="29"/>
+      <c r="E32" s="29"/>
+      <c r="F32" s="29"/>
+      <c r="G32" s="38"/>
+      <c r="H32" s="29"/>
     </row>
     <row r="33" spans="1:8">
-      <c r="A33" s="28"/>
-      <c r="B33" s="28"/>
-      <c r="C33" s="28"/>
-      <c r="D33" s="28"/>
-      <c r="E33" s="28"/>
-      <c r="F33" s="28"/>
-      <c r="G33" s="37"/>
-      <c r="H33" s="28"/>
+      <c r="A33" s="29"/>
+      <c r="B33" s="29"/>
+      <c r="C33" s="29"/>
+      <c r="D33" s="29"/>
+      <c r="E33" s="29"/>
+      <c r="F33" s="29"/>
+      <c r="G33" s="38"/>
+      <c r="H33" s="29"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4403,534 +4420,534 @@
   <dimension ref="A2:U12"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="5.5625" style="4" customWidth="1"/>
-    <col min="2" max="7" width="10.5625" style="4" customWidth="1"/>
-    <col min="8" max="8" width="20.5625" style="4" customWidth="1"/>
-    <col min="9" max="9" width="15.5625" style="4" customWidth="1"/>
-    <col min="10" max="10" width="30.5625" style="4" customWidth="1"/>
-    <col min="11" max="11" width="9" style="4"/>
-    <col min="12" max="12" width="15.5625" style="4" customWidth="1"/>
-    <col min="13" max="16" width="10.5625" style="4" customWidth="1"/>
-    <col min="17" max="17" width="9" style="4"/>
-    <col min="18" max="18" width="20.5625" style="4" customWidth="1"/>
-    <col min="19" max="20" width="10.5625" style="4" customWidth="1"/>
-    <col min="21" max="16384" width="9" style="4"/>
+    <col min="1" max="1" width="5.5625" style="5" customWidth="1"/>
+    <col min="2" max="7" width="10.5625" style="5" customWidth="1"/>
+    <col min="8" max="8" width="20.5625" style="5" customWidth="1"/>
+    <col min="9" max="9" width="15.5625" style="5" customWidth="1"/>
+    <col min="10" max="10" width="30.5625" style="5" customWidth="1"/>
+    <col min="11" max="11" width="9" style="5"/>
+    <col min="12" max="12" width="15.5625" style="5" customWidth="1"/>
+    <col min="13" max="16" width="10.5625" style="5" customWidth="1"/>
+    <col min="17" max="17" width="9" style="5"/>
+    <col min="18" max="18" width="20.5625" style="5" customWidth="1"/>
+    <col min="19" max="20" width="10.5625" style="5" customWidth="1"/>
+    <col min="21" max="16384" width="9" style="5"/>
   </cols>
   <sheetData>
     <row r="2" ht="18" spans="1:20">
-      <c r="A2" s="26" t="s">
+      <c r="A2" s="27" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="27" t="s">
+      <c r="B2" s="28" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="27" t="s">
+      <c r="C2" s="28" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="27"/>
-      <c r="E2" s="27" t="s">
+      <c r="D2" s="28"/>
+      <c r="E2" s="28" t="s">
         <v>19</v>
       </c>
-      <c r="F2" s="27" t="s">
+      <c r="F2" s="28" t="s">
         <v>20</v>
       </c>
-      <c r="G2" s="27" t="s">
+      <c r="G2" s="28" t="s">
         <v>21</v>
       </c>
-      <c r="H2" s="27" t="s">
+      <c r="H2" s="28" t="s">
         <v>22</v>
       </c>
-      <c r="I2" s="27" t="s">
+      <c r="I2" s="28" t="s">
         <v>5</v>
       </c>
-      <c r="J2" s="26" t="s">
+      <c r="J2" s="27" t="s">
         <v>23</v>
       </c>
-      <c r="L2" s="26" t="s">
+      <c r="L2" s="27" t="s">
         <v>8</v>
       </c>
-      <c r="M2" s="26" t="s">
+      <c r="M2" s="27" t="s">
         <v>9</v>
       </c>
-      <c r="N2" s="26" t="s">
+      <c r="N2" s="27" t="s">
         <v>10</v>
       </c>
-      <c r="O2" s="26" t="s">
+      <c r="O2" s="27" t="s">
         <v>11</v>
       </c>
-      <c r="P2" s="26" t="s">
+      <c r="P2" s="27" t="s">
         <v>12</v>
       </c>
-      <c r="Q2" s="26" t="s">
+      <c r="Q2" s="27" t="s">
         <v>13</v>
       </c>
-      <c r="R2" s="26" t="s">
+      <c r="R2" s="27" t="s">
         <v>14</v>
       </c>
-      <c r="S2" s="26" t="s">
+      <c r="S2" s="27" t="s">
         <v>15</v>
       </c>
-      <c r="T2" s="26" t="s">
+      <c r="T2" s="27" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="3" spans="1:21">
-      <c r="A3" s="28">
+      <c r="A3" s="29">
         <v>1</v>
       </c>
-      <c r="B3" s="28">
+      <c r="B3" s="29">
         <v>72</v>
       </c>
-      <c r="C3" s="28">
+      <c r="C3" s="29">
         <v>400000</v>
       </c>
-      <c r="D3" s="28" t="s">
+      <c r="D3" s="29" t="s">
         <v>24</v>
       </c>
-      <c r="E3" s="4">
+      <c r="E3" s="5">
         <v>25</v>
       </c>
-      <c r="F3" s="4">
+      <c r="F3" s="5">
         <v>40</v>
       </c>
-      <c r="G3" s="4">
+      <c r="G3" s="5">
         <v>15</v>
       </c>
-      <c r="H3" s="4">
+      <c r="H3" s="5">
         <f>(F3-E3)*G3/2</f>
         <v>112.5</v>
       </c>
-      <c r="I3" s="4">
+      <c r="I3" s="5">
         <v>1800</v>
       </c>
-      <c r="J3" s="4">
+      <c r="J3" s="5">
         <f>(B3*0.5*POWER(10,10))/(2*C3*I3*H3)</f>
         <v>2.22222222222222</v>
       </c>
-      <c r="L3" s="29">
+      <c r="L3" s="30">
         <f>B3/J3</f>
         <v>32.4</v>
       </c>
-      <c r="M3" s="4">
+      <c r="M3" s="5">
         <v>216</v>
       </c>
-      <c r="N3" s="32">
+      <c r="N3" s="33">
         <v>0.5</v>
       </c>
-      <c r="O3" s="4">
+      <c r="O3" s="5">
         <f>M3*N3</f>
         <v>108</v>
       </c>
-      <c r="P3" s="33">
+      <c r="P3" s="34">
         <f>O3/B3</f>
         <v>1.5</v>
       </c>
-      <c r="Q3" s="29">
+      <c r="Q3" s="30">
         <f>M3/L3</f>
         <v>6.66666666666667</v>
       </c>
-      <c r="R3" s="33">
+      <c r="R3" s="34">
         <v>2.5</v>
       </c>
-      <c r="S3" s="32">
+      <c r="S3" s="33">
         <f>SQRT((P3*0.9/(R3+5))/0.9)</f>
         <v>0.447213595499958</v>
       </c>
-      <c r="T3" s="32">
+      <c r="T3" s="33">
         <f>SQRT((N3*0.9/(R3+5))/0.9)</f>
         <v>0.258198889747161</v>
       </c>
-      <c r="U3" s="33">
+      <c r="U3" s="34">
         <f>P3/R3</f>
         <v>0.6</v>
       </c>
     </row>
     <row r="4" spans="1:20">
-      <c r="A4" s="28"/>
-      <c r="B4" s="28">
+      <c r="A4" s="29"/>
+      <c r="B4" s="29">
         <v>72</v>
       </c>
-      <c r="C4" s="28">
+      <c r="C4" s="29">
         <v>400000</v>
       </c>
-      <c r="D4" s="28" t="s">
+      <c r="D4" s="29" t="s">
         <v>24</v>
       </c>
-      <c r="E4" s="4">
+      <c r="E4" s="5">
         <v>23</v>
       </c>
-      <c r="F4" s="4">
+      <c r="F4" s="5">
         <v>40</v>
       </c>
-      <c r="G4" s="4">
+      <c r="G4" s="5">
         <v>15</v>
       </c>
-      <c r="H4" s="4">
+      <c r="H4" s="5">
         <f t="shared" ref="H4:H9" si="0">(F4-E4)*G4/2</f>
         <v>127.5</v>
       </c>
-      <c r="I4" s="4">
+      <c r="I4" s="5">
         <v>350</v>
       </c>
-      <c r="J4" s="4">
+      <c r="J4" s="5">
         <f t="shared" ref="J4:J9" si="1">(B4*0.5*POWER(10,10))/(2*C4*I4*H4)</f>
         <v>10.0840336134454</v>
       </c>
-      <c r="L4" s="29">
+      <c r="L4" s="30">
         <f t="shared" ref="L4:L9" si="2">B4/J4</f>
         <v>7.14</v>
       </c>
-      <c r="M4" s="4">
+      <c r="M4" s="5">
         <v>216</v>
       </c>
-      <c r="N4" s="32">
+      <c r="N4" s="33">
         <v>0.5</v>
       </c>
-      <c r="O4" s="4">
+      <c r="O4" s="5">
         <f t="shared" ref="O4:O9" si="3">M4*N4</f>
         <v>108</v>
       </c>
-      <c r="P4" s="33">
+      <c r="P4" s="34">
         <f t="shared" ref="P4:P9" si="4">O4/B4</f>
         <v>1.5</v>
       </c>
-      <c r="Q4" s="29">
+      <c r="Q4" s="30">
         <f t="shared" ref="Q4:Q9" si="5">M4/L4</f>
         <v>30.2521008403361</v>
       </c>
-      <c r="R4" s="33">
+      <c r="R4" s="34">
         <v>2.5</v>
       </c>
-      <c r="S4" s="32">
+      <c r="S4" s="33">
         <f t="shared" ref="S4:S9" si="6">SQRT((P4*0.9/(R4+5))/0.9)</f>
         <v>0.447213595499958</v>
       </c>
-      <c r="T4" s="32">
+      <c r="T4" s="33">
         <f t="shared" ref="T4:T9" si="7">SQRT((N4*0.9/(R4+5))/0.9)</f>
         <v>0.258198889747161</v>
       </c>
     </row>
     <row r="5" spans="2:20">
-      <c r="B5" s="28">
+      <c r="B5" s="29">
         <v>72</v>
       </c>
-      <c r="C5" s="28">
+      <c r="C5" s="29">
         <v>400000</v>
       </c>
-      <c r="D5" s="28"/>
-      <c r="E5" s="4">
+      <c r="D5" s="29"/>
+      <c r="E5" s="5">
         <v>23.13</v>
       </c>
-      <c r="F5" s="4">
+      <c r="F5" s="5">
         <v>39.88</v>
       </c>
-      <c r="G5" s="4">
+      <c r="G5" s="5">
         <v>14.48</v>
       </c>
-      <c r="H5" s="4">
+      <c r="H5" s="5">
         <f t="shared" si="0"/>
         <v>121.27</v>
       </c>
-      <c r="I5" s="4">
+      <c r="I5" s="5">
         <v>600</v>
       </c>
-      <c r="J5" s="4">
+      <c r="J5" s="5">
         <f t="shared" si="1"/>
         <v>6.18454687886534</v>
       </c>
-      <c r="L5" s="29">
+      <c r="L5" s="30">
         <f t="shared" si="2"/>
         <v>11.64192</v>
       </c>
-      <c r="M5" s="4">
+      <c r="M5" s="5">
         <v>216</v>
       </c>
-      <c r="N5" s="32">
+      <c r="N5" s="33">
         <v>0.5</v>
       </c>
-      <c r="O5" s="4">
+      <c r="O5" s="5">
         <f t="shared" si="3"/>
         <v>108</v>
       </c>
-      <c r="P5" s="33">
+      <c r="P5" s="34">
         <f t="shared" si="4"/>
         <v>1.5</v>
       </c>
-      <c r="Q5" s="29">
+      <c r="Q5" s="30">
         <f t="shared" si="5"/>
         <v>18.553640636596</v>
       </c>
-      <c r="R5" s="33">
+      <c r="R5" s="34">
         <v>2.5</v>
       </c>
-      <c r="S5" s="32">
+      <c r="S5" s="33">
         <f t="shared" si="6"/>
         <v>0.447213595499958</v>
       </c>
-      <c r="T5" s="32">
+      <c r="T5" s="33">
         <f t="shared" si="7"/>
         <v>0.258198889747161</v>
       </c>
     </row>
     <row r="6" spans="2:20">
-      <c r="B6" s="28">
+      <c r="B6" s="29">
         <v>72</v>
       </c>
-      <c r="C6" s="28">
+      <c r="C6" s="29">
         <v>400000</v>
       </c>
-      <c r="D6" s="28"/>
-      <c r="E6" s="4">
+      <c r="D6" s="29"/>
+      <c r="E6" s="5">
         <v>23.13</v>
       </c>
-      <c r="F6" s="4">
+      <c r="F6" s="5">
         <v>39.88</v>
       </c>
-      <c r="G6" s="4">
+      <c r="G6" s="5">
         <v>14.48</v>
       </c>
-      <c r="H6" s="4">
+      <c r="H6" s="5">
         <f t="shared" si="0"/>
         <v>121.27</v>
       </c>
-      <c r="I6" s="4">
+      <c r="I6" s="5">
         <v>350</v>
       </c>
-      <c r="J6" s="4">
+      <c r="J6" s="5">
         <f t="shared" si="1"/>
         <v>10.6020803637692</v>
       </c>
-      <c r="L6" s="29">
+      <c r="L6" s="30">
         <f t="shared" si="2"/>
         <v>6.79112</v>
       </c>
-      <c r="M6" s="4">
+      <c r="M6" s="5">
         <v>216</v>
       </c>
-      <c r="N6" s="32">
+      <c r="N6" s="33">
         <v>0.5</v>
       </c>
-      <c r="O6" s="4">
+      <c r="O6" s="5">
         <f t="shared" si="3"/>
         <v>108</v>
       </c>
-      <c r="P6" s="33">
+      <c r="P6" s="34">
         <f t="shared" si="4"/>
         <v>1.5</v>
       </c>
-      <c r="Q6" s="29">
+      <c r="Q6" s="30">
         <f t="shared" si="5"/>
         <v>31.8062410913075</v>
       </c>
-      <c r="R6" s="33">
+      <c r="R6" s="34">
         <v>2.5</v>
       </c>
-      <c r="S6" s="32">
+      <c r="S6" s="33">
         <f t="shared" si="6"/>
         <v>0.447213595499958</v>
       </c>
-      <c r="T6" s="32">
+      <c r="T6" s="33">
         <f t="shared" si="7"/>
         <v>0.258198889747161</v>
       </c>
     </row>
     <row r="7" spans="2:20">
-      <c r="B7" s="28">
+      <c r="B7" s="29">
         <v>72</v>
       </c>
-      <c r="C7" s="28">
+      <c r="C7" s="29">
         <v>400000</v>
       </c>
-      <c r="D7" s="4" t="s">
+      <c r="D7" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="E7" s="4">
+      <c r="E7" s="5">
         <v>23.3</v>
       </c>
-      <c r="F7" s="4">
+      <c r="F7" s="5">
         <v>40.4</v>
       </c>
-      <c r="G7" s="4">
+      <c r="G7" s="5">
         <v>15.1</v>
       </c>
-      <c r="H7" s="4">
+      <c r="H7" s="5">
         <f t="shared" si="0"/>
         <v>129.105</v>
       </c>
-      <c r="I7" s="4">
+      <c r="I7" s="5">
         <v>350</v>
       </c>
-      <c r="J7" s="4">
+      <c r="J7" s="5">
         <f t="shared" si="1"/>
         <v>9.95867151322014</v>
       </c>
-      <c r="L7" s="29">
+      <c r="L7" s="30">
         <f t="shared" si="2"/>
         <v>7.22988</v>
       </c>
-      <c r="M7" s="4">
+      <c r="M7" s="5">
         <v>216</v>
       </c>
-      <c r="N7" s="32">
+      <c r="N7" s="33">
         <v>0.5</v>
       </c>
-      <c r="O7" s="4">
+      <c r="O7" s="5">
         <f t="shared" si="3"/>
         <v>108</v>
       </c>
-      <c r="P7" s="33">
+      <c r="P7" s="34">
         <f t="shared" si="4"/>
         <v>1.5</v>
       </c>
-      <c r="Q7" s="29">
+      <c r="Q7" s="30">
         <f t="shared" si="5"/>
         <v>29.8760145396604</v>
       </c>
-      <c r="R7" s="33">
+      <c r="R7" s="34">
         <v>2.5</v>
       </c>
-      <c r="S7" s="32">
+      <c r="S7" s="33">
         <f t="shared" si="6"/>
         <v>0.447213595499958</v>
       </c>
-      <c r="T7" s="32">
+      <c r="T7" s="33">
         <f t="shared" si="7"/>
         <v>0.258198889747161</v>
       </c>
     </row>
     <row r="8" spans="2:20">
-      <c r="B8" s="28">
+      <c r="B8" s="29">
         <v>72</v>
       </c>
-      <c r="C8" s="28">
+      <c r="C8" s="29">
         <v>400000</v>
       </c>
-      <c r="D8" s="4" t="s">
+      <c r="D8" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="E8" s="4">
+      <c r="E8" s="5">
         <v>13.5</v>
       </c>
-      <c r="F8" s="4">
+      <c r="F8" s="5">
         <v>23.3</v>
       </c>
-      <c r="G8" s="4">
+      <c r="G8" s="5">
         <v>8</v>
       </c>
-      <c r="H8" s="4">
+      <c r="H8" s="5">
         <f t="shared" si="0"/>
         <v>39.2</v>
       </c>
-      <c r="I8" s="4">
+      <c r="I8" s="5">
         <v>350</v>
       </c>
-      <c r="J8" s="4">
+      <c r="J8" s="5">
         <f t="shared" si="1"/>
         <v>32.798833819242</v>
       </c>
-      <c r="L8" s="29">
+      <c r="L8" s="30">
         <f t="shared" si="2"/>
         <v>2.1952</v>
       </c>
-      <c r="M8" s="4">
+      <c r="M8" s="5">
         <v>216</v>
       </c>
-      <c r="N8" s="32">
+      <c r="N8" s="33">
         <v>0.5</v>
       </c>
-      <c r="O8" s="4">
+      <c r="O8" s="5">
         <f t="shared" si="3"/>
         <v>108</v>
       </c>
-      <c r="P8" s="33">
+      <c r="P8" s="34">
         <f t="shared" si="4"/>
         <v>1.5</v>
       </c>
-      <c r="Q8" s="29">
+      <c r="Q8" s="30">
         <f t="shared" si="5"/>
         <v>98.396501457726</v>
       </c>
-      <c r="R8" s="33">
+      <c r="R8" s="34">
         <v>2.5</v>
       </c>
-      <c r="S8" s="32">
+      <c r="S8" s="33">
         <f t="shared" si="6"/>
         <v>0.447213595499958</v>
       </c>
-      <c r="T8" s="32">
+      <c r="T8" s="33">
         <f t="shared" si="7"/>
         <v>0.258198889747161</v>
       </c>
     </row>
     <row r="9" spans="2:20">
-      <c r="B9" s="28">
+      <c r="B9" s="29">
         <v>72</v>
       </c>
-      <c r="C9" s="28">
+      <c r="C9" s="29">
         <v>400000</v>
       </c>
-      <c r="E9" s="4">
+      <c r="E9" s="5">
         <v>23.3</v>
       </c>
-      <c r="F9" s="4">
+      <c r="F9" s="5">
         <v>40.6</v>
       </c>
-      <c r="G9" s="4">
+      <c r="G9" s="5">
         <v>14.9</v>
       </c>
-      <c r="H9" s="4">
+      <c r="H9" s="5">
         <f t="shared" si="0"/>
         <v>128.885</v>
       </c>
-      <c r="I9" s="4">
+      <c r="I9" s="5">
         <v>350</v>
       </c>
-      <c r="J9" s="4">
+      <c r="J9" s="5">
         <f t="shared" si="1"/>
         <v>9.9756704481847</v>
       </c>
-      <c r="L9" s="29">
+      <c r="L9" s="30">
         <f t="shared" si="2"/>
         <v>7.21756</v>
       </c>
-      <c r="M9" s="4">
+      <c r="M9" s="5">
         <v>216</v>
       </c>
-      <c r="N9" s="32">
+      <c r="N9" s="33">
         <v>0.5</v>
       </c>
-      <c r="O9" s="4">
+      <c r="O9" s="5">
         <f t="shared" si="3"/>
         <v>108</v>
       </c>
-      <c r="P9" s="33">
+      <c r="P9" s="34">
         <f t="shared" si="4"/>
         <v>1.5</v>
       </c>
-      <c r="Q9" s="29">
+      <c r="Q9" s="30">
         <f t="shared" si="5"/>
         <v>29.9270113445541</v>
       </c>
-      <c r="R9" s="33">
+      <c r="R9" s="34">
         <v>2.5</v>
       </c>
-      <c r="S9" s="32">
+      <c r="S9" s="33">
         <f t="shared" si="6"/>
         <v>0.447213595499958</v>
       </c>
-      <c r="T9" s="32">
+      <c r="T9" s="33">
         <f t="shared" si="7"/>
         <v>0.258198889747161</v>
       </c>
     </row>
     <row r="10" spans="10:10">
-      <c r="J10" s="30"/>
+      <c r="J10" s="31"/>
     </row>
     <row r="11" spans="10:10">
-      <c r="J11" s="29"/>
+      <c r="J11" s="30"/>
     </row>
     <row r="12" spans="10:10">
-      <c r="J12" s="31"/>
+      <c r="J12" s="32"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4944,950 +4961,913 @@
   <dimension ref="B3:Y38"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="5.5625" style="4" customWidth="1"/>
-    <col min="2" max="2" width="15.5625" style="5" customWidth="1"/>
-    <col min="3" max="3" width="15.5625" style="4" customWidth="1"/>
-    <col min="4" max="4" width="5.5625" style="4" customWidth="1"/>
-    <col min="5" max="5" width="18.5625" style="4" customWidth="1"/>
-    <col min="6" max="6" width="34.6015625" style="4" customWidth="1"/>
-    <col min="7" max="12" width="18.5625" style="4" customWidth="1"/>
-    <col min="13" max="13" width="5.2265625" style="4" customWidth="1"/>
-    <col min="14" max="14" width="25.4375" style="4" customWidth="1"/>
-    <col min="15" max="17" width="5.5625" style="4" customWidth="1"/>
-    <col min="18" max="18" width="15.5625" style="4" customWidth="1"/>
-    <col min="19" max="20" width="9" style="4"/>
-    <col min="21" max="22" width="20.5625" style="4" customWidth="1"/>
-    <col min="23" max="23" width="9" style="4"/>
-    <col min="24" max="24" width="11.125" style="4"/>
-    <col min="25" max="16384" width="9" style="4"/>
+    <col min="1" max="1" width="5.5625" style="5" customWidth="1"/>
+    <col min="2" max="2" width="15.5625" style="6" customWidth="1"/>
+    <col min="3" max="3" width="15.5625" style="5" customWidth="1"/>
+    <col min="4" max="4" width="5.5625" style="5" customWidth="1"/>
+    <col min="5" max="5" width="18.5625" style="5" customWidth="1"/>
+    <col min="6" max="6" width="34.6015625" style="5" customWidth="1"/>
+    <col min="7" max="12" width="18.5625" style="5" customWidth="1"/>
+    <col min="13" max="13" width="5.2265625" style="5" customWidth="1"/>
+    <col min="14" max="14" width="25.4375" style="5" customWidth="1"/>
+    <col min="15" max="17" width="5.5625" style="5" customWidth="1"/>
+    <col min="18" max="18" width="15.5625" style="5" customWidth="1"/>
+    <col min="19" max="20" width="9" style="5"/>
+    <col min="21" max="22" width="20.5625" style="5" customWidth="1"/>
+    <col min="23" max="23" width="9" style="5"/>
+    <col min="24" max="24" width="11.125" style="5"/>
+    <col min="25" max="16384" width="9" style="5"/>
   </cols>
   <sheetData>
-    <row r="3" spans="2:4">
-      <c r="B3" s="6" t="s">
+    <row r="3" spans="2:6">
+      <c r="B3" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="C3" s="7">
+      <c r="C3" s="8">
         <v>400000</v>
       </c>
-      <c r="D3" s="7" t="s">
+      <c r="D3" s="8" t="s">
         <v>28</v>
       </c>
+      <c r="F3" s="5" t="s">
+        <v>27</v>
+      </c>
     </row>
     <row r="4" customHeight="1" spans="2:4">
-      <c r="B4" s="6" t="s">
+      <c r="B4" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="C4" s="7">
+      <c r="C4" s="8">
         <v>100</v>
       </c>
-      <c r="D4" s="7" t="s">
+      <c r="D4" s="8" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="5" customHeight="1" spans="2:4">
-      <c r="B5" s="6" t="s">
+      <c r="B5" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="C5" s="7">
+      <c r="C5" s="8">
         <f>C4/2</f>
         <v>50</v>
       </c>
-      <c r="D5" s="7" t="s">
+      <c r="D5" s="8" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="6" customHeight="1" spans="2:4">
-      <c r="B6" s="6"/>
-      <c r="C6" s="7"/>
-      <c r="D6" s="7"/>
+      <c r="B6" s="7"/>
+      <c r="C6" s="8"/>
+      <c r="D6" s="8"/>
     </row>
     <row r="7" spans="2:4">
-      <c r="B7" s="8" t="s">
+      <c r="B7" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="D7" s="7"/>
+      <c r="D7" s="8"/>
     </row>
     <row r="8" ht="18" spans="2:24">
-      <c r="B8" s="6" t="s">
+      <c r="B8" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="C8" s="9">
+      <c r="C8" s="10">
         <f>((C5*SQRT(2))/(2*3.14*C3))*1000000</f>
         <v>28.1491553020122</v>
       </c>
-      <c r="D8" s="7" t="s">
+      <c r="D8" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="F8" s="4">
-        <f>50*SQRT(2)</f>
-        <v>70.7106781186548</v>
-      </c>
-      <c r="G8" s="4">
-        <f>1/G9</f>
-        <v>5.62983106040245e-9</v>
-      </c>
-      <c r="M8" s="17"/>
-      <c r="N8" s="7" t="s">
+      <c r="M8" s="18"/>
+      <c r="N8" s="8" t="s">
         <v>35</v>
       </c>
-      <c r="O8" s="23">
+      <c r="O8" s="24">
         <v>1.4</v>
       </c>
-      <c r="P8" s="7"/>
-      <c r="S8" s="7"/>
-      <c r="T8" s="17"/>
-      <c r="U8" s="17"/>
-      <c r="V8" s="7"/>
-      <c r="W8" s="7"/>
-      <c r="X8" s="7"/>
+      <c r="P8" s="8"/>
+      <c r="S8" s="8"/>
+      <c r="T8" s="18"/>
+      <c r="U8" s="18"/>
+      <c r="V8" s="8"/>
+      <c r="W8" s="8"/>
+      <c r="X8" s="8"/>
     </row>
     <row r="9" ht="18" spans="2:24">
-      <c r="B9" s="6" t="s">
+      <c r="B9" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="C9" s="10">
+      <c r="C9" s="11">
         <f>(1/(2*3.14*C3*C5*SQRT(2)))*1000000000</f>
         <v>5.62983106040245</v>
       </c>
-      <c r="D9" s="7" t="s">
+      <c r="D9" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="F9" s="4">
-        <f>2*3.14*400000</f>
-        <v>2512000</v>
-      </c>
-      <c r="G9" s="4">
-        <f>F8*F9</f>
-        <v>177625223.434061</v>
-      </c>
-      <c r="M9" s="15"/>
-      <c r="N9" s="7" t="s">
+      <c r="M9" s="16"/>
+      <c r="N9" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="O9" s="23">
+      <c r="O9" s="24">
         <v>0.707</v>
       </c>
-      <c r="P9" s="24"/>
-      <c r="S9" s="7"/>
-      <c r="T9" s="9"/>
-      <c r="U9" s="9"/>
-      <c r="V9" s="25"/>
-      <c r="W9" s="25"/>
-      <c r="X9" s="7"/>
+      <c r="P9" s="25"/>
+      <c r="S9" s="8"/>
+      <c r="T9" s="10"/>
+      <c r="U9" s="10"/>
+      <c r="V9" s="26"/>
+      <c r="W9" s="26"/>
+      <c r="X9" s="8"/>
     </row>
     <row r="10" ht="18" spans="2:24">
-      <c r="B10" s="6" t="s">
+      <c r="B10" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="C10" s="11">
+      <c r="C10" s="12">
         <f>C9/2</f>
         <v>2.81491553020122</v>
       </c>
-      <c r="D10" s="7" t="s">
+      <c r="D10" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="E10" s="15"/>
-      <c r="F10" s="16">
-        <f>F8/F9</f>
-        <v>2.81491553020122e-5</v>
-      </c>
-      <c r="G10" s="7"/>
-      <c r="H10" s="7"/>
-      <c r="I10" s="7"/>
-      <c r="J10" s="9"/>
-      <c r="K10" s="9"/>
-      <c r="L10" s="15"/>
-      <c r="M10" s="15"/>
-      <c r="N10" s="7" t="s">
+      <c r="E10" s="16"/>
+      <c r="F10" s="17"/>
+      <c r="G10" s="8"/>
+      <c r="H10" s="8"/>
+      <c r="I10" s="8"/>
+      <c r="J10" s="10"/>
+      <c r="K10" s="10"/>
+      <c r="L10" s="16"/>
+      <c r="M10" s="16"/>
+      <c r="N10" s="8" t="s">
         <v>40</v>
       </c>
-      <c r="O10" s="23">
+      <c r="O10" s="24">
         <v>0.3</v>
       </c>
-      <c r="P10" s="7"/>
-      <c r="S10" s="7"/>
-      <c r="T10" s="7"/>
-      <c r="U10" s="7"/>
-      <c r="V10" s="7"/>
-      <c r="W10" s="7"/>
-      <c r="X10" s="7"/>
+      <c r="P10" s="8"/>
+      <c r="S10" s="8"/>
+      <c r="T10" s="8"/>
+      <c r="U10" s="8"/>
+      <c r="V10" s="8"/>
+      <c r="W10" s="8"/>
+      <c r="X10" s="8"/>
     </row>
     <row r="11" spans="2:24">
-      <c r="B11" s="12"/>
-      <c r="C11" s="7"/>
-      <c r="D11" s="7"/>
-      <c r="J11" s="9"/>
-      <c r="K11" s="9"/>
-      <c r="L11" s="15"/>
-      <c r="M11" s="15"/>
-      <c r="N11" s="7"/>
-      <c r="O11" s="7"/>
-      <c r="P11" s="7"/>
-      <c r="Q11" s="7"/>
-      <c r="R11" s="7"/>
-      <c r="S11" s="7"/>
-      <c r="T11" s="7"/>
-      <c r="U11" s="7"/>
-      <c r="V11" s="7"/>
-      <c r="W11" s="7"/>
-      <c r="X11" s="7"/>
+      <c r="B11" s="13"/>
+      <c r="C11" s="8"/>
+      <c r="D11" s="8"/>
+      <c r="J11" s="10"/>
+      <c r="K11" s="10"/>
+      <c r="L11" s="16"/>
+      <c r="M11" s="16"/>
+      <c r="N11" s="8"/>
+      <c r="O11" s="8"/>
+      <c r="P11" s="8"/>
+      <c r="Q11" s="8"/>
+      <c r="R11" s="8"/>
+      <c r="S11" s="8"/>
+      <c r="T11" s="8"/>
+      <c r="U11" s="8"/>
+      <c r="V11" s="8"/>
+      <c r="W11" s="8"/>
+      <c r="X11" s="8"/>
     </row>
     <row r="12" spans="2:24">
-      <c r="B12" s="8" t="s">
+      <c r="B12" s="9" t="s">
         <v>41</v>
       </c>
-      <c r="C12" s="13"/>
-      <c r="D12" s="7"/>
-      <c r="E12" s="17"/>
-      <c r="F12" s="17"/>
-      <c r="G12" s="17"/>
-      <c r="H12" s="17"/>
-      <c r="I12" s="17"/>
-      <c r="J12" s="21"/>
-      <c r="K12" s="21"/>
-      <c r="L12" s="22"/>
-      <c r="M12" s="22"/>
-      <c r="N12" s="7"/>
-      <c r="O12" s="7"/>
-      <c r="P12" s="7"/>
-      <c r="Q12" s="7"/>
-      <c r="R12" s="7"/>
-      <c r="S12" s="7"/>
-      <c r="T12" s="7"/>
-      <c r="U12" s="7"/>
-      <c r="V12" s="7"/>
-      <c r="W12" s="7"/>
-      <c r="X12" s="7"/>
+      <c r="C12" s="14"/>
+      <c r="D12" s="8"/>
+      <c r="E12" s="18"/>
+      <c r="F12" s="18"/>
+      <c r="G12" s="18"/>
+      <c r="H12" s="18"/>
+      <c r="I12" s="18"/>
+      <c r="J12" s="22"/>
+      <c r="K12" s="22"/>
+      <c r="L12" s="23"/>
+      <c r="M12" s="23"/>
+      <c r="N12" s="8"/>
+      <c r="O12" s="8"/>
+      <c r="P12" s="8"/>
+      <c r="Q12" s="8"/>
+      <c r="R12" s="8"/>
+      <c r="S12" s="8"/>
+      <c r="T12" s="8"/>
+      <c r="U12" s="8"/>
+      <c r="V12" s="8"/>
+      <c r="W12" s="8"/>
+      <c r="X12" s="8"/>
     </row>
     <row r="13" ht="18" spans="2:24">
-      <c r="B13" s="6" t="s">
+      <c r="B13" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="C13" s="7">
+      <c r="C13" s="8">
         <v>29</v>
       </c>
-      <c r="D13" s="7" t="s">
+      <c r="D13" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="F13" s="18">
-        <f>SQRT(C13*C15*10^-(15))</f>
-        <v>3.95727178748188e-7</v>
-      </c>
-      <c r="G13" s="19">
-        <f>C13*C15</f>
-        <v>156.6</v>
-      </c>
-      <c r="J13" s="9"/>
-      <c r="K13" s="9"/>
-      <c r="L13" s="15"/>
-      <c r="M13" s="15"/>
-      <c r="N13" s="7"/>
-      <c r="O13" s="7"/>
-      <c r="P13" s="7"/>
-      <c r="Q13" s="7"/>
-      <c r="R13" s="7"/>
-      <c r="S13" s="7"/>
-      <c r="T13" s="7"/>
-      <c r="U13" s="7"/>
-      <c r="V13" s="7"/>
-      <c r="W13" s="7"/>
-      <c r="X13" s="7"/>
+      <c r="F13" s="19"/>
+      <c r="G13" s="20"/>
+      <c r="J13" s="10"/>
+      <c r="K13" s="10"/>
+      <c r="L13" s="16"/>
+      <c r="M13" s="16"/>
+      <c r="N13" s="8"/>
+      <c r="O13" s="8"/>
+      <c r="P13" s="8"/>
+      <c r="Q13" s="8"/>
+      <c r="R13" s="8"/>
+      <c r="S13" s="8"/>
+      <c r="T13" s="8"/>
+      <c r="U13" s="8"/>
+      <c r="V13" s="8"/>
+      <c r="W13" s="8"/>
+      <c r="X13" s="8"/>
     </row>
     <row r="14" ht="18" spans="2:24">
-      <c r="B14" s="6" t="s">
+      <c r="B14" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="C14" s="14">
+      <c r="C14" s="15">
         <v>2.7</v>
       </c>
-      <c r="D14" s="7" t="s">
+      <c r="D14" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="E14" s="15"/>
-      <c r="F14" s="20">
-        <f>2*3.14*F13</f>
-        <v>2.48516668253862e-6</v>
-      </c>
-      <c r="G14" s="7"/>
-      <c r="H14" s="7"/>
-      <c r="I14" s="7"/>
-      <c r="J14" s="9"/>
-      <c r="K14" s="9"/>
-      <c r="L14" s="15"/>
-      <c r="M14" s="15"/>
-      <c r="N14" s="7"/>
-      <c r="O14" s="7"/>
-      <c r="P14" s="7"/>
-      <c r="Q14" s="7"/>
-      <c r="R14" s="7"/>
-      <c r="S14" s="7"/>
-      <c r="T14" s="7"/>
-      <c r="U14" s="7"/>
-      <c r="V14" s="7"/>
-      <c r="W14" s="7"/>
-      <c r="X14" s="7"/>
+      <c r="E14" s="16"/>
+      <c r="F14" s="21"/>
+      <c r="G14" s="8"/>
+      <c r="H14" s="8"/>
+      <c r="I14" s="8"/>
+      <c r="J14" s="10"/>
+      <c r="K14" s="10"/>
+      <c r="L14" s="16"/>
+      <c r="M14" s="16"/>
+      <c r="N14" s="8"/>
+      <c r="O14" s="8"/>
+      <c r="P14" s="8"/>
+      <c r="Q14" s="8"/>
+      <c r="R14" s="8"/>
+      <c r="S14" s="8"/>
+      <c r="T14" s="8"/>
+      <c r="U14" s="8"/>
+      <c r="V14" s="8"/>
+      <c r="W14" s="8"/>
+      <c r="X14" s="8"/>
     </row>
     <row r="15" ht="18" spans="2:25">
-      <c r="B15" s="6" t="s">
+      <c r="B15" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="C15" s="14">
+      <c r="C15" s="15">
         <f>2*C14</f>
         <v>5.4</v>
       </c>
-      <c r="D15" s="7" t="s">
+      <c r="D15" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="E15" s="7"/>
-      <c r="F15" s="20">
-        <f>1/F14</f>
-        <v>402387.496591775</v>
-      </c>
-      <c r="G15" s="15"/>
-      <c r="H15" s="15"/>
-      <c r="I15" s="15"/>
-      <c r="J15" s="7"/>
-      <c r="K15" s="9"/>
-      <c r="L15" s="9"/>
-      <c r="M15" s="9"/>
-      <c r="N15" s="9"/>
-      <c r="O15" s="7"/>
-      <c r="P15" s="7"/>
-      <c r="Q15" s="7"/>
-      <c r="R15" s="7"/>
-      <c r="S15" s="7"/>
-      <c r="T15" s="7"/>
-      <c r="U15" s="7"/>
-      <c r="V15" s="7"/>
-      <c r="W15" s="7"/>
-      <c r="X15" s="7"/>
-      <c r="Y15" s="7"/>
+      <c r="E15" s="8"/>
+      <c r="F15" s="21"/>
+      <c r="G15" s="16"/>
+      <c r="H15" s="16"/>
+      <c r="I15" s="16"/>
+      <c r="J15" s="8"/>
+      <c r="K15" s="10"/>
+      <c r="L15" s="10"/>
+      <c r="M15" s="10"/>
+      <c r="N15" s="10"/>
+      <c r="O15" s="8"/>
+      <c r="P15" s="8"/>
+      <c r="Q15" s="8"/>
+      <c r="R15" s="8"/>
+      <c r="S15" s="8"/>
+      <c r="T15" s="8"/>
+      <c r="U15" s="8"/>
+      <c r="V15" s="8"/>
+      <c r="W15" s="8"/>
+      <c r="X15" s="8"/>
+      <c r="Y15" s="8"/>
     </row>
     <row r="16" ht="18" spans="2:25">
-      <c r="B16" s="6" t="s">
+      <c r="B16" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="C16" s="9">
-        <f>C5*SQRT((C15*(POWER(10,-9))/(C13*POWER(10,-6))))</f>
+      <c r="C16" s="10">
+        <f>C5*SQRT((C15*POWER(10,-9))/(C13*POWER(10,-6)))</f>
         <v>0.682288239221013</v>
       </c>
-      <c r="D16" s="7"/>
-      <c r="E16" s="7"/>
-      <c r="F16" s="11">
-        <f>(C15*POWER(10,-9))/(C13*POWER(10,-6))</f>
-        <v>0.000186206896551724</v>
-      </c>
-      <c r="G16" s="11">
-        <f>SQRT(F16)</f>
-        <v>0.0136457647844203</v>
-      </c>
-      <c r="H16" s="7"/>
-      <c r="I16" s="7"/>
-      <c r="J16" s="7"/>
-      <c r="K16" s="7"/>
-      <c r="L16" s="7"/>
-      <c r="M16" s="7"/>
-      <c r="N16" s="7"/>
-      <c r="O16" s="7"/>
-      <c r="P16" s="7"/>
-      <c r="Q16" s="7"/>
-      <c r="R16" s="7"/>
-      <c r="S16" s="7"/>
-      <c r="T16" s="7"/>
-      <c r="U16" s="7"/>
-      <c r="V16" s="7"/>
-      <c r="W16" s="7"/>
-      <c r="X16" s="7"/>
-      <c r="Y16" s="7"/>
+      <c r="D16" s="8"/>
+      <c r="E16" s="8"/>
+      <c r="F16" s="12"/>
+      <c r="G16" s="12"/>
+      <c r="H16" s="8"/>
+      <c r="I16" s="8"/>
+      <c r="J16" s="8"/>
+      <c r="K16" s="8"/>
+      <c r="L16" s="8"/>
+      <c r="M16" s="8"/>
+      <c r="N16" s="8"/>
+      <c r="O16" s="8"/>
+      <c r="P16" s="8"/>
+      <c r="Q16" s="8"/>
+      <c r="R16" s="8"/>
+      <c r="S16" s="8"/>
+      <c r="T16" s="8"/>
+      <c r="U16" s="8"/>
+      <c r="V16" s="8"/>
+      <c r="W16" s="8"/>
+      <c r="X16" s="8"/>
+      <c r="Y16" s="8"/>
     </row>
     <row r="17" ht="18" spans="2:25">
-      <c r="B17" s="6" t="s">
+      <c r="B17" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="C17" s="9">
+      <c r="C17" s="10">
         <f>1/(2*3.14*SQRT((C13/POWER(10,6))*(C15/POWER(10,9))))</f>
         <v>402387.496591775</v>
       </c>
-      <c r="D17" s="7" t="s">
+      <c r="D17" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="E17" s="7"/>
-      <c r="F17" s="7"/>
-      <c r="G17" s="7">
-        <f>50/G16</f>
-        <v>3664.1405439647</v>
-      </c>
-      <c r="H17" s="7"/>
-      <c r="I17" s="7"/>
-      <c r="J17" s="7"/>
-      <c r="K17" s="7"/>
-      <c r="L17" s="7"/>
-      <c r="M17" s="7"/>
-      <c r="N17" s="7"/>
-      <c r="O17" s="7"/>
-      <c r="P17" s="7"/>
-      <c r="Q17" s="7"/>
-      <c r="R17" s="7"/>
-      <c r="S17" s="7"/>
-      <c r="T17" s="7"/>
-      <c r="U17" s="7"/>
-      <c r="V17" s="7"/>
-      <c r="W17" s="7"/>
-      <c r="X17" s="7"/>
-      <c r="Y17" s="7"/>
+      <c r="E17" s="8"/>
+      <c r="F17" s="8"/>
+      <c r="G17" s="8"/>
+      <c r="H17" s="8"/>
+      <c r="I17" s="8"/>
+      <c r="J17" s="8"/>
+      <c r="K17" s="8"/>
+      <c r="L17" s="8"/>
+      <c r="M17" s="8"/>
+      <c r="N17" s="8"/>
+      <c r="O17" s="8"/>
+      <c r="P17" s="8"/>
+      <c r="Q17" s="8"/>
+      <c r="R17" s="8"/>
+      <c r="S17" s="8"/>
+      <c r="T17" s="8"/>
+      <c r="U17" s="8"/>
+      <c r="V17" s="8"/>
+      <c r="W17" s="8"/>
+      <c r="X17" s="8"/>
+      <c r="Y17" s="8"/>
     </row>
     <row r="18" ht="18" spans="2:25">
-      <c r="B18" s="6" t="s">
+      <c r="B18" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="C18" s="9">
+      <c r="C18" s="10">
         <f>20*LOG10(C16)</f>
         <v>-3.3206422940395</v>
       </c>
-      <c r="D18" s="7" t="s">
+      <c r="D18" s="8" t="s">
         <v>48</v>
       </c>
-      <c r="E18" s="7"/>
-      <c r="F18" s="7"/>
-      <c r="G18" s="7"/>
-      <c r="H18" s="7"/>
-      <c r="I18" s="7"/>
-      <c r="J18" s="7"/>
-      <c r="K18" s="7"/>
-      <c r="L18" s="7"/>
-      <c r="M18" s="7"/>
-      <c r="N18" s="7"/>
-      <c r="O18" s="7"/>
-      <c r="P18" s="7"/>
-      <c r="Q18" s="7"/>
-      <c r="R18" s="7"/>
-      <c r="S18" s="7"/>
-      <c r="T18" s="7"/>
-      <c r="U18" s="7"/>
-      <c r="V18" s="7"/>
-      <c r="W18" s="7"/>
-      <c r="X18" s="7"/>
-      <c r="Y18" s="7"/>
+      <c r="E18" s="8"/>
+      <c r="F18" s="8"/>
+      <c r="G18" s="8"/>
+      <c r="H18" s="8"/>
+      <c r="I18" s="8"/>
+      <c r="J18" s="8"/>
+      <c r="K18" s="8"/>
+      <c r="L18" s="8"/>
+      <c r="M18" s="8"/>
+      <c r="N18" s="8"/>
+      <c r="O18" s="8"/>
+      <c r="P18" s="8"/>
+      <c r="Q18" s="8"/>
+      <c r="R18" s="8"/>
+      <c r="S18" s="8"/>
+      <c r="T18" s="8"/>
+      <c r="U18" s="8"/>
+      <c r="V18" s="8"/>
+      <c r="W18" s="8"/>
+      <c r="X18" s="8"/>
+      <c r="Y18" s="8"/>
     </row>
     <row r="19" spans="2:25">
-      <c r="B19" s="12"/>
-      <c r="C19" s="7"/>
-      <c r="D19" s="7"/>
-      <c r="E19" s="7"/>
-      <c r="F19" s="7"/>
-      <c r="G19" s="7"/>
-      <c r="H19" s="7"/>
-      <c r="I19" s="7"/>
-      <c r="J19" s="7"/>
-      <c r="K19" s="7"/>
-      <c r="L19" s="7"/>
-      <c r="M19" s="7"/>
-      <c r="N19" s="7"/>
-      <c r="O19" s="7"/>
-      <c r="P19" s="7"/>
-      <c r="Q19" s="7"/>
-      <c r="R19" s="7"/>
-      <c r="S19" s="7"/>
-      <c r="T19" s="7"/>
-      <c r="U19" s="7"/>
-      <c r="V19" s="7"/>
-      <c r="W19" s="7"/>
-      <c r="X19" s="7"/>
-      <c r="Y19" s="7"/>
+      <c r="B19" s="13"/>
+      <c r="C19" s="8"/>
+      <c r="D19" s="8"/>
+      <c r="E19" s="8"/>
+      <c r="F19" s="8"/>
+      <c r="G19" s="8"/>
+      <c r="H19" s="8"/>
+      <c r="I19" s="8"/>
+      <c r="J19" s="8"/>
+      <c r="K19" s="8"/>
+      <c r="L19" s="8"/>
+      <c r="M19" s="8"/>
+      <c r="N19" s="8"/>
+      <c r="O19" s="8"/>
+      <c r="P19" s="8"/>
+      <c r="Q19" s="8"/>
+      <c r="R19" s="8"/>
+      <c r="S19" s="8"/>
+      <c r="T19" s="8"/>
+      <c r="U19" s="8"/>
+      <c r="V19" s="8"/>
+      <c r="W19" s="8"/>
+      <c r="X19" s="8"/>
+      <c r="Y19" s="8"/>
     </row>
     <row r="20" spans="2:25">
-      <c r="B20" s="12"/>
-      <c r="C20" s="7"/>
-      <c r="D20" s="7"/>
-      <c r="E20" s="7"/>
-      <c r="F20" s="7"/>
-      <c r="G20" s="7"/>
-      <c r="H20" s="7"/>
-      <c r="I20" s="7"/>
-      <c r="J20" s="7"/>
-      <c r="K20" s="7"/>
-      <c r="L20" s="7"/>
-      <c r="M20" s="7"/>
-      <c r="N20" s="7"/>
-      <c r="O20" s="7"/>
-      <c r="P20" s="7"/>
-      <c r="Q20" s="7"/>
-      <c r="R20" s="7"/>
-      <c r="S20" s="7"/>
-      <c r="T20" s="7"/>
-      <c r="U20" s="7"/>
-      <c r="V20" s="7"/>
-      <c r="W20" s="7"/>
-      <c r="X20" s="7"/>
-      <c r="Y20" s="7"/>
+      <c r="B20" s="13"/>
+      <c r="C20" s="8"/>
+      <c r="D20" s="8"/>
+      <c r="E20" s="8"/>
+      <c r="F20" s="8"/>
+      <c r="G20" s="8"/>
+      <c r="H20" s="8"/>
+      <c r="I20" s="8"/>
+      <c r="J20" s="8"/>
+      <c r="K20" s="8"/>
+      <c r="L20" s="8"/>
+      <c r="M20" s="8"/>
+      <c r="N20" s="8"/>
+      <c r="O20" s="8"/>
+      <c r="P20" s="8"/>
+      <c r="Q20" s="8"/>
+      <c r="R20" s="8"/>
+      <c r="S20" s="8"/>
+      <c r="T20" s="8"/>
+      <c r="U20" s="8"/>
+      <c r="V20" s="8"/>
+      <c r="W20" s="8"/>
+      <c r="X20" s="8"/>
+      <c r="Y20" s="8"/>
     </row>
     <row r="21" spans="2:25">
-      <c r="B21" s="12"/>
-      <c r="C21" s="7"/>
-      <c r="D21" s="7"/>
-      <c r="E21" s="7"/>
-      <c r="F21" s="7"/>
-      <c r="G21" s="7"/>
-      <c r="H21" s="7"/>
-      <c r="I21" s="7"/>
-      <c r="J21" s="7"/>
-      <c r="K21" s="7"/>
-      <c r="L21" s="7"/>
-      <c r="M21" s="7"/>
-      <c r="N21" s="7"/>
-      <c r="O21" s="7"/>
-      <c r="P21" s="7"/>
-      <c r="Q21" s="7"/>
-      <c r="R21" s="7"/>
-      <c r="S21" s="7"/>
-      <c r="T21" s="7"/>
-      <c r="U21" s="7"/>
-      <c r="V21" s="7"/>
-      <c r="W21" s="7"/>
-      <c r="X21" s="7"/>
-      <c r="Y21" s="7"/>
+      <c r="B21" s="13"/>
+      <c r="C21" s="8"/>
+      <c r="D21" s="8"/>
+      <c r="E21" s="8"/>
+      <c r="F21" s="8"/>
+      <c r="G21" s="8"/>
+      <c r="H21" s="8"/>
+      <c r="I21" s="8"/>
+      <c r="J21" s="8"/>
+      <c r="K21" s="8"/>
+      <c r="L21" s="8"/>
+      <c r="M21" s="8"/>
+      <c r="N21" s="8"/>
+      <c r="O21" s="8"/>
+      <c r="P21" s="8"/>
+      <c r="Q21" s="8"/>
+      <c r="R21" s="8"/>
+      <c r="S21" s="8"/>
+      <c r="T21" s="8"/>
+      <c r="U21" s="8"/>
+      <c r="V21" s="8"/>
+      <c r="W21" s="8"/>
+      <c r="X21" s="8"/>
+      <c r="Y21" s="8"/>
     </row>
     <row r="22" spans="2:25">
-      <c r="B22" s="12"/>
-      <c r="C22" s="7"/>
-      <c r="D22" s="7"/>
-      <c r="E22" s="7"/>
-      <c r="F22" s="7"/>
-      <c r="G22" s="7"/>
-      <c r="H22" s="7"/>
-      <c r="I22" s="7"/>
-      <c r="J22" s="7"/>
-      <c r="K22" s="7"/>
-      <c r="L22" s="7"/>
-      <c r="M22" s="7"/>
-      <c r="N22" s="7"/>
-      <c r="O22" s="7"/>
-      <c r="P22" s="7"/>
-      <c r="Q22" s="7"/>
-      <c r="R22" s="7"/>
-      <c r="S22" s="7"/>
-      <c r="T22" s="7"/>
-      <c r="U22" s="7"/>
-      <c r="V22" s="7"/>
-      <c r="W22" s="7"/>
-      <c r="X22" s="7"/>
-      <c r="Y22" s="7"/>
+      <c r="B22" s="13"/>
+      <c r="C22" s="8"/>
+      <c r="D22" s="8"/>
+      <c r="E22" s="8"/>
+      <c r="F22" s="8"/>
+      <c r="G22" s="8"/>
+      <c r="H22" s="8"/>
+      <c r="I22" s="8"/>
+      <c r="J22" s="8"/>
+      <c r="K22" s="8"/>
+      <c r="L22" s="8"/>
+      <c r="M22" s="8"/>
+      <c r="N22" s="8"/>
+      <c r="O22" s="8"/>
+      <c r="P22" s="8"/>
+      <c r="Q22" s="8"/>
+      <c r="R22" s="8"/>
+      <c r="S22" s="8"/>
+      <c r="T22" s="8"/>
+      <c r="U22" s="8"/>
+      <c r="V22" s="8"/>
+      <c r="W22" s="8"/>
+      <c r="X22" s="8"/>
+      <c r="Y22" s="8"/>
     </row>
     <row r="23" spans="2:25">
-      <c r="B23" s="12"/>
-      <c r="C23" s="7"/>
-      <c r="D23" s="7"/>
-      <c r="E23" s="7"/>
-      <c r="F23" s="7"/>
-      <c r="G23" s="7"/>
-      <c r="H23" s="7"/>
-      <c r="I23" s="7"/>
-      <c r="J23" s="7"/>
-      <c r="K23" s="7"/>
-      <c r="L23" s="7"/>
-      <c r="M23" s="7"/>
-      <c r="N23" s="7"/>
-      <c r="O23" s="7"/>
-      <c r="P23" s="7"/>
-      <c r="Q23" s="7"/>
-      <c r="R23" s="7"/>
-      <c r="S23" s="7"/>
-      <c r="T23" s="7"/>
-      <c r="U23" s="7"/>
-      <c r="V23" s="7"/>
-      <c r="W23" s="7"/>
-      <c r="X23" s="7"/>
-      <c r="Y23" s="7"/>
+      <c r="B23" s="13"/>
+      <c r="C23" s="8"/>
+      <c r="D23" s="8"/>
+      <c r="E23" s="8"/>
+      <c r="F23" s="8"/>
+      <c r="G23" s="8"/>
+      <c r="H23" s="8"/>
+      <c r="I23" s="8"/>
+      <c r="J23" s="8"/>
+      <c r="K23" s="8"/>
+      <c r="L23" s="8"/>
+      <c r="M23" s="8"/>
+      <c r="N23" s="8"/>
+      <c r="O23" s="8"/>
+      <c r="P23" s="8"/>
+      <c r="Q23" s="8"/>
+      <c r="R23" s="8"/>
+      <c r="S23" s="8"/>
+      <c r="T23" s="8"/>
+      <c r="U23" s="8"/>
+      <c r="V23" s="8"/>
+      <c r="W23" s="8"/>
+      <c r="X23" s="8"/>
+      <c r="Y23" s="8"/>
     </row>
     <row r="24" spans="2:25">
-      <c r="B24" s="12"/>
-      <c r="C24" s="7"/>
-      <c r="D24" s="7"/>
-      <c r="E24" s="7"/>
-      <c r="F24" s="7"/>
-      <c r="G24" s="7"/>
-      <c r="H24" s="7"/>
-      <c r="I24" s="7"/>
-      <c r="J24" s="7"/>
-      <c r="K24" s="7"/>
-      <c r="L24" s="7"/>
-      <c r="M24" s="7"/>
-      <c r="N24" s="7"/>
-      <c r="O24" s="7"/>
-      <c r="P24" s="7"/>
-      <c r="Q24" s="7"/>
-      <c r="R24" s="7"/>
-      <c r="S24" s="7"/>
-      <c r="T24" s="7"/>
-      <c r="U24" s="7"/>
-      <c r="V24" s="7"/>
-      <c r="W24" s="7"/>
-      <c r="X24" s="7"/>
-      <c r="Y24" s="7"/>
+      <c r="B24" s="13"/>
+      <c r="C24" s="8"/>
+      <c r="D24" s="8"/>
+      <c r="E24" s="8"/>
+      <c r="F24" s="8"/>
+      <c r="G24" s="8"/>
+      <c r="H24" s="8"/>
+      <c r="I24" s="8"/>
+      <c r="J24" s="8"/>
+      <c r="K24" s="8"/>
+      <c r="L24" s="8"/>
+      <c r="M24" s="8"/>
+      <c r="N24" s="8"/>
+      <c r="O24" s="8"/>
+      <c r="P24" s="8"/>
+      <c r="Q24" s="8"/>
+      <c r="R24" s="8"/>
+      <c r="S24" s="8"/>
+      <c r="T24" s="8"/>
+      <c r="U24" s="8"/>
+      <c r="V24" s="8"/>
+      <c r="W24" s="8"/>
+      <c r="X24" s="8"/>
+      <c r="Y24" s="8"/>
     </row>
     <row r="25" spans="2:25">
-      <c r="B25" s="12"/>
-      <c r="C25" s="7"/>
-      <c r="D25" s="7"/>
-      <c r="E25" s="7"/>
-      <c r="F25" s="7"/>
-      <c r="G25" s="7"/>
-      <c r="H25" s="7"/>
-      <c r="I25" s="7"/>
-      <c r="J25" s="7"/>
-      <c r="K25" s="7"/>
-      <c r="L25" s="7"/>
-      <c r="M25" s="7"/>
-      <c r="N25" s="7"/>
-      <c r="O25" s="7"/>
-      <c r="P25" s="7"/>
-      <c r="Q25" s="7"/>
-      <c r="R25" s="7"/>
-      <c r="S25" s="7"/>
-      <c r="T25" s="7"/>
-      <c r="U25" s="7"/>
-      <c r="V25" s="7"/>
-      <c r="W25" s="7"/>
-      <c r="X25" s="7"/>
-      <c r="Y25" s="7"/>
+      <c r="B25" s="13"/>
+      <c r="C25" s="8"/>
+      <c r="D25" s="8"/>
+      <c r="E25" s="8"/>
+      <c r="F25" s="8"/>
+      <c r="G25" s="8"/>
+      <c r="H25" s="8"/>
+      <c r="I25" s="8"/>
+      <c r="J25" s="8"/>
+      <c r="K25" s="8"/>
+      <c r="L25" s="8"/>
+      <c r="M25" s="8"/>
+      <c r="N25" s="8"/>
+      <c r="O25" s="8"/>
+      <c r="P25" s="8"/>
+      <c r="Q25" s="8"/>
+      <c r="R25" s="8"/>
+      <c r="S25" s="8"/>
+      <c r="T25" s="8"/>
+      <c r="U25" s="8"/>
+      <c r="V25" s="8"/>
+      <c r="W25" s="8"/>
+      <c r="X25" s="8"/>
+      <c r="Y25" s="8"/>
     </row>
     <row r="26" spans="2:25">
-      <c r="B26" s="12"/>
-      <c r="C26" s="7"/>
-      <c r="D26" s="7"/>
-      <c r="E26" s="7"/>
-      <c r="F26" s="7"/>
-      <c r="G26" s="7"/>
-      <c r="H26" s="7"/>
-      <c r="I26" s="7"/>
-      <c r="J26" s="7"/>
-      <c r="K26" s="7"/>
-      <c r="L26" s="7"/>
-      <c r="M26" s="7"/>
-      <c r="N26" s="7"/>
-      <c r="O26" s="7"/>
-      <c r="P26" s="7"/>
-      <c r="Q26" s="7"/>
-      <c r="R26" s="7"/>
-      <c r="S26" s="7"/>
-      <c r="T26" s="7"/>
-      <c r="U26" s="7"/>
-      <c r="V26" s="7"/>
-      <c r="W26" s="7"/>
-      <c r="X26" s="7"/>
-      <c r="Y26" s="7"/>
+      <c r="B26" s="13"/>
+      <c r="C26" s="8"/>
+      <c r="D26" s="8"/>
+      <c r="E26" s="8"/>
+      <c r="F26" s="8"/>
+      <c r="G26" s="8"/>
+      <c r="H26" s="8"/>
+      <c r="I26" s="8"/>
+      <c r="J26" s="8"/>
+      <c r="K26" s="8"/>
+      <c r="L26" s="8"/>
+      <c r="M26" s="8"/>
+      <c r="N26" s="8"/>
+      <c r="O26" s="8"/>
+      <c r="P26" s="8"/>
+      <c r="Q26" s="8"/>
+      <c r="R26" s="8"/>
+      <c r="S26" s="8"/>
+      <c r="T26" s="8"/>
+      <c r="U26" s="8"/>
+      <c r="V26" s="8"/>
+      <c r="W26" s="8"/>
+      <c r="X26" s="8"/>
+      <c r="Y26" s="8"/>
     </row>
     <row r="27" spans="2:25">
-      <c r="B27" s="12"/>
-      <c r="C27" s="7"/>
-      <c r="D27" s="7"/>
-      <c r="E27" s="7"/>
-      <c r="F27" s="7"/>
-      <c r="G27" s="7"/>
-      <c r="H27" s="7"/>
-      <c r="I27" s="7"/>
-      <c r="J27" s="7"/>
-      <c r="K27" s="7"/>
-      <c r="L27" s="7"/>
-      <c r="M27" s="7"/>
-      <c r="N27" s="7"/>
-      <c r="O27" s="7"/>
-      <c r="P27" s="7"/>
-      <c r="Q27" s="7"/>
-      <c r="R27" s="7"/>
-      <c r="S27" s="7"/>
-      <c r="T27" s="7"/>
-      <c r="U27" s="7"/>
-      <c r="V27" s="7"/>
-      <c r="W27" s="7"/>
-      <c r="X27" s="7"/>
-      <c r="Y27" s="7"/>
+      <c r="B27" s="13"/>
+      <c r="C27" s="8"/>
+      <c r="D27" s="8"/>
+      <c r="E27" s="8"/>
+      <c r="F27" s="8"/>
+      <c r="G27" s="8"/>
+      <c r="H27" s="8"/>
+      <c r="I27" s="8"/>
+      <c r="J27" s="8"/>
+      <c r="K27" s="8"/>
+      <c r="L27" s="8"/>
+      <c r="M27" s="8"/>
+      <c r="N27" s="8"/>
+      <c r="O27" s="8"/>
+      <c r="P27" s="8"/>
+      <c r="Q27" s="8"/>
+      <c r="R27" s="8"/>
+      <c r="S27" s="8"/>
+      <c r="T27" s="8"/>
+      <c r="U27" s="8"/>
+      <c r="V27" s="8"/>
+      <c r="W27" s="8"/>
+      <c r="X27" s="8"/>
+      <c r="Y27" s="8"/>
     </row>
     <row r="28" spans="2:25">
-      <c r="B28" s="12"/>
-      <c r="C28" s="7"/>
-      <c r="D28" s="7"/>
-      <c r="E28" s="7"/>
-      <c r="F28" s="7"/>
-      <c r="G28" s="7"/>
-      <c r="H28" s="7"/>
-      <c r="I28" s="7"/>
-      <c r="J28" s="7"/>
-      <c r="K28" s="7"/>
-      <c r="L28" s="7"/>
-      <c r="M28" s="7"/>
-      <c r="N28" s="7"/>
-      <c r="O28" s="7"/>
-      <c r="P28" s="7"/>
-      <c r="Q28" s="7"/>
-      <c r="R28" s="7"/>
-      <c r="S28" s="7"/>
-      <c r="T28" s="7"/>
-      <c r="U28" s="7"/>
-      <c r="V28" s="7"/>
-      <c r="W28" s="7"/>
-      <c r="X28" s="7"/>
-      <c r="Y28" s="7"/>
+      <c r="B28" s="13"/>
+      <c r="C28" s="8"/>
+      <c r="D28" s="8"/>
+      <c r="E28" s="8"/>
+      <c r="F28" s="8"/>
+      <c r="G28" s="8"/>
+      <c r="H28" s="8"/>
+      <c r="I28" s="8"/>
+      <c r="J28" s="8"/>
+      <c r="K28" s="8"/>
+      <c r="L28" s="8"/>
+      <c r="M28" s="8"/>
+      <c r="N28" s="8"/>
+      <c r="O28" s="8"/>
+      <c r="P28" s="8"/>
+      <c r="Q28" s="8"/>
+      <c r="R28" s="8"/>
+      <c r="S28" s="8"/>
+      <c r="T28" s="8"/>
+      <c r="U28" s="8"/>
+      <c r="V28" s="8"/>
+      <c r="W28" s="8"/>
+      <c r="X28" s="8"/>
+      <c r="Y28" s="8"/>
     </row>
     <row r="29" spans="2:25">
-      <c r="B29" s="12"/>
-      <c r="C29" s="7"/>
-      <c r="D29" s="7"/>
-      <c r="E29" s="7"/>
-      <c r="F29" s="7"/>
-      <c r="G29" s="7"/>
-      <c r="H29" s="7"/>
-      <c r="I29" s="7"/>
-      <c r="J29" s="7"/>
-      <c r="K29" s="7"/>
-      <c r="L29" s="7"/>
-      <c r="M29" s="7"/>
-      <c r="N29" s="7"/>
-      <c r="O29" s="7"/>
-      <c r="P29" s="7"/>
-      <c r="Q29" s="7"/>
-      <c r="R29" s="7"/>
-      <c r="S29" s="7"/>
-      <c r="T29" s="7"/>
-      <c r="U29" s="7"/>
-      <c r="V29" s="7"/>
-      <c r="W29" s="7"/>
-      <c r="X29" s="7"/>
-      <c r="Y29" s="7"/>
+      <c r="B29" s="13"/>
+      <c r="C29" s="8"/>
+      <c r="D29" s="8"/>
+      <c r="E29" s="8"/>
+      <c r="F29" s="8"/>
+      <c r="G29" s="8"/>
+      <c r="H29" s="8"/>
+      <c r="I29" s="8"/>
+      <c r="J29" s="8"/>
+      <c r="K29" s="8"/>
+      <c r="L29" s="8"/>
+      <c r="M29" s="8"/>
+      <c r="N29" s="8"/>
+      <c r="O29" s="8"/>
+      <c r="P29" s="8"/>
+      <c r="Q29" s="8"/>
+      <c r="R29" s="8"/>
+      <c r="S29" s="8"/>
+      <c r="T29" s="8"/>
+      <c r="U29" s="8"/>
+      <c r="V29" s="8"/>
+      <c r="W29" s="8"/>
+      <c r="X29" s="8"/>
+      <c r="Y29" s="8"/>
     </row>
     <row r="30" spans="2:25">
-      <c r="B30" s="12"/>
-      <c r="C30" s="7"/>
-      <c r="D30" s="7"/>
-      <c r="E30" s="7"/>
-      <c r="F30" s="7"/>
-      <c r="G30" s="7"/>
-      <c r="H30" s="7"/>
-      <c r="I30" s="7"/>
-      <c r="J30" s="7"/>
-      <c r="K30" s="7"/>
-      <c r="L30" s="7"/>
-      <c r="M30" s="7"/>
-      <c r="N30" s="7"/>
-      <c r="O30" s="7"/>
-      <c r="P30" s="7"/>
-      <c r="Q30" s="7"/>
-      <c r="R30" s="7"/>
-      <c r="S30" s="7"/>
-      <c r="T30" s="7"/>
-      <c r="U30" s="7"/>
-      <c r="V30" s="7"/>
-      <c r="W30" s="7"/>
-      <c r="X30" s="7"/>
-      <c r="Y30" s="7"/>
+      <c r="B30" s="13"/>
+      <c r="C30" s="8"/>
+      <c r="D30" s="8"/>
+      <c r="E30" s="8"/>
+      <c r="F30" s="8"/>
+      <c r="G30" s="8"/>
+      <c r="H30" s="8"/>
+      <c r="I30" s="8"/>
+      <c r="J30" s="8"/>
+      <c r="K30" s="8"/>
+      <c r="L30" s="8"/>
+      <c r="M30" s="8"/>
+      <c r="N30" s="8"/>
+      <c r="O30" s="8"/>
+      <c r="P30" s="8"/>
+      <c r="Q30" s="8"/>
+      <c r="R30" s="8"/>
+      <c r="S30" s="8"/>
+      <c r="T30" s="8"/>
+      <c r="U30" s="8"/>
+      <c r="V30" s="8"/>
+      <c r="W30" s="8"/>
+      <c r="X30" s="8"/>
+      <c r="Y30" s="8"/>
     </row>
     <row r="31" spans="2:25">
-      <c r="B31" s="12"/>
-      <c r="C31" s="7"/>
-      <c r="D31" s="7"/>
-      <c r="E31" s="7"/>
-      <c r="F31" s="7"/>
-      <c r="G31" s="7"/>
-      <c r="H31" s="7"/>
-      <c r="I31" s="7"/>
-      <c r="J31" s="7"/>
-      <c r="K31" s="7"/>
-      <c r="L31" s="7"/>
-      <c r="M31" s="7"/>
-      <c r="N31" s="7"/>
-      <c r="O31" s="7"/>
-      <c r="P31" s="7"/>
-      <c r="Q31" s="7"/>
-      <c r="R31" s="7"/>
-      <c r="S31" s="7"/>
-      <c r="T31" s="7"/>
-      <c r="U31" s="7"/>
-      <c r="V31" s="7"/>
-      <c r="W31" s="7"/>
-      <c r="X31" s="7"/>
-      <c r="Y31" s="7"/>
+      <c r="B31" s="13"/>
+      <c r="C31" s="8"/>
+      <c r="D31" s="8"/>
+      <c r="E31" s="8"/>
+      <c r="F31" s="8"/>
+      <c r="G31" s="8"/>
+      <c r="H31" s="8"/>
+      <c r="I31" s="8"/>
+      <c r="J31" s="8"/>
+      <c r="K31" s="8"/>
+      <c r="L31" s="8"/>
+      <c r="M31" s="8"/>
+      <c r="N31" s="8"/>
+      <c r="O31" s="8"/>
+      <c r="P31" s="8"/>
+      <c r="Q31" s="8"/>
+      <c r="R31" s="8"/>
+      <c r="S31" s="8"/>
+      <c r="T31" s="8"/>
+      <c r="U31" s="8"/>
+      <c r="V31" s="8"/>
+      <c r="W31" s="8"/>
+      <c r="X31" s="8"/>
+      <c r="Y31" s="8"/>
     </row>
     <row r="32" spans="2:25">
-      <c r="B32" s="12"/>
-      <c r="C32" s="7"/>
-      <c r="D32" s="7"/>
-      <c r="E32" s="7"/>
-      <c r="F32" s="7"/>
-      <c r="G32" s="7"/>
-      <c r="H32" s="7"/>
-      <c r="I32" s="7"/>
-      <c r="J32" s="7"/>
-      <c r="K32" s="7"/>
-      <c r="L32" s="7"/>
-      <c r="M32" s="7"/>
-      <c r="N32" s="7"/>
-      <c r="O32" s="7"/>
-      <c r="P32" s="7"/>
-      <c r="Q32" s="7"/>
-      <c r="R32" s="7"/>
-      <c r="S32" s="7"/>
-      <c r="T32" s="7"/>
-      <c r="U32" s="7"/>
-      <c r="V32" s="7"/>
-      <c r="W32" s="7"/>
-      <c r="X32" s="7"/>
-      <c r="Y32" s="7"/>
+      <c r="B32" s="13"/>
+      <c r="C32" s="8"/>
+      <c r="D32" s="8"/>
+      <c r="E32" s="8"/>
+      <c r="F32" s="8"/>
+      <c r="G32" s="8"/>
+      <c r="H32" s="8"/>
+      <c r="I32" s="8"/>
+      <c r="J32" s="8"/>
+      <c r="K32" s="8"/>
+      <c r="L32" s="8"/>
+      <c r="M32" s="8"/>
+      <c r="N32" s="8"/>
+      <c r="O32" s="8"/>
+      <c r="P32" s="8"/>
+      <c r="Q32" s="8"/>
+      <c r="R32" s="8"/>
+      <c r="S32" s="8"/>
+      <c r="T32" s="8"/>
+      <c r="U32" s="8"/>
+      <c r="V32" s="8"/>
+      <c r="W32" s="8"/>
+      <c r="X32" s="8"/>
+      <c r="Y32" s="8"/>
     </row>
     <row r="33" spans="2:25">
-      <c r="B33" s="12"/>
-      <c r="C33" s="7"/>
-      <c r="D33" s="7"/>
-      <c r="E33" s="7"/>
-      <c r="F33" s="7"/>
-      <c r="G33" s="7"/>
-      <c r="H33" s="7"/>
-      <c r="I33" s="7"/>
-      <c r="J33" s="7"/>
-      <c r="K33" s="7"/>
-      <c r="L33" s="7"/>
-      <c r="M33" s="7"/>
-      <c r="N33" s="7"/>
-      <c r="O33" s="7"/>
-      <c r="P33" s="7"/>
-      <c r="Q33" s="7"/>
-      <c r="R33" s="7"/>
-      <c r="S33" s="7"/>
-      <c r="T33" s="7"/>
-      <c r="U33" s="7"/>
-      <c r="V33" s="7"/>
-      <c r="W33" s="7"/>
-      <c r="X33" s="7"/>
-      <c r="Y33" s="7"/>
+      <c r="B33" s="13"/>
+      <c r="C33" s="8"/>
+      <c r="D33" s="8"/>
+      <c r="E33" s="8"/>
+      <c r="F33" s="8"/>
+      <c r="G33" s="8"/>
+      <c r="H33" s="8"/>
+      <c r="I33" s="8"/>
+      <c r="J33" s="8"/>
+      <c r="K33" s="8"/>
+      <c r="L33" s="8"/>
+      <c r="M33" s="8"/>
+      <c r="N33" s="8"/>
+      <c r="O33" s="8"/>
+      <c r="P33" s="8"/>
+      <c r="Q33" s="8"/>
+      <c r="R33" s="8"/>
+      <c r="S33" s="8"/>
+      <c r="T33" s="8"/>
+      <c r="U33" s="8"/>
+      <c r="V33" s="8"/>
+      <c r="W33" s="8"/>
+      <c r="X33" s="8"/>
+      <c r="Y33" s="8"/>
     </row>
     <row r="34" spans="2:25">
-      <c r="B34" s="12"/>
-      <c r="C34" s="7"/>
-      <c r="D34" s="7"/>
-      <c r="E34" s="7"/>
-      <c r="F34" s="7"/>
-      <c r="G34" s="7"/>
-      <c r="H34" s="7"/>
-      <c r="I34" s="7"/>
-      <c r="J34" s="7"/>
-      <c r="K34" s="7"/>
-      <c r="L34" s="7"/>
-      <c r="M34" s="7"/>
-      <c r="N34" s="7"/>
-      <c r="O34" s="7"/>
-      <c r="P34" s="7"/>
-      <c r="Q34" s="7"/>
-      <c r="R34" s="7"/>
-      <c r="S34" s="7"/>
-      <c r="T34" s="7"/>
-      <c r="U34" s="7"/>
-      <c r="V34" s="7"/>
-      <c r="W34" s="7"/>
-      <c r="X34" s="7"/>
-      <c r="Y34" s="7"/>
+      <c r="B34" s="13"/>
+      <c r="C34" s="8"/>
+      <c r="D34" s="8"/>
+      <c r="E34" s="8"/>
+      <c r="F34" s="8"/>
+      <c r="G34" s="8"/>
+      <c r="H34" s="8"/>
+      <c r="I34" s="8"/>
+      <c r="J34" s="8"/>
+      <c r="K34" s="8"/>
+      <c r="L34" s="8"/>
+      <c r="M34" s="8"/>
+      <c r="N34" s="8"/>
+      <c r="O34" s="8"/>
+      <c r="P34" s="8"/>
+      <c r="Q34" s="8"/>
+      <c r="R34" s="8"/>
+      <c r="S34" s="8"/>
+      <c r="T34" s="8"/>
+      <c r="U34" s="8"/>
+      <c r="V34" s="8"/>
+      <c r="W34" s="8"/>
+      <c r="X34" s="8"/>
+      <c r="Y34" s="8"/>
     </row>
     <row r="35" spans="2:25">
-      <c r="B35" s="12"/>
-      <c r="C35" s="7"/>
-      <c r="D35" s="7"/>
-      <c r="E35" s="7"/>
-      <c r="F35" s="7"/>
-      <c r="G35" s="7"/>
-      <c r="H35" s="7"/>
-      <c r="I35" s="7"/>
-      <c r="J35" s="7"/>
-      <c r="K35" s="7"/>
-      <c r="L35" s="7"/>
-      <c r="M35" s="7"/>
-      <c r="N35" s="7"/>
-      <c r="O35" s="7"/>
-      <c r="P35" s="7"/>
-      <c r="Q35" s="7"/>
-      <c r="R35" s="7"/>
-      <c r="S35" s="7"/>
-      <c r="T35" s="7"/>
-      <c r="U35" s="7"/>
-      <c r="V35" s="7"/>
-      <c r="W35" s="7"/>
-      <c r="X35" s="7"/>
-      <c r="Y35" s="7"/>
+      <c r="B35" s="13"/>
+      <c r="C35" s="8"/>
+      <c r="D35" s="8"/>
+      <c r="E35" s="8"/>
+      <c r="F35" s="8"/>
+      <c r="G35" s="8"/>
+      <c r="H35" s="8"/>
+      <c r="I35" s="8"/>
+      <c r="J35" s="8"/>
+      <c r="K35" s="8"/>
+      <c r="L35" s="8"/>
+      <c r="M35" s="8"/>
+      <c r="N35" s="8"/>
+      <c r="O35" s="8"/>
+      <c r="P35" s="8"/>
+      <c r="Q35" s="8"/>
+      <c r="R35" s="8"/>
+      <c r="S35" s="8"/>
+      <c r="T35" s="8"/>
+      <c r="U35" s="8"/>
+      <c r="V35" s="8"/>
+      <c r="W35" s="8"/>
+      <c r="X35" s="8"/>
+      <c r="Y35" s="8"/>
     </row>
     <row r="36" spans="2:25">
-      <c r="B36" s="12"/>
-      <c r="C36" s="7"/>
-      <c r="D36" s="7"/>
-      <c r="E36" s="7"/>
-      <c r="F36" s="7"/>
-      <c r="G36" s="7"/>
-      <c r="H36" s="7"/>
-      <c r="I36" s="7"/>
-      <c r="J36" s="7"/>
-      <c r="K36" s="7"/>
-      <c r="L36" s="7"/>
-      <c r="M36" s="7"/>
-      <c r="N36" s="7"/>
-      <c r="O36" s="7"/>
-      <c r="P36" s="7"/>
-      <c r="Q36" s="7"/>
-      <c r="R36" s="7"/>
-      <c r="S36" s="7"/>
-      <c r="T36" s="7"/>
-      <c r="U36" s="7"/>
-      <c r="V36" s="7"/>
-      <c r="W36" s="7"/>
-      <c r="X36" s="7"/>
-      <c r="Y36" s="7"/>
+      <c r="B36" s="13"/>
+      <c r="C36" s="8"/>
+      <c r="D36" s="8"/>
+      <c r="E36" s="8"/>
+      <c r="F36" s="8"/>
+      <c r="G36" s="8"/>
+      <c r="H36" s="8"/>
+      <c r="I36" s="8"/>
+      <c r="J36" s="8"/>
+      <c r="K36" s="8"/>
+      <c r="L36" s="8"/>
+      <c r="M36" s="8"/>
+      <c r="N36" s="8"/>
+      <c r="O36" s="8"/>
+      <c r="P36" s="8"/>
+      <c r="Q36" s="8"/>
+      <c r="R36" s="8"/>
+      <c r="S36" s="8"/>
+      <c r="T36" s="8"/>
+      <c r="U36" s="8"/>
+      <c r="V36" s="8"/>
+      <c r="W36" s="8"/>
+      <c r="X36" s="8"/>
+      <c r="Y36" s="8"/>
     </row>
     <row r="37" spans="2:25">
-      <c r="B37" s="12"/>
-      <c r="C37" s="7"/>
-      <c r="D37" s="7"/>
-      <c r="E37" s="7"/>
-      <c r="F37" s="7"/>
-      <c r="G37" s="7"/>
-      <c r="H37" s="7"/>
-      <c r="I37" s="7"/>
-      <c r="J37" s="7"/>
-      <c r="K37" s="7"/>
-      <c r="L37" s="7"/>
-      <c r="M37" s="7"/>
-      <c r="N37" s="7"/>
-      <c r="O37" s="7"/>
-      <c r="P37" s="7"/>
-      <c r="Q37" s="7"/>
-      <c r="R37" s="7"/>
-      <c r="S37" s="7"/>
-      <c r="T37" s="7"/>
-      <c r="U37" s="7"/>
-      <c r="V37" s="7"/>
-      <c r="W37" s="7"/>
-      <c r="X37" s="7"/>
-      <c r="Y37" s="7"/>
+      <c r="B37" s="13"/>
+      <c r="C37" s="8"/>
+      <c r="D37" s="8"/>
+      <c r="E37" s="8"/>
+      <c r="F37" s="8"/>
+      <c r="G37" s="8"/>
+      <c r="H37" s="8"/>
+      <c r="I37" s="8"/>
+      <c r="J37" s="8"/>
+      <c r="K37" s="8"/>
+      <c r="L37" s="8"/>
+      <c r="M37" s="8"/>
+      <c r="N37" s="8"/>
+      <c r="O37" s="8"/>
+      <c r="P37" s="8"/>
+      <c r="Q37" s="8"/>
+      <c r="R37" s="8"/>
+      <c r="S37" s="8"/>
+      <c r="T37" s="8"/>
+      <c r="U37" s="8"/>
+      <c r="V37" s="8"/>
+      <c r="W37" s="8"/>
+      <c r="X37" s="8"/>
+      <c r="Y37" s="8"/>
     </row>
     <row r="38" spans="2:25">
-      <c r="B38" s="12"/>
-      <c r="C38" s="7"/>
-      <c r="D38" s="7"/>
-      <c r="E38" s="7"/>
-      <c r="F38" s="7"/>
-      <c r="G38" s="7"/>
-      <c r="H38" s="7"/>
-      <c r="I38" s="7"/>
-      <c r="J38" s="7"/>
-      <c r="K38" s="7"/>
-      <c r="L38" s="7"/>
-      <c r="M38" s="7"/>
-      <c r="N38" s="7"/>
-      <c r="O38" s="7"/>
-      <c r="P38" s="7"/>
-      <c r="Q38" s="7"/>
-      <c r="R38" s="7"/>
-      <c r="S38" s="7"/>
-      <c r="T38" s="7"/>
-      <c r="U38" s="7"/>
-      <c r="V38" s="7"/>
-      <c r="W38" s="7"/>
-      <c r="X38" s="7"/>
-      <c r="Y38" s="7"/>
+      <c r="B38" s="13"/>
+      <c r="C38" s="8"/>
+      <c r="D38" s="8"/>
+      <c r="E38" s="8"/>
+      <c r="F38" s="8"/>
+      <c r="G38" s="8"/>
+      <c r="H38" s="8"/>
+      <c r="I38" s="8"/>
+      <c r="J38" s="8"/>
+      <c r="K38" s="8"/>
+      <c r="L38" s="8"/>
+      <c r="M38" s="8"/>
+      <c r="N38" s="8"/>
+      <c r="O38" s="8"/>
+      <c r="P38" s="8"/>
+      <c r="Q38" s="8"/>
+      <c r="R38" s="8"/>
+      <c r="S38" s="8"/>
+      <c r="T38" s="8"/>
+      <c r="U38" s="8"/>
+      <c r="V38" s="8"/>
+      <c r="W38" s="8"/>
+      <c r="X38" s="8"/>
+      <c r="Y38" s="8"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -5901,306 +5881,306 @@
   <dimension ref="B1:F18"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.8" outlineLevelCol="5"/>
   <cols>
-    <col min="1" max="4" width="9" style="1"/>
-    <col min="5" max="5" width="6.875" style="1" customWidth="1"/>
-    <col min="6" max="6" width="26.1640625" style="1" customWidth="1"/>
-    <col min="7" max="16384" width="9" style="1"/>
+    <col min="1" max="4" width="9" style="2"/>
+    <col min="5" max="5" width="6.875" style="2" customWidth="1"/>
+    <col min="6" max="6" width="26.1640625" style="2" customWidth="1"/>
+    <col min="7" max="16384" width="9" style="2"/>
   </cols>
   <sheetData>
     <row r="1" spans="2:3">
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="2" spans="2:6">
-      <c r="B2" s="2">
+      <c r="B2" s="3">
         <v>10</v>
       </c>
-      <c r="C2" s="2">
+      <c r="C2" s="3">
         <v>-0.1</v>
       </c>
-      <c r="D2" s="2">
+      <c r="D2" s="3">
         <v>0.989</v>
       </c>
-      <c r="E2" s="3">
+      <c r="E2" s="4">
         <v>0.989</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="F2" s="3" t="s">
         <v>51</v>
       </c>
     </row>
     <row r="3" spans="2:6">
-      <c r="B3" s="2">
+      <c r="B3" s="3">
         <v>50</v>
       </c>
-      <c r="C3" s="2">
+      <c r="C3" s="3">
         <v>-0.2</v>
       </c>
-      <c r="D3" s="2">
+      <c r="D3" s="3">
         <v>0.977</v>
       </c>
-      <c r="E3" s="3">
+      <c r="E3" s="4">
         <v>0.977</v>
       </c>
-      <c r="F3" s="2" t="s">
+      <c r="F3" s="3" t="s">
         <v>51</v>
       </c>
     </row>
     <row r="4" spans="2:6">
-      <c r="B4" s="2">
+      <c r="B4" s="3">
         <v>100</v>
       </c>
-      <c r="C4" s="2">
+      <c r="C4" s="3">
         <v>-0.8</v>
       </c>
-      <c r="D4" s="2">
+      <c r="D4" s="3">
         <v>0.912</v>
       </c>
-      <c r="E4" s="3">
+      <c r="E4" s="4">
         <v>0.912</v>
       </c>
-      <c r="F4" s="2" t="s">
+      <c r="F4" s="3" t="s">
         <v>52</v>
       </c>
     </row>
     <row r="5" spans="2:6">
-      <c r="B5" s="2">
+      <c r="B5" s="3">
         <v>150</v>
       </c>
-      <c r="C5" s="2">
+      <c r="C5" s="3">
         <v>-1.8</v>
       </c>
-      <c r="D5" s="2">
+      <c r="D5" s="3">
         <v>0.813</v>
       </c>
-      <c r="E5" s="3">
+      <c r="E5" s="4">
         <v>0.813</v>
       </c>
-      <c r="F5" s="2" t="s">
+      <c r="F5" s="3" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="6" spans="2:6">
-      <c r="B6" s="2">
+      <c r="B6" s="3">
         <v>200</v>
       </c>
-      <c r="C6" s="2">
+      <c r="C6" s="3">
         <v>-3.2</v>
       </c>
-      <c r="D6" s="2">
+      <c r="D6" s="3">
         <v>0.692</v>
       </c>
-      <c r="E6" s="3">
+      <c r="E6" s="4">
         <v>0.692</v>
       </c>
-      <c r="F6" s="2" t="s">
+      <c r="F6" s="3" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="7" spans="2:6">
-      <c r="B7" s="2">
+      <c r="B7" s="3">
         <v>250</v>
       </c>
-      <c r="C7" s="2">
+      <c r="C7" s="3">
         <v>-2.8</v>
       </c>
-      <c r="D7" s="2">
+      <c r="D7" s="3">
         <v>0.724</v>
       </c>
-      <c r="E7" s="3">
+      <c r="E7" s="4">
         <v>0.724</v>
       </c>
-      <c r="F7" s="2" t="s">
+      <c r="F7" s="3" t="s">
         <v>54</v>
       </c>
     </row>
     <row r="8" spans="2:6">
-      <c r="B8" s="2">
+      <c r="B8" s="3">
         <v>283</v>
       </c>
-      <c r="C8" s="2">
+      <c r="C8" s="3">
         <v>-3</v>
       </c>
-      <c r="D8" s="2">
+      <c r="D8" s="3">
         <v>0.708</v>
       </c>
-      <c r="E8" s="3">
+      <c r="E8" s="4">
         <v>0.708</v>
       </c>
-      <c r="F8" s="2" t="s">
+      <c r="F8" s="3" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="9" spans="2:6">
-      <c r="B9" s="2">
+      <c r="B9" s="3">
         <v>300</v>
       </c>
-      <c r="C9" s="2">
+      <c r="C9" s="3">
         <v>-3.5</v>
       </c>
-      <c r="D9" s="2">
+      <c r="D9" s="3">
         <v>0.668</v>
       </c>
-      <c r="E9" s="3">
+      <c r="E9" s="4">
         <v>0.668</v>
       </c>
-      <c r="F9" s="2" t="s">
+      <c r="F9" s="3" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="10" spans="2:6">
-      <c r="B10" s="2">
+      <c r="B10" s="3">
         <v>350</v>
       </c>
-      <c r="C10" s="2">
+      <c r="C10" s="3">
         <v>-4.2</v>
       </c>
-      <c r="D10" s="2">
+      <c r="D10" s="3">
         <v>0.617</v>
       </c>
-      <c r="E10" s="3">
+      <c r="E10" s="4">
         <v>0.617</v>
       </c>
-      <c r="F10" s="2" t="s">
+      <c r="F10" s="3" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="11" spans="2:6">
-      <c r="B11" s="2">
+      <c r="B11" s="3">
         <v>400</v>
       </c>
-      <c r="C11" s="2">
+      <c r="C11" s="3">
         <v>-4.7</v>
       </c>
-      <c r="D11" s="2">
+      <c r="D11" s="3">
         <v>0.585</v>
       </c>
-      <c r="E11" s="3">
+      <c r="E11" s="4">
         <v>0.585</v>
       </c>
-      <c r="F11" s="2" t="s">
+      <c r="F11" s="3" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="12" spans="2:6">
-      <c r="B12" s="2">
+      <c r="B12" s="3">
         <v>450</v>
       </c>
-      <c r="C12" s="2">
+      <c r="C12" s="3">
         <v>-5.3</v>
       </c>
-      <c r="D12" s="2">
+      <c r="D12" s="3">
         <v>0.544</v>
       </c>
-      <c r="E12" s="3">
+      <c r="E12" s="4">
         <v>0.544</v>
       </c>
-      <c r="F12" s="2" t="s">
+      <c r="F12" s="3" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="13" spans="2:6">
-      <c r="B13" s="2">
+      <c r="B13" s="3">
         <v>500</v>
       </c>
-      <c r="C13" s="2">
+      <c r="C13" s="3">
         <v>-6</v>
       </c>
-      <c r="D13" s="2">
+      <c r="D13" s="3">
         <v>0.501</v>
       </c>
-      <c r="E13" s="3">
+      <c r="E13" s="4">
         <v>0.501</v>
       </c>
-      <c r="F13" s="2" t="s">
+      <c r="F13" s="3" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="14" spans="2:6">
-      <c r="B14" s="2">
+      <c r="B14" s="3">
         <v>600</v>
       </c>
-      <c r="C14" s="2">
+      <c r="C14" s="3">
         <v>-7.8</v>
       </c>
-      <c r="D14" s="2">
+      <c r="D14" s="3">
         <v>0.407</v>
       </c>
-      <c r="E14" s="3">
+      <c r="E14" s="4">
         <v>0.407</v>
       </c>
-      <c r="F14" s="2" t="s">
+      <c r="F14" s="3" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="15" spans="2:6">
-      <c r="B15" s="2">
+      <c r="B15" s="3">
         <v>700</v>
       </c>
-      <c r="C15" s="2">
+      <c r="C15" s="3">
         <v>-10.2</v>
       </c>
-      <c r="D15" s="2">
+      <c r="D15" s="3">
         <v>0.307</v>
       </c>
-      <c r="E15" s="3">
+      <c r="E15" s="4">
         <v>0.307</v>
       </c>
-      <c r="F15" s="2" t="s">
+      <c r="F15" s="3" t="s">
         <v>60</v>
       </c>
     </row>
     <row r="16" spans="2:6">
-      <c r="B16" s="2">
+      <c r="B16" s="3">
         <v>800</v>
       </c>
-      <c r="C16" s="2">
+      <c r="C16" s="3">
         <v>-13.1</v>
       </c>
-      <c r="D16" s="2">
+      <c r="D16" s="3">
         <v>0.221</v>
       </c>
-      <c r="E16" s="3">
+      <c r="E16" s="4">
         <v>0.221</v>
       </c>
-      <c r="F16" s="2" t="s">
+      <c r="F16" s="3" t="s">
         <v>60</v>
       </c>
     </row>
     <row r="17" spans="2:6">
-      <c r="B17" s="2">
+      <c r="B17" s="3">
         <v>900</v>
       </c>
-      <c r="C17" s="2">
+      <c r="C17" s="3">
         <v>-16.4</v>
       </c>
-      <c r="D17" s="2">
+      <c r="D17" s="3">
         <v>0.151</v>
       </c>
-      <c r="E17" s="3">
+      <c r="E17" s="4">
         <v>0.151</v>
       </c>
-      <c r="F17" s="2" t="s">
+      <c r="F17" s="3" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="18" spans="2:6">
-      <c r="B18" s="2">
+      <c r="B18" s="3">
         <v>1000</v>
       </c>
-      <c r="C18" s="2">
+      <c r="C18" s="3">
         <v>-20</v>
       </c>
-      <c r="D18" s="2">
+      <c r="D18" s="3">
         <v>0.1</v>
       </c>
-      <c r="E18" s="3">
+      <c r="E18" s="4">
         <v>0.1</v>
       </c>
-      <c r="F18" s="2" t="s">
+      <c r="F18" s="3" t="s">
         <v>61</v>
       </c>
     </row>
@@ -6209,4 +6189,51 @@
   <headerFooter/>
   <drawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:F2"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.8" outlineLevelRow="1" outlineLevelCol="5"/>
+  <cols>
+    <col min="6" max="6" width="12.6875"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4">
+      <c r="A1" t="s">
+        <v>62</v>
+      </c>
+      <c r="B1" t="s">
+        <v>63</v>
+      </c>
+      <c r="C1" t="s">
+        <v>64</v>
+      </c>
+      <c r="D1" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2">
+        <v>100</v>
+      </c>
+      <c r="C2">
+        <v>29</v>
+      </c>
+      <c r="D2">
+        <v>2.7</v>
+      </c>
+      <c r="F2" s="1">
+        <f>1+(A2*((C2*POWER(10,-6))/(B2/2))*2*(D2*POWER(10,-9)))+POWER(A2,2)</f>
+        <v>2</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
modified:   Ferrite Transformer Calculation.xlsx 	modified:   README.md 	deleted:    hardware/CTL-1.0/CTL-1.0-backups/CTL-1.0-2025-06-04_105918.zip 	new file:   hardware/CTL-1.0/CTL-1.0-backups/CTL-1.0-2025-07-31_095618.zip 	deleted:    hardware/CTL-1.0/~CTL-1.0.kicad_sch.lck 	deleted:    hardware/XF-1.0/XF-1.0-backups/XF-1.0-2025-07-14_112815.zip 	deleted:    hardware/XF-1.0/XF-1.0-backups/XF-1.0-2025-07-15_150114.zip 	deleted:    hardware/XF-1.0/XF-1.0-backups/XF-1.0-2025-07-15_150614.zip 	new file:   hardware/XF-1.0/XF-1.0-backups/XF-1.0-2025-07-31_161825.zip 	new file:   hardware/XF-1.0/XF-1.0-backups/XF-1.0-2025-07-31_163521.zip 	new file:   hardware/XF-1.0/XF-1.0-backups/XF-1.0-2025-08-01_083038.zip 	modified:   pic/.DS_Store 	modified:   pic/Reverse Engineering/.DS_Store 	new file:   pic/Skin-Effect.drawio 	new file:   pic/skin-effect.png
</commit_message>
<xml_diff>
--- a/Ferrite Transformer Calculation.xlsx
+++ b/Ferrite Transformer Calculation.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="28800" windowHeight="13060" activeTab="4"/>
+    <workbookView windowWidth="28800" windowHeight="14080" activeTab="4"/>
   </bookViews>
   <sheets>
     <sheet name="ETD" sheetId="1" r:id="rId1"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="66">
   <si>
     <t>#</t>
   </si>
@@ -1359,6 +1359,13 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
       <t>C</t>
     </r>
     <r>
@@ -1799,20 +1806,6 @@
       <vertAlign val="subscript"/>
       <sz val="10"/>
       <color theme="1"/>
-      <name val="Arial"/>
-      <charset val="134"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="10"/>
-      <color theme="1"/>
-      <name val="Arial Bold"/>
-      <charset val="134"/>
-    </font>
-    <font>
-      <vertAlign val="subscript"/>
-      <sz val="10"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -1826,13 +1819,18 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <vertAlign val="superscript"/>
+      <vertAlign val="subscript"/>
       <sz val="10"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="Arial"/>
       <charset val="134"/>
-      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial Bold"/>
+      <charset val="134"/>
     </font>
     <font>
       <vertAlign val="superscript"/>
@@ -1848,6 +1846,15 @@
       <color theme="1"/>
       <name val="Arial Bold"/>
       <charset val="134"/>
+    </font>
+    <font>
+      <b/>
+      <vertAlign val="superscript"/>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="33">
@@ -6194,42 +6201,137 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:F2"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.8" outlineLevelRow="1" outlineLevelCol="5"/>
+  <dimension ref="A1:I5"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.8" outlineLevelRow="4"/>
   <cols>
-    <col min="6" max="6" width="12.6875"/>
+    <col min="7" max="7" width="12.6875"/>
+    <col min="8" max="8" width="9.5"/>
+    <col min="9" max="9" width="12.6875"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4">
+    <row r="1" spans="1:5">
       <c r="A1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B1" t="s">
         <v>62</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>63</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>64</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="2" spans="1:6">
+    <row r="2" spans="1:9">
       <c r="A2">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="B2">
+        <f>2*3.14*A2</f>
+        <v>62.8</v>
+      </c>
+      <c r="C2">
         <v>100</v>
       </c>
-      <c r="C2">
+      <c r="D2">
         <v>29</v>
       </c>
-      <c r="D2">
+      <c r="E2">
         <v>2.7</v>
       </c>
-      <c r="F2" s="1">
-        <f>1+(A2*((C2*POWER(10,-6))/(B2/2))*2*(D2*POWER(10,-9)))+POWER(A2,2)</f>
-        <v>2</v>
+      <c r="G2" s="1">
+        <f>1+(B2*((D2*POWER(10,-6))/(C2/2))*2*(E2*POWER(10,-9)))+POWER(B2,2)</f>
+        <v>3944.84</v>
+      </c>
+      <c r="H2" s="1">
+        <f>1/G2</f>
+        <v>0.000253495705782744</v>
+      </c>
+      <c r="I2">
+        <f>1/SQRT((1-B2^2*D2*2*E2)^2+(B2*(D2/(C2/2))*2*E2)^2)</f>
+        <v>1.61915951369643e-6</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8">
+      <c r="A3">
+        <v>100</v>
+      </c>
+      <c r="B3">
+        <f>2*3.14*A3</f>
+        <v>628</v>
+      </c>
+      <c r="C3">
+        <v>100</v>
+      </c>
+      <c r="D3">
+        <v>29</v>
+      </c>
+      <c r="E3">
+        <v>2.7</v>
+      </c>
+      <c r="G3" s="1">
+        <f>1+(B3*((D3*POWER(10,-6))/(C3/2))*2*(E3*POWER(10,-9)))+POWER(B3,2)</f>
+        <v>394385</v>
+      </c>
+      <c r="H3" s="1">
+        <f>1/G3</f>
+        <v>2.53559339224362e-6</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8">
+      <c r="A4">
+        <v>1000</v>
+      </c>
+      <c r="B4">
+        <f>2*3.14*A4</f>
+        <v>6280</v>
+      </c>
+      <c r="C4">
+        <v>100</v>
+      </c>
+      <c r="D4">
+        <v>29</v>
+      </c>
+      <c r="E4">
+        <v>2.7</v>
+      </c>
+      <c r="G4" s="1">
+        <f>1+(B4*((D4*POWER(10,-6))/(C4/2))*2*(E4*POWER(10,-9)))+POWER(B4,2)</f>
+        <v>39438401</v>
+      </c>
+      <c r="H4" s="1">
+        <f>1/G4</f>
+        <v>2.53559975720111e-8</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8">
+      <c r="A5">
+        <v>10000</v>
+      </c>
+      <c r="B5">
+        <f>2*3.14*A5</f>
+        <v>62800</v>
+      </c>
+      <c r="C5">
+        <v>100</v>
+      </c>
+      <c r="D5">
+        <v>29</v>
+      </c>
+      <c r="E5">
+        <v>2.7</v>
+      </c>
+      <c r="G5" s="1">
+        <f>1+(B5*((D5*POWER(10,-6))/(C5/2))*2*(E5*POWER(10,-9)))+POWER(B5,2)</f>
+        <v>3943840001</v>
+      </c>
+      <c r="H5" s="1">
+        <f>1/G5</f>
+        <v>2.53559982085085e-10</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
modified:   Ferrite Transformer Calculation.xlsx 	modified:   README.md 	modified:   pic/PWM.drawio
</commit_message>
<xml_diff>
--- a/Ferrite Transformer Calculation.xlsx
+++ b/Ferrite Transformer Calculation.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="27660" windowHeight="12960" activeTab="3"/>
+    <workbookView windowWidth="27660" windowHeight="13060" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="ETD" sheetId="1" r:id="rId1"/>
@@ -1736,28 +1736,19 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <b/>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial Bold"/>
+      <charset val="134"/>
+    </font>
+    <font>
       <vertAlign val="subscript"/>
       <sz val="10"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <vertAlign val="superscript"/>
-      <sz val="10"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="10"/>
-      <color theme="1"/>
-      <name val="Arial Bold"/>
-      <charset val="134"/>
     </font>
     <font>
       <vertAlign val="subscript"/>
@@ -1770,8 +1761,9 @@
       <vertAlign val="superscript"/>
       <sz val="10"/>
       <color theme="1"/>
-      <name val="Arial"/>
+      <name val="Calibri"/>
       <charset val="134"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <b/>
@@ -1782,6 +1774,7 @@
       <charset val="134"/>
     </font>
     <font>
+      <b/>
       <vertAlign val="superscript"/>
       <sz val="10"/>
       <color theme="1"/>
@@ -1789,13 +1782,32 @@
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <vertAlign val="superscript"/>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <charset val="134"/>
+    </font>
   </fonts>
-  <fills count="34">
+  <fills count="36">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -2122,7 +2134,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -2146,16 +2158,16 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="5" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="7" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="8" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
@@ -2164,102 +2176,126 @@
     <xf numFmtId="0" fontId="17" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="45">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="178" fontId="1" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="178" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="178" fontId="1" fillId="3" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="1" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="180" fontId="1" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="179" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="180" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="1" fillId="3" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="180" fontId="1" fillId="3" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1">
@@ -2283,6 +2319,9 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="181" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2295,7 +2334,7 @@
     <xf numFmtId="185" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1">
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -2307,13 +2346,13 @@
     <xf numFmtId="41" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="1" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1">
+    <xf numFmtId="41" fontId="1" fillId="4" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="186" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="186" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1">
+    <xf numFmtId="186" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="176" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1">
@@ -2325,16 +2364,16 @@
     <xf numFmtId="188" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="187" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="188" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1">
+    <xf numFmtId="187" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="188" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="41" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1">
+    <xf numFmtId="41" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -2891,538 +2930,538 @@
   <dimension ref="A1:U33"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="5.5625" style="28" customWidth="1"/>
-    <col min="2" max="4" width="10.5625" style="28" customWidth="1"/>
-    <col min="5" max="5" width="20.5625" style="28" customWidth="1"/>
-    <col min="6" max="6" width="15.5625" style="28" customWidth="1"/>
-    <col min="7" max="7" width="30.5625" style="31" customWidth="1"/>
-    <col min="8" max="8" width="10.5625" style="28" customWidth="1"/>
-    <col min="9" max="9" width="15.5625" style="5" customWidth="1"/>
-    <col min="10" max="13" width="10.5625" style="5" customWidth="1"/>
-    <col min="14" max="14" width="9" style="5"/>
-    <col min="15" max="15" width="20.5625" style="5" customWidth="1"/>
-    <col min="16" max="17" width="10.5625" style="5" customWidth="1"/>
-    <col min="18" max="16384" width="9" style="5"/>
+    <col min="1" max="1" width="5.5625" style="37" customWidth="1"/>
+    <col min="2" max="4" width="10.5625" style="37" customWidth="1"/>
+    <col min="5" max="5" width="20.5625" style="37" customWidth="1"/>
+    <col min="6" max="6" width="15.5625" style="37" customWidth="1"/>
+    <col min="7" max="7" width="30.5625" style="40" customWidth="1"/>
+    <col min="8" max="8" width="10.5625" style="37" customWidth="1"/>
+    <col min="9" max="9" width="15.5625" style="13" customWidth="1"/>
+    <col min="10" max="13" width="10.5625" style="13" customWidth="1"/>
+    <col min="14" max="14" width="9" style="13"/>
+    <col min="15" max="15" width="20.5625" style="13" customWidth="1"/>
+    <col min="16" max="17" width="10.5625" style="13" customWidth="1"/>
+    <col min="18" max="16384" width="9" style="13"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8">
-      <c r="A1" s="5"/>
-      <c r="B1" s="5"/>
-      <c r="C1" s="5"/>
-      <c r="D1" s="5"/>
-      <c r="E1" s="5"/>
-      <c r="F1" s="5"/>
-      <c r="G1" s="17"/>
-      <c r="H1" s="5"/>
-    </row>
-    <row r="2" s="30" customFormat="1" ht="18" spans="1:21">
-      <c r="A2" s="17" t="s">
+      <c r="A1" s="13"/>
+      <c r="B1" s="13"/>
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
+      <c r="E1" s="13"/>
+      <c r="F1" s="13"/>
+      <c r="G1" s="26"/>
+      <c r="H1" s="13"/>
+    </row>
+    <row r="2" s="39" customFormat="1" ht="18" spans="1:21">
+      <c r="A2" s="26" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="18" t="s">
+      <c r="B2" s="27" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="18" t="s">
+      <c r="C2" s="27" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="18" t="s">
+      <c r="D2" s="27" t="s">
         <v>3</v>
       </c>
-      <c r="E2" s="18" t="s">
+      <c r="E2" s="27" t="s">
         <v>4</v>
       </c>
-      <c r="F2" s="18" t="s">
+      <c r="F2" s="27" t="s">
         <v>5</v>
       </c>
-      <c r="G2" s="17" t="s">
+      <c r="G2" s="26" t="s">
         <v>6</v>
       </c>
-      <c r="H2" s="18" t="s">
+      <c r="H2" s="27" t="s">
         <v>7</v>
       </c>
-      <c r="I2" s="17" t="s">
+      <c r="I2" s="26" t="s">
         <v>8</v>
       </c>
-      <c r="J2" s="17" t="s">
+      <c r="J2" s="26" t="s">
         <v>9</v>
       </c>
-      <c r="K2" s="17" t="s">
+      <c r="K2" s="26" t="s">
         <v>10</v>
       </c>
-      <c r="L2" s="17" t="s">
+      <c r="L2" s="26" t="s">
         <v>11</v>
       </c>
-      <c r="M2" s="17" t="s">
+      <c r="M2" s="26" t="s">
         <v>12</v>
       </c>
-      <c r="N2" s="17" t="s">
+      <c r="N2" s="26" t="s">
         <v>13</v>
       </c>
-      <c r="O2" s="17" t="s">
+      <c r="O2" s="26" t="s">
         <v>14</v>
       </c>
-      <c r="P2" s="17" t="s">
+      <c r="P2" s="26" t="s">
         <v>15</v>
       </c>
-      <c r="Q2" s="17" t="s">
+      <c r="Q2" s="26" t="s">
         <v>16</v>
       </c>
-      <c r="R2" s="17" t="s">
+      <c r="R2" s="26" t="s">
         <v>17</v>
       </c>
-      <c r="S2" s="17" t="s">
+      <c r="S2" s="26" t="s">
         <v>18</v>
       </c>
-      <c r="T2" s="17" t="s">
+      <c r="T2" s="26" t="s">
         <v>17</v>
       </c>
-      <c r="U2" s="17" t="s">
+      <c r="U2" s="26" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="3" spans="1:21">
-      <c r="A3" s="19">
+      <c r="A3" s="28">
         <v>1</v>
       </c>
-      <c r="B3" s="19">
+      <c r="B3" s="28">
         <v>72</v>
       </c>
-      <c r="C3" s="19">
+      <c r="C3" s="28">
         <v>400000</v>
       </c>
-      <c r="D3" s="19">
+      <c r="D3" s="28">
         <v>10</v>
       </c>
-      <c r="E3" s="32">
+      <c r="E3" s="41">
         <f>3.14*POWER(D3,2)/4</f>
         <v>78.5</v>
       </c>
-      <c r="F3" s="32">
+      <c r="F3" s="41">
         <v>1898.58</v>
       </c>
-      <c r="G3" s="33">
+      <c r="G3" s="42">
         <f>(B3*POWER(10,10))/(4*C3*F3*E3)</f>
         <v>3.01935345175506</v>
       </c>
-      <c r="H3" s="34" t="str">
+      <c r="H3" s="43" t="str">
         <f>IF((B3*POWER(10,10))/(4*C3*G3*E3)&gt;1200,IF((B3*POWER(10,10))/(4*C3*G3*E3)&lt;2000,"OK","NG"),"NG")</f>
         <v>OK</v>
       </c>
-      <c r="I3" s="28">
+      <c r="I3" s="37">
         <f>B3/G3</f>
         <v>23.8461648</v>
       </c>
-      <c r="J3" s="28">
+      <c r="J3" s="37">
         <f>B3*3</f>
         <v>216</v>
       </c>
-      <c r="K3" s="25">
+      <c r="K3" s="34">
         <v>0.5</v>
       </c>
-      <c r="L3" s="28">
+      <c r="L3" s="37">
         <f>J3*K3</f>
         <v>108</v>
       </c>
-      <c r="M3" s="25">
+      <c r="M3" s="34">
         <f>L3/B3</f>
         <v>1.5</v>
       </c>
-      <c r="N3" s="28">
+      <c r="N3" s="37">
         <f>J3/I3</f>
         <v>9.05806035526518</v>
       </c>
-      <c r="O3" s="28">
+      <c r="O3" s="37">
         <v>1.5</v>
       </c>
-      <c r="P3" s="35">
+      <c r="P3" s="44">
         <f>SQRT((M3*0.9/(O3+5))/0.9)</f>
         <v>0.480384461415261</v>
       </c>
-      <c r="Q3" s="35">
+      <c r="Q3" s="44">
         <f>SQRT((K3*0.9/(O3+5))/0.9)</f>
         <v>0.277350098112615</v>
       </c>
-      <c r="R3" s="5">
+      <c r="R3" s="13">
         <v>1</v>
       </c>
-      <c r="S3" s="5">
+      <c r="S3" s="13">
         <v>1</v>
       </c>
-      <c r="T3" s="5">
+      <c r="T3" s="13">
         <f>IF(((M3*0.9/(O3+5)))/(R3*R3*1)&lt;1,1,((M3*0.9/(O3+5))/(R3*R3*1)))</f>
         <v>1</v>
       </c>
-      <c r="U3" s="5">
+      <c r="U3" s="13">
         <f>IF(((K3*0.9/(O3+5)))/(S3*S3*1)&lt;1,1,((K3*0.9/(O3+5))/(S3*S3*1)))</f>
         <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:21">
-      <c r="A4" s="19">
+      <c r="A4" s="28">
         <v>2</v>
       </c>
-      <c r="B4" s="19">
+      <c r="B4" s="28">
         <v>72</v>
       </c>
-      <c r="C4" s="19">
+      <c r="C4" s="28">
         <v>400000</v>
       </c>
-      <c r="D4" s="19">
+      <c r="D4" s="28">
         <v>10</v>
       </c>
-      <c r="E4" s="32">
+      <c r="E4" s="41">
         <f>3.14*POWER(D4,2)/4</f>
         <v>78.5</v>
       </c>
-      <c r="F4" s="32">
+      <c r="F4" s="41">
         <v>1898.58</v>
       </c>
-      <c r="G4" s="33">
+      <c r="G4" s="42">
         <f>(B4*POWER(10,10))/(4*C4*F4*E4)</f>
         <v>3.01935345175506</v>
       </c>
-      <c r="H4" s="34" t="str">
+      <c r="H4" s="43" t="str">
         <f>IF((B4*POWER(10,10))/(4*C4*G4*E4)&gt;1200,IF((B4*POWER(10,10))/(4*C4*G4*E4)&lt;2000,"OK","NG"),"NG")</f>
         <v>OK</v>
       </c>
-      <c r="I4" s="28">
+      <c r="I4" s="37">
         <f>B4/G4</f>
         <v>23.8461648</v>
       </c>
-      <c r="J4" s="28">
+      <c r="J4" s="37">
         <f>B4*3</f>
         <v>216</v>
       </c>
-      <c r="K4" s="25">
+      <c r="K4" s="34">
         <v>0.5</v>
       </c>
-      <c r="L4" s="28">
+      <c r="L4" s="37">
         <f>J4*K4</f>
         <v>108</v>
       </c>
-      <c r="M4" s="25">
+      <c r="M4" s="34">
         <f>L4/B4</f>
         <v>1.5</v>
       </c>
-      <c r="N4" s="28">
+      <c r="N4" s="37">
         <f>J4/I4</f>
         <v>9.05806035526518</v>
       </c>
-      <c r="O4" s="28">
+      <c r="O4" s="37">
         <v>1.5</v>
       </c>
-      <c r="P4" s="35">
+      <c r="P4" s="44">
         <f>SQRT((M4*0.9/(O4+5))/0.9)</f>
         <v>0.480384461415261</v>
       </c>
-      <c r="Q4" s="35">
+      <c r="Q4" s="44">
         <f>SQRT((K4*0.9/(O4+5))/0.9)</f>
         <v>0.277350098112615</v>
       </c>
-      <c r="R4" s="5">
+      <c r="R4" s="13">
         <v>1</v>
       </c>
-      <c r="S4" s="5">
+      <c r="S4" s="13">
         <v>1</v>
       </c>
-      <c r="T4" s="5">
+      <c r="T4" s="13">
         <f>IF(((M4*0.9/(O4+5)))/(R4*R4*1)&lt;1,1,((M4*0.9/(O4+5))/(R4*R4*1)))</f>
         <v>1</v>
       </c>
-      <c r="U4" s="5">
+      <c r="U4" s="13">
         <f>IF(((K4*0.9/(O4+5)))/(S4*S4*1)&lt;1,1,((K4*0.9/(O4+5))/(S4*S4*1)))</f>
         <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:8">
-      <c r="A5" s="19"/>
-      <c r="B5" s="19"/>
-      <c r="C5" s="19"/>
-      <c r="D5" s="19"/>
-      <c r="E5" s="19"/>
-      <c r="F5" s="19"/>
-      <c r="G5" s="33"/>
-      <c r="H5" s="19"/>
+      <c r="A5" s="28"/>
+      <c r="B5" s="28"/>
+      <c r="C5" s="28"/>
+      <c r="D5" s="28"/>
+      <c r="E5" s="28"/>
+      <c r="F5" s="28"/>
+      <c r="G5" s="42"/>
+      <c r="H5" s="28"/>
     </row>
     <row r="6" spans="1:8">
-      <c r="A6" s="19"/>
-      <c r="B6" s="19"/>
-      <c r="C6" s="19"/>
-      <c r="D6" s="19"/>
-      <c r="E6" s="19"/>
-      <c r="F6" s="19"/>
-      <c r="G6" s="33"/>
-      <c r="H6" s="19"/>
+      <c r="A6" s="28"/>
+      <c r="B6" s="28"/>
+      <c r="C6" s="28"/>
+      <c r="D6" s="28"/>
+      <c r="E6" s="28"/>
+      <c r="F6" s="28"/>
+      <c r="G6" s="42"/>
+      <c r="H6" s="28"/>
     </row>
     <row r="7" spans="1:8">
-      <c r="A7" s="19"/>
-      <c r="B7" s="19"/>
-      <c r="C7" s="19"/>
-      <c r="D7" s="19"/>
-      <c r="E7" s="19"/>
-      <c r="F7" s="19"/>
-      <c r="G7" s="33"/>
-      <c r="H7" s="19"/>
+      <c r="A7" s="28"/>
+      <c r="B7" s="28"/>
+      <c r="C7" s="28"/>
+      <c r="D7" s="28"/>
+      <c r="E7" s="28"/>
+      <c r="F7" s="28"/>
+      <c r="G7" s="42"/>
+      <c r="H7" s="28"/>
     </row>
     <row r="8" spans="1:8">
-      <c r="A8" s="19"/>
-      <c r="B8" s="19"/>
-      <c r="C8" s="19"/>
-      <c r="D8" s="19"/>
-      <c r="E8" s="19"/>
-      <c r="F8" s="19"/>
-      <c r="G8" s="33"/>
-      <c r="H8" s="19"/>
+      <c r="A8" s="28"/>
+      <c r="B8" s="28"/>
+      <c r="C8" s="28"/>
+      <c r="D8" s="28"/>
+      <c r="E8" s="28"/>
+      <c r="F8" s="28"/>
+      <c r="G8" s="42"/>
+      <c r="H8" s="28"/>
     </row>
     <row r="9" spans="1:8">
-      <c r="A9" s="19"/>
-      <c r="B9" s="19"/>
-      <c r="C9" s="19"/>
-      <c r="D9" s="19"/>
-      <c r="E9" s="19"/>
-      <c r="F9" s="19"/>
-      <c r="G9" s="33"/>
-      <c r="H9" s="19"/>
+      <c r="A9" s="28"/>
+      <c r="B9" s="28"/>
+      <c r="C9" s="28"/>
+      <c r="D9" s="28"/>
+      <c r="E9" s="28"/>
+      <c r="F9" s="28"/>
+      <c r="G9" s="42"/>
+      <c r="H9" s="28"/>
     </row>
     <row r="10" spans="1:8">
-      <c r="A10" s="19"/>
-      <c r="B10" s="19"/>
-      <c r="C10" s="19"/>
-      <c r="D10" s="19"/>
-      <c r="E10" s="19"/>
-      <c r="F10" s="19"/>
-      <c r="G10" s="33"/>
-      <c r="H10" s="19"/>
+      <c r="A10" s="28"/>
+      <c r="B10" s="28"/>
+      <c r="C10" s="28"/>
+      <c r="D10" s="28"/>
+      <c r="E10" s="28"/>
+      <c r="F10" s="28"/>
+      <c r="G10" s="42"/>
+      <c r="H10" s="28"/>
     </row>
     <row r="11" spans="1:8">
-      <c r="A11" s="19"/>
-      <c r="B11" s="19"/>
-      <c r="C11" s="19"/>
-      <c r="D11" s="19"/>
-      <c r="E11" s="19"/>
-      <c r="F11" s="19"/>
-      <c r="G11" s="33"/>
-      <c r="H11" s="19"/>
+      <c r="A11" s="28"/>
+      <c r="B11" s="28"/>
+      <c r="C11" s="28"/>
+      <c r="D11" s="28"/>
+      <c r="E11" s="28"/>
+      <c r="F11" s="28"/>
+      <c r="G11" s="42"/>
+      <c r="H11" s="28"/>
     </row>
     <row r="12" spans="1:8">
-      <c r="A12" s="19"/>
-      <c r="B12" s="19"/>
-      <c r="C12" s="19"/>
-      <c r="D12" s="19"/>
-      <c r="E12" s="19"/>
-      <c r="F12" s="19"/>
-      <c r="G12" s="33"/>
-      <c r="H12" s="19"/>
+      <c r="A12" s="28"/>
+      <c r="B12" s="28"/>
+      <c r="C12" s="28"/>
+      <c r="D12" s="28"/>
+      <c r="E12" s="28"/>
+      <c r="F12" s="28"/>
+      <c r="G12" s="42"/>
+      <c r="H12" s="28"/>
     </row>
     <row r="13" spans="1:8">
-      <c r="A13" s="19"/>
-      <c r="B13" s="19"/>
-      <c r="C13" s="19"/>
-      <c r="D13" s="19"/>
-      <c r="E13" s="19"/>
-      <c r="F13" s="19"/>
-      <c r="G13" s="33"/>
-      <c r="H13" s="19"/>
+      <c r="A13" s="28"/>
+      <c r="B13" s="28"/>
+      <c r="C13" s="28"/>
+      <c r="D13" s="28"/>
+      <c r="E13" s="28"/>
+      <c r="F13" s="28"/>
+      <c r="G13" s="42"/>
+      <c r="H13" s="28"/>
     </row>
     <row r="14" spans="1:8">
-      <c r="A14" s="19"/>
-      <c r="B14" s="19"/>
-      <c r="C14" s="19"/>
-      <c r="D14" s="19"/>
-      <c r="E14" s="19"/>
-      <c r="F14" s="19"/>
-      <c r="G14" s="33"/>
-      <c r="H14" s="19"/>
+      <c r="A14" s="28"/>
+      <c r="B14" s="28"/>
+      <c r="C14" s="28"/>
+      <c r="D14" s="28"/>
+      <c r="E14" s="28"/>
+      <c r="F14" s="28"/>
+      <c r="G14" s="42"/>
+      <c r="H14" s="28"/>
     </row>
     <row r="15" spans="1:8">
-      <c r="A15" s="19"/>
-      <c r="B15" s="19"/>
-      <c r="C15" s="19"/>
-      <c r="D15" s="19"/>
-      <c r="E15" s="19"/>
-      <c r="F15" s="19"/>
-      <c r="G15" s="33"/>
-      <c r="H15" s="19"/>
+      <c r="A15" s="28"/>
+      <c r="B15" s="28"/>
+      <c r="C15" s="28"/>
+      <c r="D15" s="28"/>
+      <c r="E15" s="28"/>
+      <c r="F15" s="28"/>
+      <c r="G15" s="42"/>
+      <c r="H15" s="28"/>
     </row>
     <row r="16" spans="1:8">
-      <c r="A16" s="19"/>
-      <c r="B16" s="19"/>
-      <c r="C16" s="19"/>
-      <c r="D16" s="19"/>
-      <c r="E16" s="19"/>
-      <c r="F16" s="19"/>
-      <c r="G16" s="33"/>
-      <c r="H16" s="19"/>
+      <c r="A16" s="28"/>
+      <c r="B16" s="28"/>
+      <c r="C16" s="28"/>
+      <c r="D16" s="28"/>
+      <c r="E16" s="28"/>
+      <c r="F16" s="28"/>
+      <c r="G16" s="42"/>
+      <c r="H16" s="28"/>
     </row>
     <row r="17" spans="1:8">
-      <c r="A17" s="19"/>
-      <c r="B17" s="19"/>
-      <c r="C17" s="19"/>
-      <c r="D17" s="19"/>
-      <c r="E17" s="19"/>
-      <c r="F17" s="19"/>
-      <c r="G17" s="33"/>
-      <c r="H17" s="19"/>
+      <c r="A17" s="28"/>
+      <c r="B17" s="28"/>
+      <c r="C17" s="28"/>
+      <c r="D17" s="28"/>
+      <c r="E17" s="28"/>
+      <c r="F17" s="28"/>
+      <c r="G17" s="42"/>
+      <c r="H17" s="28"/>
     </row>
     <row r="18" spans="1:8">
-      <c r="A18" s="19"/>
-      <c r="B18" s="19"/>
-      <c r="C18" s="19"/>
-      <c r="D18" s="19"/>
-      <c r="E18" s="19"/>
-      <c r="F18" s="19"/>
-      <c r="G18" s="33"/>
-      <c r="H18" s="19"/>
+      <c r="A18" s="28"/>
+      <c r="B18" s="28"/>
+      <c r="C18" s="28"/>
+      <c r="D18" s="28"/>
+      <c r="E18" s="28"/>
+      <c r="F18" s="28"/>
+      <c r="G18" s="42"/>
+      <c r="H18" s="28"/>
     </row>
     <row r="19" spans="1:8">
-      <c r="A19" s="19"/>
-      <c r="B19" s="19"/>
-      <c r="C19" s="19"/>
-      <c r="D19" s="19"/>
-      <c r="E19" s="19"/>
-      <c r="F19" s="19"/>
-      <c r="G19" s="33"/>
-      <c r="H19" s="19"/>
+      <c r="A19" s="28"/>
+      <c r="B19" s="28"/>
+      <c r="C19" s="28"/>
+      <c r="D19" s="28"/>
+      <c r="E19" s="28"/>
+      <c r="F19" s="28"/>
+      <c r="G19" s="42"/>
+      <c r="H19" s="28"/>
     </row>
     <row r="20" spans="1:8">
-      <c r="A20" s="19"/>
-      <c r="B20" s="19"/>
-      <c r="C20" s="19"/>
-      <c r="D20" s="19"/>
-      <c r="E20" s="19"/>
-      <c r="F20" s="19"/>
-      <c r="G20" s="33"/>
-      <c r="H20" s="19"/>
+      <c r="A20" s="28"/>
+      <c r="B20" s="28"/>
+      <c r="C20" s="28"/>
+      <c r="D20" s="28"/>
+      <c r="E20" s="28"/>
+      <c r="F20" s="28"/>
+      <c r="G20" s="42"/>
+      <c r="H20" s="28"/>
     </row>
     <row r="21" spans="1:8">
-      <c r="A21" s="19"/>
-      <c r="B21" s="19"/>
-      <c r="C21" s="19"/>
-      <c r="D21" s="19"/>
-      <c r="E21" s="19"/>
-      <c r="F21" s="19"/>
-      <c r="G21" s="33"/>
-      <c r="H21" s="19"/>
+      <c r="A21" s="28"/>
+      <c r="B21" s="28"/>
+      <c r="C21" s="28"/>
+      <c r="D21" s="28"/>
+      <c r="E21" s="28"/>
+      <c r="F21" s="28"/>
+      <c r="G21" s="42"/>
+      <c r="H21" s="28"/>
     </row>
     <row r="22" spans="1:8">
-      <c r="A22" s="19"/>
-      <c r="B22" s="19"/>
-      <c r="C22" s="19"/>
-      <c r="D22" s="19"/>
-      <c r="E22" s="19"/>
-      <c r="F22" s="19"/>
-      <c r="G22" s="33"/>
-      <c r="H22" s="19"/>
+      <c r="A22" s="28"/>
+      <c r="B22" s="28"/>
+      <c r="C22" s="28"/>
+      <c r="D22" s="28"/>
+      <c r="E22" s="28"/>
+      <c r="F22" s="28"/>
+      <c r="G22" s="42"/>
+      <c r="H22" s="28"/>
     </row>
     <row r="23" spans="1:8">
-      <c r="A23" s="19"/>
-      <c r="B23" s="19"/>
-      <c r="C23" s="19"/>
-      <c r="D23" s="19"/>
-      <c r="E23" s="19"/>
-      <c r="F23" s="19"/>
-      <c r="G23" s="33"/>
-      <c r="H23" s="19"/>
+      <c r="A23" s="28"/>
+      <c r="B23" s="28"/>
+      <c r="C23" s="28"/>
+      <c r="D23" s="28"/>
+      <c r="E23" s="28"/>
+      <c r="F23" s="28"/>
+      <c r="G23" s="42"/>
+      <c r="H23" s="28"/>
     </row>
     <row r="24" spans="1:8">
-      <c r="A24" s="19"/>
-      <c r="B24" s="19"/>
-      <c r="C24" s="19"/>
-      <c r="D24" s="19"/>
-      <c r="E24" s="19"/>
-      <c r="F24" s="19"/>
-      <c r="G24" s="33"/>
-      <c r="H24" s="19"/>
+      <c r="A24" s="28"/>
+      <c r="B24" s="28"/>
+      <c r="C24" s="28"/>
+      <c r="D24" s="28"/>
+      <c r="E24" s="28"/>
+      <c r="F24" s="28"/>
+      <c r="G24" s="42"/>
+      <c r="H24" s="28"/>
     </row>
     <row r="25" spans="1:8">
-      <c r="A25" s="19"/>
-      <c r="B25" s="19"/>
-      <c r="C25" s="19"/>
-      <c r="D25" s="19"/>
-      <c r="E25" s="19"/>
-      <c r="F25" s="19"/>
-      <c r="G25" s="33"/>
-      <c r="H25" s="19"/>
+      <c r="A25" s="28"/>
+      <c r="B25" s="28"/>
+      <c r="C25" s="28"/>
+      <c r="D25" s="28"/>
+      <c r="E25" s="28"/>
+      <c r="F25" s="28"/>
+      <c r="G25" s="42"/>
+      <c r="H25" s="28"/>
     </row>
     <row r="26" spans="1:8">
-      <c r="A26" s="19"/>
-      <c r="B26" s="19"/>
-      <c r="C26" s="19"/>
-      <c r="D26" s="19"/>
-      <c r="E26" s="19"/>
-      <c r="F26" s="19"/>
-      <c r="G26" s="33"/>
-      <c r="H26" s="19"/>
+      <c r="A26" s="28"/>
+      <c r="B26" s="28"/>
+      <c r="C26" s="28"/>
+      <c r="D26" s="28"/>
+      <c r="E26" s="28"/>
+      <c r="F26" s="28"/>
+      <c r="G26" s="42"/>
+      <c r="H26" s="28"/>
     </row>
     <row r="27" spans="1:8">
-      <c r="A27" s="19"/>
-      <c r="B27" s="19"/>
-      <c r="C27" s="19"/>
-      <c r="D27" s="19"/>
-      <c r="E27" s="19"/>
-      <c r="F27" s="19"/>
-      <c r="G27" s="33"/>
-      <c r="H27" s="19"/>
+      <c r="A27" s="28"/>
+      <c r="B27" s="28"/>
+      <c r="C27" s="28"/>
+      <c r="D27" s="28"/>
+      <c r="E27" s="28"/>
+      <c r="F27" s="28"/>
+      <c r="G27" s="42"/>
+      <c r="H27" s="28"/>
     </row>
     <row r="28" spans="1:8">
-      <c r="A28" s="19"/>
-      <c r="B28" s="19"/>
-      <c r="C28" s="19"/>
-      <c r="D28" s="19"/>
-      <c r="E28" s="19"/>
-      <c r="F28" s="19"/>
-      <c r="G28" s="33"/>
-      <c r="H28" s="19"/>
+      <c r="A28" s="28"/>
+      <c r="B28" s="28"/>
+      <c r="C28" s="28"/>
+      <c r="D28" s="28"/>
+      <c r="E28" s="28"/>
+      <c r="F28" s="28"/>
+      <c r="G28" s="42"/>
+      <c r="H28" s="28"/>
     </row>
     <row r="29" spans="1:8">
-      <c r="A29" s="19"/>
-      <c r="B29" s="19"/>
-      <c r="C29" s="19"/>
-      <c r="D29" s="19"/>
-      <c r="E29" s="19"/>
-      <c r="F29" s="19"/>
-      <c r="G29" s="33"/>
-      <c r="H29" s="19"/>
+      <c r="A29" s="28"/>
+      <c r="B29" s="28"/>
+      <c r="C29" s="28"/>
+      <c r="D29" s="28"/>
+      <c r="E29" s="28"/>
+      <c r="F29" s="28"/>
+      <c r="G29" s="42"/>
+      <c r="H29" s="28"/>
     </row>
     <row r="30" spans="1:8">
-      <c r="A30" s="19"/>
-      <c r="B30" s="19"/>
-      <c r="C30" s="19"/>
-      <c r="D30" s="19"/>
-      <c r="E30" s="19"/>
-      <c r="F30" s="19"/>
-      <c r="G30" s="33"/>
-      <c r="H30" s="19"/>
+      <c r="A30" s="28"/>
+      <c r="B30" s="28"/>
+      <c r="C30" s="28"/>
+      <c r="D30" s="28"/>
+      <c r="E30" s="28"/>
+      <c r="F30" s="28"/>
+      <c r="G30" s="42"/>
+      <c r="H30" s="28"/>
     </row>
     <row r="31" spans="1:8">
-      <c r="A31" s="19"/>
-      <c r="B31" s="19"/>
-      <c r="C31" s="19"/>
-      <c r="D31" s="19"/>
-      <c r="E31" s="19"/>
-      <c r="F31" s="19"/>
-      <c r="G31" s="33"/>
-      <c r="H31" s="19"/>
+      <c r="A31" s="28"/>
+      <c r="B31" s="28"/>
+      <c r="C31" s="28"/>
+      <c r="D31" s="28"/>
+      <c r="E31" s="28"/>
+      <c r="F31" s="28"/>
+      <c r="G31" s="42"/>
+      <c r="H31" s="28"/>
     </row>
     <row r="32" spans="1:8">
-      <c r="A32" s="19"/>
-      <c r="B32" s="19"/>
-      <c r="C32" s="19"/>
-      <c r="D32" s="19"/>
-      <c r="E32" s="19"/>
-      <c r="F32" s="19"/>
-      <c r="G32" s="33"/>
-      <c r="H32" s="19"/>
+      <c r="A32" s="28"/>
+      <c r="B32" s="28"/>
+      <c r="C32" s="28"/>
+      <c r="D32" s="28"/>
+      <c r="E32" s="28"/>
+      <c r="F32" s="28"/>
+      <c r="G32" s="42"/>
+      <c r="H32" s="28"/>
     </row>
     <row r="33" spans="1:8">
-      <c r="A33" s="19"/>
-      <c r="B33" s="19"/>
-      <c r="C33" s="19"/>
-      <c r="D33" s="19"/>
-      <c r="E33" s="19"/>
-      <c r="F33" s="19"/>
-      <c r="G33" s="33"/>
-      <c r="H33" s="19"/>
+      <c r="A33" s="28"/>
+      <c r="B33" s="28"/>
+      <c r="C33" s="28"/>
+      <c r="D33" s="28"/>
+      <c r="E33" s="28"/>
+      <c r="F33" s="28"/>
+      <c r="G33" s="42"/>
+      <c r="H33" s="28"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3436,657 +3475,657 @@
   <dimension ref="A2:U12"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="5.5625" style="5" customWidth="1"/>
-    <col min="2" max="7" width="10.5625" style="5" customWidth="1"/>
-    <col min="8" max="8" width="20.5625" style="5" customWidth="1"/>
-    <col min="9" max="9" width="15.5625" style="5" customWidth="1"/>
-    <col min="10" max="10" width="30.5625" style="5" customWidth="1"/>
-    <col min="11" max="11" width="9" style="5"/>
-    <col min="12" max="12" width="15.5625" style="5" customWidth="1"/>
-    <col min="13" max="16" width="10.5625" style="5" customWidth="1"/>
-    <col min="17" max="17" width="9" style="5"/>
-    <col min="18" max="18" width="20.5625" style="5" customWidth="1"/>
-    <col min="19" max="20" width="10.5625" style="5" customWidth="1"/>
-    <col min="21" max="16384" width="9" style="5"/>
+    <col min="1" max="1" width="5.5625" style="13" customWidth="1"/>
+    <col min="2" max="7" width="10.5625" style="13" customWidth="1"/>
+    <col min="8" max="8" width="20.5625" style="13" customWidth="1"/>
+    <col min="9" max="9" width="15.5625" style="13" customWidth="1"/>
+    <col min="10" max="10" width="30.5625" style="13" customWidth="1"/>
+    <col min="11" max="11" width="9" style="13"/>
+    <col min="12" max="12" width="15.5625" style="13" customWidth="1"/>
+    <col min="13" max="16" width="10.5625" style="13" customWidth="1"/>
+    <col min="17" max="17" width="9" style="13"/>
+    <col min="18" max="18" width="20.5625" style="13" customWidth="1"/>
+    <col min="19" max="20" width="10.5625" style="13" customWidth="1"/>
+    <col min="21" max="16384" width="9" style="13"/>
   </cols>
   <sheetData>
     <row r="2" ht="18" spans="1:20">
-      <c r="A2" s="17" t="s">
+      <c r="A2" s="26" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="18" t="s">
+      <c r="B2" s="27" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="18" t="s">
+      <c r="C2" s="27" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="18"/>
-      <c r="E2" s="18" t="s">
+      <c r="D2" s="27"/>
+      <c r="E2" s="27" t="s">
         <v>19</v>
       </c>
-      <c r="F2" s="18" t="s">
+      <c r="F2" s="27" t="s">
         <v>20</v>
       </c>
-      <c r="G2" s="18" t="s">
+      <c r="G2" s="27" t="s">
         <v>21</v>
       </c>
-      <c r="H2" s="18" t="s">
+      <c r="H2" s="27" t="s">
         <v>22</v>
       </c>
-      <c r="I2" s="18" t="s">
+      <c r="I2" s="27" t="s">
         <v>5</v>
       </c>
-      <c r="J2" s="17" t="s">
+      <c r="J2" s="26" t="s">
         <v>23</v>
       </c>
-      <c r="L2" s="17" t="s">
+      <c r="L2" s="26" t="s">
         <v>8</v>
       </c>
-      <c r="M2" s="17" t="s">
+      <c r="M2" s="26" t="s">
         <v>9</v>
       </c>
-      <c r="N2" s="17" t="s">
+      <c r="N2" s="26" t="s">
         <v>10</v>
       </c>
-      <c r="O2" s="17" t="s">
+      <c r="O2" s="26" t="s">
         <v>11</v>
       </c>
-      <c r="P2" s="17" t="s">
+      <c r="P2" s="26" t="s">
         <v>12</v>
       </c>
-      <c r="Q2" s="17" t="s">
+      <c r="Q2" s="26" t="s">
         <v>13</v>
       </c>
-      <c r="R2" s="17" t="s">
+      <c r="R2" s="26" t="s">
         <v>14</v>
       </c>
-      <c r="S2" s="17" t="s">
+      <c r="S2" s="26" t="s">
         <v>15</v>
       </c>
-      <c r="T2" s="17" t="s">
+      <c r="T2" s="26" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="3" spans="1:21">
-      <c r="A3" s="19">
+      <c r="A3" s="28">
         <v>1</v>
       </c>
-      <c r="B3" s="19">
+      <c r="B3" s="28">
         <v>72</v>
       </c>
-      <c r="C3" s="19">
+      <c r="C3" s="28">
         <v>400000</v>
       </c>
-      <c r="D3" s="19" t="s">
+      <c r="D3" s="28" t="s">
         <v>24</v>
       </c>
-      <c r="E3" s="5">
+      <c r="E3" s="13">
         <v>25</v>
       </c>
-      <c r="F3" s="5">
+      <c r="F3" s="13">
         <v>40</v>
       </c>
-      <c r="G3" s="5">
+      <c r="G3" s="13">
         <v>15</v>
       </c>
-      <c r="H3" s="5">
+      <c r="H3" s="13">
         <f>(F3-E3)*G3/2</f>
         <v>112.5</v>
       </c>
-      <c r="I3" s="5">
+      <c r="I3" s="13">
         <v>1800</v>
       </c>
-      <c r="J3" s="5">
+      <c r="J3" s="13">
         <f>(B3*0.5*POWER(10,10))/(2*C3*I3*H3)</f>
         <v>2.22222222222222</v>
       </c>
-      <c r="L3" s="21">
+      <c r="L3" s="30">
         <f>B3/J3</f>
         <v>32.4</v>
       </c>
-      <c r="M3" s="5">
+      <c r="M3" s="13">
         <v>216</v>
       </c>
-      <c r="N3" s="24">
+      <c r="N3" s="33">
         <v>0.5</v>
       </c>
-      <c r="O3" s="5">
+      <c r="O3" s="13">
         <f>M3*N3</f>
         <v>108</v>
       </c>
-      <c r="P3" s="25">
+      <c r="P3" s="34">
         <f>O3/B3</f>
         <v>1.5</v>
       </c>
-      <c r="Q3" s="28">
+      <c r="Q3" s="37">
         <f>M3/L3</f>
         <v>6.66666666666667</v>
       </c>
-      <c r="R3" s="25">
+      <c r="R3" s="34">
         <v>2.5</v>
       </c>
-      <c r="S3" s="24">
+      <c r="S3" s="33">
         <f>SQRT((P3*0.9/(R3+5))/0.9)</f>
         <v>0.447213595499958</v>
       </c>
-      <c r="T3" s="24">
+      <c r="T3" s="33">
         <f>SQRT((N3*0.9/(R3+5))/0.9)</f>
         <v>0.258198889747161</v>
       </c>
-      <c r="U3" s="25">
+      <c r="U3" s="34">
         <f>P3/R3</f>
         <v>0.6</v>
       </c>
     </row>
-    <row r="4" s="16" customFormat="1" spans="1:20">
-      <c r="A4" s="20"/>
-      <c r="B4" s="20">
+    <row r="4" s="25" customFormat="1" spans="1:20">
+      <c r="A4" s="29"/>
+      <c r="B4" s="29">
         <v>72</v>
       </c>
-      <c r="C4" s="20">
+      <c r="C4" s="29">
         <v>400000</v>
       </c>
-      <c r="D4" s="20" t="s">
+      <c r="D4" s="29" t="s">
         <v>24</v>
       </c>
-      <c r="E4" s="16">
+      <c r="E4" s="25">
         <v>23</v>
       </c>
-      <c r="F4" s="16">
+      <c r="F4" s="25">
         <v>40</v>
       </c>
-      <c r="G4" s="16">
+      <c r="G4" s="25">
         <v>15</v>
       </c>
-      <c r="H4" s="16">
+      <c r="H4" s="25">
         <f t="shared" ref="H4:H11" si="0">(F4-E4)*G4/2</f>
         <v>127.5</v>
       </c>
-      <c r="I4" s="16">
+      <c r="I4" s="25">
         <v>350</v>
       </c>
-      <c r="J4" s="16">
+      <c r="J4" s="25">
         <f t="shared" ref="J4:J11" si="1">(B4*0.5*POWER(10,10))/(2*C4*I4*H4)</f>
         <v>10.0840336134454</v>
       </c>
-      <c r="L4" s="22">
+      <c r="L4" s="31">
         <f t="shared" ref="L4:L11" si="2">B4/J4</f>
         <v>7.14</v>
       </c>
-      <c r="M4" s="16">
+      <c r="M4" s="25">
         <v>216</v>
       </c>
-      <c r="N4" s="26">
+      <c r="N4" s="35">
         <v>0.5</v>
       </c>
-      <c r="O4" s="16">
+      <c r="O4" s="25">
         <f t="shared" ref="O4:O11" si="3">M4*N4</f>
         <v>108</v>
       </c>
-      <c r="P4" s="27">
+      <c r="P4" s="36">
         <f t="shared" ref="P4:P11" si="4">O4/B4</f>
         <v>1.5</v>
       </c>
-      <c r="Q4" s="29">
+      <c r="Q4" s="38">
         <f t="shared" ref="Q4:Q11" si="5">M4/L4</f>
         <v>30.2521008403361</v>
       </c>
-      <c r="R4" s="27">
+      <c r="R4" s="36">
         <v>2.5</v>
       </c>
-      <c r="S4" s="26">
+      <c r="S4" s="35">
         <f t="shared" ref="S4:S11" si="6">SQRT((P4*0.9/(R4+5))/0.9)</f>
         <v>0.447213595499958</v>
       </c>
-      <c r="T4" s="26">
+      <c r="T4" s="35">
         <f t="shared" ref="T4:T11" si="7">SQRT((N4*0.9/(R4+5))/0.9)</f>
         <v>0.258198889747161</v>
       </c>
     </row>
     <row r="5" spans="2:20">
-      <c r="B5" s="19">
+      <c r="B5" s="28">
         <v>72</v>
       </c>
-      <c r="C5" s="19">
+      <c r="C5" s="28">
         <v>400000</v>
       </c>
-      <c r="D5" s="19"/>
-      <c r="E5" s="5">
+      <c r="D5" s="28"/>
+      <c r="E5" s="13">
         <v>23.13</v>
       </c>
-      <c r="F5" s="5">
+      <c r="F5" s="13">
         <v>39.88</v>
       </c>
-      <c r="G5" s="5">
+      <c r="G5" s="13">
         <v>14.48</v>
       </c>
-      <c r="H5" s="5">
+      <c r="H5" s="13">
         <f t="shared" si="0"/>
         <v>121.27</v>
       </c>
-      <c r="I5" s="5">
+      <c r="I5" s="13">
         <v>600</v>
       </c>
-      <c r="J5" s="5">
+      <c r="J5" s="13">
         <f t="shared" si="1"/>
         <v>6.18454687886534</v>
       </c>
-      <c r="L5" s="21">
+      <c r="L5" s="30">
         <f t="shared" si="2"/>
         <v>11.64192</v>
       </c>
-      <c r="M5" s="5">
+      <c r="M5" s="13">
         <v>216</v>
       </c>
-      <c r="N5" s="24">
+      <c r="N5" s="33">
         <v>0.5</v>
       </c>
-      <c r="O5" s="5">
+      <c r="O5" s="13">
         <f t="shared" si="3"/>
         <v>108</v>
       </c>
-      <c r="P5" s="25">
+      <c r="P5" s="34">
         <f t="shared" si="4"/>
         <v>1.5</v>
       </c>
-      <c r="Q5" s="28">
+      <c r="Q5" s="37">
         <f t="shared" si="5"/>
         <v>18.553640636596</v>
       </c>
-      <c r="R5" s="25">
+      <c r="R5" s="34">
         <v>2.5</v>
       </c>
-      <c r="S5" s="24">
+      <c r="S5" s="33">
         <f t="shared" si="6"/>
         <v>0.447213595499958</v>
       </c>
-      <c r="T5" s="24">
+      <c r="T5" s="33">
         <f t="shared" si="7"/>
         <v>0.258198889747161</v>
       </c>
     </row>
     <row r="6" spans="2:20">
-      <c r="B6" s="19">
+      <c r="B6" s="28">
         <v>72</v>
       </c>
-      <c r="C6" s="19">
+      <c r="C6" s="28">
         <v>400000</v>
       </c>
-      <c r="D6" s="19"/>
-      <c r="E6" s="5">
+      <c r="D6" s="28"/>
+      <c r="E6" s="13">
         <v>23.13</v>
       </c>
-      <c r="F6" s="5">
+      <c r="F6" s="13">
         <v>39.88</v>
       </c>
-      <c r="G6" s="5">
+      <c r="G6" s="13">
         <v>14.48</v>
       </c>
-      <c r="H6" s="5">
+      <c r="H6" s="13">
         <f t="shared" si="0"/>
         <v>121.27</v>
       </c>
-      <c r="I6" s="5">
+      <c r="I6" s="13">
         <v>350</v>
       </c>
-      <c r="J6" s="5">
+      <c r="J6" s="13">
         <f t="shared" si="1"/>
         <v>10.6020803637692</v>
       </c>
-      <c r="L6" s="21">
+      <c r="L6" s="30">
         <f t="shared" si="2"/>
         <v>6.79112</v>
       </c>
-      <c r="M6" s="5">
+      <c r="M6" s="13">
         <v>216</v>
       </c>
-      <c r="N6" s="24">
+      <c r="N6" s="33">
         <v>0.5</v>
       </c>
-      <c r="O6" s="5">
+      <c r="O6" s="13">
         <f t="shared" si="3"/>
         <v>108</v>
       </c>
-      <c r="P6" s="25">
+      <c r="P6" s="34">
         <f t="shared" si="4"/>
         <v>1.5</v>
       </c>
-      <c r="Q6" s="28">
+      <c r="Q6" s="37">
         <f t="shared" si="5"/>
         <v>31.8062410913075</v>
       </c>
-      <c r="R6" s="25">
+      <c r="R6" s="34">
         <v>2.5</v>
       </c>
-      <c r="S6" s="24">
+      <c r="S6" s="33">
         <f t="shared" si="6"/>
         <v>0.447213595499958</v>
       </c>
-      <c r="T6" s="24">
+      <c r="T6" s="33">
         <f t="shared" si="7"/>
         <v>0.258198889747161</v>
       </c>
     </row>
     <row r="7" spans="2:20">
-      <c r="B7" s="19">
+      <c r="B7" s="28">
         <v>72</v>
       </c>
-      <c r="C7" s="19">
+      <c r="C7" s="28">
         <v>400000</v>
       </c>
-      <c r="D7" s="5" t="s">
+      <c r="D7" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="E7" s="5">
+      <c r="E7" s="13">
         <v>23.3</v>
       </c>
-      <c r="F7" s="5">
+      <c r="F7" s="13">
         <v>40.4</v>
       </c>
-      <c r="G7" s="5">
+      <c r="G7" s="13">
         <v>15.1</v>
       </c>
-      <c r="H7" s="5">
+      <c r="H7" s="13">
         <f t="shared" si="0"/>
         <v>129.105</v>
       </c>
-      <c r="I7" s="5">
+      <c r="I7" s="13">
         <v>350</v>
       </c>
-      <c r="J7" s="5">
+      <c r="J7" s="13">
         <f t="shared" si="1"/>
         <v>9.95867151322014</v>
       </c>
-      <c r="L7" s="21">
+      <c r="L7" s="30">
         <f t="shared" si="2"/>
         <v>7.22988</v>
       </c>
-      <c r="M7" s="5">
+      <c r="M7" s="13">
         <v>216</v>
       </c>
-      <c r="N7" s="24">
+      <c r="N7" s="33">
         <v>0.5</v>
       </c>
-      <c r="O7" s="5">
+      <c r="O7" s="13">
         <f t="shared" si="3"/>
         <v>108</v>
       </c>
-      <c r="P7" s="25">
+      <c r="P7" s="34">
         <f t="shared" si="4"/>
         <v>1.5</v>
       </c>
-      <c r="Q7" s="28">
+      <c r="Q7" s="37">
         <f t="shared" si="5"/>
         <v>29.8760145396604</v>
       </c>
-      <c r="R7" s="25">
+      <c r="R7" s="34">
         <v>2.5</v>
       </c>
-      <c r="S7" s="24">
+      <c r="S7" s="33">
         <f t="shared" si="6"/>
         <v>0.447213595499958</v>
       </c>
-      <c r="T7" s="24">
+      <c r="T7" s="33">
         <f t="shared" si="7"/>
         <v>0.258198889747161</v>
       </c>
     </row>
     <row r="8" spans="2:20">
-      <c r="B8" s="19">
+      <c r="B8" s="28">
         <v>72</v>
       </c>
-      <c r="C8" s="19">
+      <c r="C8" s="28">
         <v>400000</v>
       </c>
-      <c r="D8" s="5" t="s">
+      <c r="D8" s="13" t="s">
         <v>26</v>
       </c>
-      <c r="E8" s="5">
+      <c r="E8" s="13">
         <v>13.5</v>
       </c>
-      <c r="F8" s="5">
+      <c r="F8" s="13">
         <v>23.3</v>
       </c>
-      <c r="G8" s="5">
+      <c r="G8" s="13">
         <v>8</v>
       </c>
-      <c r="H8" s="5">
+      <c r="H8" s="13">
         <f t="shared" si="0"/>
         <v>39.2</v>
       </c>
-      <c r="I8" s="5">
+      <c r="I8" s="13">
         <v>350</v>
       </c>
-      <c r="J8" s="5">
+      <c r="J8" s="13">
         <f t="shared" si="1"/>
         <v>32.798833819242</v>
       </c>
-      <c r="L8" s="21">
+      <c r="L8" s="30">
         <f t="shared" si="2"/>
         <v>2.1952</v>
       </c>
-      <c r="M8" s="5">
+      <c r="M8" s="13">
         <v>216</v>
       </c>
-      <c r="N8" s="24">
+      <c r="N8" s="33">
         <v>0.5</v>
       </c>
-      <c r="O8" s="5">
+      <c r="O8" s="13">
         <f t="shared" si="3"/>
         <v>108</v>
       </c>
-      <c r="P8" s="25">
+      <c r="P8" s="34">
         <f t="shared" si="4"/>
         <v>1.5</v>
       </c>
-      <c r="Q8" s="28">
+      <c r="Q8" s="37">
         <f t="shared" si="5"/>
         <v>98.396501457726</v>
       </c>
-      <c r="R8" s="25">
+      <c r="R8" s="34">
         <v>2.5</v>
       </c>
-      <c r="S8" s="24">
+      <c r="S8" s="33">
         <f t="shared" si="6"/>
         <v>0.447213595499958</v>
       </c>
-      <c r="T8" s="24">
+      <c r="T8" s="33">
         <f t="shared" si="7"/>
         <v>0.258198889747161</v>
       </c>
     </row>
     <row r="9" spans="2:20">
-      <c r="B9" s="19">
+      <c r="B9" s="28">
         <v>72</v>
       </c>
-      <c r="C9" s="19">
+      <c r="C9" s="28">
         <v>400000</v>
       </c>
-      <c r="E9" s="5">
+      <c r="E9" s="13">
         <v>23.3</v>
       </c>
-      <c r="F9" s="5">
+      <c r="F9" s="13">
         <v>40.6</v>
       </c>
-      <c r="G9" s="5">
+      <c r="G9" s="13">
         <v>14.9</v>
       </c>
-      <c r="H9" s="5">
+      <c r="H9" s="13">
         <f t="shared" si="0"/>
         <v>128.885</v>
       </c>
-      <c r="I9" s="5">
+      <c r="I9" s="13">
         <v>350</v>
       </c>
-      <c r="J9" s="5">
+      <c r="J9" s="13">
         <f t="shared" si="1"/>
         <v>9.9756704481847</v>
       </c>
-      <c r="L9" s="21">
+      <c r="L9" s="30">
         <f t="shared" si="2"/>
         <v>7.21756</v>
       </c>
-      <c r="M9" s="5">
+      <c r="M9" s="13">
         <v>216</v>
       </c>
-      <c r="N9" s="24">
+      <c r="N9" s="33">
         <v>0.5</v>
       </c>
-      <c r="O9" s="5">
+      <c r="O9" s="13">
         <f t="shared" si="3"/>
         <v>108</v>
       </c>
-      <c r="P9" s="25">
+      <c r="P9" s="34">
         <f t="shared" si="4"/>
         <v>1.5</v>
       </c>
-      <c r="Q9" s="28">
+      <c r="Q9" s="37">
         <f t="shared" si="5"/>
         <v>29.9270113445541</v>
       </c>
-      <c r="R9" s="25">
+      <c r="R9" s="34">
         <v>2.5</v>
       </c>
-      <c r="S9" s="24">
+      <c r="S9" s="33">
         <f t="shared" si="6"/>
         <v>0.447213595499958</v>
       </c>
-      <c r="T9" s="24">
+      <c r="T9" s="33">
         <f t="shared" si="7"/>
         <v>0.258198889747161</v>
       </c>
     </row>
     <row r="10" spans="2:20">
-      <c r="B10" s="19">
+      <c r="B10" s="28">
         <v>72</v>
       </c>
-      <c r="C10" s="19">
+      <c r="C10" s="28">
         <v>400000</v>
       </c>
-      <c r="D10" s="19" t="s">
+      <c r="D10" s="28" t="s">
         <v>24</v>
       </c>
-      <c r="E10" s="5">
+      <c r="E10" s="13">
         <v>23</v>
       </c>
-      <c r="F10" s="5">
+      <c r="F10" s="13">
         <v>40</v>
       </c>
-      <c r="G10" s="5">
+      <c r="G10" s="13">
         <v>15</v>
       </c>
-      <c r="H10" s="5">
+      <c r="H10" s="13">
         <f t="shared" si="0"/>
         <v>127.5</v>
       </c>
-      <c r="I10" s="5">
+      <c r="I10" s="13">
         <v>350</v>
       </c>
-      <c r="J10" s="5">
+      <c r="J10" s="13">
         <f t="shared" si="1"/>
         <v>10.0840336134454</v>
       </c>
-      <c r="L10" s="21">
+      <c r="L10" s="30">
         <f t="shared" si="2"/>
         <v>7.14</v>
       </c>
-      <c r="M10" s="5">
+      <c r="M10" s="13">
         <f>72*7</f>
         <v>504</v>
       </c>
-      <c r="N10" s="24">
+      <c r="N10" s="33">
         <v>0.5</v>
       </c>
-      <c r="O10" s="5">
+      <c r="O10" s="13">
         <f t="shared" si="3"/>
         <v>252</v>
       </c>
-      <c r="P10" s="25">
+      <c r="P10" s="34">
         <f t="shared" si="4"/>
         <v>3.5</v>
       </c>
-      <c r="Q10" s="28">
+      <c r="Q10" s="37">
         <f t="shared" si="5"/>
         <v>70.5882352941176</v>
       </c>
-      <c r="R10" s="25">
+      <c r="R10" s="34">
         <v>2.5</v>
       </c>
-      <c r="S10" s="24">
+      <c r="S10" s="33">
         <f t="shared" si="6"/>
         <v>0.683130051063973</v>
       </c>
-      <c r="T10" s="24">
+      <c r="T10" s="33">
         <f t="shared" si="7"/>
         <v>0.258198889747161</v>
       </c>
     </row>
-    <row r="11" s="16" customFormat="1" spans="2:20">
-      <c r="B11" s="20">
+    <row r="11" s="25" customFormat="1" spans="2:20">
+      <c r="B11" s="29">
         <v>72</v>
       </c>
-      <c r="C11" s="20">
+      <c r="C11" s="29">
         <v>200000</v>
       </c>
-      <c r="D11" s="20" t="s">
+      <c r="D11" s="29" t="s">
         <v>24</v>
       </c>
-      <c r="E11" s="16">
+      <c r="E11" s="25">
         <v>23</v>
       </c>
-      <c r="F11" s="16">
+      <c r="F11" s="25">
         <v>40</v>
       </c>
-      <c r="G11" s="16">
+      <c r="G11" s="25">
         <v>15</v>
       </c>
-      <c r="H11" s="16">
+      <c r="H11" s="25">
         <f t="shared" si="0"/>
         <v>127.5</v>
       </c>
-      <c r="I11" s="16">
+      <c r="I11" s="25">
         <v>350</v>
       </c>
-      <c r="J11" s="16">
+      <c r="J11" s="25">
         <f t="shared" si="1"/>
         <v>20.1680672268908</v>
       </c>
-      <c r="L11" s="22">
+      <c r="L11" s="31">
         <f t="shared" si="2"/>
         <v>3.57</v>
       </c>
-      <c r="M11" s="16">
+      <c r="M11" s="25">
         <v>504</v>
       </c>
-      <c r="N11" s="26">
+      <c r="N11" s="35">
         <v>0.5</v>
       </c>
-      <c r="O11" s="16">
+      <c r="O11" s="25">
         <f t="shared" si="3"/>
         <v>252</v>
       </c>
-      <c r="P11" s="27">
+      <c r="P11" s="36">
         <f t="shared" si="4"/>
         <v>3.5</v>
       </c>
-      <c r="Q11" s="29">
+      <c r="Q11" s="38">
         <f t="shared" si="5"/>
         <v>141.176470588235</v>
       </c>
-      <c r="R11" s="27">
+      <c r="R11" s="36">
         <v>2.5</v>
       </c>
-      <c r="S11" s="26">
+      <c r="S11" s="35">
         <f t="shared" si="6"/>
         <v>0.683130051063973</v>
       </c>
-      <c r="T11" s="26">
+      <c r="T11" s="35">
         <f t="shared" si="7"/>
         <v>0.258198889747161</v>
       </c>
     </row>
     <row r="12" spans="10:10">
-      <c r="J12" s="23"/>
+      <c r="J12" s="32"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4100,921 +4139,924 @@
   <dimension ref="B3:Y34"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="5.5625" style="5" customWidth="1"/>
-    <col min="2" max="2" width="15.5625" style="6" customWidth="1"/>
-    <col min="3" max="3" width="15.5625" style="5" customWidth="1"/>
-    <col min="4" max="4" width="5.5625" style="5" customWidth="1"/>
-    <col min="5" max="5" width="15.5625" style="5" customWidth="1"/>
-    <col min="6" max="6" width="5.5625" style="5" customWidth="1"/>
-    <col min="7" max="7" width="15.5625" style="5" customWidth="1"/>
-    <col min="8" max="8" width="5.5625" style="5" customWidth="1"/>
-    <col min="9" max="9" width="15.5625" style="5" customWidth="1"/>
-    <col min="10" max="10" width="5.5625" style="5" customWidth="1"/>
-    <col min="11" max="12" width="18.5625" style="5" customWidth="1"/>
-    <col min="13" max="13" width="5.2265625" style="5" customWidth="1"/>
-    <col min="14" max="14" width="25.4375" style="5" customWidth="1"/>
-    <col min="15" max="17" width="5.5625" style="5" customWidth="1"/>
-    <col min="18" max="18" width="15.5625" style="5" customWidth="1"/>
-    <col min="19" max="20" width="9" style="5"/>
-    <col min="21" max="22" width="20.5625" style="5" customWidth="1"/>
-    <col min="23" max="23" width="9" style="5"/>
-    <col min="24" max="24" width="11.125" style="5"/>
-    <col min="25" max="16384" width="9" style="5"/>
+    <col min="1" max="1" width="5.5625" style="13" customWidth="1"/>
+    <col min="2" max="2" width="15.5625" style="14" customWidth="1"/>
+    <col min="3" max="3" width="15.5625" style="13" customWidth="1"/>
+    <col min="4" max="4" width="5.5625" style="13" customWidth="1"/>
+    <col min="5" max="5" width="15.5625" style="13" customWidth="1"/>
+    <col min="6" max="6" width="5.5625" style="13" customWidth="1"/>
+    <col min="7" max="7" width="15.5625" style="13" customWidth="1"/>
+    <col min="8" max="8" width="5.5625" style="13" customWidth="1"/>
+    <col min="9" max="9" width="15.5625" style="13" customWidth="1"/>
+    <col min="10" max="10" width="14.359375" style="13" customWidth="1"/>
+    <col min="11" max="12" width="18.5625" style="13" customWidth="1"/>
+    <col min="13" max="13" width="5.2265625" style="13" customWidth="1"/>
+    <col min="14" max="14" width="25.4375" style="13" customWidth="1"/>
+    <col min="15" max="17" width="5.5625" style="13" customWidth="1"/>
+    <col min="18" max="18" width="15.5625" style="13" customWidth="1"/>
+    <col min="19" max="20" width="9" style="13"/>
+    <col min="21" max="22" width="20.5625" style="13" customWidth="1"/>
+    <col min="23" max="23" width="9" style="13"/>
+    <col min="24" max="24" width="11.125" style="13"/>
+    <col min="25" max="16384" width="9" style="13"/>
   </cols>
   <sheetData>
-    <row r="3" spans="2:6">
-      <c r="B3" s="1" t="s">
+    <row r="3" spans="2:10">
+      <c r="B3" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="C3" s="2">
+      <c r="C3" s="5">
         <v>400000</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="D3" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="E3" s="2">
+      <c r="E3" s="5">
         <v>400000</v>
       </c>
-      <c r="F3" s="2" t="s">
+      <c r="F3" s="5" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="4" customHeight="1" spans="2:6">
-      <c r="B4" s="1" t="s">
+      <c r="I3" s="5"/>
+      <c r="J3" s="20"/>
+    </row>
+    <row r="4" customHeight="1" spans="2:9">
+      <c r="B4" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="C4" s="2">
+      <c r="C4" s="5">
         <v>100</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="D4" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="E4" s="2">
+      <c r="E4" s="5">
         <v>500</v>
       </c>
-      <c r="F4" s="2" t="s">
+      <c r="F4" s="5" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="5" customHeight="1" spans="2:6">
-      <c r="B5" s="1" t="s">
+      <c r="I4" s="5"/>
+    </row>
+    <row r="5" customHeight="1" spans="2:9">
+      <c r="B5" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="C5" s="2">
+      <c r="C5" s="5">
         <f>C4/2</f>
         <v>50</v>
       </c>
-      <c r="D5" s="2" t="s">
+      <c r="D5" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="E5" s="2">
+      <c r="E5" s="5">
         <f>E4/2</f>
         <v>250</v>
       </c>
-      <c r="F5" s="2" t="s">
+      <c r="F5" s="5" t="s">
         <v>30</v>
       </c>
+      <c r="I5" s="5"/>
     </row>
     <row r="6" ht="18" spans="2:24">
-      <c r="B6" s="1" t="s">
+      <c r="B6" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="C6" s="3">
+      <c r="C6" s="9">
         <f>((C5*SQRT(2))/(2*3.14*C3))*1000000</f>
         <v>28.1491553020122</v>
       </c>
-      <c r="D6" s="2" t="s">
+      <c r="D6" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="E6" s="3">
+      <c r="E6" s="9">
         <f>((E5*SQRT(2))/(2*3.14*E3))*1000000</f>
         <v>140.745776510061</v>
       </c>
-      <c r="F6" s="2" t="s">
+      <c r="F6" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="M6" s="12"/>
-      <c r="N6" s="2" t="s">
+      <c r="M6" s="21"/>
+      <c r="N6" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="O6" s="13">
+      <c r="O6" s="22">
         <v>1.4</v>
       </c>
-      <c r="P6" s="2"/>
-      <c r="S6" s="2"/>
-      <c r="T6" s="12"/>
-      <c r="U6" s="12"/>
-      <c r="V6" s="2"/>
-      <c r="W6" s="2"/>
-      <c r="X6" s="2"/>
+      <c r="P6" s="5"/>
+      <c r="S6" s="5"/>
+      <c r="T6" s="21"/>
+      <c r="U6" s="21"/>
+      <c r="V6" s="5"/>
+      <c r="W6" s="5"/>
+      <c r="X6" s="5"/>
     </row>
     <row r="7" ht="18" spans="2:24">
-      <c r="B7" s="1" t="s">
+      <c r="B7" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="C7" s="4">
+      <c r="C7" s="10">
         <f>(1/(2*3.14*C3*C5*SQRT(2)))*1000000000</f>
         <v>5.62983106040245</v>
       </c>
-      <c r="D7" s="2" t="s">
+      <c r="D7" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="E7" s="4">
+      <c r="E7" s="10">
         <f>(1/(2*3.14*E3*E5*SQRT(2)))*1000000000</f>
         <v>1.12596621208049</v>
       </c>
-      <c r="F7" s="2" t="s">
+      <c r="F7" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="M7" s="11"/>
-      <c r="N7" s="2" t="s">
+      <c r="M7" s="19"/>
+      <c r="N7" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="O7" s="13">
+      <c r="O7" s="22">
         <v>0.707</v>
       </c>
-      <c r="P7" s="14"/>
-      <c r="S7" s="2"/>
-      <c r="T7" s="3"/>
-      <c r="U7" s="3"/>
-      <c r="V7" s="15"/>
-      <c r="W7" s="15"/>
-      <c r="X7" s="2"/>
+      <c r="P7" s="23"/>
+      <c r="S7" s="5"/>
+      <c r="T7" s="9"/>
+      <c r="U7" s="9"/>
+      <c r="V7" s="24"/>
+      <c r="W7" s="24"/>
+      <c r="X7" s="5"/>
     </row>
     <row r="8" ht="18" spans="2:24">
-      <c r="B8" s="1" t="s">
+      <c r="B8" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="C8" s="7">
+      <c r="C8" s="15">
         <f>C7/2</f>
         <v>2.81491553020122</v>
       </c>
-      <c r="D8" s="2" t="s">
+      <c r="D8" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="E8" s="7">
+      <c r="E8" s="15">
         <f>E7/2</f>
         <v>0.562983106040245</v>
       </c>
-      <c r="F8" s="2" t="s">
+      <c r="F8" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="G8" s="2"/>
-      <c r="H8" s="2"/>
-      <c r="I8" s="2"/>
-      <c r="J8" s="3"/>
-      <c r="K8" s="3"/>
-      <c r="L8" s="11"/>
-      <c r="M8" s="11"/>
-      <c r="N8" s="2" t="s">
+      <c r="G8" s="5"/>
+      <c r="H8" s="5"/>
+      <c r="I8" s="5"/>
+      <c r="J8" s="9"/>
+      <c r="K8" s="9"/>
+      <c r="L8" s="19"/>
+      <c r="M8" s="19"/>
+      <c r="N8" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="O8" s="13">
+      <c r="O8" s="22">
         <v>0.3</v>
       </c>
-      <c r="P8" s="2"/>
-      <c r="S8" s="2"/>
-      <c r="T8" s="2"/>
-      <c r="U8" s="2"/>
-      <c r="V8" s="2"/>
-      <c r="W8" s="2"/>
-      <c r="X8" s="2"/>
+      <c r="P8" s="5"/>
+      <c r="S8" s="5"/>
+      <c r="T8" s="5"/>
+      <c r="U8" s="5"/>
+      <c r="V8" s="5"/>
+      <c r="W8" s="5"/>
+      <c r="X8" s="5"/>
     </row>
     <row r="9" ht="18" spans="2:24">
-      <c r="B9" s="1" t="s">
+      <c r="B9" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="C9" s="2">
+      <c r="C9" s="5">
         <v>29</v>
       </c>
-      <c r="D9" s="2" t="s">
+      <c r="D9" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="E9" s="2">
+      <c r="E9" s="5">
         <v>140.7</v>
       </c>
-      <c r="F9" s="2" t="s">
+      <c r="F9" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="G9" s="10"/>
-      <c r="J9" s="3"/>
-      <c r="K9" s="3"/>
-      <c r="L9" s="11"/>
-      <c r="M9" s="11"/>
-      <c r="N9" s="2"/>
-      <c r="O9" s="2"/>
-      <c r="P9" s="2"/>
-      <c r="Q9" s="2"/>
-      <c r="R9" s="2"/>
-      <c r="S9" s="2"/>
-      <c r="T9" s="2"/>
-      <c r="U9" s="2"/>
-      <c r="V9" s="2"/>
-      <c r="W9" s="2"/>
-      <c r="X9" s="2"/>
+      <c r="G9" s="18"/>
+      <c r="J9" s="9"/>
+      <c r="K9" s="9"/>
+      <c r="L9" s="19"/>
+      <c r="M9" s="19"/>
+      <c r="N9" s="5"/>
+      <c r="O9" s="5"/>
+      <c r="P9" s="5"/>
+      <c r="Q9" s="5"/>
+      <c r="R9" s="5"/>
+      <c r="S9" s="5"/>
+      <c r="T9" s="5"/>
+      <c r="U9" s="5"/>
+      <c r="V9" s="5"/>
+      <c r="W9" s="5"/>
+      <c r="X9" s="5"/>
     </row>
     <row r="10" ht="18" spans="2:24">
-      <c r="B10" s="1" t="s">
+      <c r="B10" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="C10" s="8">
+      <c r="C10" s="16">
         <v>2.7</v>
       </c>
-      <c r="D10" s="2" t="s">
+      <c r="D10" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="E10" s="8">
+      <c r="E10" s="16">
         <v>0.56</v>
       </c>
-      <c r="F10" s="2" t="s">
+      <c r="F10" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="G10" s="2"/>
-      <c r="H10" s="2"/>
-      <c r="I10" s="2"/>
-      <c r="J10" s="3"/>
-      <c r="K10" s="3"/>
-      <c r="L10" s="11"/>
-      <c r="M10" s="11"/>
-      <c r="N10" s="2"/>
-      <c r="O10" s="2"/>
-      <c r="P10" s="2"/>
-      <c r="Q10" s="2"/>
-      <c r="R10" s="2"/>
-      <c r="S10" s="2"/>
-      <c r="T10" s="2"/>
-      <c r="U10" s="2"/>
-      <c r="V10" s="2"/>
-      <c r="W10" s="2"/>
-      <c r="X10" s="2"/>
+      <c r="G10" s="5"/>
+      <c r="H10" s="5"/>
+      <c r="I10" s="5"/>
+      <c r="J10" s="9"/>
+      <c r="K10" s="9"/>
+      <c r="L10" s="19"/>
+      <c r="M10" s="19"/>
+      <c r="N10" s="5"/>
+      <c r="O10" s="5"/>
+      <c r="P10" s="5"/>
+      <c r="Q10" s="5"/>
+      <c r="R10" s="5"/>
+      <c r="S10" s="5"/>
+      <c r="T10" s="5"/>
+      <c r="U10" s="5"/>
+      <c r="V10" s="5"/>
+      <c r="W10" s="5"/>
+      <c r="X10" s="5"/>
     </row>
     <row r="11" ht="18" spans="2:25">
-      <c r="B11" s="1" t="s">
+      <c r="B11" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="C11" s="8">
+      <c r="C11" s="16">
         <f>2*C10</f>
         <v>5.4</v>
       </c>
-      <c r="D11" s="2" t="s">
+      <c r="D11" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="E11" s="8">
+      <c r="E11" s="16">
         <f>2*E10</f>
         <v>1.12</v>
       </c>
-      <c r="F11" s="2" t="s">
+      <c r="F11" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="G11" s="11"/>
-      <c r="H11" s="11"/>
-      <c r="I11" s="11"/>
-      <c r="J11" s="2"/>
-      <c r="K11" s="3"/>
-      <c r="L11" s="3"/>
-      <c r="M11" s="3"/>
-      <c r="N11" s="3"/>
-      <c r="O11" s="2"/>
-      <c r="P11" s="2"/>
-      <c r="Q11" s="2"/>
-      <c r="R11" s="2"/>
-      <c r="S11" s="2"/>
-      <c r="T11" s="2"/>
-      <c r="U11" s="2"/>
-      <c r="V11" s="2"/>
-      <c r="W11" s="2"/>
-      <c r="X11" s="2"/>
-      <c r="Y11" s="2"/>
+      <c r="G11" s="19"/>
+      <c r="H11" s="19"/>
+      <c r="I11" s="19"/>
+      <c r="J11" s="5"/>
+      <c r="K11" s="9"/>
+      <c r="L11" s="9"/>
+      <c r="M11" s="9"/>
+      <c r="N11" s="9"/>
+      <c r="O11" s="5"/>
+      <c r="P11" s="5"/>
+      <c r="Q11" s="5"/>
+      <c r="R11" s="5"/>
+      <c r="S11" s="5"/>
+      <c r="T11" s="5"/>
+      <c r="U11" s="5"/>
+      <c r="V11" s="5"/>
+      <c r="W11" s="5"/>
+      <c r="X11" s="5"/>
+      <c r="Y11" s="5"/>
     </row>
     <row r="12" ht="18" spans="2:25">
-      <c r="B12" s="1" t="s">
+      <c r="B12" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="C12" s="3">
+      <c r="C12" s="9">
         <f>C5*SQRT((C11*POWER(10,-9))/(C9*POWER(10,-6)))</f>
         <v>0.682288239221013</v>
       </c>
-      <c r="D12" s="2"/>
-      <c r="E12" s="3">
+      <c r="D12" s="5"/>
+      <c r="E12" s="9">
         <f>E5*SQRT((E11*POWER(10,-9))/(E9*POWER(10,-6)))</f>
         <v>0.705345615858598</v>
       </c>
-      <c r="F12" s="2"/>
-      <c r="G12" s="7"/>
-      <c r="H12" s="2"/>
-      <c r="I12" s="2"/>
-      <c r="J12" s="2"/>
-      <c r="K12" s="2"/>
-      <c r="L12" s="2"/>
-      <c r="M12" s="2"/>
-      <c r="N12" s="2"/>
-      <c r="O12" s="2"/>
-      <c r="P12" s="2"/>
-      <c r="Q12" s="2"/>
-      <c r="R12" s="2"/>
-      <c r="S12" s="2"/>
-      <c r="T12" s="2"/>
-      <c r="U12" s="2"/>
-      <c r="V12" s="2"/>
-      <c r="W12" s="2"/>
-      <c r="X12" s="2"/>
-      <c r="Y12" s="2"/>
+      <c r="F12" s="5"/>
+      <c r="G12" s="15"/>
+      <c r="H12" s="5"/>
+      <c r="I12" s="5"/>
+      <c r="J12" s="5"/>
+      <c r="K12" s="5"/>
+      <c r="L12" s="5"/>
+      <c r="M12" s="5"/>
+      <c r="N12" s="5"/>
+      <c r="O12" s="5"/>
+      <c r="P12" s="5"/>
+      <c r="Q12" s="5"/>
+      <c r="R12" s="5"/>
+      <c r="S12" s="5"/>
+      <c r="T12" s="5"/>
+      <c r="U12" s="5"/>
+      <c r="V12" s="5"/>
+      <c r="W12" s="5"/>
+      <c r="X12" s="5"/>
+      <c r="Y12" s="5"/>
     </row>
     <row r="13" ht="18" spans="2:25">
-      <c r="B13" s="1" t="s">
+      <c r="B13" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="C13" s="3">
+      <c r="C13" s="9">
         <f>1/(2*3.14*SQRT((C9/POWER(10,6))*(C11/POWER(10,9))))</f>
         <v>402387.496591775</v>
       </c>
-      <c r="D13" s="2" t="s">
+      <c r="D13" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="E13" s="3">
+      <c r="E13" s="9">
         <f>1/(2*3.14*SQRT((E9/POWER(10,6))*(E11/POWER(10,9))))</f>
         <v>401129.217390013</v>
       </c>
-      <c r="F13" s="2" t="s">
+      <c r="F13" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="G13" s="2"/>
-      <c r="H13" s="2"/>
-      <c r="I13" s="2"/>
-      <c r="J13" s="2"/>
-      <c r="K13" s="2"/>
-      <c r="L13" s="2"/>
-      <c r="M13" s="2"/>
-      <c r="N13" s="2"/>
-      <c r="O13" s="2"/>
-      <c r="P13" s="2"/>
-      <c r="Q13" s="2"/>
-      <c r="R13" s="2"/>
-      <c r="S13" s="2"/>
-      <c r="T13" s="2"/>
-      <c r="U13" s="2"/>
-      <c r="V13" s="2"/>
-      <c r="W13" s="2"/>
-      <c r="X13" s="2"/>
-      <c r="Y13" s="2"/>
+      <c r="G13" s="5"/>
+      <c r="H13" s="5"/>
+      <c r="I13" s="5"/>
+      <c r="J13" s="5"/>
+      <c r="K13" s="5"/>
+      <c r="L13" s="5"/>
+      <c r="M13" s="5"/>
+      <c r="N13" s="5"/>
+      <c r="O13" s="5"/>
+      <c r="P13" s="5"/>
+      <c r="Q13" s="5"/>
+      <c r="R13" s="5"/>
+      <c r="S13" s="5"/>
+      <c r="T13" s="5"/>
+      <c r="U13" s="5"/>
+      <c r="V13" s="5"/>
+      <c r="W13" s="5"/>
+      <c r="X13" s="5"/>
+      <c r="Y13" s="5"/>
     </row>
     <row r="14" ht="18" spans="2:25">
-      <c r="B14" s="1" t="s">
+      <c r="B14" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="C14" s="3">
+      <c r="C14" s="9">
         <f>20*LOG10(C12)</f>
         <v>-3.3206422940395</v>
       </c>
-      <c r="D14" s="2" t="s">
+      <c r="D14" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="E14" s="3">
+      <c r="E14" s="9">
         <f>20*LOG10(E12)</f>
         <v>-3.03196057420489</v>
       </c>
-      <c r="F14" s="2" t="s">
+      <c r="F14" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="G14" s="2"/>
-      <c r="H14" s="2"/>
-      <c r="I14" s="2"/>
-      <c r="J14" s="2"/>
-      <c r="K14" s="2"/>
-      <c r="L14" s="2"/>
-      <c r="M14" s="2"/>
-      <c r="N14" s="2"/>
-      <c r="O14" s="2"/>
-      <c r="P14" s="2"/>
-      <c r="Q14" s="2"/>
-      <c r="R14" s="2"/>
-      <c r="S14" s="2"/>
-      <c r="T14" s="2"/>
-      <c r="U14" s="2"/>
-      <c r="V14" s="2"/>
-      <c r="W14" s="2"/>
-      <c r="X14" s="2"/>
-      <c r="Y14" s="2"/>
+      <c r="G14" s="5"/>
+      <c r="H14" s="5"/>
+      <c r="J14" s="5"/>
+      <c r="K14" s="5"/>
+      <c r="L14" s="5"/>
+      <c r="M14" s="5"/>
+      <c r="N14" s="5"/>
+      <c r="O14" s="5"/>
+      <c r="P14" s="5"/>
+      <c r="Q14" s="5"/>
+      <c r="R14" s="5"/>
+      <c r="S14" s="5"/>
+      <c r="T14" s="5"/>
+      <c r="U14" s="5"/>
+      <c r="V14" s="5"/>
+      <c r="W14" s="5"/>
+      <c r="X14" s="5"/>
+      <c r="Y14" s="5"/>
     </row>
     <row r="15" spans="2:25">
-      <c r="B15" s="9"/>
-      <c r="C15" s="2"/>
-      <c r="D15" s="2"/>
-      <c r="E15" s="2"/>
-      <c r="F15" s="2"/>
-      <c r="G15" s="2"/>
-      <c r="H15" s="2"/>
-      <c r="I15" s="2"/>
-      <c r="J15" s="2"/>
-      <c r="K15" s="2"/>
-      <c r="L15" s="2"/>
-      <c r="M15" s="2"/>
-      <c r="N15" s="2"/>
-      <c r="O15" s="2"/>
-      <c r="P15" s="2"/>
-      <c r="Q15" s="2"/>
-      <c r="R15" s="2"/>
-      <c r="S15" s="2"/>
-      <c r="T15" s="2"/>
-      <c r="U15" s="2"/>
-      <c r="V15" s="2"/>
-      <c r="W15" s="2"/>
-      <c r="X15" s="2"/>
-      <c r="Y15" s="2"/>
+      <c r="B15" s="17"/>
+      <c r="C15" s="5"/>
+      <c r="D15" s="5"/>
+      <c r="E15" s="5"/>
+      <c r="F15" s="5"/>
+      <c r="G15" s="5"/>
+      <c r="H15" s="5"/>
+      <c r="I15" s="5"/>
+      <c r="J15" s="5"/>
+      <c r="K15" s="5"/>
+      <c r="L15" s="5"/>
+      <c r="M15" s="5"/>
+      <c r="N15" s="5"/>
+      <c r="O15" s="5"/>
+      <c r="P15" s="5"/>
+      <c r="Q15" s="5"/>
+      <c r="R15" s="5"/>
+      <c r="S15" s="5"/>
+      <c r="T15" s="5"/>
+      <c r="U15" s="5"/>
+      <c r="V15" s="5"/>
+      <c r="W15" s="5"/>
+      <c r="X15" s="5"/>
+      <c r="Y15" s="5"/>
     </row>
     <row r="16" spans="2:25">
-      <c r="B16" s="9"/>
-      <c r="C16" s="2"/>
-      <c r="D16" s="2"/>
-      <c r="E16" s="2"/>
-      <c r="F16" s="2"/>
-      <c r="G16" s="2"/>
-      <c r="H16" s="2"/>
-      <c r="I16" s="2"/>
-      <c r="J16" s="2"/>
-      <c r="K16" s="2"/>
-      <c r="L16" s="2"/>
-      <c r="M16" s="2"/>
-      <c r="N16" s="2"/>
-      <c r="O16" s="2"/>
-      <c r="P16" s="2"/>
-      <c r="Q16" s="2"/>
-      <c r="R16" s="2"/>
-      <c r="S16" s="2"/>
-      <c r="T16" s="2"/>
-      <c r="U16" s="2"/>
-      <c r="V16" s="2"/>
-      <c r="W16" s="2"/>
-      <c r="X16" s="2"/>
-      <c r="Y16" s="2"/>
+      <c r="B16" s="17"/>
+      <c r="C16" s="5"/>
+      <c r="D16" s="5"/>
+      <c r="E16" s="5"/>
+      <c r="F16" s="5"/>
+      <c r="G16" s="5"/>
+      <c r="H16" s="5"/>
+      <c r="I16" s="5"/>
+      <c r="J16" s="5"/>
+      <c r="K16" s="5"/>
+      <c r="L16" s="5"/>
+      <c r="M16" s="5"/>
+      <c r="N16" s="5"/>
+      <c r="O16" s="5"/>
+      <c r="P16" s="5"/>
+      <c r="Q16" s="5"/>
+      <c r="R16" s="5"/>
+      <c r="S16" s="5"/>
+      <c r="T16" s="5"/>
+      <c r="U16" s="5"/>
+      <c r="V16" s="5"/>
+      <c r="W16" s="5"/>
+      <c r="X16" s="5"/>
+      <c r="Y16" s="5"/>
     </row>
     <row r="17" spans="2:25">
-      <c r="B17" s="9"/>
-      <c r="C17" s="2"/>
-      <c r="D17" s="2"/>
-      <c r="E17" s="2"/>
-      <c r="F17" s="2"/>
-      <c r="G17" s="2"/>
-      <c r="H17" s="2"/>
-      <c r="I17" s="2"/>
-      <c r="J17" s="2"/>
-      <c r="K17" s="2"/>
-      <c r="L17" s="2"/>
-      <c r="M17" s="2"/>
-      <c r="N17" s="2"/>
-      <c r="O17" s="2"/>
-      <c r="P17" s="2"/>
-      <c r="Q17" s="2"/>
-      <c r="R17" s="2"/>
-      <c r="S17" s="2"/>
-      <c r="T17" s="2"/>
-      <c r="U17" s="2"/>
-      <c r="V17" s="2"/>
-      <c r="W17" s="2"/>
-      <c r="X17" s="2"/>
-      <c r="Y17" s="2"/>
+      <c r="B17" s="17"/>
+      <c r="C17" s="5"/>
+      <c r="D17" s="5"/>
+      <c r="E17" s="5"/>
+      <c r="F17" s="5"/>
+      <c r="G17" s="5"/>
+      <c r="H17" s="5"/>
+      <c r="I17" s="5"/>
+      <c r="J17" s="5"/>
+      <c r="K17" s="5"/>
+      <c r="L17" s="5"/>
+      <c r="M17" s="5"/>
+      <c r="N17" s="5"/>
+      <c r="O17" s="5"/>
+      <c r="P17" s="5"/>
+      <c r="Q17" s="5"/>
+      <c r="R17" s="5"/>
+      <c r="S17" s="5"/>
+      <c r="T17" s="5"/>
+      <c r="U17" s="5"/>
+      <c r="V17" s="5"/>
+      <c r="W17" s="5"/>
+      <c r="X17" s="5"/>
+      <c r="Y17" s="5"/>
     </row>
     <row r="18" spans="2:25">
-      <c r="B18" s="9"/>
-      <c r="C18" s="2"/>
-      <c r="D18" s="2"/>
-      <c r="E18" s="2"/>
-      <c r="F18" s="2"/>
-      <c r="G18" s="2"/>
-      <c r="H18" s="2"/>
-      <c r="I18" s="2"/>
-      <c r="J18" s="2"/>
-      <c r="K18" s="2"/>
-      <c r="L18" s="2"/>
-      <c r="M18" s="2"/>
-      <c r="N18" s="2"/>
-      <c r="O18" s="2"/>
-      <c r="P18" s="2"/>
-      <c r="Q18" s="2"/>
-      <c r="R18" s="2"/>
-      <c r="S18" s="2"/>
-      <c r="T18" s="2"/>
-      <c r="U18" s="2"/>
-      <c r="V18" s="2"/>
-      <c r="W18" s="2"/>
-      <c r="X18" s="2"/>
-      <c r="Y18" s="2"/>
+      <c r="B18" s="17"/>
+      <c r="C18" s="5"/>
+      <c r="D18" s="5"/>
+      <c r="E18" s="5"/>
+      <c r="F18" s="5"/>
+      <c r="G18" s="5"/>
+      <c r="H18" s="5"/>
+      <c r="I18" s="5"/>
+      <c r="J18" s="5"/>
+      <c r="K18" s="5"/>
+      <c r="L18" s="5"/>
+      <c r="M18" s="5"/>
+      <c r="N18" s="5"/>
+      <c r="O18" s="5"/>
+      <c r="P18" s="5"/>
+      <c r="Q18" s="5"/>
+      <c r="R18" s="5"/>
+      <c r="S18" s="5"/>
+      <c r="T18" s="5"/>
+      <c r="U18" s="5"/>
+      <c r="V18" s="5"/>
+      <c r="W18" s="5"/>
+      <c r="X18" s="5"/>
+      <c r="Y18" s="5"/>
     </row>
     <row r="19" spans="2:25">
-      <c r="B19" s="9"/>
-      <c r="C19" s="2"/>
-      <c r="D19" s="2"/>
-      <c r="E19" s="2"/>
-      <c r="F19" s="2"/>
-      <c r="G19" s="2"/>
-      <c r="H19" s="2"/>
-      <c r="I19" s="2"/>
-      <c r="J19" s="2"/>
-      <c r="K19" s="2"/>
-      <c r="L19" s="2"/>
-      <c r="M19" s="2"/>
-      <c r="N19" s="2"/>
-      <c r="O19" s="2"/>
-      <c r="P19" s="2"/>
-      <c r="Q19" s="2"/>
-      <c r="R19" s="2"/>
-      <c r="S19" s="2"/>
-      <c r="T19" s="2"/>
-      <c r="U19" s="2"/>
-      <c r="V19" s="2"/>
-      <c r="W19" s="2"/>
-      <c r="X19" s="2"/>
-      <c r="Y19" s="2"/>
+      <c r="B19" s="17"/>
+      <c r="C19" s="5"/>
+      <c r="D19" s="5"/>
+      <c r="E19" s="5"/>
+      <c r="F19" s="5"/>
+      <c r="G19" s="5"/>
+      <c r="H19" s="5"/>
+      <c r="I19" s="5"/>
+      <c r="J19" s="5"/>
+      <c r="K19" s="5"/>
+      <c r="L19" s="5"/>
+      <c r="M19" s="5"/>
+      <c r="N19" s="5"/>
+      <c r="O19" s="5"/>
+      <c r="P19" s="5"/>
+      <c r="Q19" s="5"/>
+      <c r="R19" s="5"/>
+      <c r="S19" s="5"/>
+      <c r="T19" s="5"/>
+      <c r="U19" s="5"/>
+      <c r="V19" s="5"/>
+      <c r="W19" s="5"/>
+      <c r="X19" s="5"/>
+      <c r="Y19" s="5"/>
     </row>
     <row r="20" spans="2:25">
-      <c r="B20" s="9"/>
-      <c r="C20" s="2"/>
-      <c r="D20" s="2"/>
-      <c r="E20" s="2"/>
-      <c r="F20" s="2"/>
-      <c r="G20" s="2"/>
-      <c r="H20" s="2"/>
-      <c r="I20" s="2"/>
-      <c r="J20" s="2"/>
-      <c r="K20" s="2"/>
-      <c r="L20" s="2"/>
-      <c r="M20" s="2"/>
-      <c r="N20" s="2"/>
-      <c r="O20" s="2"/>
-      <c r="P20" s="2"/>
-      <c r="Q20" s="2"/>
-      <c r="R20" s="2"/>
-      <c r="S20" s="2"/>
-      <c r="T20" s="2"/>
-      <c r="U20" s="2"/>
-      <c r="V20" s="2"/>
-      <c r="W20" s="2"/>
-      <c r="X20" s="2"/>
-      <c r="Y20" s="2"/>
+      <c r="B20" s="17"/>
+      <c r="C20" s="5"/>
+      <c r="D20" s="5"/>
+      <c r="E20" s="5"/>
+      <c r="F20" s="5"/>
+      <c r="G20" s="5"/>
+      <c r="H20" s="5"/>
+      <c r="I20" s="5"/>
+      <c r="J20" s="5"/>
+      <c r="K20" s="5"/>
+      <c r="L20" s="5"/>
+      <c r="M20" s="5"/>
+      <c r="N20" s="5"/>
+      <c r="O20" s="5"/>
+      <c r="P20" s="5"/>
+      <c r="Q20" s="5"/>
+      <c r="R20" s="5"/>
+      <c r="S20" s="5"/>
+      <c r="T20" s="5"/>
+      <c r="U20" s="5"/>
+      <c r="V20" s="5"/>
+      <c r="W20" s="5"/>
+      <c r="X20" s="5"/>
+      <c r="Y20" s="5"/>
     </row>
     <row r="21" spans="2:25">
-      <c r="B21" s="9"/>
-      <c r="C21" s="2"/>
-      <c r="D21" s="2"/>
-      <c r="E21" s="2"/>
-      <c r="F21" s="2"/>
-      <c r="G21" s="2"/>
-      <c r="H21" s="2"/>
-      <c r="I21" s="2"/>
-      <c r="J21" s="2"/>
-      <c r="K21" s="2"/>
-      <c r="L21" s="2"/>
-      <c r="M21" s="2"/>
-      <c r="N21" s="2"/>
-      <c r="O21" s="2"/>
-      <c r="P21" s="2"/>
-      <c r="Q21" s="2"/>
-      <c r="R21" s="2"/>
-      <c r="S21" s="2"/>
-      <c r="T21" s="2"/>
-      <c r="U21" s="2"/>
-      <c r="V21" s="2"/>
-      <c r="W21" s="2"/>
-      <c r="X21" s="2"/>
-      <c r="Y21" s="2"/>
+      <c r="B21" s="17"/>
+      <c r="C21" s="5"/>
+      <c r="D21" s="5"/>
+      <c r="E21" s="5"/>
+      <c r="F21" s="5"/>
+      <c r="G21" s="5"/>
+      <c r="H21" s="5"/>
+      <c r="I21" s="5"/>
+      <c r="J21" s="5"/>
+      <c r="K21" s="5"/>
+      <c r="L21" s="5"/>
+      <c r="M21" s="5"/>
+      <c r="N21" s="5"/>
+      <c r="O21" s="5"/>
+      <c r="P21" s="5"/>
+      <c r="Q21" s="5"/>
+      <c r="R21" s="5"/>
+      <c r="S21" s="5"/>
+      <c r="T21" s="5"/>
+      <c r="U21" s="5"/>
+      <c r="V21" s="5"/>
+      <c r="W21" s="5"/>
+      <c r="X21" s="5"/>
+      <c r="Y21" s="5"/>
     </row>
     <row r="22" spans="2:25">
-      <c r="B22" s="9"/>
-      <c r="C22" s="2"/>
-      <c r="D22" s="2"/>
-      <c r="E22" s="2"/>
-      <c r="F22" s="2"/>
-      <c r="G22" s="2"/>
-      <c r="H22" s="2"/>
-      <c r="I22" s="2"/>
-      <c r="J22" s="2"/>
-      <c r="K22" s="2"/>
-      <c r="L22" s="2"/>
-      <c r="M22" s="2"/>
-      <c r="N22" s="2"/>
-      <c r="O22" s="2"/>
-      <c r="P22" s="2"/>
-      <c r="Q22" s="2"/>
-      <c r="R22" s="2"/>
-      <c r="S22" s="2"/>
-      <c r="T22" s="2"/>
-      <c r="U22" s="2"/>
-      <c r="V22" s="2"/>
-      <c r="W22" s="2"/>
-      <c r="X22" s="2"/>
-      <c r="Y22" s="2"/>
+      <c r="B22" s="17"/>
+      <c r="C22" s="5"/>
+      <c r="D22" s="5"/>
+      <c r="E22" s="5"/>
+      <c r="F22" s="5"/>
+      <c r="G22" s="5"/>
+      <c r="H22" s="5"/>
+      <c r="I22" s="5"/>
+      <c r="J22" s="5"/>
+      <c r="K22" s="5"/>
+      <c r="L22" s="5"/>
+      <c r="M22" s="5"/>
+      <c r="N22" s="5"/>
+      <c r="O22" s="5"/>
+      <c r="P22" s="5"/>
+      <c r="Q22" s="5"/>
+      <c r="R22" s="5"/>
+      <c r="S22" s="5"/>
+      <c r="T22" s="5"/>
+      <c r="U22" s="5"/>
+      <c r="V22" s="5"/>
+      <c r="W22" s="5"/>
+      <c r="X22" s="5"/>
+      <c r="Y22" s="5"/>
     </row>
     <row r="23" spans="2:25">
-      <c r="B23" s="9"/>
-      <c r="C23" s="2"/>
-      <c r="D23" s="2"/>
-      <c r="E23" s="2"/>
-      <c r="F23" s="2"/>
-      <c r="G23" s="2"/>
-      <c r="H23" s="2"/>
-      <c r="I23" s="2"/>
-      <c r="J23" s="2"/>
-      <c r="K23" s="2"/>
-      <c r="L23" s="2"/>
-      <c r="M23" s="2"/>
-      <c r="N23" s="2"/>
-      <c r="O23" s="2"/>
-      <c r="P23" s="2"/>
-      <c r="Q23" s="2"/>
-      <c r="R23" s="2"/>
-      <c r="S23" s="2"/>
-      <c r="T23" s="2"/>
-      <c r="U23" s="2"/>
-      <c r="V23" s="2"/>
-      <c r="W23" s="2"/>
-      <c r="X23" s="2"/>
-      <c r="Y23" s="2"/>
+      <c r="B23" s="17"/>
+      <c r="C23" s="5"/>
+      <c r="D23" s="5"/>
+      <c r="E23" s="5"/>
+      <c r="F23" s="5"/>
+      <c r="G23" s="5"/>
+      <c r="H23" s="5"/>
+      <c r="I23" s="5"/>
+      <c r="J23" s="5"/>
+      <c r="K23" s="5"/>
+      <c r="L23" s="5"/>
+      <c r="M23" s="5"/>
+      <c r="N23" s="5"/>
+      <c r="O23" s="5"/>
+      <c r="P23" s="5"/>
+      <c r="Q23" s="5"/>
+      <c r="R23" s="5"/>
+      <c r="S23" s="5"/>
+      <c r="T23" s="5"/>
+      <c r="U23" s="5"/>
+      <c r="V23" s="5"/>
+      <c r="W23" s="5"/>
+      <c r="X23" s="5"/>
+      <c r="Y23" s="5"/>
     </row>
     <row r="24" spans="2:25">
-      <c r="B24" s="9"/>
-      <c r="C24" s="2"/>
-      <c r="D24" s="2"/>
-      <c r="E24" s="2"/>
-      <c r="F24" s="2"/>
-      <c r="G24" s="2"/>
-      <c r="H24" s="2"/>
-      <c r="I24" s="2"/>
-      <c r="J24" s="2"/>
-      <c r="K24" s="2"/>
-      <c r="L24" s="2"/>
-      <c r="M24" s="2"/>
-      <c r="N24" s="2"/>
-      <c r="O24" s="2"/>
-      <c r="P24" s="2"/>
-      <c r="Q24" s="2"/>
-      <c r="R24" s="2"/>
-      <c r="S24" s="2"/>
-      <c r="T24" s="2"/>
-      <c r="U24" s="2"/>
-      <c r="V24" s="2"/>
-      <c r="W24" s="2"/>
-      <c r="X24" s="2"/>
-      <c r="Y24" s="2"/>
+      <c r="B24" s="17"/>
+      <c r="C24" s="5"/>
+      <c r="D24" s="5"/>
+      <c r="E24" s="5"/>
+      <c r="F24" s="5"/>
+      <c r="G24" s="5"/>
+      <c r="H24" s="5"/>
+      <c r="I24" s="5"/>
+      <c r="J24" s="5"/>
+      <c r="K24" s="5"/>
+      <c r="L24" s="5"/>
+      <c r="M24" s="5"/>
+      <c r="N24" s="5"/>
+      <c r="O24" s="5"/>
+      <c r="P24" s="5"/>
+      <c r="Q24" s="5"/>
+      <c r="R24" s="5"/>
+      <c r="S24" s="5"/>
+      <c r="T24" s="5"/>
+      <c r="U24" s="5"/>
+      <c r="V24" s="5"/>
+      <c r="W24" s="5"/>
+      <c r="X24" s="5"/>
+      <c r="Y24" s="5"/>
     </row>
     <row r="25" spans="2:25">
-      <c r="B25" s="9"/>
-      <c r="C25" s="2"/>
-      <c r="D25" s="2"/>
-      <c r="E25" s="2"/>
-      <c r="F25" s="2"/>
-      <c r="G25" s="2"/>
-      <c r="H25" s="2"/>
-      <c r="I25" s="2"/>
-      <c r="J25" s="2"/>
-      <c r="K25" s="2"/>
-      <c r="L25" s="2"/>
-      <c r="M25" s="2"/>
-      <c r="N25" s="2"/>
-      <c r="O25" s="2"/>
-      <c r="P25" s="2"/>
-      <c r="Q25" s="2"/>
-      <c r="R25" s="2"/>
-      <c r="S25" s="2"/>
-      <c r="T25" s="2"/>
-      <c r="U25" s="2"/>
-      <c r="V25" s="2"/>
-      <c r="W25" s="2"/>
-      <c r="X25" s="2"/>
-      <c r="Y25" s="2"/>
+      <c r="B25" s="17"/>
+      <c r="C25" s="5"/>
+      <c r="D25" s="5"/>
+      <c r="E25" s="5"/>
+      <c r="F25" s="5"/>
+      <c r="G25" s="5"/>
+      <c r="H25" s="5"/>
+      <c r="I25" s="5"/>
+      <c r="J25" s="5"/>
+      <c r="K25" s="5"/>
+      <c r="L25" s="5"/>
+      <c r="M25" s="5"/>
+      <c r="N25" s="5"/>
+      <c r="O25" s="5"/>
+      <c r="P25" s="5"/>
+      <c r="Q25" s="5"/>
+      <c r="R25" s="5"/>
+      <c r="S25" s="5"/>
+      <c r="T25" s="5"/>
+      <c r="U25" s="5"/>
+      <c r="V25" s="5"/>
+      <c r="W25" s="5"/>
+      <c r="X25" s="5"/>
+      <c r="Y25" s="5"/>
     </row>
     <row r="26" spans="2:25">
-      <c r="B26" s="9"/>
-      <c r="C26" s="2"/>
-      <c r="D26" s="2"/>
-      <c r="E26" s="2"/>
-      <c r="F26" s="2"/>
-      <c r="G26" s="2"/>
-      <c r="H26" s="2"/>
-      <c r="I26" s="2"/>
-      <c r="J26" s="2"/>
-      <c r="K26" s="2"/>
-      <c r="L26" s="2"/>
-      <c r="M26" s="2"/>
-      <c r="N26" s="2"/>
-      <c r="O26" s="2"/>
-      <c r="P26" s="2"/>
-      <c r="Q26" s="2"/>
-      <c r="R26" s="2"/>
-      <c r="S26" s="2"/>
-      <c r="T26" s="2"/>
-      <c r="U26" s="2"/>
-      <c r="V26" s="2"/>
-      <c r="W26" s="2"/>
-      <c r="X26" s="2"/>
-      <c r="Y26" s="2"/>
+      <c r="B26" s="17"/>
+      <c r="C26" s="5"/>
+      <c r="D26" s="5"/>
+      <c r="E26" s="5"/>
+      <c r="F26" s="5"/>
+      <c r="G26" s="5"/>
+      <c r="H26" s="5"/>
+      <c r="I26" s="5"/>
+      <c r="J26" s="5"/>
+      <c r="K26" s="5"/>
+      <c r="L26" s="5"/>
+      <c r="M26" s="5"/>
+      <c r="N26" s="5"/>
+      <c r="O26" s="5"/>
+      <c r="P26" s="5"/>
+      <c r="Q26" s="5"/>
+      <c r="R26" s="5"/>
+      <c r="S26" s="5"/>
+      <c r="T26" s="5"/>
+      <c r="U26" s="5"/>
+      <c r="V26" s="5"/>
+      <c r="W26" s="5"/>
+      <c r="X26" s="5"/>
+      <c r="Y26" s="5"/>
     </row>
     <row r="27" spans="2:25">
-      <c r="B27" s="9"/>
-      <c r="C27" s="2"/>
-      <c r="D27" s="2"/>
-      <c r="E27" s="2"/>
-      <c r="F27" s="2"/>
-      <c r="G27" s="2"/>
-      <c r="H27" s="2"/>
-      <c r="I27" s="2"/>
-      <c r="J27" s="2"/>
-      <c r="K27" s="2"/>
-      <c r="L27" s="2"/>
-      <c r="M27" s="2"/>
-      <c r="N27" s="2"/>
-      <c r="O27" s="2"/>
-      <c r="P27" s="2"/>
-      <c r="Q27" s="2"/>
-      <c r="R27" s="2"/>
-      <c r="S27" s="2"/>
-      <c r="T27" s="2"/>
-      <c r="U27" s="2"/>
-      <c r="V27" s="2"/>
-      <c r="W27" s="2"/>
-      <c r="X27" s="2"/>
-      <c r="Y27" s="2"/>
+      <c r="B27" s="17"/>
+      <c r="C27" s="5"/>
+      <c r="D27" s="5"/>
+      <c r="E27" s="5"/>
+      <c r="F27" s="5"/>
+      <c r="G27" s="5"/>
+      <c r="H27" s="5"/>
+      <c r="I27" s="5"/>
+      <c r="J27" s="5"/>
+      <c r="K27" s="5"/>
+      <c r="L27" s="5"/>
+      <c r="M27" s="5"/>
+      <c r="N27" s="5"/>
+      <c r="O27" s="5"/>
+      <c r="P27" s="5"/>
+      <c r="Q27" s="5"/>
+      <c r="R27" s="5"/>
+      <c r="S27" s="5"/>
+      <c r="T27" s="5"/>
+      <c r="U27" s="5"/>
+      <c r="V27" s="5"/>
+      <c r="W27" s="5"/>
+      <c r="X27" s="5"/>
+      <c r="Y27" s="5"/>
     </row>
     <row r="28" spans="2:25">
-      <c r="B28" s="9"/>
-      <c r="C28" s="2"/>
-      <c r="D28" s="2"/>
-      <c r="E28" s="2"/>
-      <c r="F28" s="2"/>
-      <c r="G28" s="2"/>
-      <c r="H28" s="2"/>
-      <c r="I28" s="2"/>
-      <c r="J28" s="2"/>
-      <c r="K28" s="2"/>
-      <c r="L28" s="2"/>
-      <c r="M28" s="2"/>
-      <c r="N28" s="2"/>
-      <c r="O28" s="2"/>
-      <c r="P28" s="2"/>
-      <c r="Q28" s="2"/>
-      <c r="R28" s="2"/>
-      <c r="S28" s="2"/>
-      <c r="T28" s="2"/>
-      <c r="U28" s="2"/>
-      <c r="V28" s="2"/>
-      <c r="W28" s="2"/>
-      <c r="X28" s="2"/>
-      <c r="Y28" s="2"/>
+      <c r="B28" s="17"/>
+      <c r="C28" s="5"/>
+      <c r="D28" s="5"/>
+      <c r="E28" s="5"/>
+      <c r="F28" s="5"/>
+      <c r="G28" s="5"/>
+      <c r="H28" s="5"/>
+      <c r="I28" s="5"/>
+      <c r="J28" s="5"/>
+      <c r="K28" s="5"/>
+      <c r="L28" s="5"/>
+      <c r="M28" s="5"/>
+      <c r="N28" s="5"/>
+      <c r="O28" s="5"/>
+      <c r="P28" s="5"/>
+      <c r="Q28" s="5"/>
+      <c r="R28" s="5"/>
+      <c r="S28" s="5"/>
+      <c r="T28" s="5"/>
+      <c r="U28" s="5"/>
+      <c r="V28" s="5"/>
+      <c r="W28" s="5"/>
+      <c r="X28" s="5"/>
+      <c r="Y28" s="5"/>
     </row>
     <row r="29" spans="2:25">
-      <c r="B29" s="9"/>
-      <c r="C29" s="2"/>
-      <c r="D29" s="2"/>
-      <c r="E29" s="2"/>
-      <c r="F29" s="2"/>
-      <c r="G29" s="2"/>
-      <c r="H29" s="2"/>
-      <c r="I29" s="2"/>
-      <c r="J29" s="2"/>
-      <c r="K29" s="2"/>
-      <c r="L29" s="2"/>
-      <c r="M29" s="2"/>
-      <c r="N29" s="2"/>
-      <c r="O29" s="2"/>
-      <c r="P29" s="2"/>
-      <c r="Q29" s="2"/>
-      <c r="R29" s="2"/>
-      <c r="S29" s="2"/>
-      <c r="T29" s="2"/>
-      <c r="U29" s="2"/>
-      <c r="V29" s="2"/>
-      <c r="W29" s="2"/>
-      <c r="X29" s="2"/>
-      <c r="Y29" s="2"/>
+      <c r="B29" s="17"/>
+      <c r="C29" s="5"/>
+      <c r="D29" s="5"/>
+      <c r="E29" s="5"/>
+      <c r="F29" s="5"/>
+      <c r="G29" s="5"/>
+      <c r="H29" s="5"/>
+      <c r="I29" s="5"/>
+      <c r="J29" s="5"/>
+      <c r="K29" s="5"/>
+      <c r="L29" s="5"/>
+      <c r="M29" s="5"/>
+      <c r="N29" s="5"/>
+      <c r="O29" s="5"/>
+      <c r="P29" s="5"/>
+      <c r="Q29" s="5"/>
+      <c r="R29" s="5"/>
+      <c r="S29" s="5"/>
+      <c r="T29" s="5"/>
+      <c r="U29" s="5"/>
+      <c r="V29" s="5"/>
+      <c r="W29" s="5"/>
+      <c r="X29" s="5"/>
+      <c r="Y29" s="5"/>
     </row>
     <row r="30" spans="2:25">
-      <c r="B30" s="9"/>
-      <c r="C30" s="2"/>
-      <c r="D30" s="2"/>
-      <c r="E30" s="2"/>
-      <c r="F30" s="2"/>
-      <c r="G30" s="2"/>
-      <c r="H30" s="2"/>
-      <c r="I30" s="2"/>
-      <c r="J30" s="2"/>
-      <c r="K30" s="2"/>
-      <c r="L30" s="2"/>
-      <c r="M30" s="2"/>
-      <c r="N30" s="2"/>
-      <c r="O30" s="2"/>
-      <c r="P30" s="2"/>
-      <c r="Q30" s="2"/>
-      <c r="R30" s="2"/>
-      <c r="S30" s="2"/>
-      <c r="T30" s="2"/>
-      <c r="U30" s="2"/>
-      <c r="V30" s="2"/>
-      <c r="W30" s="2"/>
-      <c r="X30" s="2"/>
-      <c r="Y30" s="2"/>
+      <c r="B30" s="17"/>
+      <c r="C30" s="5"/>
+      <c r="D30" s="5"/>
+      <c r="E30" s="5"/>
+      <c r="F30" s="5"/>
+      <c r="G30" s="5"/>
+      <c r="H30" s="5"/>
+      <c r="I30" s="5"/>
+      <c r="J30" s="5"/>
+      <c r="K30" s="5"/>
+      <c r="L30" s="5"/>
+      <c r="M30" s="5"/>
+      <c r="N30" s="5"/>
+      <c r="O30" s="5"/>
+      <c r="P30" s="5"/>
+      <c r="Q30" s="5"/>
+      <c r="R30" s="5"/>
+      <c r="S30" s="5"/>
+      <c r="T30" s="5"/>
+      <c r="U30" s="5"/>
+      <c r="V30" s="5"/>
+      <c r="W30" s="5"/>
+      <c r="X30" s="5"/>
+      <c r="Y30" s="5"/>
     </row>
     <row r="31" spans="2:25">
-      <c r="B31" s="9"/>
-      <c r="C31" s="2"/>
-      <c r="D31" s="2"/>
-      <c r="E31" s="2"/>
-      <c r="F31" s="2"/>
-      <c r="G31" s="2"/>
-      <c r="H31" s="2"/>
-      <c r="I31" s="2"/>
-      <c r="J31" s="2"/>
-      <c r="K31" s="2"/>
-      <c r="L31" s="2"/>
-      <c r="M31" s="2"/>
-      <c r="N31" s="2"/>
-      <c r="O31" s="2"/>
-      <c r="P31" s="2"/>
-      <c r="Q31" s="2"/>
-      <c r="R31" s="2"/>
-      <c r="S31" s="2"/>
-      <c r="T31" s="2"/>
-      <c r="U31" s="2"/>
-      <c r="V31" s="2"/>
-      <c r="W31" s="2"/>
-      <c r="X31" s="2"/>
-      <c r="Y31" s="2"/>
+      <c r="B31" s="17"/>
+      <c r="C31" s="5"/>
+      <c r="D31" s="5"/>
+      <c r="E31" s="5"/>
+      <c r="F31" s="5"/>
+      <c r="G31" s="5"/>
+      <c r="H31" s="5"/>
+      <c r="I31" s="5"/>
+      <c r="J31" s="5"/>
+      <c r="K31" s="5"/>
+      <c r="L31" s="5"/>
+      <c r="M31" s="5"/>
+      <c r="N31" s="5"/>
+      <c r="O31" s="5"/>
+      <c r="P31" s="5"/>
+      <c r="Q31" s="5"/>
+      <c r="R31" s="5"/>
+      <c r="S31" s="5"/>
+      <c r="T31" s="5"/>
+      <c r="U31" s="5"/>
+      <c r="V31" s="5"/>
+      <c r="W31" s="5"/>
+      <c r="X31" s="5"/>
+      <c r="Y31" s="5"/>
     </row>
     <row r="32" spans="2:25">
-      <c r="B32" s="9"/>
-      <c r="C32" s="2"/>
-      <c r="D32" s="2"/>
-      <c r="E32" s="2"/>
-      <c r="F32" s="2"/>
-      <c r="G32" s="2"/>
-      <c r="H32" s="2"/>
-      <c r="I32" s="2"/>
-      <c r="J32" s="2"/>
-      <c r="K32" s="2"/>
-      <c r="L32" s="2"/>
-      <c r="M32" s="2"/>
-      <c r="N32" s="2"/>
-      <c r="O32" s="2"/>
-      <c r="P32" s="2"/>
-      <c r="Q32" s="2"/>
-      <c r="R32" s="2"/>
-      <c r="S32" s="2"/>
-      <c r="T32" s="2"/>
-      <c r="U32" s="2"/>
-      <c r="V32" s="2"/>
-      <c r="W32" s="2"/>
-      <c r="X32" s="2"/>
-      <c r="Y32" s="2"/>
+      <c r="B32" s="17"/>
+      <c r="C32" s="5"/>
+      <c r="D32" s="5"/>
+      <c r="E32" s="5"/>
+      <c r="F32" s="5"/>
+      <c r="G32" s="5"/>
+      <c r="H32" s="5"/>
+      <c r="I32" s="5"/>
+      <c r="J32" s="5"/>
+      <c r="K32" s="5"/>
+      <c r="L32" s="5"/>
+      <c r="M32" s="5"/>
+      <c r="N32" s="5"/>
+      <c r="O32" s="5"/>
+      <c r="P32" s="5"/>
+      <c r="Q32" s="5"/>
+      <c r="R32" s="5"/>
+      <c r="S32" s="5"/>
+      <c r="T32" s="5"/>
+      <c r="U32" s="5"/>
+      <c r="V32" s="5"/>
+      <c r="W32" s="5"/>
+      <c r="X32" s="5"/>
+      <c r="Y32" s="5"/>
     </row>
     <row r="33" spans="2:25">
-      <c r="B33" s="9"/>
-      <c r="C33" s="2"/>
-      <c r="D33" s="2"/>
-      <c r="E33" s="2"/>
-      <c r="F33" s="2"/>
-      <c r="G33" s="2"/>
-      <c r="H33" s="2"/>
-      <c r="I33" s="2"/>
-      <c r="J33" s="2"/>
-      <c r="K33" s="2"/>
-      <c r="L33" s="2"/>
-      <c r="M33" s="2"/>
-      <c r="N33" s="2"/>
-      <c r="O33" s="2"/>
-      <c r="P33" s="2"/>
-      <c r="Q33" s="2"/>
-      <c r="R33" s="2"/>
-      <c r="S33" s="2"/>
-      <c r="T33" s="2"/>
-      <c r="U33" s="2"/>
-      <c r="V33" s="2"/>
-      <c r="W33" s="2"/>
-      <c r="X33" s="2"/>
-      <c r="Y33" s="2"/>
+      <c r="B33" s="17"/>
+      <c r="C33" s="5"/>
+      <c r="D33" s="5"/>
+      <c r="E33" s="5"/>
+      <c r="F33" s="5"/>
+      <c r="G33" s="5"/>
+      <c r="H33" s="5"/>
+      <c r="I33" s="5"/>
+      <c r="J33" s="5"/>
+      <c r="K33" s="5"/>
+      <c r="L33" s="5"/>
+      <c r="M33" s="5"/>
+      <c r="N33" s="5"/>
+      <c r="O33" s="5"/>
+      <c r="P33" s="5"/>
+      <c r="Q33" s="5"/>
+      <c r="R33" s="5"/>
+      <c r="S33" s="5"/>
+      <c r="T33" s="5"/>
+      <c r="U33" s="5"/>
+      <c r="V33" s="5"/>
+      <c r="W33" s="5"/>
+      <c r="X33" s="5"/>
+      <c r="Y33" s="5"/>
     </row>
     <row r="34" spans="2:25">
-      <c r="B34" s="9"/>
-      <c r="C34" s="2"/>
-      <c r="D34" s="2"/>
-      <c r="E34" s="2"/>
-      <c r="F34" s="2"/>
-      <c r="G34" s="2"/>
-      <c r="H34" s="2"/>
-      <c r="I34" s="2"/>
-      <c r="J34" s="2"/>
-      <c r="K34" s="2"/>
-      <c r="L34" s="2"/>
-      <c r="M34" s="2"/>
-      <c r="N34" s="2"/>
-      <c r="O34" s="2"/>
-      <c r="P34" s="2"/>
-      <c r="Q34" s="2"/>
-      <c r="R34" s="2"/>
-      <c r="S34" s="2"/>
-      <c r="T34" s="2"/>
-      <c r="U34" s="2"/>
-      <c r="V34" s="2"/>
-      <c r="W34" s="2"/>
-      <c r="X34" s="2"/>
-      <c r="Y34" s="2"/>
+      <c r="B34" s="17"/>
+      <c r="C34" s="5"/>
+      <c r="D34" s="5"/>
+      <c r="E34" s="5"/>
+      <c r="F34" s="5"/>
+      <c r="G34" s="5"/>
+      <c r="H34" s="5"/>
+      <c r="I34" s="5"/>
+      <c r="J34" s="5"/>
+      <c r="K34" s="5"/>
+      <c r="L34" s="5"/>
+      <c r="M34" s="5"/>
+      <c r="N34" s="5"/>
+      <c r="O34" s="5"/>
+      <c r="P34" s="5"/>
+      <c r="Q34" s="5"/>
+      <c r="R34" s="5"/>
+      <c r="S34" s="5"/>
+      <c r="T34" s="5"/>
+      <c r="U34" s="5"/>
+      <c r="V34" s="5"/>
+      <c r="W34" s="5"/>
+      <c r="X34" s="5"/>
+      <c r="Y34" s="5"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -5025,7 +5067,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="B2:M10"/>
+  <dimension ref="B2:M12"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.8"/>
   <cols>
     <col min="2" max="2" width="15.5625" customWidth="1"/>
@@ -5037,409 +5079,501 @@
   </cols>
   <sheetData>
     <row r="2" ht="18" spans="2:13">
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="C2" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="D2" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="E2" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="F2" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="G2" s="1" t="s">
+      <c r="G2" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="H2" s="1" t="s">
+      <c r="H2" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="I2" s="1" t="s">
+      <c r="I2" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="J2" s="1" t="s">
+      <c r="J2" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="K2" s="1" t="s">
+      <c r="K2" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="L2" s="1" t="s">
+      <c r="L2" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="M2" s="1" t="s">
+      <c r="M2" s="3" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="3" spans="2:13">
-      <c r="B3" s="2">
+    <row r="3" s="1" customFormat="1" spans="2:13">
+      <c r="B3" s="4">
         <v>400000</v>
       </c>
-      <c r="C3" s="2">
+      <c r="C3" s="4">
         <v>100</v>
       </c>
-      <c r="D3" s="2">
+      <c r="D3" s="4">
         <f>C3/2</f>
         <v>50</v>
       </c>
-      <c r="E3" s="3">
+      <c r="E3" s="7">
         <f>((D3*SQRT(2))/(2*3.14*B3))*1000000</f>
         <v>28.1491553020122</v>
       </c>
-      <c r="F3" s="4">
+      <c r="F3" s="8">
         <f>(1/(2*3.14*B3*D3*SQRT(2)))*1000000000</f>
         <v>5.62983106040245</v>
       </c>
-      <c r="G3" s="3">
+      <c r="G3" s="7">
         <f>F3/2</f>
         <v>2.81491553020122</v>
       </c>
-      <c r="H3" s="3">
+      <c r="H3" s="7">
         <v>28.14</v>
       </c>
-      <c r="I3" s="3">
+      <c r="I3" s="7">
         <v>2.7</v>
       </c>
-      <c r="J3" s="3">
+      <c r="J3" s="7">
         <f>2*I3</f>
         <v>5.4</v>
       </c>
-      <c r="K3" s="3">
+      <c r="K3" s="7">
         <f>D3*SQRT((J3*POWER(10,-9))/(H3*POWER(10,-6)))</f>
         <v>0.692635644809415</v>
       </c>
-      <c r="L3" s="3">
+      <c r="L3" s="7">
         <f>1/(2*3.14*SQRT((H3/POWER(10,6))*(J3/POWER(10,9))))</f>
         <v>408490.000477362</v>
       </c>
-      <c r="M3" s="3">
+      <c r="M3" s="7">
         <f>20*LOG10(K3)</f>
         <v>-3.18990324603721</v>
       </c>
     </row>
     <row r="4" spans="2:13">
-      <c r="B4" s="2">
+      <c r="B4" s="5">
         <v>200000</v>
       </c>
-      <c r="C4" s="2">
+      <c r="C4" s="5">
         <v>100</v>
       </c>
-      <c r="D4" s="2">
-        <f t="shared" ref="D4:D10" si="0">C4/2</f>
+      <c r="D4" s="5">
+        <f>C4/2</f>
         <v>50</v>
       </c>
-      <c r="E4" s="3">
-        <f t="shared" ref="E4:E10" si="1">((D4*SQRT(2))/(2*3.14*B4))*1000000</f>
+      <c r="E4" s="9">
+        <f>((D4*SQRT(2))/(2*3.14*B4))*1000000</f>
         <v>56.2983106040245</v>
       </c>
-      <c r="F4" s="4">
-        <f t="shared" ref="F4:F10" si="2">(1/(2*3.14*B4*D4*SQRT(2)))*1000000000</f>
+      <c r="F4" s="10">
+        <f>(1/(2*3.14*B4*D4*SQRT(2)))*1000000000</f>
         <v>11.2596621208049</v>
       </c>
-      <c r="G4" s="3">
-        <f t="shared" ref="G4:G10" si="3">F4/2</f>
+      <c r="G4" s="9">
+        <f>F4/2</f>
         <v>5.62983106040245</v>
       </c>
-      <c r="H4" s="3">
+      <c r="H4" s="9">
         <v>56.2</v>
       </c>
-      <c r="I4" s="3">
+      <c r="I4" s="9">
         <v>5.6</v>
       </c>
-      <c r="J4" s="3">
-        <f t="shared" ref="J4:J10" si="4">2*I4</f>
+      <c r="J4" s="9">
+        <f>2*I4</f>
         <v>11.2</v>
       </c>
-      <c r="K4" s="3">
-        <f t="shared" ref="K4:K10" si="5">D4*SQRT((J4*POWER(10,-9))/(H4*POWER(10,-6)))</f>
+      <c r="K4" s="9">
+        <f>D4*SQRT((J4*POWER(10,-9))/(H4*POWER(10,-6)))</f>
         <v>0.705847462678301</v>
       </c>
-      <c r="L4" s="3">
-        <f t="shared" ref="L4:L10" si="6">1/(2*3.14*SQRT((H4/POWER(10,6))*(J4/POWER(10,9))))</f>
+      <c r="L4" s="9">
+        <f>1/(2*3.14*SQRT((H4/POWER(10,6))*(J4/POWER(10,9))))</f>
         <v>200707.308541373</v>
       </c>
-      <c r="M4" s="3">
-        <f t="shared" ref="M4:M10" si="7">20*LOG10(K4)</f>
+      <c r="M4" s="9">
+        <f>20*LOG10(K4)</f>
         <v>-3.02578284226842</v>
       </c>
     </row>
     <row r="5" spans="2:13">
-      <c r="B5" s="2">
+      <c r="B5" s="5">
+        <v>100000</v>
+      </c>
+      <c r="C5" s="5">
+        <v>100</v>
+      </c>
+      <c r="D5" s="5">
+        <f>C5/2</f>
+        <v>50</v>
+      </c>
+      <c r="E5" s="9">
+        <f>((D5*SQRT(2))/(2*3.14*B5))*1000000</f>
+        <v>112.596621208049</v>
+      </c>
+      <c r="F5" s="10">
+        <f>(1/(2*3.14*B5*D5*SQRT(2)))*1000000000</f>
+        <v>22.5193242416098</v>
+      </c>
+      <c r="G5" s="9">
+        <f>F5/2</f>
+        <v>11.2596621208049</v>
+      </c>
+      <c r="H5" s="9">
+        <v>112</v>
+      </c>
+      <c r="I5" s="9">
+        <v>10</v>
+      </c>
+      <c r="J5" s="9">
+        <f>2*I5</f>
+        <v>20</v>
+      </c>
+      <c r="K5" s="9">
+        <f>D5*SQRT((J5*POWER(10,-9))/(H5*POWER(10,-6)))</f>
+        <v>0.668153104781061</v>
+      </c>
+      <c r="L5" s="9">
+        <f>1/(2*3.14*SQRT((H5/POWER(10,6))*(J5/POWER(10,9))))</f>
+        <v>106393.8064938</v>
+      </c>
+      <c r="M5" s="9">
+        <f>20*LOG10(K5)</f>
+        <v>-3.50248018334163</v>
+      </c>
+    </row>
+    <row r="6" spans="2:13">
+      <c r="B6" s="5">
         <v>25000</v>
       </c>
-      <c r="C5" s="2">
+      <c r="C6" s="5">
         <v>100</v>
       </c>
-      <c r="D5" s="2">
+      <c r="D6" s="5">
+        <f t="shared" ref="D6:D12" si="0">C6/2</f>
+        <v>50</v>
+      </c>
+      <c r="E6" s="9">
+        <f t="shared" ref="E6:E12" si="1">((D6*SQRT(2))/(2*3.14*B6))*1000000</f>
+        <v>450.386484832196</v>
+      </c>
+      <c r="F6" s="10">
+        <f t="shared" ref="F6:F12" si="2">(1/(2*3.14*B6*D6*SQRT(2)))*1000000000</f>
+        <v>90.0772969664392</v>
+      </c>
+      <c r="G6" s="9">
+        <f t="shared" ref="G6:G12" si="3">F6/2</f>
+        <v>45.0386484832196</v>
+      </c>
+      <c r="H6" s="9">
+        <v>450.4</v>
+      </c>
+      <c r="I6" s="9">
+        <v>47</v>
+      </c>
+      <c r="J6" s="9">
+        <f t="shared" ref="J6:J12" si="4">2*I6</f>
+        <v>94</v>
+      </c>
+      <c r="K6" s="9">
+        <f t="shared" ref="K6:K12" si="5">D6*SQRT((J6*POWER(10,-9))/(H6*POWER(10,-6)))</f>
+        <v>0.722328482717481</v>
+      </c>
+      <c r="L6" s="9">
+        <f t="shared" ref="L6:L12" si="6">1/(2*3.14*SQRT((H6/POWER(10,6))*(J6/POWER(10,9))))</f>
+        <v>24472.438091797</v>
+      </c>
+      <c r="M6" s="9">
+        <f t="shared" ref="M6:M12" si="7">20*LOG10(K6)</f>
+        <v>-2.82530519571553</v>
+      </c>
+    </row>
+    <row r="7" spans="2:13">
+      <c r="B7" s="5">
+        <v>20000</v>
+      </c>
+      <c r="C7" s="5">
+        <v>100</v>
+      </c>
+      <c r="D7" s="5">
         <f t="shared" si="0"/>
         <v>50</v>
       </c>
-      <c r="E5" s="3">
-        <f t="shared" si="1"/>
-        <v>450.386484832196</v>
-      </c>
-      <c r="F5" s="4">
-        <f t="shared" si="2"/>
-        <v>90.0772969664392</v>
-      </c>
-      <c r="G5" s="3">
-        <f t="shared" si="3"/>
-        <v>45.0386484832196</v>
-      </c>
-      <c r="H5" s="3">
-        <v>450.4</v>
-      </c>
-      <c r="I5" s="3">
-        <v>47</v>
-      </c>
-      <c r="J5" s="3">
-        <f t="shared" si="4"/>
-        <v>94</v>
-      </c>
-      <c r="K5" s="3">
-        <f t="shared" si="5"/>
-        <v>0.722328482717481</v>
-      </c>
-      <c r="L5" s="3">
-        <f t="shared" si="6"/>
-        <v>24472.438091797</v>
-      </c>
-      <c r="M5" s="3">
-        <f t="shared" si="7"/>
-        <v>-2.82530519571553</v>
-      </c>
-    </row>
-    <row r="6" spans="2:13">
-      <c r="B6" s="2">
-        <v>20000</v>
-      </c>
-      <c r="C6" s="2">
-        <v>100</v>
-      </c>
-      <c r="D6" s="2">
-        <f t="shared" si="0"/>
-        <v>50</v>
-      </c>
-      <c r="E6" s="3">
+      <c r="E7" s="9">
         <f t="shared" si="1"/>
         <v>562.983106040245</v>
       </c>
-      <c r="F6" s="4">
+      <c r="F7" s="10">
         <f t="shared" si="2"/>
         <v>112.596621208049</v>
       </c>
-      <c r="G6" s="3">
+      <c r="G7" s="9">
         <f t="shared" si="3"/>
         <v>56.2983106040245</v>
       </c>
-      <c r="H6" s="3">
+      <c r="H7" s="9">
         <v>563</v>
       </c>
-      <c r="I6" s="3">
+      <c r="I7" s="9">
         <v>56</v>
       </c>
-      <c r="J6" s="3">
+      <c r="J7" s="9">
         <f t="shared" si="4"/>
         <v>112</v>
       </c>
-      <c r="K6" s="3">
+      <c r="K7" s="9">
         <f t="shared" si="5"/>
         <v>0.70522032131709</v>
       </c>
-      <c r="L6" s="3">
+      <c r="L7" s="9">
         <f t="shared" si="6"/>
         <v>20052.8981266233</v>
       </c>
-      <c r="M6" s="3">
+      <c r="M7" s="9">
         <f t="shared" si="7"/>
         <v>-3.03350363509127</v>
       </c>
     </row>
-    <row r="7" spans="2:13">
-      <c r="B7" s="2">
+    <row r="8" s="2" customFormat="1" spans="2:13">
+      <c r="B8" s="6">
         <v>400000</v>
       </c>
-      <c r="C7" s="2">
+      <c r="C8" s="6">
         <v>500</v>
       </c>
-      <c r="D7" s="2">
+      <c r="D8" s="6">
         <f t="shared" si="0"/>
         <v>250</v>
       </c>
-      <c r="E7" s="3">
+      <c r="E8" s="11">
         <f t="shared" si="1"/>
         <v>140.745776510061</v>
       </c>
-      <c r="F7" s="4">
+      <c r="F8" s="12">
         <f t="shared" si="2"/>
         <v>1.12596621208049</v>
       </c>
-      <c r="G7" s="3">
+      <c r="G8" s="11">
         <f t="shared" si="3"/>
         <v>0.562983106040245</v>
       </c>
-      <c r="H7" s="3">
+      <c r="H8" s="11">
         <v>140.7</v>
       </c>
-      <c r="I7" s="3">
+      <c r="I8" s="11">
         <v>0.56</v>
       </c>
-      <c r="J7" s="3">
+      <c r="J8" s="11">
         <f t="shared" si="4"/>
         <v>1.12</v>
       </c>
-      <c r="K7" s="3">
+      <c r="K8" s="11">
         <f t="shared" si="5"/>
         <v>0.705345615858598</v>
       </c>
-      <c r="L7" s="3">
+      <c r="L8" s="11">
         <f t="shared" si="6"/>
         <v>401129.217390013</v>
       </c>
-      <c r="M7" s="3">
+      <c r="M8" s="11">
         <f t="shared" si="7"/>
         <v>-3.03196057420489</v>
       </c>
     </row>
-    <row r="8" spans="2:13">
-      <c r="B8" s="2">
+    <row r="9" spans="2:13">
+      <c r="B9" s="5">
         <v>200000</v>
       </c>
-      <c r="C8" s="2">
+      <c r="C9" s="5">
         <v>500</v>
       </c>
-      <c r="D8" s="2">
+      <c r="D9" s="5">
         <f t="shared" si="0"/>
         <v>250</v>
       </c>
-      <c r="E8" s="3">
+      <c r="E9" s="9">
         <f t="shared" si="1"/>
         <v>281.491553020122</v>
       </c>
-      <c r="F8" s="4">
+      <c r="F9" s="10">
         <f t="shared" si="2"/>
         <v>2.25193242416098</v>
       </c>
-      <c r="G8" s="3">
+      <c r="G9" s="9">
         <f t="shared" si="3"/>
         <v>1.12596621208049</v>
       </c>
-      <c r="H8" s="3">
+      <c r="H9" s="9">
         <v>281.5</v>
       </c>
-      <c r="I8" s="3">
+      <c r="I9" s="9">
         <v>1</v>
       </c>
-      <c r="J8" s="3">
+      <c r="J9" s="9">
         <f t="shared" si="4"/>
         <v>2</v>
       </c>
-      <c r="K8" s="3">
+      <c r="K9" s="9">
         <f t="shared" si="5"/>
         <v>0.666370567755029</v>
       </c>
-      <c r="L8" s="3">
+      <c r="L9" s="9">
         <f t="shared" si="6"/>
         <v>212219.926036633</v>
       </c>
-      <c r="M8" s="3">
+      <c r="M9" s="9">
         <f t="shared" si="7"/>
         <v>-3.52568386179308</v>
       </c>
     </row>
-    <row r="9" spans="2:13">
-      <c r="B9" s="2">
+    <row r="10" spans="2:13">
+      <c r="B10" s="5">
         <v>25000</v>
       </c>
-      <c r="C9" s="2">
+      <c r="C10" s="5">
         <v>500</v>
       </c>
-      <c r="D9" s="2">
+      <c r="D10" s="5">
         <f t="shared" si="0"/>
         <v>250</v>
       </c>
-      <c r="E9" s="3">
+      <c r="E10" s="9">
         <f t="shared" si="1"/>
         <v>2251.93242416098</v>
       </c>
-      <c r="F9" s="4">
+      <c r="F10" s="10">
         <f t="shared" si="2"/>
         <v>18.0154593932878</v>
       </c>
-      <c r="G9" s="3">
+      <c r="G10" s="9">
         <f t="shared" si="3"/>
         <v>9.00772969664392</v>
       </c>
-      <c r="H9" s="3">
+      <c r="H10" s="9">
         <v>2252</v>
       </c>
-      <c r="I9" s="3">
+      <c r="I10" s="9">
         <v>8.6</v>
       </c>
-      <c r="J9" s="3">
+      <c r="J10" s="9">
         <f t="shared" si="4"/>
         <v>17.2</v>
       </c>
-      <c r="K9" s="3">
+      <c r="K10" s="9">
         <f t="shared" si="5"/>
         <v>0.690907709891793</v>
       </c>
-      <c r="L9" s="3">
+      <c r="L10" s="9">
         <f t="shared" si="6"/>
         <v>25585.3840131756</v>
       </c>
-      <c r="M9" s="3">
+      <c r="M10" s="9">
         <f t="shared" si="7"/>
         <v>-3.21159921927684</v>
       </c>
     </row>
-    <row r="10" spans="2:13">
-      <c r="B10" s="2">
+    <row r="11" spans="2:13">
+      <c r="B11" s="5">
         <v>20000</v>
       </c>
-      <c r="C10" s="2">
+      <c r="C11" s="5">
         <v>500</v>
       </c>
-      <c r="D10" s="2">
+      <c r="D11" s="5">
         <f t="shared" si="0"/>
         <v>250</v>
       </c>
-      <c r="E10" s="3">
+      <c r="E11" s="9">
         <f t="shared" si="1"/>
         <v>2814.91553020122</v>
       </c>
-      <c r="F10" s="4">
+      <c r="F11" s="10">
         <f t="shared" si="2"/>
         <v>22.5193242416098</v>
       </c>
-      <c r="G10" s="3">
+      <c r="G11" s="9">
         <f t="shared" si="3"/>
         <v>11.2596621208049</v>
       </c>
-      <c r="H10" s="3">
+      <c r="H11" s="9">
         <v>2815</v>
       </c>
-      <c r="I10" s="3">
+      <c r="I11" s="9">
         <v>10</v>
       </c>
-      <c r="J10" s="3">
+      <c r="J11" s="9">
         <f t="shared" si="4"/>
         <v>20</v>
       </c>
-      <c r="K10" s="3">
+      <c r="K11" s="9">
         <f t="shared" si="5"/>
         <v>0.666370567755029</v>
       </c>
-      <c r="L10" s="3">
+      <c r="L11" s="9">
         <f t="shared" si="6"/>
         <v>21221.9926036634</v>
       </c>
-      <c r="M10" s="3">
+      <c r="M11" s="9">
         <f t="shared" si="7"/>
         <v>-3.52568386179308</v>
+      </c>
+    </row>
+    <row r="12" s="2" customFormat="1" spans="2:13">
+      <c r="B12" s="6">
+        <v>100000</v>
+      </c>
+      <c r="C12" s="6">
+        <v>500</v>
+      </c>
+      <c r="D12" s="6">
+        <f t="shared" si="0"/>
+        <v>250</v>
+      </c>
+      <c r="E12" s="11">
+        <f t="shared" si="1"/>
+        <v>562.983106040245</v>
+      </c>
+      <c r="F12" s="12">
+        <f t="shared" si="2"/>
+        <v>4.50386484832196</v>
+      </c>
+      <c r="G12" s="11">
+        <f t="shared" si="3"/>
+        <v>2.25193242416098</v>
+      </c>
+      <c r="H12" s="11">
+        <v>560</v>
+      </c>
+      <c r="I12" s="11">
+        <v>2.2</v>
+      </c>
+      <c r="J12" s="11">
+        <f t="shared" si="4"/>
+        <v>4.4</v>
+      </c>
+      <c r="K12" s="11">
+        <f t="shared" si="5"/>
+        <v>0.700764888226735</v>
+      </c>
+      <c r="L12" s="11">
+        <f t="shared" si="6"/>
+        <v>101442.514219273</v>
+      </c>
+      <c r="M12" s="11">
+        <f t="shared" si="7"/>
+        <v>-3.08855333175938</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
modified:   Ferrite Transformer Calculation.xlsx 	modified:   README.md 	modified:   firmware/ESP32-S3 PWM/src/main.cpp
</commit_message>
<xml_diff>
--- a/Ferrite Transformer Calculation.xlsx
+++ b/Ferrite Transformer Calculation.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="27660" windowHeight="13060" activeTab="3"/>
+    <workbookView windowWidth="27660" windowHeight="13060" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="ETD" sheetId="1" r:id="rId1"/>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="47">
   <si>
     <t>#</t>
   </si>
@@ -1790,7 +1790,7 @@
       <charset val="134"/>
     </font>
   </fonts>
-  <fills count="36">
+  <fills count="37">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1812,6 +1812,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="5" tint="0.8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.6"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -2134,7 +2140,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -2158,16 +2164,16 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="6" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="7" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="8" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="8" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="8" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="9" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
@@ -2176,89 +2182,89 @@
     <xf numFmtId="0" fontId="17" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="45">
+  <cellXfs count="51">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -2349,13 +2355,19 @@
     <xf numFmtId="41" fontId="1" fillId="4" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="41" fontId="1" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="186" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="186" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="176" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1">
+    <xf numFmtId="186" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="187" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1">
@@ -2370,10 +2382,22 @@
     <xf numFmtId="188" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="187" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="188" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="41" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="41" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="188" fontId="1" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -2930,12 +2954,12 @@
   <dimension ref="A1:U33"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="5.5625" style="37" customWidth="1"/>
-    <col min="2" max="4" width="10.5625" style="37" customWidth="1"/>
-    <col min="5" max="5" width="20.5625" style="37" customWidth="1"/>
-    <col min="6" max="6" width="15.5625" style="37" customWidth="1"/>
-    <col min="7" max="7" width="30.5625" style="40" customWidth="1"/>
-    <col min="8" max="8" width="10.5625" style="37" customWidth="1"/>
+    <col min="1" max="1" width="5.5625" style="41" customWidth="1"/>
+    <col min="2" max="4" width="10.5625" style="41" customWidth="1"/>
+    <col min="5" max="5" width="20.5625" style="41" customWidth="1"/>
+    <col min="6" max="6" width="15.5625" style="41" customWidth="1"/>
+    <col min="7" max="7" width="30.5625" style="46" customWidth="1"/>
+    <col min="8" max="8" width="10.5625" style="41" customWidth="1"/>
     <col min="9" max="9" width="15.5625" style="13" customWidth="1"/>
     <col min="10" max="13" width="10.5625" style="13" customWidth="1"/>
     <col min="14" max="14" width="9" style="13"/>
@@ -2954,7 +2978,7 @@
       <c r="G1" s="26"/>
       <c r="H1" s="13"/>
     </row>
-    <row r="2" s="39" customFormat="1" ht="18" spans="1:21">
+    <row r="2" s="45" customFormat="1" ht="18" spans="1:21">
       <c r="A2" s="26" t="s">
         <v>0</v>
       </c>
@@ -3032,52 +3056,52 @@
       <c r="D3" s="28">
         <v>10</v>
       </c>
-      <c r="E3" s="41">
+      <c r="E3" s="47">
         <f>3.14*POWER(D3,2)/4</f>
         <v>78.5</v>
       </c>
-      <c r="F3" s="41">
+      <c r="F3" s="47">
         <v>1898.58</v>
       </c>
-      <c r="G3" s="42">
+      <c r="G3" s="48">
         <f>(B3*POWER(10,10))/(4*C3*F3*E3)</f>
         <v>3.01935345175506</v>
       </c>
-      <c r="H3" s="43" t="str">
+      <c r="H3" s="49" t="str">
         <f>IF((B3*POWER(10,10))/(4*C3*G3*E3)&gt;1200,IF((B3*POWER(10,10))/(4*C3*G3*E3)&lt;2000,"OK","NG"),"NG")</f>
         <v>OK</v>
       </c>
-      <c r="I3" s="37">
+      <c r="I3" s="41">
         <f>B3/G3</f>
         <v>23.8461648</v>
       </c>
-      <c r="J3" s="37">
+      <c r="J3" s="41">
         <f>B3*3</f>
         <v>216</v>
       </c>
-      <c r="K3" s="34">
+      <c r="K3" s="36">
         <v>0.5</v>
       </c>
-      <c r="L3" s="37">
+      <c r="L3" s="41">
         <f>J3*K3</f>
         <v>108</v>
       </c>
-      <c r="M3" s="34">
+      <c r="M3" s="36">
         <f>L3/B3</f>
         <v>1.5</v>
       </c>
-      <c r="N3" s="37">
+      <c r="N3" s="41">
         <f>J3/I3</f>
         <v>9.05806035526518</v>
       </c>
-      <c r="O3" s="37">
+      <c r="O3" s="41">
         <v>1.5</v>
       </c>
-      <c r="P3" s="44">
+      <c r="P3" s="50">
         <f>SQRT((M3*0.9/(O3+5))/0.9)</f>
         <v>0.480384461415261</v>
       </c>
-      <c r="Q3" s="44">
+      <c r="Q3" s="50">
         <f>SQRT((K3*0.9/(O3+5))/0.9)</f>
         <v>0.277350098112615</v>
       </c>
@@ -3109,52 +3133,52 @@
       <c r="D4" s="28">
         <v>10</v>
       </c>
-      <c r="E4" s="41">
+      <c r="E4" s="47">
         <f>3.14*POWER(D4,2)/4</f>
         <v>78.5</v>
       </c>
-      <c r="F4" s="41">
+      <c r="F4" s="47">
         <v>1898.58</v>
       </c>
-      <c r="G4" s="42">
+      <c r="G4" s="48">
         <f>(B4*POWER(10,10))/(4*C4*F4*E4)</f>
         <v>3.01935345175506</v>
       </c>
-      <c r="H4" s="43" t="str">
+      <c r="H4" s="49" t="str">
         <f>IF((B4*POWER(10,10))/(4*C4*G4*E4)&gt;1200,IF((B4*POWER(10,10))/(4*C4*G4*E4)&lt;2000,"OK","NG"),"NG")</f>
         <v>OK</v>
       </c>
-      <c r="I4" s="37">
+      <c r="I4" s="41">
         <f>B4/G4</f>
         <v>23.8461648</v>
       </c>
-      <c r="J4" s="37">
+      <c r="J4" s="41">
         <f>B4*3</f>
         <v>216</v>
       </c>
-      <c r="K4" s="34">
+      <c r="K4" s="36">
         <v>0.5</v>
       </c>
-      <c r="L4" s="37">
+      <c r="L4" s="41">
         <f>J4*K4</f>
         <v>108</v>
       </c>
-      <c r="M4" s="34">
+      <c r="M4" s="36">
         <f>L4/B4</f>
         <v>1.5</v>
       </c>
-      <c r="N4" s="37">
+      <c r="N4" s="41">
         <f>J4/I4</f>
         <v>9.05806035526518</v>
       </c>
-      <c r="O4" s="37">
+      <c r="O4" s="41">
         <v>1.5</v>
       </c>
-      <c r="P4" s="44">
+      <c r="P4" s="50">
         <f>SQRT((M4*0.9/(O4+5))/0.9)</f>
         <v>0.480384461415261</v>
       </c>
-      <c r="Q4" s="44">
+      <c r="Q4" s="50">
         <f>SQRT((K4*0.9/(O4+5))/0.9)</f>
         <v>0.277350098112615</v>
       </c>
@@ -3180,7 +3204,7 @@
       <c r="D5" s="28"/>
       <c r="E5" s="28"/>
       <c r="F5" s="28"/>
-      <c r="G5" s="42"/>
+      <c r="G5" s="48"/>
       <c r="H5" s="28"/>
     </row>
     <row r="6" spans="1:8">
@@ -3190,7 +3214,7 @@
       <c r="D6" s="28"/>
       <c r="E6" s="28"/>
       <c r="F6" s="28"/>
-      <c r="G6" s="42"/>
+      <c r="G6" s="48"/>
       <c r="H6" s="28"/>
     </row>
     <row r="7" spans="1:8">
@@ -3200,7 +3224,7 @@
       <c r="D7" s="28"/>
       <c r="E7" s="28"/>
       <c r="F7" s="28"/>
-      <c r="G7" s="42"/>
+      <c r="G7" s="48"/>
       <c r="H7" s="28"/>
     </row>
     <row r="8" spans="1:8">
@@ -3210,7 +3234,7 @@
       <c r="D8" s="28"/>
       <c r="E8" s="28"/>
       <c r="F8" s="28"/>
-      <c r="G8" s="42"/>
+      <c r="G8" s="48"/>
       <c r="H8" s="28"/>
     </row>
     <row r="9" spans="1:8">
@@ -3220,7 +3244,7 @@
       <c r="D9" s="28"/>
       <c r="E9" s="28"/>
       <c r="F9" s="28"/>
-      <c r="G9" s="42"/>
+      <c r="G9" s="48"/>
       <c r="H9" s="28"/>
     </row>
     <row r="10" spans="1:8">
@@ -3230,7 +3254,7 @@
       <c r="D10" s="28"/>
       <c r="E10" s="28"/>
       <c r="F10" s="28"/>
-      <c r="G10" s="42"/>
+      <c r="G10" s="48"/>
       <c r="H10" s="28"/>
     </row>
     <row r="11" spans="1:8">
@@ -3240,7 +3264,7 @@
       <c r="D11" s="28"/>
       <c r="E11" s="28"/>
       <c r="F11" s="28"/>
-      <c r="G11" s="42"/>
+      <c r="G11" s="48"/>
       <c r="H11" s="28"/>
     </row>
     <row r="12" spans="1:8">
@@ -3250,7 +3274,7 @@
       <c r="D12" s="28"/>
       <c r="E12" s="28"/>
       <c r="F12" s="28"/>
-      <c r="G12" s="42"/>
+      <c r="G12" s="48"/>
       <c r="H12" s="28"/>
     </row>
     <row r="13" spans="1:8">
@@ -3260,7 +3284,7 @@
       <c r="D13" s="28"/>
       <c r="E13" s="28"/>
       <c r="F13" s="28"/>
-      <c r="G13" s="42"/>
+      <c r="G13" s="48"/>
       <c r="H13" s="28"/>
     </row>
     <row r="14" spans="1:8">
@@ -3270,7 +3294,7 @@
       <c r="D14" s="28"/>
       <c r="E14" s="28"/>
       <c r="F14" s="28"/>
-      <c r="G14" s="42"/>
+      <c r="G14" s="48"/>
       <c r="H14" s="28"/>
     </row>
     <row r="15" spans="1:8">
@@ -3280,7 +3304,7 @@
       <c r="D15" s="28"/>
       <c r="E15" s="28"/>
       <c r="F15" s="28"/>
-      <c r="G15" s="42"/>
+      <c r="G15" s="48"/>
       <c r="H15" s="28"/>
     </row>
     <row r="16" spans="1:8">
@@ -3290,7 +3314,7 @@
       <c r="D16" s="28"/>
       <c r="E16" s="28"/>
       <c r="F16" s="28"/>
-      <c r="G16" s="42"/>
+      <c r="G16" s="48"/>
       <c r="H16" s="28"/>
     </row>
     <row r="17" spans="1:8">
@@ -3300,7 +3324,7 @@
       <c r="D17" s="28"/>
       <c r="E17" s="28"/>
       <c r="F17" s="28"/>
-      <c r="G17" s="42"/>
+      <c r="G17" s="48"/>
       <c r="H17" s="28"/>
     </row>
     <row r="18" spans="1:8">
@@ -3310,7 +3334,7 @@
       <c r="D18" s="28"/>
       <c r="E18" s="28"/>
       <c r="F18" s="28"/>
-      <c r="G18" s="42"/>
+      <c r="G18" s="48"/>
       <c r="H18" s="28"/>
     </row>
     <row r="19" spans="1:8">
@@ -3320,7 +3344,7 @@
       <c r="D19" s="28"/>
       <c r="E19" s="28"/>
       <c r="F19" s="28"/>
-      <c r="G19" s="42"/>
+      <c r="G19" s="48"/>
       <c r="H19" s="28"/>
     </row>
     <row r="20" spans="1:8">
@@ -3330,7 +3354,7 @@
       <c r="D20" s="28"/>
       <c r="E20" s="28"/>
       <c r="F20" s="28"/>
-      <c r="G20" s="42"/>
+      <c r="G20" s="48"/>
       <c r="H20" s="28"/>
     </row>
     <row r="21" spans="1:8">
@@ -3340,7 +3364,7 @@
       <c r="D21" s="28"/>
       <c r="E21" s="28"/>
       <c r="F21" s="28"/>
-      <c r="G21" s="42"/>
+      <c r="G21" s="48"/>
       <c r="H21" s="28"/>
     </row>
     <row r="22" spans="1:8">
@@ -3350,7 +3374,7 @@
       <c r="D22" s="28"/>
       <c r="E22" s="28"/>
       <c r="F22" s="28"/>
-      <c r="G22" s="42"/>
+      <c r="G22" s="48"/>
       <c r="H22" s="28"/>
     </row>
     <row r="23" spans="1:8">
@@ -3360,7 +3384,7 @@
       <c r="D23" s="28"/>
       <c r="E23" s="28"/>
       <c r="F23" s="28"/>
-      <c r="G23" s="42"/>
+      <c r="G23" s="48"/>
       <c r="H23" s="28"/>
     </row>
     <row r="24" spans="1:8">
@@ -3370,7 +3394,7 @@
       <c r="D24" s="28"/>
       <c r="E24" s="28"/>
       <c r="F24" s="28"/>
-      <c r="G24" s="42"/>
+      <c r="G24" s="48"/>
       <c r="H24" s="28"/>
     </row>
     <row r="25" spans="1:8">
@@ -3380,7 +3404,7 @@
       <c r="D25" s="28"/>
       <c r="E25" s="28"/>
       <c r="F25" s="28"/>
-      <c r="G25" s="42"/>
+      <c r="G25" s="48"/>
       <c r="H25" s="28"/>
     </row>
     <row r="26" spans="1:8">
@@ -3390,7 +3414,7 @@
       <c r="D26" s="28"/>
       <c r="E26" s="28"/>
       <c r="F26" s="28"/>
-      <c r="G26" s="42"/>
+      <c r="G26" s="48"/>
       <c r="H26" s="28"/>
     </row>
     <row r="27" spans="1:8">
@@ -3400,7 +3424,7 @@
       <c r="D27" s="28"/>
       <c r="E27" s="28"/>
       <c r="F27" s="28"/>
-      <c r="G27" s="42"/>
+      <c r="G27" s="48"/>
       <c r="H27" s="28"/>
     </row>
     <row r="28" spans="1:8">
@@ -3410,7 +3434,7 @@
       <c r="D28" s="28"/>
       <c r="E28" s="28"/>
       <c r="F28" s="28"/>
-      <c r="G28" s="42"/>
+      <c r="G28" s="48"/>
       <c r="H28" s="28"/>
     </row>
     <row r="29" spans="1:8">
@@ -3420,7 +3444,7 @@
       <c r="D29" s="28"/>
       <c r="E29" s="28"/>
       <c r="F29" s="28"/>
-      <c r="G29" s="42"/>
+      <c r="G29" s="48"/>
       <c r="H29" s="28"/>
     </row>
     <row r="30" spans="1:8">
@@ -3430,7 +3454,7 @@
       <c r="D30" s="28"/>
       <c r="E30" s="28"/>
       <c r="F30" s="28"/>
-      <c r="G30" s="42"/>
+      <c r="G30" s="48"/>
       <c r="H30" s="28"/>
     </row>
     <row r="31" spans="1:8">
@@ -3440,7 +3464,7 @@
       <c r="D31" s="28"/>
       <c r="E31" s="28"/>
       <c r="F31" s="28"/>
-      <c r="G31" s="42"/>
+      <c r="G31" s="48"/>
       <c r="H31" s="28"/>
     </row>
     <row r="32" spans="1:8">
@@ -3450,7 +3474,7 @@
       <c r="D32" s="28"/>
       <c r="E32" s="28"/>
       <c r="F32" s="28"/>
-      <c r="G32" s="42"/>
+      <c r="G32" s="48"/>
       <c r="H32" s="28"/>
     </row>
     <row r="33" spans="1:8">
@@ -3460,7 +3484,7 @@
       <c r="D33" s="28"/>
       <c r="E33" s="28"/>
       <c r="F33" s="28"/>
-      <c r="G33" s="42"/>
+      <c r="G33" s="48"/>
       <c r="H33" s="28"/>
     </row>
   </sheetData>
@@ -3472,7 +3496,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A2:U12"/>
+  <dimension ref="A2:V13"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="5.5625" style="13" customWidth="1"/>
@@ -3579,45 +3603,45 @@
         <f>(B3*0.5*POWER(10,10))/(2*C3*I3*H3)</f>
         <v>2.22222222222222</v>
       </c>
-      <c r="L3" s="30">
+      <c r="L3" s="32">
         <f>B3/J3</f>
         <v>32.4</v>
       </c>
       <c r="M3" s="13">
         <v>216</v>
       </c>
-      <c r="N3" s="33">
+      <c r="N3" s="35">
         <v>0.5</v>
       </c>
       <c r="O3" s="13">
         <f>M3*N3</f>
         <v>108</v>
       </c>
-      <c r="P3" s="34">
+      <c r="P3" s="36">
         <f>O3/B3</f>
         <v>1.5</v>
       </c>
-      <c r="Q3" s="37">
+      <c r="Q3" s="41">
         <f>M3/L3</f>
         <v>6.66666666666667</v>
       </c>
-      <c r="R3" s="34">
+      <c r="R3" s="36">
         <v>2.5</v>
       </c>
-      <c r="S3" s="33">
+      <c r="S3" s="35">
         <f>SQRT((P3*0.9/(R3+5))/0.9)</f>
         <v>0.447213595499958</v>
       </c>
-      <c r="T3" s="33">
+      <c r="T3" s="35">
         <f>SQRT((N3*0.9/(R3+5))/0.9)</f>
         <v>0.258198889747161</v>
       </c>
-      <c r="U3" s="34">
-        <f>P3/R3</f>
-        <v>0.6</v>
-      </c>
-    </row>
-    <row r="4" s="25" customFormat="1" spans="1:20">
+      <c r="U3" s="36">
+        <f>SQRT((4*P3)/(3.14*R3))</f>
+        <v>0.874260378943872</v>
+      </c>
+    </row>
+    <row r="4" s="25" customFormat="1" spans="1:22">
       <c r="A4" s="29"/>
       <c r="B4" s="29">
         <v>72</v>
@@ -3629,57 +3653,65 @@
         <v>24</v>
       </c>
       <c r="E4" s="25">
-        <v>23</v>
+        <v>23.3</v>
       </c>
       <c r="F4" s="25">
-        <v>40</v>
+        <v>40.4</v>
       </c>
       <c r="G4" s="25">
-        <v>15</v>
+        <v>15.1</v>
       </c>
       <c r="H4" s="25">
-        <f t="shared" ref="H4:H11" si="0">(F4-E4)*G4/2</f>
-        <v>127.5</v>
+        <f t="shared" ref="H4:H13" si="0">(F4-E4)*G4/2</f>
+        <v>129.105</v>
       </c>
       <c r="I4" s="25">
         <v>350</v>
       </c>
       <c r="J4" s="25">
-        <f t="shared" ref="J4:J11" si="1">(B4*0.5*POWER(10,10))/(2*C4*I4*H4)</f>
-        <v>10.0840336134454</v>
-      </c>
-      <c r="L4" s="31">
-        <f t="shared" ref="L4:L11" si="2">B4/J4</f>
-        <v>7.14</v>
+        <f t="shared" ref="J4:J13" si="1">(B4*0.5*POWER(10,10))/(2*C4*I4*H4)</f>
+        <v>9.95867151322014</v>
+      </c>
+      <c r="L4" s="33">
+        <f t="shared" ref="L4:L13" si="2">B4/J4</f>
+        <v>7.22988</v>
       </c>
       <c r="M4" s="25">
         <v>216</v>
       </c>
-      <c r="N4" s="35">
+      <c r="N4" s="37">
         <v>0.5</v>
       </c>
       <c r="O4" s="25">
         <f t="shared" ref="O4:O11" si="3">M4*N4</f>
         <v>108</v>
       </c>
-      <c r="P4" s="36">
-        <f t="shared" ref="P4:P11" si="4">O4/B4</f>
+      <c r="P4" s="38">
+        <f t="shared" ref="P4:P13" si="4">O4/B4</f>
         <v>1.5</v>
       </c>
-      <c r="Q4" s="38">
-        <f t="shared" ref="Q4:Q11" si="5">M4/L4</f>
-        <v>30.2521008403361</v>
-      </c>
-      <c r="R4" s="36">
-        <v>2.5</v>
-      </c>
-      <c r="S4" s="35">
-        <f t="shared" ref="S4:S11" si="6">SQRT((P4*0.9/(R4+5))/0.9)</f>
-        <v>0.447213595499958</v>
-      </c>
-      <c r="T4" s="35">
-        <f t="shared" ref="T4:T11" si="7">SQRT((N4*0.9/(R4+5))/0.9)</f>
-        <v>0.258198889747161</v>
+      <c r="Q4" s="42">
+        <f t="shared" ref="Q4:Q13" si="5">M4/L4</f>
+        <v>29.8760145396604</v>
+      </c>
+      <c r="R4" s="38">
+        <v>1.5</v>
+      </c>
+      <c r="S4" s="37">
+        <f t="shared" ref="S4:S13" si="6">SQRT((P4*0.9/(R4+5))/0.9)</f>
+        <v>0.480384461415261</v>
+      </c>
+      <c r="T4" s="37">
+        <f t="shared" ref="T4:T13" si="7">SQRT((N4*0.9/(R4+5))/0.9)</f>
+        <v>0.277350098112615</v>
+      </c>
+      <c r="U4" s="36">
+        <f>SQRT((4*P4)/(3.14*R4))</f>
+        <v>1.1286652959662</v>
+      </c>
+      <c r="V4" s="36">
+        <f>SQRT((4*N4)/(3.14*R4))</f>
+        <v>0.651635212451075</v>
       </c>
     </row>
     <row r="5" spans="2:20">
@@ -3710,36 +3742,36 @@
         <f t="shared" si="1"/>
         <v>6.18454687886534</v>
       </c>
-      <c r="L5" s="30">
+      <c r="L5" s="32">
         <f t="shared" si="2"/>
         <v>11.64192</v>
       </c>
       <c r="M5" s="13">
         <v>216</v>
       </c>
-      <c r="N5" s="33">
+      <c r="N5" s="35">
         <v>0.5</v>
       </c>
       <c r="O5" s="13">
         <f t="shared" si="3"/>
         <v>108</v>
       </c>
-      <c r="P5" s="34">
+      <c r="P5" s="36">
         <f t="shared" si="4"/>
         <v>1.5</v>
       </c>
-      <c r="Q5" s="37">
+      <c r="Q5" s="41">
         <f t="shared" si="5"/>
         <v>18.553640636596</v>
       </c>
-      <c r="R5" s="34">
+      <c r="R5" s="36">
         <v>2.5</v>
       </c>
-      <c r="S5" s="33">
+      <c r="S5" s="35">
         <f t="shared" si="6"/>
         <v>0.447213595499958</v>
       </c>
-      <c r="T5" s="33">
+      <c r="T5" s="35">
         <f t="shared" si="7"/>
         <v>0.258198889747161</v>
       </c>
@@ -3772,36 +3804,36 @@
         <f t="shared" si="1"/>
         <v>10.6020803637692</v>
       </c>
-      <c r="L6" s="30">
+      <c r="L6" s="32">
         <f t="shared" si="2"/>
         <v>6.79112</v>
       </c>
       <c r="M6" s="13">
         <v>216</v>
       </c>
-      <c r="N6" s="33">
+      <c r="N6" s="35">
         <v>0.5</v>
       </c>
       <c r="O6" s="13">
         <f t="shared" si="3"/>
         <v>108</v>
       </c>
-      <c r="P6" s="34">
+      <c r="P6" s="36">
         <f t="shared" si="4"/>
         <v>1.5</v>
       </c>
-      <c r="Q6" s="37">
+      <c r="Q6" s="41">
         <f t="shared" si="5"/>
         <v>31.8062410913075</v>
       </c>
-      <c r="R6" s="34">
+      <c r="R6" s="36">
         <v>2.5</v>
       </c>
-      <c r="S6" s="33">
+      <c r="S6" s="35">
         <f t="shared" si="6"/>
         <v>0.447213595499958</v>
       </c>
-      <c r="T6" s="33">
+      <c r="T6" s="35">
         <f t="shared" si="7"/>
         <v>0.258198889747161</v>
       </c>
@@ -3836,36 +3868,36 @@
         <f t="shared" si="1"/>
         <v>9.95867151322014</v>
       </c>
-      <c r="L7" s="30">
+      <c r="L7" s="32">
         <f t="shared" si="2"/>
         <v>7.22988</v>
       </c>
       <c r="M7" s="13">
         <v>216</v>
       </c>
-      <c r="N7" s="33">
+      <c r="N7" s="35">
         <v>0.5</v>
       </c>
       <c r="O7" s="13">
         <f t="shared" si="3"/>
         <v>108</v>
       </c>
-      <c r="P7" s="34">
+      <c r="P7" s="36">
         <f t="shared" si="4"/>
         <v>1.5</v>
       </c>
-      <c r="Q7" s="37">
+      <c r="Q7" s="41">
         <f t="shared" si="5"/>
         <v>29.8760145396604</v>
       </c>
-      <c r="R7" s="34">
+      <c r="R7" s="36">
         <v>2.5</v>
       </c>
-      <c r="S7" s="33">
+      <c r="S7" s="35">
         <f t="shared" si="6"/>
         <v>0.447213595499958</v>
       </c>
-      <c r="T7" s="33">
+      <c r="T7" s="35">
         <f t="shared" si="7"/>
         <v>0.258198889747161</v>
       </c>
@@ -3900,36 +3932,36 @@
         <f t="shared" si="1"/>
         <v>32.798833819242</v>
       </c>
-      <c r="L8" s="30">
+      <c r="L8" s="32">
         <f t="shared" si="2"/>
         <v>2.1952</v>
       </c>
       <c r="M8" s="13">
         <v>216</v>
       </c>
-      <c r="N8" s="33">
+      <c r="N8" s="35">
         <v>0.5</v>
       </c>
       <c r="O8" s="13">
         <f t="shared" si="3"/>
         <v>108</v>
       </c>
-      <c r="P8" s="34">
+      <c r="P8" s="36">
         <f t="shared" si="4"/>
         <v>1.5</v>
       </c>
-      <c r="Q8" s="37">
+      <c r="Q8" s="41">
         <f t="shared" si="5"/>
         <v>98.396501457726</v>
       </c>
-      <c r="R8" s="34">
+      <c r="R8" s="36">
         <v>2.5</v>
       </c>
-      <c r="S8" s="33">
+      <c r="S8" s="35">
         <f t="shared" si="6"/>
         <v>0.447213595499958</v>
       </c>
-      <c r="T8" s="33">
+      <c r="T8" s="35">
         <f t="shared" si="7"/>
         <v>0.258198889747161</v>
       </c>
@@ -3961,36 +3993,36 @@
         <f t="shared" si="1"/>
         <v>9.9756704481847</v>
       </c>
-      <c r="L9" s="30">
+      <c r="L9" s="32">
         <f t="shared" si="2"/>
         <v>7.21756</v>
       </c>
       <c r="M9" s="13">
         <v>216</v>
       </c>
-      <c r="N9" s="33">
+      <c r="N9" s="35">
         <v>0.5</v>
       </c>
       <c r="O9" s="13">
         <f t="shared" si="3"/>
         <v>108</v>
       </c>
-      <c r="P9" s="34">
+      <c r="P9" s="36">
         <f t="shared" si="4"/>
         <v>1.5</v>
       </c>
-      <c r="Q9" s="37">
+      <c r="Q9" s="41">
         <f t="shared" si="5"/>
         <v>29.9270113445541</v>
       </c>
-      <c r="R9" s="34">
+      <c r="R9" s="36">
         <v>2.5</v>
       </c>
-      <c r="S9" s="33">
+      <c r="S9" s="35">
         <f t="shared" si="6"/>
         <v>0.447213595499958</v>
       </c>
-      <c r="T9" s="33">
+      <c r="T9" s="35">
         <f t="shared" si="7"/>
         <v>0.258198889747161</v>
       </c>
@@ -4025,7 +4057,7 @@
         <f t="shared" si="1"/>
         <v>10.0840336134454</v>
       </c>
-      <c r="L10" s="30">
+      <c r="L10" s="32">
         <f t="shared" si="2"/>
         <v>7.14</v>
       </c>
@@ -4033,99 +4065,248 @@
         <f>72*7</f>
         <v>504</v>
       </c>
-      <c r="N10" s="33">
+      <c r="N10" s="35">
         <v>0.5</v>
       </c>
       <c r="O10" s="13">
         <f t="shared" si="3"/>
         <v>252</v>
       </c>
-      <c r="P10" s="34">
+      <c r="P10" s="36">
         <f t="shared" si="4"/>
         <v>3.5</v>
       </c>
-      <c r="Q10" s="37">
+      <c r="Q10" s="41">
         <f t="shared" si="5"/>
         <v>70.5882352941176</v>
       </c>
-      <c r="R10" s="34">
+      <c r="R10" s="36">
         <v>2.5</v>
       </c>
-      <c r="S10" s="33">
+      <c r="S10" s="35">
         <f t="shared" si="6"/>
         <v>0.683130051063973</v>
       </c>
-      <c r="T10" s="33">
+      <c r="T10" s="35">
         <f t="shared" si="7"/>
         <v>0.258198889747161</v>
       </c>
     </row>
-    <row r="11" s="25" customFormat="1" spans="2:20">
+    <row r="11" s="25" customFormat="1" spans="2:22">
       <c r="B11" s="29">
         <v>72</v>
       </c>
       <c r="C11" s="29">
-        <v>200000</v>
+        <v>100000</v>
       </c>
       <c r="D11" s="29" t="s">
         <v>24</v>
       </c>
       <c r="E11" s="25">
-        <v>23</v>
+        <v>23.3</v>
       </c>
       <c r="F11" s="25">
-        <v>40</v>
+        <v>40.4</v>
       </c>
       <c r="G11" s="25">
-        <v>15</v>
+        <v>15.1</v>
       </c>
       <c r="H11" s="25">
         <f t="shared" si="0"/>
-        <v>127.5</v>
+        <v>129.105</v>
       </c>
       <c r="I11" s="25">
         <v>350</v>
       </c>
       <c r="J11" s="25">
         <f t="shared" si="1"/>
-        <v>20.1680672268908</v>
-      </c>
-      <c r="L11" s="31">
+        <v>39.8346860528805</v>
+      </c>
+      <c r="L11" s="33">
         <f t="shared" si="2"/>
-        <v>3.57</v>
+        <v>1.80747</v>
       </c>
       <c r="M11" s="25">
         <v>504</v>
       </c>
-      <c r="N11" s="35">
+      <c r="N11" s="37">
+        <v>0.2</v>
+      </c>
+      <c r="O11" s="37">
+        <f t="shared" ref="O11:O13" si="8">M11*N11</f>
+        <v>100.8</v>
+      </c>
+      <c r="P11" s="38">
+        <f t="shared" si="4"/>
+        <v>1.4</v>
+      </c>
+      <c r="Q11" s="42">
+        <f t="shared" si="5"/>
+        <v>278.842802370164</v>
+      </c>
+      <c r="R11" s="38">
+        <v>1.5</v>
+      </c>
+      <c r="S11" s="37">
+        <f t="shared" si="6"/>
+        <v>0.464095480892257</v>
+      </c>
+      <c r="T11" s="37">
+        <f t="shared" si="7"/>
+        <v>0.175411603861406</v>
+      </c>
+      <c r="U11" s="36">
+        <f t="shared" ref="U11:U13" si="9">SQRT((4*P11)/(3.14*R11))</f>
+        <v>1.09039426827971</v>
+      </c>
+      <c r="V11" s="36">
+        <f t="shared" ref="V11:V13" si="10">SQRT((4*N11)/(3.14*R11))</f>
+        <v>0.412130294982622</v>
+      </c>
+    </row>
+    <row r="12" spans="2:22">
+      <c r="B12" s="30">
+        <v>48</v>
+      </c>
+      <c r="C12" s="30">
+        <v>400000</v>
+      </c>
+      <c r="D12" s="30" t="s">
+        <v>24</v>
+      </c>
+      <c r="E12" s="31">
+        <v>23.3</v>
+      </c>
+      <c r="F12" s="31">
+        <v>40.4</v>
+      </c>
+      <c r="G12" s="31">
+        <v>15.1</v>
+      </c>
+      <c r="H12" s="31">
+        <f t="shared" si="0"/>
+        <v>129.105</v>
+      </c>
+      <c r="I12" s="31">
+        <v>350</v>
+      </c>
+      <c r="J12" s="31">
+        <v>7</v>
+      </c>
+      <c r="K12" s="31"/>
+      <c r="L12" s="34">
+        <f>B12/J12</f>
+        <v>6.85714285714286</v>
+      </c>
+      <c r="M12" s="31">
+        <v>200</v>
+      </c>
+      <c r="N12" s="39">
         <v>0.5</v>
       </c>
-      <c r="O11" s="25">
-        <f t="shared" si="3"/>
-        <v>252</v>
-      </c>
-      <c r="P11" s="36">
+      <c r="O12" s="31">
+        <f t="shared" si="8"/>
+        <v>100</v>
+      </c>
+      <c r="P12" s="40">
         <f t="shared" si="4"/>
-        <v>3.5</v>
-      </c>
-      <c r="Q11" s="38">
+        <v>2.08333333333333</v>
+      </c>
+      <c r="Q12" s="43">
         <f t="shared" si="5"/>
-        <v>141.176470588235</v>
-      </c>
-      <c r="R11" s="36">
-        <v>2.5</v>
-      </c>
-      <c r="S11" s="35">
+        <v>29.1666666666667</v>
+      </c>
+      <c r="R12" s="40">
+        <v>1.5</v>
+      </c>
+      <c r="S12" s="39">
         <f t="shared" si="6"/>
-        <v>0.683130051063973</v>
-      </c>
-      <c r="T11" s="35">
+        <v>0.566138517072298</v>
+      </c>
+      <c r="T12" s="39">
         <f t="shared" si="7"/>
-        <v>0.258198889747161</v>
-      </c>
-    </row>
-    <row r="12" spans="10:10">
-      <c r="J12" s="32"/>
+        <v>0.277350098112615</v>
+      </c>
+      <c r="U12" s="44">
+        <f t="shared" si="9"/>
+        <v>1.33014480744604</v>
+      </c>
+      <c r="V12" s="44">
+        <f t="shared" si="10"/>
+        <v>0.651635212451075</v>
+      </c>
+    </row>
+    <row r="13" spans="2:22">
+      <c r="B13" s="30">
+        <v>48</v>
+      </c>
+      <c r="C13" s="30">
+        <v>100000</v>
+      </c>
+      <c r="D13" s="30" t="s">
+        <v>24</v>
+      </c>
+      <c r="E13" s="31">
+        <v>23.3</v>
+      </c>
+      <c r="F13" s="31">
+        <v>40.4</v>
+      </c>
+      <c r="G13" s="31">
+        <v>15.1</v>
+      </c>
+      <c r="H13" s="31">
+        <f t="shared" si="0"/>
+        <v>129.105</v>
+      </c>
+      <c r="I13" s="31">
+        <v>350</v>
+      </c>
+      <c r="J13" s="31">
+        <v>27</v>
+      </c>
+      <c r="K13" s="31"/>
+      <c r="L13" s="34">
+        <f t="shared" si="2"/>
+        <v>1.77777777777778</v>
+      </c>
+      <c r="M13" s="31">
+        <v>500</v>
+      </c>
+      <c r="N13" s="39">
+        <v>0.2</v>
+      </c>
+      <c r="O13" s="39">
+        <f t="shared" si="8"/>
+        <v>100</v>
+      </c>
+      <c r="P13" s="40">
+        <f t="shared" si="4"/>
+        <v>2.08333333333333</v>
+      </c>
+      <c r="Q13" s="43">
+        <f t="shared" si="5"/>
+        <v>281.25</v>
+      </c>
+      <c r="R13" s="40">
+        <v>1.5</v>
+      </c>
+      <c r="S13" s="39">
+        <f t="shared" si="6"/>
+        <v>0.566138517072298</v>
+      </c>
+      <c r="T13" s="39">
+        <f t="shared" si="7"/>
+        <v>0.175411603861406</v>
+      </c>
+      <c r="U13" s="44">
+        <f t="shared" si="9"/>
+        <v>1.33014480744604</v>
+      </c>
+      <c r="V13" s="44">
+        <f t="shared" si="10"/>
+        <v>0.412130294982622</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>